<commit_message>
Add spreadsheet formulas for CPM calculations
</commit_message>
<xml_diff>
--- a/AC Tasks.xlsx
+++ b/AC Tasks.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="149">
   <si>
     <t xml:space="preserve">Id</t>
   </si>
@@ -62,6 +62,24 @@
     <t xml:space="preserve">Date</t>
   </si>
   <si>
+    <t xml:space="preserve">Duration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slack</t>
+  </si>
+  <si>
     <t xml:space="preserve">T0</t>
   </si>
   <si>
@@ -435,6 +453,9 @@
   </si>
   <si>
     <t xml:space="preserve">all sections done</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project Finish</t>
   </si>
   <si>
     <t xml:space="preserve">All estimates in days</t>
@@ -661,7 +682,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M63"/>
+  <dimension ref="A1:S65"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.21"/>
@@ -715,84 +736,134 @@
       <c r="M1" s="0" t="s">
         <v>12</v>
       </c>
+      <c r="N1" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="0" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
+      </c>
+      <c r="N2" s="0" t="n">
+        <f aca="false">IF(H2&lt;&gt;"",H2,IF(AND(I2&lt;&gt;"",J2&lt;&gt;""),(I2+J2)/2,0))</f>
+        <v>0</v>
+      </c>
+      <c r="P2" s="0" t="n">
+        <f aca="false">O2+N2</f>
+        <v>0</v>
+      </c>
+      <c r="Q2" s="0" t="n">
+        <f aca="false">SUMPRODUCT(MIN(IF(($D$2:$D$63=$A2)+($E$2:$E$63=$A2)+($F$2:$F$63=$A2)+($G$2:$G$63=$A2)&gt;0,$R$2:$R$63,$N$65)))</f>
+        <v>0</v>
+      </c>
+      <c r="R2" s="0" t="n">
+        <f aca="false">Q2-N2</f>
+        <v>0</v>
+      </c>
+      <c r="S2" s="0" t="n">
+        <f aca="false">R2-O2</f>
+        <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="H3" s="0" t="n">
         <v>8</v>
       </c>
+      <c r="N3" s="0" t="n">
+        <f aca="false">IF(H3&lt;&gt;"",H3,IF(AND(I3&lt;&gt;"",J3&lt;&gt;""),(I3+J3)/2,0))</f>
+        <v>8</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="H4" s="0" t="n">
         <v>7</v>
       </c>
+      <c r="N4" s="0" t="n">
+        <f aca="false">IF(H4&lt;&gt;"",H4,IF(AND(I4&lt;&gt;"",J4&lt;&gt;""),(I4+J4)/2,0))</f>
+        <v>7</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="H5" s="0" t="n">
         <v>3</v>
       </c>
+      <c r="N5" s="0" t="n">
+        <f aca="false">IF(H5&lt;&gt;"",H5,IF(AND(I5&lt;&gt;"",J5&lt;&gt;""),(I5+J5)/2,0))</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I6" s="0" t="n">
         <v>5</v>
@@ -801,92 +872,112 @@
         <v>10</v>
       </c>
       <c r="K6" s="0" t="s">
-        <v>25</v>
+        <v>31</v>
+      </c>
+      <c r="N6" s="0" t="n">
+        <f aca="false">IF(H6&lt;&gt;"",H6,IF(AND(I6&lt;&gt;"",J6&lt;&gt;""),(I6+J6)/2,0))</f>
+        <v>7.5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="H7" s="0" t="n">
         <v>10</v>
       </c>
       <c r="L7" s="0" t="s">
-        <v>25</v>
+        <v>31</v>
+      </c>
+      <c r="N7" s="0" t="n">
+        <f aca="false">IF(H7&lt;&gt;"",H7,IF(AND(I7&lt;&gt;"",J7&lt;&gt;""),(I7+J7)/2,0))</f>
+        <v>10</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C8" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="0" t="s">
-        <v>23</v>
-      </c>
       <c r="H8" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="N8" s="0" t="n">
+        <f aca="false">IF(H8&lt;&gt;"",H8,IF(AND(I8&lt;&gt;"",J8&lt;&gt;""),(I8+J8)/2,0))</f>
         <v>5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="H9" s="0" t="n">
         <v>10</v>
       </c>
+      <c r="N9" s="0" t="n">
+        <f aca="false">IF(H9&lt;&gt;"",H9,IF(AND(I9&lt;&gt;"",J9&lt;&gt;""),(I9+J9)/2,0))</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
+      </c>
+      <c r="N10" s="0" t="n">
+        <f aca="false">IF(H10&lt;&gt;"",H10,IF(AND(I10&lt;&gt;"",J10&lt;&gt;""),(I10+J10)/2,0))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="I11" s="0" t="n">
         <v>21</v>
@@ -894,53 +985,65 @@
       <c r="J11" s="0" t="n">
         <v>23</v>
       </c>
+      <c r="N11" s="0" t="n">
+        <f aca="false">IF(H11&lt;&gt;"",H11,IF(AND(I11&lt;&gt;"",J11&lt;&gt;""),(I11+J11)/2,0))</f>
+        <v>22</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="H12" s="0" t="n">
         <v>10</v>
       </c>
+      <c r="N12" s="0" t="n">
+        <f aca="false">IF(H12&lt;&gt;"",H12,IF(AND(I12&lt;&gt;"",J12&lt;&gt;""),(I12+J12)/2,0))</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" s="0" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="0" t="s">
-        <v>33</v>
-      </c>
       <c r="C13" s="0" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="H13" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="N13" s="0" t="n">
+        <f aca="false">IF(H13&lt;&gt;"",H13,IF(AND(I13&lt;&gt;"",J13&lt;&gt;""),(I13+J13)/2,0))</f>
         <v>5</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" s="0" t="s">
         <v>41</v>
-      </c>
-      <c r="B14" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="C14" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" s="0" t="s">
-        <v>35</v>
       </c>
       <c r="I14" s="0" t="n">
         <v>15</v>
@@ -949,95 +1052,115 @@
         <v>21</v>
       </c>
       <c r="L14" s="0" t="s">
-        <v>25</v>
+        <v>31</v>
+      </c>
+      <c r="N14" s="0" t="n">
+        <f aca="false">IF(H14&lt;&gt;"",H14,IF(AND(I14&lt;&gt;"",J14&lt;&gt;""),(I14+J14)/2,0))</f>
+        <v>18</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="H15" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="N15" s="0" t="n">
+        <f aca="false">IF(H15&lt;&gt;"",H15,IF(AND(I15&lt;&gt;"",J15&lt;&gt;""),(I15+J15)/2,0))</f>
         <v>5</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="H16" s="0" t="n">
         <v>10</v>
       </c>
+      <c r="N16" s="0" t="n">
+        <f aca="false">IF(H16&lt;&gt;"",H16,IF(AND(I16&lt;&gt;"",J16&lt;&gt;""),(I16+J16)/2,0))</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="H17" s="0" t="n">
         <v>3</v>
       </c>
+      <c r="N17" s="0" t="n">
+        <f aca="false">IF(H17&lt;&gt;"",H17,IF(AND(I17&lt;&gt;"",J17&lt;&gt;""),(I17+J17)/2,0))</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="H18" s="0" t="n">
         <v>10</v>
       </c>
+      <c r="N18" s="0" t="n">
+        <f aca="false">IF(H18&lt;&gt;"",H18,IF(AND(I18&lt;&gt;"",J18&lt;&gt;""),(I18+J18)/2,0))</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B19" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="D19" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="E19" s="0" t="s">
         <v>51</v>
-      </c>
-      <c r="B19" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="C19" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="D19" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="E19" s="0" t="s">
-        <v>45</v>
       </c>
       <c r="I19" s="0" t="n">
         <v>5</v>
@@ -1045,252 +1168,308 @@
       <c r="J19" s="0" t="n">
         <v>8</v>
       </c>
+      <c r="N19" s="0" t="n">
+        <f aca="false">IF(H19&lt;&gt;"",H19,IF(AND(I19&lt;&gt;"",J19&lt;&gt;""),(I19+J19)/2,0))</f>
+        <v>6.5</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="D20" s="0" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="H20" s="0" t="n">
         <v>10</v>
       </c>
+      <c r="N20" s="0" t="n">
+        <f aca="false">IF(H20&lt;&gt;"",H20,IF(AND(I20&lt;&gt;"",J20&lt;&gt;""),(I20+J20)/2,0))</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C21" s="0" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="D21" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
+      </c>
+      <c r="N21" s="0" t="n">
+        <f aca="false">IF(H21&lt;&gt;"",H21,IF(AND(I21&lt;&gt;"",J21&lt;&gt;""),(I21+J21)/2,0))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="H22" s="0" t="n">
         <v>16</v>
       </c>
+      <c r="N22" s="0" t="n">
+        <f aca="false">IF(H22&lt;&gt;"",H22,IF(AND(I22&lt;&gt;"",J22&lt;&gt;""),(I22+J22)/2,0))</f>
+        <v>16</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="D23" s="0" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="H23" s="0" t="n">
         <v>2</v>
       </c>
+      <c r="N23" s="0" t="n">
+        <f aca="false">IF(H23&lt;&gt;"",H23,IF(AND(I23&lt;&gt;"",J23&lt;&gt;""),(I23+J23)/2,0))</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D24" s="0" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="H24" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="N24" s="0" t="n">
+        <f aca="false">IF(H24&lt;&gt;"",H24,IF(AND(I24&lt;&gt;"",J24&lt;&gt;""),(I24+J24)/2,0))</f>
         <v>5</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="D25" s="0" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="H25" s="0" t="n">
         <v>15</v>
       </c>
+      <c r="N25" s="0" t="n">
+        <f aca="false">IF(H25&lt;&gt;"",H25,IF(AND(I25&lt;&gt;"",J25&lt;&gt;""),(I25+J25)/2,0))</f>
+        <v>15</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D26" s="0" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H26" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="N26" s="0" t="n">
+        <f aca="false">IF(H26&lt;&gt;"",H26,IF(AND(I26&lt;&gt;"",J26&lt;&gt;""),(I26+J26)/2,0))</f>
         <v>5</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="H27" s="0" t="n">
         <v>25</v>
       </c>
+      <c r="N27" s="0" t="n">
+        <f aca="false">IF(H27&lt;&gt;"",H27,IF(AND(I27&lt;&gt;"",J27&lt;&gt;""),(I27+J27)/2,0))</f>
+        <v>25</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B28" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="C28" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="D28" s="0" t="s">
+        <v>76</v>
+      </c>
+      <c r="E28" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="F28" s="0" t="s">
         <v>69</v>
-      </c>
-      <c r="B28" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="C28" s="0" t="s">
-        <v>50</v>
-      </c>
-      <c r="D28" s="0" t="s">
-        <v>70</v>
-      </c>
-      <c r="E28" s="0" t="s">
-        <v>71</v>
-      </c>
-      <c r="F28" s="0" t="s">
-        <v>63</v>
       </c>
       <c r="H28" s="0" t="n">
         <v>20</v>
       </c>
+      <c r="N28" s="0" t="n">
+        <f aca="false">IF(H28&lt;&gt;"",H28,IF(AND(I28&lt;&gt;"",J28&lt;&gt;""),(I28+J28)/2,0))</f>
+        <v>20</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="H29" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="N29" s="0" t="n">
+        <f aca="false">IF(H29&lt;&gt;"",H29,IF(AND(I29&lt;&gt;"",J29&lt;&gt;""),(I29+J29)/2,0))</f>
         <v>5</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B30" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="C30" s="0" t="s">
+        <v>80</v>
+      </c>
+      <c r="D30" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="E30" s="0" t="s">
         <v>73</v>
-      </c>
-      <c r="B30" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="C30" s="0" t="s">
-        <v>74</v>
-      </c>
-      <c r="D30" s="0" t="s">
-        <v>58</v>
-      </c>
-      <c r="E30" s="0" t="s">
-        <v>67</v>
       </c>
       <c r="H30" s="0" t="n">
         <v>20</v>
       </c>
+      <c r="N30" s="0" t="n">
+        <f aca="false">IF(H30&lt;&gt;"",H30,IF(AND(I30&lt;&gt;"",J30&lt;&gt;""),(I30+J30)/2,0))</f>
+        <v>20</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C31" s="0" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="D31" s="0" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="H31" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="N31" s="0" t="n">
+        <f aca="false">IF(H31&lt;&gt;"",H31,IF(AND(I31&lt;&gt;"",J31&lt;&gt;""),(I31+J31)/2,0))</f>
         <v>5</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B32" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="C32" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="D32" s="0" t="s">
         <v>76</v>
       </c>
-      <c r="B32" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="C32" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="D32" s="0" t="s">
-        <v>70</v>
-      </c>
       <c r="H32" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="N32" s="0" t="n">
+        <f aca="false">IF(H32&lt;&gt;"",H32,IF(AND(I32&lt;&gt;"",J32&lt;&gt;""),(I32+J32)/2,0))</f>
         <v>5</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C33" s="0" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D33" s="0" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="I33" s="0" t="n">
         <v>5</v>
@@ -1298,124 +1477,152 @@
       <c r="J33" s="0" t="n">
         <v>8</v>
       </c>
+      <c r="N33" s="0" t="n">
+        <f aca="false">IF(H33&lt;&gt;"",H33,IF(AND(I33&lt;&gt;"",J33&lt;&gt;""),(I33+J33)/2,0))</f>
+        <v>6.5</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C34" s="0" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="D34" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
+      </c>
+      <c r="N34" s="0" t="n">
+        <f aca="false">IF(H34&lt;&gt;"",H34,IF(AND(I34&lt;&gt;"",J34&lt;&gt;""),(I34+J34)/2,0))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C35" s="0" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="D35" s="0" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="H35" s="0" t="n">
         <v>3</v>
       </c>
+      <c r="N35" s="0" t="n">
+        <f aca="false">IF(H35&lt;&gt;"",H35,IF(AND(I35&lt;&gt;"",J35&lt;&gt;""),(I35+J35)/2,0))</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C36" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="D36" s="0" t="s">
         <v>86</v>
-      </c>
-      <c r="D36" s="0" t="s">
-        <v>80</v>
       </c>
       <c r="H36" s="0" t="n">
         <v>10</v>
       </c>
+      <c r="N36" s="0" t="n">
+        <f aca="false">IF(H36&lt;&gt;"",H36,IF(AND(I36&lt;&gt;"",J36&lt;&gt;""),(I36+J36)/2,0))</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B37" s="0" t="s">
         <v>87</v>
       </c>
-      <c r="B37" s="0" t="s">
-        <v>81</v>
-      </c>
       <c r="C37" s="0" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="D37" s="0" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="H37" s="0" t="n">
         <v>15</v>
       </c>
+      <c r="N37" s="0" t="n">
+        <f aca="false">IF(H37&lt;&gt;"",H37,IF(AND(I37&lt;&gt;"",J37&lt;&gt;""),(I37+J37)/2,0))</f>
+        <v>15</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D38" s="0" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="H38" s="0" t="n">
         <v>15</v>
       </c>
+      <c r="N38" s="0" t="n">
+        <f aca="false">IF(H38&lt;&gt;"",H38,IF(AND(I38&lt;&gt;"",J38&lt;&gt;""),(I38+J38)/2,0))</f>
+        <v>15</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B39" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="C39" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="D39" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="E39" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="F39" s="0" t="s">
         <v>91</v>
       </c>
-      <c r="B39" s="0" t="s">
-        <v>81</v>
-      </c>
-      <c r="C39" s="0" t="s">
-        <v>50</v>
-      </c>
-      <c r="D39" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="E39" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="F39" s="0" t="s">
-        <v>85</v>
-      </c>
       <c r="H39" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="N39" s="0" t="n">
+        <f aca="false">IF(H39&lt;&gt;"",H39,IF(AND(I39&lt;&gt;"",J39&lt;&gt;""),(I39+J39)/2,0))</f>
         <v>5</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C40" s="0" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D40" s="0" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="I40" s="0" t="n">
         <v>5</v>
@@ -1423,36 +1630,44 @@
       <c r="J40" s="0" t="n">
         <v>8</v>
       </c>
+      <c r="N40" s="0" t="n">
+        <f aca="false">IF(H40&lt;&gt;"",H40,IF(AND(I40&lt;&gt;"",J40&lt;&gt;""),(I40+J40)/2,0))</f>
+        <v>6.5</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C41" s="0" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D41" s="0" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="H41" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="N41" s="0" t="n">
+        <f aca="false">IF(H41&lt;&gt;"",H41,IF(AND(I41&lt;&gt;"",J41&lt;&gt;""),(I41+J41)/2,0))</f>
         <v>5</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C42" s="0" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D42" s="0" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="I42" s="0" t="n">
         <v>20</v>
@@ -1461,166 +1676,202 @@
         <v>28</v>
       </c>
       <c r="L42" s="0" t="s">
-        <v>97</v>
+        <v>103</v>
+      </c>
+      <c r="N42" s="0" t="n">
+        <f aca="false">IF(H42&lt;&gt;"",H42,IF(AND(I42&lt;&gt;"",J42&lt;&gt;""),(I42+J42)/2,0))</f>
+        <v>24</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C43" s="0" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D43" s="0" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="H43" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="N43" s="0" t="n">
+        <f aca="false">IF(H43&lt;&gt;"",H43,IF(AND(I43&lt;&gt;"",J43&lt;&gt;""),(I43+J43)/2,0))</f>
         <v>5</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C44" s="0" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="D44" s="0" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="E44" s="0" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="H44" s="0" t="n">
         <v>9</v>
       </c>
+      <c r="N44" s="0" t="n">
+        <f aca="false">IF(H44&lt;&gt;"",H44,IF(AND(I44&lt;&gt;"",J44&lt;&gt;""),(I44+J44)/2,0))</f>
+        <v>9</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C45" s="0" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="D45" s="0" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="H45" s="0" t="n">
         <v>3</v>
       </c>
+      <c r="N45" s="0" t="n">
+        <f aca="false">IF(H45&lt;&gt;"",H45,IF(AND(I45&lt;&gt;"",J45&lt;&gt;""),(I45+J45)/2,0))</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C46" s="0" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="H46" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="N46" s="0" t="n">
+        <f aca="false">IF(H46&lt;&gt;"",H46,IF(AND(I46&lt;&gt;"",J46&lt;&gt;""),(I46+J46)/2,0))</f>
         <v>5</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B47" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="C47" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="D47" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="E47" s="0" t="s">
         <v>106</v>
-      </c>
-      <c r="B47" s="0" t="s">
-        <v>81</v>
-      </c>
-      <c r="C47" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="D47" s="0" t="s">
-        <v>104</v>
-      </c>
-      <c r="E47" s="0" t="s">
-        <v>100</v>
       </c>
       <c r="H47" s="0" t="n">
         <v>10</v>
       </c>
+      <c r="N47" s="0" t="n">
+        <f aca="false">IF(H47&lt;&gt;"",H47,IF(AND(I47&lt;&gt;"",J47&lt;&gt;""),(I47+J47)/2,0))</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B48" s="0" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C48" s="0" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="D48" s="0" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H48" s="0" t="n">
         <v>10</v>
       </c>
+      <c r="N48" s="0" t="n">
+        <f aca="false">IF(H48&lt;&gt;"",H48,IF(AND(I48&lt;&gt;"",J48&lt;&gt;""),(I48+J48)/2,0))</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B49" s="0" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C49" s="0" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="M49" s="2" t="n">
         <v>40080</v>
       </c>
+      <c r="N49" s="0" t="n">
+        <f aca="false">IF(H49&lt;&gt;"",H49,IF(AND(I49&lt;&gt;"",J49&lt;&gt;""),(I49+J49)/2,0))</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C50" s="0" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="D50" s="0" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="M50" s="2" t="n">
         <v>40161</v>
       </c>
+      <c r="N50" s="0" t="n">
+        <f aca="false">IF(H50&lt;&gt;"",H50,IF(AND(I50&lt;&gt;"",J50&lt;&gt;""),(I50+J50)/2,0))</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B51" s="0" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C51" s="0" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="D51" s="0" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="I51" s="0" t="n">
         <v>5</v>
@@ -1628,33 +1879,41 @@
       <c r="J51" s="0" t="n">
         <v>10</v>
       </c>
+      <c r="N51" s="0" t="n">
+        <f aca="false">IF(H51&lt;&gt;"",H51,IF(AND(I51&lt;&gt;"",J51&lt;&gt;""),(I51+J51)/2,0))</f>
+        <v>7.5</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B52" s="0" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C52" s="0" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="D52" s="0" t="s">
-        <v>16</v>
+        <v>22</v>
+      </c>
+      <c r="N52" s="0" t="n">
+        <f aca="false">IF(H52&lt;&gt;"",H52,IF(AND(I52&lt;&gt;"",J52&lt;&gt;""),(I52+J52)/2,0))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B53" s="0" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C53" s="0" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="D53" s="0" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="I53" s="0" t="n">
         <v>14</v>
@@ -1662,36 +1921,44 @@
       <c r="J53" s="0" t="n">
         <v>28</v>
       </c>
+      <c r="N53" s="0" t="n">
+        <f aca="false">IF(H53&lt;&gt;"",H53,IF(AND(I53&lt;&gt;"",J53&lt;&gt;""),(I53+J53)/2,0))</f>
+        <v>21</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B54" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="C54" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="D54" s="0" t="s">
         <v>119</v>
       </c>
-      <c r="B54" s="0" t="s">
-        <v>108</v>
-      </c>
-      <c r="C54" s="0" t="s">
-        <v>120</v>
-      </c>
-      <c r="D54" s="0" t="s">
-        <v>113</v>
-      </c>
       <c r="E54" s="0" t="s">
-        <v>117</v>
+        <v>123</v>
+      </c>
+      <c r="N54" s="0" t="n">
+        <f aca="false">IF(H54&lt;&gt;"",H54,IF(AND(I54&lt;&gt;"",J54&lt;&gt;""),(I54+J54)/2,0))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="B55" s="0" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C55" s="0" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="D55" s="0" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="I55" s="0" t="n">
         <v>0.5</v>
@@ -1699,150 +1966,191 @@
       <c r="J55" s="0" t="n">
         <v>1</v>
       </c>
+      <c r="N55" s="0" t="n">
+        <f aca="false">IF(H55&lt;&gt;"",H55,IF(AND(I55&lt;&gt;"",J55&lt;&gt;""),(I55+J55)/2,0))</f>
+        <v>0.75</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="B56" s="0" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C56" s="0" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>113</v>
+        <v>119</v>
+      </c>
+      <c r="N56" s="0" t="n">
+        <f aca="false">IF(H56&lt;&gt;"",H56,IF(AND(I56&lt;&gt;"",J56&lt;&gt;""),(I56+J56)/2,0))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="B57" s="0" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C57" s="0" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="D57" s="0" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="H57" s="0" t="n">
         <v>365</v>
       </c>
+      <c r="N57" s="0" t="n">
+        <f aca="false">IF(H57&lt;&gt;"",H57,IF(AND(I57&lt;&gt;"",J57&lt;&gt;""),(I57+J57)/2,0))</f>
+        <v>365</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B58" s="0" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C58" s="0" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="H58" s="0" t="n">
         <v>4</v>
       </c>
+      <c r="N58" s="0" t="n">
+        <f aca="false">IF(H58&lt;&gt;"",H58,IF(AND(I58&lt;&gt;"",J58&lt;&gt;""),(I58+J58)/2,0))</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B59" s="0" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C59" s="0" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="D59" s="0" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="F59" s="0" t="s">
-        <v>98</v>
+        <v>104</v>
+      </c>
+      <c r="N59" s="0" t="n">
+        <f aca="false">IF(H59&lt;&gt;"",H59,IF(AND(I59&lt;&gt;"",J59&lt;&gt;""),(I59+J59)/2,0))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B60" s="0" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C60" s="0" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="D60" s="0" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="F60" s="0" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="G60" s="0" t="s">
-        <v>65</v>
+        <v>71</v>
+      </c>
+      <c r="N60" s="0" t="n">
+        <f aca="false">IF(H60&lt;&gt;"",H60,IF(AND(I60&lt;&gt;"",J60&lt;&gt;""),(I60+J60)/2,0))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B61" s="0" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C61" s="0" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>30</v>
+        <v>36</v>
+      </c>
+      <c r="N61" s="0" t="n">
+        <f aca="false">IF(H61&lt;&gt;"",H61,IF(AND(I61&lt;&gt;"",J61&lt;&gt;""),(I61+J61)/2,0))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B62" s="0" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C62" s="0" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="E62" s="0" t="s">
-        <v>53</v>
+        <v>59</v>
+      </c>
+      <c r="N62" s="0" t="n">
+        <f aca="false">IF(H62&lt;&gt;"",H62,IF(AND(I62&lt;&gt;"",J62&lt;&gt;""),(I62+J62)/2,0))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B63" s="0" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C63" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="D63" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="E63" s="0" t="s">
         <v>137</v>
       </c>
-      <c r="D63" s="0" t="s">
+      <c r="F63" s="0" t="s">
         <v>135</v>
       </c>
-      <c r="E63" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F63" s="0" t="s">
-        <v>129</v>
-      </c>
       <c r="G63" s="0" t="s">
-        <v>133</v>
+        <v>139</v>
+      </c>
+      <c r="N63" s="0" t="n">
+        <f aca="false">IF(H63&lt;&gt;"",H63,IF(AND(I63&lt;&gt;"",J63&lt;&gt;""),(I63+J63)/2,0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M65" s="0" t="s">
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -1869,22 +2177,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="39.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="35.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="42.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="50.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="40.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Parse CPM calculations from CSV into Elm
</commit_message>
<xml_diff>
--- a/AC Tasks.xlsx
+++ b/AC Tasks.xlsx
@@ -772,21 +772,25 @@
         <f aca="false">IF(H2&lt;&gt;"",H2,IF(AND(I2&lt;&gt;"",J2&lt;&gt;""),(I2+J2)/2,0))</f>
         <v>0</v>
       </c>
+      <c r="O2" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D2,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E2,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F2,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G2,$A$2:$A$63,0)),0))</f>
+        <v>0</v>
+      </c>
       <c r="P2" s="0" t="n">
         <f aca="false">O2+N2</f>
         <v>0</v>
       </c>
       <c r="Q2" s="0" t="n">
-        <f aca="false">SUMPRODUCT(MIN(IF(($D$2:$D$63=$A2)+($E$2:$E$63=$A2)+($F$2:$F$63=$A2)+($G$2:$G$63=$A2)&gt;0,$R$2:$R$63,$N$65)))</f>
-        <v>0</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A2)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A2)),IF(COUNTIF($E$2:$E$63,$A2)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A2)),IF(COUNTIF($F$2:$F$63,$A2)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A2)),IF(COUNTIF($G$2:$G$63,$A2)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A2)))</f>
+        <v>19.5</v>
       </c>
       <c r="R2" s="0" t="n">
         <f aca="false">Q2-N2</f>
-        <v>0</v>
+        <v>19.5</v>
       </c>
       <c r="S2" s="0" t="n">
         <f aca="false">R2-O2</f>
-        <v>0</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -809,6 +813,26 @@
         <f aca="false">IF(H3&lt;&gt;"",H3,IF(AND(I3&lt;&gt;"",J3&lt;&gt;""),(I3+J3)/2,0))</f>
         <v>8</v>
       </c>
+      <c r="O3" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D3,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E3,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F3,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G3,$A$2:$A$63,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="P3" s="0" t="n">
+        <f aca="false">O3+N3</f>
+        <v>8</v>
+      </c>
+      <c r="Q3" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A3)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A3)),IF(COUNTIF($E$2:$E$63,$A3)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A3)),IF(COUNTIF($F$2:$F$63,$A3)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A3)),IF(COUNTIF($G$2:$G$63,$A3)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A3)))</f>
+        <v>27.5</v>
+      </c>
+      <c r="R3" s="0" t="n">
+        <f aca="false">Q3-N3</f>
+        <v>19.5</v>
+      </c>
+      <c r="S3" s="0" t="n">
+        <f aca="false">R3-O3</f>
+        <v>19.5</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
@@ -830,6 +854,26 @@
         <f aca="false">IF(H4&lt;&gt;"",H4,IF(AND(I4&lt;&gt;"",J4&lt;&gt;""),(I4+J4)/2,0))</f>
         <v>7</v>
       </c>
+      <c r="O4" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D4,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E4,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F4,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G4,$A$2:$A$63,0)),0))</f>
+        <v>8</v>
+      </c>
+      <c r="P4" s="0" t="n">
+        <f aca="false">O4+N4</f>
+        <v>15</v>
+      </c>
+      <c r="Q4" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A4)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A4)),IF(COUNTIF($E$2:$E$63,$A4)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A4)),IF(COUNTIF($F$2:$F$63,$A4)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A4)),IF(COUNTIF($G$2:$G$63,$A4)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A4)))</f>
+        <v>34.5</v>
+      </c>
+      <c r="R4" s="0" t="n">
+        <f aca="false">Q4-N4</f>
+        <v>27.5</v>
+      </c>
+      <c r="S4" s="0" t="n">
+        <f aca="false">R4-O4</f>
+        <v>19.5</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
@@ -851,6 +895,26 @@
         <f aca="false">IF(H5&lt;&gt;"",H5,IF(AND(I5&lt;&gt;"",J5&lt;&gt;""),(I5+J5)/2,0))</f>
         <v>3</v>
       </c>
+      <c r="O5" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D5,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E5,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F5,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G5,$A$2:$A$63,0)),0))</f>
+        <v>15</v>
+      </c>
+      <c r="P5" s="0" t="n">
+        <f aca="false">O5+N5</f>
+        <v>18</v>
+      </c>
+      <c r="Q5" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A5)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A5)),IF(COUNTIF($E$2:$E$63,$A5)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A5)),IF(COUNTIF($F$2:$F$63,$A5)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A5)),IF(COUNTIF($G$2:$G$63,$A5)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A5)))</f>
+        <v>37.5</v>
+      </c>
+      <c r="R5" s="0" t="n">
+        <f aca="false">Q5-N5</f>
+        <v>34.5</v>
+      </c>
+      <c r="S5" s="0" t="n">
+        <f aca="false">R5-O5</f>
+        <v>19.5</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
@@ -878,6 +942,26 @@
         <f aca="false">IF(H6&lt;&gt;"",H6,IF(AND(I6&lt;&gt;"",J6&lt;&gt;""),(I6+J6)/2,0))</f>
         <v>7.5</v>
       </c>
+      <c r="O6" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D6,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E6,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F6,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G6,$A$2:$A$63,0)),0))</f>
+        <v>18</v>
+      </c>
+      <c r="P6" s="0" t="n">
+        <f aca="false">O6+N6</f>
+        <v>25.5</v>
+      </c>
+      <c r="Q6" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A6)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A6)),IF(COUNTIF($E$2:$E$63,$A6)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A6)),IF(COUNTIF($F$2:$F$63,$A6)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A6)),IF(COUNTIF($G$2:$G$63,$A6)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A6)))</f>
+        <v>45</v>
+      </c>
+      <c r="R6" s="0" t="n">
+        <f aca="false">Q6-N6</f>
+        <v>37.5</v>
+      </c>
+      <c r="S6" s="0" t="n">
+        <f aca="false">R6-O6</f>
+        <v>19.5</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
@@ -902,6 +986,26 @@
         <f aca="false">IF(H7&lt;&gt;"",H7,IF(AND(I7&lt;&gt;"",J7&lt;&gt;""),(I7+J7)/2,0))</f>
         <v>10</v>
       </c>
+      <c r="O7" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D7,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E7,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F7,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G7,$A$2:$A$63,0)),0))</f>
+        <v>25.5</v>
+      </c>
+      <c r="P7" s="0" t="n">
+        <f aca="false">O7+N7</f>
+        <v>35.5</v>
+      </c>
+      <c r="Q7" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A7)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A7)),IF(COUNTIF($E$2:$E$63,$A7)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A7)),IF(COUNTIF($F$2:$F$63,$A7)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A7)),IF(COUNTIF($G$2:$G$63,$A7)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A7)))</f>
+        <v>55</v>
+      </c>
+      <c r="R7" s="0" t="n">
+        <f aca="false">Q7-N7</f>
+        <v>45</v>
+      </c>
+      <c r="S7" s="0" t="n">
+        <f aca="false">R7-O7</f>
+        <v>19.5</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
@@ -923,6 +1027,26 @@
         <f aca="false">IF(H8&lt;&gt;"",H8,IF(AND(I8&lt;&gt;"",J8&lt;&gt;""),(I8+J8)/2,0))</f>
         <v>5</v>
       </c>
+      <c r="O8" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D8,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E8,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F8,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G8,$A$2:$A$63,0)),0))</f>
+        <v>25.5</v>
+      </c>
+      <c r="P8" s="0" t="n">
+        <f aca="false">O8+N8</f>
+        <v>30.5</v>
+      </c>
+      <c r="Q8" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A8)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A8)),IF(COUNTIF($E$2:$E$63,$A8)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A8)),IF(COUNTIF($F$2:$F$63,$A8)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A8)),IF(COUNTIF($G$2:$G$63,$A8)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A8)))</f>
+        <v>55</v>
+      </c>
+      <c r="R8" s="0" t="n">
+        <f aca="false">Q8-N8</f>
+        <v>50</v>
+      </c>
+      <c r="S8" s="0" t="n">
+        <f aca="false">R8-O8</f>
+        <v>24.5</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
@@ -947,6 +1071,26 @@
         <f aca="false">IF(H9&lt;&gt;"",H9,IF(AND(I9&lt;&gt;"",J9&lt;&gt;""),(I9+J9)/2,0))</f>
         <v>10</v>
       </c>
+      <c r="O9" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D9,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E9,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F9,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G9,$A$2:$A$63,0)),0))</f>
+        <v>35.5</v>
+      </c>
+      <c r="P9" s="0" t="n">
+        <f aca="false">O9+N9</f>
+        <v>45.5</v>
+      </c>
+      <c r="Q9" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A9)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A9)),IF(COUNTIF($E$2:$E$63,$A9)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A9)),IF(COUNTIF($F$2:$F$63,$A9)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A9)),IF(COUNTIF($G$2:$G$63,$A9)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A9)))</f>
+        <v>65</v>
+      </c>
+      <c r="R9" s="0" t="n">
+        <f aca="false">Q9-N9</f>
+        <v>55</v>
+      </c>
+      <c r="S9" s="0" t="n">
+        <f aca="false">R9-O9</f>
+        <v>19.5</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
@@ -965,6 +1109,26 @@
         <f aca="false">IF(H10&lt;&gt;"",H10,IF(AND(I10&lt;&gt;"",J10&lt;&gt;""),(I10+J10)/2,0))</f>
         <v>0</v>
       </c>
+      <c r="O10" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D10,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E10,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F10,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G10,$A$2:$A$63,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="P10" s="0" t="n">
+        <f aca="false">O10+N10</f>
+        <v>0</v>
+      </c>
+      <c r="Q10" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A10)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A10)),IF(COUNTIF($E$2:$E$63,$A10)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A10)),IF(COUNTIF($F$2:$F$63,$A10)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A10)),IF(COUNTIF($G$2:$G$63,$A10)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A10)))</f>
+        <v>0</v>
+      </c>
+      <c r="R10" s="0" t="n">
+        <f aca="false">Q10-N10</f>
+        <v>0</v>
+      </c>
+      <c r="S10" s="0" t="n">
+        <f aca="false">R10-O10</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
@@ -989,6 +1153,26 @@
         <f aca="false">IF(H11&lt;&gt;"",H11,IF(AND(I11&lt;&gt;"",J11&lt;&gt;""),(I11+J11)/2,0))</f>
         <v>22</v>
       </c>
+      <c r="O11" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D11,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E11,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F11,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G11,$A$2:$A$63,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="P11" s="0" t="n">
+        <f aca="false">O11+N11</f>
+        <v>22</v>
+      </c>
+      <c r="Q11" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A11)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A11)),IF(COUNTIF($E$2:$E$63,$A11)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A11)),IF(COUNTIF($F$2:$F$63,$A11)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A11)),IF(COUNTIF($G$2:$G$63,$A11)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A11)))</f>
+        <v>22</v>
+      </c>
+      <c r="R11" s="0" t="n">
+        <f aca="false">Q11-N11</f>
+        <v>0</v>
+      </c>
+      <c r="S11" s="0" t="n">
+        <f aca="false">R11-O11</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
@@ -1010,6 +1194,26 @@
         <f aca="false">IF(H12&lt;&gt;"",H12,IF(AND(I12&lt;&gt;"",J12&lt;&gt;""),(I12+J12)/2,0))</f>
         <v>10</v>
       </c>
+      <c r="O12" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D12,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E12,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F12,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G12,$A$2:$A$63,0)),0))</f>
+        <v>22</v>
+      </c>
+      <c r="P12" s="0" t="n">
+        <f aca="false">O12+N12</f>
+        <v>32</v>
+      </c>
+      <c r="Q12" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A12)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A12)),IF(COUNTIF($E$2:$E$63,$A12)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A12)),IF(COUNTIF($F$2:$F$63,$A12)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A12)),IF(COUNTIF($G$2:$G$63,$A12)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A12)))</f>
+        <v>42</v>
+      </c>
+      <c r="R12" s="0" t="n">
+        <f aca="false">Q12-N12</f>
+        <v>32</v>
+      </c>
+      <c r="S12" s="0" t="n">
+        <f aca="false">R12-O12</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
@@ -1031,6 +1235,26 @@
         <f aca="false">IF(H13&lt;&gt;"",H13,IF(AND(I13&lt;&gt;"",J13&lt;&gt;""),(I13+J13)/2,0))</f>
         <v>5</v>
       </c>
+      <c r="O13" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D13,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E13,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F13,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G13,$A$2:$A$63,0)),0))</f>
+        <v>22</v>
+      </c>
+      <c r="P13" s="0" t="n">
+        <f aca="false">O13+N13</f>
+        <v>27</v>
+      </c>
+      <c r="Q13" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A13)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A13)),IF(COUNTIF($E$2:$E$63,$A13)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A13)),IF(COUNTIF($F$2:$F$63,$A13)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A13)),IF(COUNTIF($G$2:$G$63,$A13)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A13)))</f>
+        <v>42</v>
+      </c>
+      <c r="R13" s="0" t="n">
+        <f aca="false">Q13-N13</f>
+        <v>37</v>
+      </c>
+      <c r="S13" s="0" t="n">
+        <f aca="false">R13-O13</f>
+        <v>15</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
@@ -1058,6 +1282,26 @@
         <f aca="false">IF(H14&lt;&gt;"",H14,IF(AND(I14&lt;&gt;"",J14&lt;&gt;""),(I14+J14)/2,0))</f>
         <v>18</v>
       </c>
+      <c r="O14" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D14,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E14,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F14,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G14,$A$2:$A$63,0)),0))</f>
+        <v>22</v>
+      </c>
+      <c r="P14" s="0" t="n">
+        <f aca="false">O14+N14</f>
+        <v>40</v>
+      </c>
+      <c r="Q14" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A14)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A14)),IF(COUNTIF($E$2:$E$63,$A14)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A14)),IF(COUNTIF($F$2:$F$63,$A14)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A14)),IF(COUNTIF($G$2:$G$63,$A14)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A14)))</f>
+        <v>40</v>
+      </c>
+      <c r="R14" s="0" t="n">
+        <f aca="false">Q14-N14</f>
+        <v>22</v>
+      </c>
+      <c r="S14" s="0" t="n">
+        <f aca="false">R14-O14</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
@@ -1079,6 +1323,26 @@
         <f aca="false">IF(H15&lt;&gt;"",H15,IF(AND(I15&lt;&gt;"",J15&lt;&gt;""),(I15+J15)/2,0))</f>
         <v>5</v>
       </c>
+      <c r="O15" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D15,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E15,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F15,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G15,$A$2:$A$63,0)),0))</f>
+        <v>40</v>
+      </c>
+      <c r="P15" s="0" t="n">
+        <f aca="false">O15+N15</f>
+        <v>45</v>
+      </c>
+      <c r="Q15" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A15)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A15)),IF(COUNTIF($E$2:$E$63,$A15)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A15)),IF(COUNTIF($F$2:$F$63,$A15)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A15)),IF(COUNTIF($G$2:$G$63,$A15)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A15)))</f>
+        <v>45</v>
+      </c>
+      <c r="R15" s="0" t="n">
+        <f aca="false">Q15-N15</f>
+        <v>40</v>
+      </c>
+      <c r="S15" s="0" t="n">
+        <f aca="false">R15-O15</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
@@ -1100,6 +1364,26 @@
         <f aca="false">IF(H16&lt;&gt;"",H16,IF(AND(I16&lt;&gt;"",J16&lt;&gt;""),(I16+J16)/2,0))</f>
         <v>10</v>
       </c>
+      <c r="O16" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D16,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E16,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F16,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G16,$A$2:$A$63,0)),0))</f>
+        <v>45</v>
+      </c>
+      <c r="P16" s="0" t="n">
+        <f aca="false">O16+N16</f>
+        <v>55</v>
+      </c>
+      <c r="Q16" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A16)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A16)),IF(COUNTIF($E$2:$E$63,$A16)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A16)),IF(COUNTIF($F$2:$F$63,$A16)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A16)),IF(COUNTIF($G$2:$G$63,$A16)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A16)))</f>
+        <v>55</v>
+      </c>
+      <c r="R16" s="0" t="n">
+        <f aca="false">Q16-N16</f>
+        <v>45</v>
+      </c>
+      <c r="S16" s="0" t="n">
+        <f aca="false">R16-O16</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
@@ -1124,6 +1408,26 @@
         <f aca="false">IF(H17&lt;&gt;"",H17,IF(AND(I17&lt;&gt;"",J17&lt;&gt;""),(I17+J17)/2,0))</f>
         <v>3</v>
       </c>
+      <c r="O17" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D17,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E17,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F17,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G17,$A$2:$A$63,0)),0))</f>
+        <v>32</v>
+      </c>
+      <c r="P17" s="0" t="n">
+        <f aca="false">O17+N17</f>
+        <v>35</v>
+      </c>
+      <c r="Q17" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A17)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A17)),IF(COUNTIF($E$2:$E$63,$A17)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A17)),IF(COUNTIF($F$2:$F$63,$A17)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A17)),IF(COUNTIF($G$2:$G$63,$A17)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A17)))</f>
+        <v>45</v>
+      </c>
+      <c r="R17" s="0" t="n">
+        <f aca="false">Q17-N17</f>
+        <v>42</v>
+      </c>
+      <c r="S17" s="0" t="n">
+        <f aca="false">R17-O17</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
@@ -1145,6 +1449,26 @@
         <f aca="false">IF(H18&lt;&gt;"",H18,IF(AND(I18&lt;&gt;"",J18&lt;&gt;""),(I18+J18)/2,0))</f>
         <v>10</v>
       </c>
+      <c r="O18" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D18,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E18,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F18,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G18,$A$2:$A$63,0)),0))</f>
+        <v>35</v>
+      </c>
+      <c r="P18" s="0" t="n">
+        <f aca="false">O18+N18</f>
+        <v>45</v>
+      </c>
+      <c r="Q18" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A18)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A18)),IF(COUNTIF($E$2:$E$63,$A18)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A18)),IF(COUNTIF($F$2:$F$63,$A18)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A18)),IF(COUNTIF($G$2:$G$63,$A18)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A18)))</f>
+        <v>55</v>
+      </c>
+      <c r="R18" s="0" t="n">
+        <f aca="false">Q18-N18</f>
+        <v>45</v>
+      </c>
+      <c r="S18" s="0" t="n">
+        <f aca="false">R18-O18</f>
+        <v>10</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
@@ -1172,6 +1496,26 @@
         <f aca="false">IF(H19&lt;&gt;"",H19,IF(AND(I19&lt;&gt;"",J19&lt;&gt;""),(I19+J19)/2,0))</f>
         <v>6.5</v>
       </c>
+      <c r="O19" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D19,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E19,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F19,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G19,$A$2:$A$63,0)),0))</f>
+        <v>55</v>
+      </c>
+      <c r="P19" s="0" t="n">
+        <f aca="false">O19+N19</f>
+        <v>61.5</v>
+      </c>
+      <c r="Q19" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A19)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A19)),IF(COUNTIF($E$2:$E$63,$A19)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A19)),IF(COUNTIF($F$2:$F$63,$A19)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A19)),IF(COUNTIF($G$2:$G$63,$A19)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A19)))</f>
+        <v>65</v>
+      </c>
+      <c r="R19" s="0" t="n">
+        <f aca="false">Q19-N19</f>
+        <v>58.5</v>
+      </c>
+      <c r="S19" s="0" t="n">
+        <f aca="false">R19-O19</f>
+        <v>3.5</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
@@ -1196,6 +1540,26 @@
         <f aca="false">IF(H20&lt;&gt;"",H20,IF(AND(I20&lt;&gt;"",J20&lt;&gt;""),(I20+J20)/2,0))</f>
         <v>10</v>
       </c>
+      <c r="O20" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D20,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E20,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F20,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G20,$A$2:$A$63,0)),0))</f>
+        <v>55</v>
+      </c>
+      <c r="P20" s="0" t="n">
+        <f aca="false">O20+N20</f>
+        <v>65</v>
+      </c>
+      <c r="Q20" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A20)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A20)),IF(COUNTIF($E$2:$E$63,$A20)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A20)),IF(COUNTIF($F$2:$F$63,$A20)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A20)),IF(COUNTIF($G$2:$G$63,$A20)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A20)))</f>
+        <v>65</v>
+      </c>
+      <c r="R20" s="0" t="n">
+        <f aca="false">Q20-N20</f>
+        <v>55</v>
+      </c>
+      <c r="S20" s="0" t="n">
+        <f aca="false">R20-O20</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
@@ -1214,6 +1578,26 @@
         <f aca="false">IF(H21&lt;&gt;"",H21,IF(AND(I21&lt;&gt;"",J21&lt;&gt;""),(I21+J21)/2,0))</f>
         <v>0</v>
       </c>
+      <c r="O21" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D21,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E21,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F21,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G21,$A$2:$A$63,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="P21" s="0" t="n">
+        <f aca="false">O21+N21</f>
+        <v>0</v>
+      </c>
+      <c r="Q21" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A21)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A21)),IF(COUNTIF($E$2:$E$63,$A21)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A21)),IF(COUNTIF($F$2:$F$63,$A21)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A21)),IF(COUNTIF($G$2:$G$63,$A21)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A21)))</f>
+        <v>3</v>
+      </c>
+      <c r="R21" s="0" t="n">
+        <f aca="false">Q21-N21</f>
+        <v>3</v>
+      </c>
+      <c r="S21" s="0" t="n">
+        <f aca="false">R21-O21</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
@@ -1235,6 +1619,26 @@
         <f aca="false">IF(H22&lt;&gt;"",H22,IF(AND(I22&lt;&gt;"",J22&lt;&gt;""),(I22+J22)/2,0))</f>
         <v>16</v>
       </c>
+      <c r="O22" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D22,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E22,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F22,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G22,$A$2:$A$63,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="P22" s="0" t="n">
+        <f aca="false">O22+N22</f>
+        <v>16</v>
+      </c>
+      <c r="Q22" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A22)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A22)),IF(COUNTIF($E$2:$E$63,$A22)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A22)),IF(COUNTIF($F$2:$F$63,$A22)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A22)),IF(COUNTIF($G$2:$G$63,$A22)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A22)))</f>
+        <v>45</v>
+      </c>
+      <c r="R22" s="0" t="n">
+        <f aca="false">Q22-N22</f>
+        <v>29</v>
+      </c>
+      <c r="S22" s="0" t="n">
+        <f aca="false">R22-O22</f>
+        <v>29</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
@@ -1256,6 +1660,26 @@
         <f aca="false">IF(H23&lt;&gt;"",H23,IF(AND(I23&lt;&gt;"",J23&lt;&gt;""),(I23+J23)/2,0))</f>
         <v>2</v>
       </c>
+      <c r="O23" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D23,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E23,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F23,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G23,$A$2:$A$63,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="P23" s="0" t="n">
+        <f aca="false">O23+N23</f>
+        <v>2</v>
+      </c>
+      <c r="Q23" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A23)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A23)),IF(COUNTIF($E$2:$E$63,$A23)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A23)),IF(COUNTIF($F$2:$F$63,$A23)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A23)),IF(COUNTIF($G$2:$G$63,$A23)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A23)))</f>
+        <v>5</v>
+      </c>
+      <c r="R23" s="0" t="n">
+        <f aca="false">Q23-N23</f>
+        <v>3</v>
+      </c>
+      <c r="S23" s="0" t="n">
+        <f aca="false">R23-O23</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
@@ -1277,6 +1701,26 @@
         <f aca="false">IF(H24&lt;&gt;"",H24,IF(AND(I24&lt;&gt;"",J24&lt;&gt;""),(I24+J24)/2,0))</f>
         <v>5</v>
       </c>
+      <c r="O24" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D24,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E24,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F24,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G24,$A$2:$A$63,0)),0))</f>
+        <v>2</v>
+      </c>
+      <c r="P24" s="0" t="n">
+        <f aca="false">O24+N24</f>
+        <v>7</v>
+      </c>
+      <c r="Q24" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A24)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A24)),IF(COUNTIF($E$2:$E$63,$A24)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A24)),IF(COUNTIF($F$2:$F$63,$A24)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A24)),IF(COUNTIF($G$2:$G$63,$A24)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A24)))</f>
+        <v>60</v>
+      </c>
+      <c r="R24" s="0" t="n">
+        <f aca="false">Q24-N24</f>
+        <v>55</v>
+      </c>
+      <c r="S24" s="0" t="n">
+        <f aca="false">R24-O24</f>
+        <v>53</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
@@ -1298,6 +1742,26 @@
         <f aca="false">IF(H25&lt;&gt;"",H25,IF(AND(I25&lt;&gt;"",J25&lt;&gt;""),(I25+J25)/2,0))</f>
         <v>15</v>
       </c>
+      <c r="O25" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D25,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E25,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F25,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G25,$A$2:$A$63,0)),0))</f>
+        <v>2</v>
+      </c>
+      <c r="P25" s="0" t="n">
+        <f aca="false">O25+N25</f>
+        <v>17</v>
+      </c>
+      <c r="Q25" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A25)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A25)),IF(COUNTIF($E$2:$E$63,$A25)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A25)),IF(COUNTIF($F$2:$F$63,$A25)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A25)),IF(COUNTIF($G$2:$G$63,$A25)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A25)))</f>
+        <v>20</v>
+      </c>
+      <c r="R25" s="0" t="n">
+        <f aca="false">Q25-N25</f>
+        <v>5</v>
+      </c>
+      <c r="S25" s="0" t="n">
+        <f aca="false">R25-O25</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
@@ -1319,6 +1783,26 @@
         <f aca="false">IF(H26&lt;&gt;"",H26,IF(AND(I26&lt;&gt;"",J26&lt;&gt;""),(I26+J26)/2,0))</f>
         <v>5</v>
       </c>
+      <c r="O26" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D26,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E26,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F26,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G26,$A$2:$A$63,0)),0))</f>
+        <v>7</v>
+      </c>
+      <c r="P26" s="0" t="n">
+        <f aca="false">O26+N26</f>
+        <v>12</v>
+      </c>
+      <c r="Q26" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A26)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A26)),IF(COUNTIF($E$2:$E$63,$A26)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A26)),IF(COUNTIF($F$2:$F$63,$A26)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A26)),IF(COUNTIF($G$2:$G$63,$A26)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A26)))</f>
+        <v>65</v>
+      </c>
+      <c r="R26" s="0" t="n">
+        <f aca="false">Q26-N26</f>
+        <v>60</v>
+      </c>
+      <c r="S26" s="0" t="n">
+        <f aca="false">R26-O26</f>
+        <v>53</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
@@ -1340,6 +1824,26 @@
         <f aca="false">IF(H27&lt;&gt;"",H27,IF(AND(I27&lt;&gt;"",J27&lt;&gt;""),(I27+J27)/2,0))</f>
         <v>25</v>
       </c>
+      <c r="O27" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D27,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E27,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F27,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G27,$A$2:$A$63,0)),0))</f>
+        <v>17</v>
+      </c>
+      <c r="P27" s="0" t="n">
+        <f aca="false">O27+N27</f>
+        <v>42</v>
+      </c>
+      <c r="Q27" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A27)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A27)),IF(COUNTIF($E$2:$E$63,$A27)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A27)),IF(COUNTIF($F$2:$F$63,$A27)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A27)),IF(COUNTIF($G$2:$G$63,$A27)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A27)))</f>
+        <v>45</v>
+      </c>
+      <c r="R27" s="0" t="n">
+        <f aca="false">Q27-N27</f>
+        <v>20</v>
+      </c>
+      <c r="S27" s="0" t="n">
+        <f aca="false">R27-O27</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
@@ -1367,6 +1871,26 @@
         <f aca="false">IF(H28&lt;&gt;"",H28,IF(AND(I28&lt;&gt;"",J28&lt;&gt;""),(I28+J28)/2,0))</f>
         <v>20</v>
       </c>
+      <c r="O28" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D28,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E28,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F28,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G28,$A$2:$A$63,0)),0))</f>
+        <v>17</v>
+      </c>
+      <c r="P28" s="0" t="n">
+        <f aca="false">O28+N28</f>
+        <v>37</v>
+      </c>
+      <c r="Q28" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A28)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A28)),IF(COUNTIF($E$2:$E$63,$A28)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A28)),IF(COUNTIF($F$2:$F$63,$A28)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A28)),IF(COUNTIF($G$2:$G$63,$A28)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A28)))</f>
+        <v>58.5</v>
+      </c>
+      <c r="R28" s="0" t="n">
+        <f aca="false">Q28-N28</f>
+        <v>38.5</v>
+      </c>
+      <c r="S28" s="0" t="n">
+        <f aca="false">R28-O28</f>
+        <v>21.5</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
@@ -1388,6 +1912,26 @@
         <f aca="false">IF(H29&lt;&gt;"",H29,IF(AND(I29&lt;&gt;"",J29&lt;&gt;""),(I29+J29)/2,0))</f>
         <v>5</v>
       </c>
+      <c r="O29" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D29,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E29,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F29,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G29,$A$2:$A$63,0)),0))</f>
+        <v>7</v>
+      </c>
+      <c r="P29" s="0" t="n">
+        <f aca="false">O29+N29</f>
+        <v>12</v>
+      </c>
+      <c r="Q29" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A29)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A29)),IF(COUNTIF($E$2:$E$63,$A29)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A29)),IF(COUNTIF($F$2:$F$63,$A29)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A29)),IF(COUNTIF($G$2:$G$63,$A29)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A29)))</f>
+        <v>38.5</v>
+      </c>
+      <c r="R29" s="0" t="n">
+        <f aca="false">Q29-N29</f>
+        <v>33.5</v>
+      </c>
+      <c r="S29" s="0" t="n">
+        <f aca="false">R29-O29</f>
+        <v>26.5</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
@@ -1412,6 +1956,26 @@
         <f aca="false">IF(H30&lt;&gt;"",H30,IF(AND(I30&lt;&gt;"",J30&lt;&gt;""),(I30+J30)/2,0))</f>
         <v>20</v>
       </c>
+      <c r="O30" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D30,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E30,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F30,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G30,$A$2:$A$63,0)),0))</f>
+        <v>42</v>
+      </c>
+      <c r="P30" s="0" t="n">
+        <f aca="false">O30+N30</f>
+        <v>62</v>
+      </c>
+      <c r="Q30" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A30)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A30)),IF(COUNTIF($E$2:$E$63,$A30)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A30)),IF(COUNTIF($F$2:$F$63,$A30)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A30)),IF(COUNTIF($G$2:$G$63,$A30)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A30)))</f>
+        <v>65</v>
+      </c>
+      <c r="R30" s="0" t="n">
+        <f aca="false">Q30-N30</f>
+        <v>45</v>
+      </c>
+      <c r="S30" s="0" t="n">
+        <f aca="false">R30-O30</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
@@ -1433,6 +1997,26 @@
         <f aca="false">IF(H31&lt;&gt;"",H31,IF(AND(I31&lt;&gt;"",J31&lt;&gt;""),(I31+J31)/2,0))</f>
         <v>5</v>
       </c>
+      <c r="O31" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D31,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E31,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F31,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G31,$A$2:$A$63,0)),0))</f>
+        <v>2</v>
+      </c>
+      <c r="P31" s="0" t="n">
+        <f aca="false">O31+N31</f>
+        <v>7</v>
+      </c>
+      <c r="Q31" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A31)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A31)),IF(COUNTIF($E$2:$E$63,$A31)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A31)),IF(COUNTIF($F$2:$F$63,$A31)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A31)),IF(COUNTIF($G$2:$G$63,$A31)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A31)))</f>
+        <v>33.5</v>
+      </c>
+      <c r="R31" s="0" t="n">
+        <f aca="false">Q31-N31</f>
+        <v>28.5</v>
+      </c>
+      <c r="S31" s="0" t="n">
+        <f aca="false">R31-O31</f>
+        <v>26.5</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
@@ -1454,6 +2038,26 @@
         <f aca="false">IF(H32&lt;&gt;"",H32,IF(AND(I32&lt;&gt;"",J32&lt;&gt;""),(I32+J32)/2,0))</f>
         <v>5</v>
       </c>
+      <c r="O32" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D32,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E32,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F32,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G32,$A$2:$A$63,0)),0))</f>
+        <v>7</v>
+      </c>
+      <c r="P32" s="0" t="n">
+        <f aca="false">O32+N32</f>
+        <v>12</v>
+      </c>
+      <c r="Q32" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A32)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A32)),IF(COUNTIF($E$2:$E$63,$A32)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A32)),IF(COUNTIF($F$2:$F$63,$A32)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A32)),IF(COUNTIF($G$2:$G$63,$A32)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A32)))</f>
+        <v>65</v>
+      </c>
+      <c r="R32" s="0" t="n">
+        <f aca="false">Q32-N32</f>
+        <v>60</v>
+      </c>
+      <c r="S32" s="0" t="n">
+        <f aca="false">R32-O32</f>
+        <v>53</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
@@ -1481,6 +2085,26 @@
         <f aca="false">IF(H33&lt;&gt;"",H33,IF(AND(I33&lt;&gt;"",J33&lt;&gt;""),(I33+J33)/2,0))</f>
         <v>6.5</v>
       </c>
+      <c r="O33" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D33,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E33,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F33,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G33,$A$2:$A$63,0)),0))</f>
+        <v>42</v>
+      </c>
+      <c r="P33" s="0" t="n">
+        <f aca="false">O33+N33</f>
+        <v>48.5</v>
+      </c>
+      <c r="Q33" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A33)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A33)),IF(COUNTIF($E$2:$E$63,$A33)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A33)),IF(COUNTIF($F$2:$F$63,$A33)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A33)),IF(COUNTIF($G$2:$G$63,$A33)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A33)))</f>
+        <v>65</v>
+      </c>
+      <c r="R33" s="0" t="n">
+        <f aca="false">Q33-N33</f>
+        <v>58.5</v>
+      </c>
+      <c r="S33" s="0" t="n">
+        <f aca="false">R33-O33</f>
+        <v>16.5</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
@@ -1499,6 +2123,26 @@
         <f aca="false">IF(H34&lt;&gt;"",H34,IF(AND(I34&lt;&gt;"",J34&lt;&gt;""),(I34+J34)/2,0))</f>
         <v>0</v>
       </c>
+      <c r="O34" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D34,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E34,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F34,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G34,$A$2:$A$63,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="P34" s="0" t="n">
+        <f aca="false">O34+N34</f>
+        <v>0</v>
+      </c>
+      <c r="Q34" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A34)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A34)),IF(COUNTIF($E$2:$E$63,$A34)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A34)),IF(COUNTIF($F$2:$F$63,$A34)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A34)),IF(COUNTIF($G$2:$G$63,$A34)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A34)))</f>
+        <v>26.5</v>
+      </c>
+      <c r="R34" s="0" t="n">
+        <f aca="false">Q34-N34</f>
+        <v>26.5</v>
+      </c>
+      <c r="S34" s="0" t="n">
+        <f aca="false">R34-O34</f>
+        <v>26.5</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
@@ -1520,6 +2164,26 @@
         <f aca="false">IF(H35&lt;&gt;"",H35,IF(AND(I35&lt;&gt;"",J35&lt;&gt;""),(I35+J35)/2,0))</f>
         <v>3</v>
       </c>
+      <c r="O35" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D35,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E35,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F35,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G35,$A$2:$A$63,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="P35" s="0" t="n">
+        <f aca="false">O35+N35</f>
+        <v>3</v>
+      </c>
+      <c r="Q35" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A35)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A35)),IF(COUNTIF($E$2:$E$63,$A35)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A35)),IF(COUNTIF($F$2:$F$63,$A35)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A35)),IF(COUNTIF($G$2:$G$63,$A35)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A35)))</f>
+        <v>29.5</v>
+      </c>
+      <c r="R35" s="0" t="n">
+        <f aca="false">Q35-N35</f>
+        <v>26.5</v>
+      </c>
+      <c r="S35" s="0" t="n">
+        <f aca="false">R35-O35</f>
+        <v>26.5</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
@@ -1541,6 +2205,26 @@
         <f aca="false">IF(H36&lt;&gt;"",H36,IF(AND(I36&lt;&gt;"",J36&lt;&gt;""),(I36+J36)/2,0))</f>
         <v>10</v>
       </c>
+      <c r="O36" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D36,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E36,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F36,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G36,$A$2:$A$63,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="P36" s="0" t="n">
+        <f aca="false">O36+N36</f>
+        <v>10</v>
+      </c>
+      <c r="Q36" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A36)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A36)),IF(COUNTIF($E$2:$E$63,$A36)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A36)),IF(COUNTIF($F$2:$F$63,$A36)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A36)),IF(COUNTIF($G$2:$G$63,$A36)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A36)))</f>
+        <v>45</v>
+      </c>
+      <c r="R36" s="0" t="n">
+        <f aca="false">Q36-N36</f>
+        <v>35</v>
+      </c>
+      <c r="S36" s="0" t="n">
+        <f aca="false">R36-O36</f>
+        <v>35</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
@@ -1562,6 +2246,26 @@
         <f aca="false">IF(H37&lt;&gt;"",H37,IF(AND(I37&lt;&gt;"",J37&lt;&gt;""),(I37+J37)/2,0))</f>
         <v>15</v>
       </c>
+      <c r="O37" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D37,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E37,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F37,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G37,$A$2:$A$63,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="P37" s="0" t="n">
+        <f aca="false">O37+N37</f>
+        <v>15</v>
+      </c>
+      <c r="Q37" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A37)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A37)),IF(COUNTIF($E$2:$E$63,$A37)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A37)),IF(COUNTIF($F$2:$F$63,$A37)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A37)),IF(COUNTIF($G$2:$G$63,$A37)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A37)))</f>
+        <v>45</v>
+      </c>
+      <c r="R37" s="0" t="n">
+        <f aca="false">Q37-N37</f>
+        <v>30</v>
+      </c>
+      <c r="S37" s="0" t="n">
+        <f aca="false">R37-O37</f>
+        <v>30</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
@@ -1583,6 +2287,26 @@
         <f aca="false">IF(H38&lt;&gt;"",H38,IF(AND(I38&lt;&gt;"",J38&lt;&gt;""),(I38+J38)/2,0))</f>
         <v>15</v>
       </c>
+      <c r="O38" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D38,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E38,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F38,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G38,$A$2:$A$63,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="P38" s="0" t="n">
+        <f aca="false">O38+N38</f>
+        <v>15</v>
+      </c>
+      <c r="Q38" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A38)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A38)),IF(COUNTIF($E$2:$E$63,$A38)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A38)),IF(COUNTIF($F$2:$F$63,$A38)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A38)),IF(COUNTIF($G$2:$G$63,$A38)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A38)))</f>
+        <v>45</v>
+      </c>
+      <c r="R38" s="0" t="n">
+        <f aca="false">Q38-N38</f>
+        <v>30</v>
+      </c>
+      <c r="S38" s="0" t="n">
+        <f aca="false">R38-O38</f>
+        <v>30</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
@@ -1610,6 +2334,26 @@
         <f aca="false">IF(H39&lt;&gt;"",H39,IF(AND(I39&lt;&gt;"",J39&lt;&gt;""),(I39+J39)/2,0))</f>
         <v>5</v>
       </c>
+      <c r="O39" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D39,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E39,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F39,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G39,$A$2:$A$63,0)),0))</f>
+        <v>15</v>
+      </c>
+      <c r="P39" s="0" t="n">
+        <f aca="false">O39+N39</f>
+        <v>20</v>
+      </c>
+      <c r="Q39" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A39)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A39)),IF(COUNTIF($E$2:$E$63,$A39)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A39)),IF(COUNTIF($F$2:$F$63,$A39)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A39)),IF(COUNTIF($G$2:$G$63,$A39)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A39)))</f>
+        <v>50</v>
+      </c>
+      <c r="R39" s="0" t="n">
+        <f aca="false">Q39-N39</f>
+        <v>45</v>
+      </c>
+      <c r="S39" s="0" t="n">
+        <f aca="false">R39-O39</f>
+        <v>30</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
@@ -1634,6 +2378,26 @@
         <f aca="false">IF(H40&lt;&gt;"",H40,IF(AND(I40&lt;&gt;"",J40&lt;&gt;""),(I40+J40)/2,0))</f>
         <v>6.5</v>
       </c>
+      <c r="O40" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D40,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E40,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F40,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G40,$A$2:$A$63,0)),0))</f>
+        <v>3</v>
+      </c>
+      <c r="P40" s="0" t="n">
+        <f aca="false">O40+N40</f>
+        <v>9.5</v>
+      </c>
+      <c r="Q40" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A40)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A40)),IF(COUNTIF($E$2:$E$63,$A40)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A40)),IF(COUNTIF($F$2:$F$63,$A40)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A40)),IF(COUNTIF($G$2:$G$63,$A40)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A40)))</f>
+        <v>36</v>
+      </c>
+      <c r="R40" s="0" t="n">
+        <f aca="false">Q40-N40</f>
+        <v>29.5</v>
+      </c>
+      <c r="S40" s="0" t="n">
+        <f aca="false">R40-O40</f>
+        <v>26.5</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
@@ -1655,6 +2419,26 @@
         <f aca="false">IF(H41&lt;&gt;"",H41,IF(AND(I41&lt;&gt;"",J41&lt;&gt;""),(I41+J41)/2,0))</f>
         <v>5</v>
       </c>
+      <c r="O41" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D41,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E41,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F41,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G41,$A$2:$A$63,0)),0))</f>
+        <v>15</v>
+      </c>
+      <c r="P41" s="0" t="n">
+        <f aca="false">O41+N41</f>
+        <v>20</v>
+      </c>
+      <c r="Q41" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A41)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A41)),IF(COUNTIF($E$2:$E$63,$A41)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A41)),IF(COUNTIF($F$2:$F$63,$A41)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A41)),IF(COUNTIF($G$2:$G$63,$A41)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A41)))</f>
+        <v>438.25</v>
+      </c>
+      <c r="R41" s="0" t="n">
+        <f aca="false">Q41-N41</f>
+        <v>433.25</v>
+      </c>
+      <c r="S41" s="0" t="n">
+        <f aca="false">R41-O41</f>
+        <v>418.25</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
@@ -1682,6 +2466,26 @@
         <f aca="false">IF(H42&lt;&gt;"",H42,IF(AND(I42&lt;&gt;"",J42&lt;&gt;""),(I42+J42)/2,0))</f>
         <v>24</v>
       </c>
+      <c r="O42" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D42,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E42,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F42,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G42,$A$2:$A$63,0)),0))</f>
+        <v>9.5</v>
+      </c>
+      <c r="P42" s="0" t="n">
+        <f aca="false">O42+N42</f>
+        <v>33.5</v>
+      </c>
+      <c r="Q42" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A42)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A42)),IF(COUNTIF($E$2:$E$63,$A42)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A42)),IF(COUNTIF($F$2:$F$63,$A42)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A42)),IF(COUNTIF($G$2:$G$63,$A42)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A42)))</f>
+        <v>60</v>
+      </c>
+      <c r="R42" s="0" t="n">
+        <f aca="false">Q42-N42</f>
+        <v>36</v>
+      </c>
+      <c r="S42" s="0" t="n">
+        <f aca="false">R42-O42</f>
+        <v>26.5</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
@@ -1703,6 +2507,26 @@
         <f aca="false">IF(H43&lt;&gt;"",H43,IF(AND(I43&lt;&gt;"",J43&lt;&gt;""),(I43+J43)/2,0))</f>
         <v>5</v>
       </c>
+      <c r="O43" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D43,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E43,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F43,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G43,$A$2:$A$63,0)),0))</f>
+        <v>33.5</v>
+      </c>
+      <c r="P43" s="0" t="n">
+        <f aca="false">O43+N43</f>
+        <v>38.5</v>
+      </c>
+      <c r="Q43" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A43)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A43)),IF(COUNTIF($E$2:$E$63,$A43)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A43)),IF(COUNTIF($F$2:$F$63,$A43)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A43)),IF(COUNTIF($G$2:$G$63,$A43)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A43)))</f>
+        <v>65</v>
+      </c>
+      <c r="R43" s="0" t="n">
+        <f aca="false">Q43-N43</f>
+        <v>60</v>
+      </c>
+      <c r="S43" s="0" t="n">
+        <f aca="false">R43-O43</f>
+        <v>26.5</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
@@ -1727,6 +2551,26 @@
         <f aca="false">IF(H44&lt;&gt;"",H44,IF(AND(I44&lt;&gt;"",J44&lt;&gt;""),(I44+J44)/2,0))</f>
         <v>9</v>
       </c>
+      <c r="O44" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D44,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E44,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F44,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G44,$A$2:$A$63,0)),0))</f>
+        <v>15</v>
+      </c>
+      <c r="P44" s="0" t="n">
+        <f aca="false">O44+N44</f>
+        <v>24</v>
+      </c>
+      <c r="Q44" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A44)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A44)),IF(COUNTIF($E$2:$E$63,$A44)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A44)),IF(COUNTIF($F$2:$F$63,$A44)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A44)),IF(COUNTIF($G$2:$G$63,$A44)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A44)))</f>
+        <v>55</v>
+      </c>
+      <c r="R44" s="0" t="n">
+        <f aca="false">Q44-N44</f>
+        <v>46</v>
+      </c>
+      <c r="S44" s="0" t="n">
+        <f aca="false">R44-O44</f>
+        <v>31</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
@@ -1751,6 +2595,26 @@
         <f aca="false">IF(H45&lt;&gt;"",H45,IF(AND(I45&lt;&gt;"",J45&lt;&gt;""),(I45+J45)/2,0))</f>
         <v>3</v>
       </c>
+      <c r="O45" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D45,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E45,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F45,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G45,$A$2:$A$63,0)),0))</f>
+        <v>15</v>
+      </c>
+      <c r="P45" s="0" t="n">
+        <f aca="false">O45+N45</f>
+        <v>18</v>
+      </c>
+      <c r="Q45" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A45)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A45)),IF(COUNTIF($E$2:$E$63,$A45)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A45)),IF(COUNTIF($F$2:$F$63,$A45)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A45)),IF(COUNTIF($G$2:$G$63,$A45)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A45)))</f>
+        <v>438.25</v>
+      </c>
+      <c r="R45" s="0" t="n">
+        <f aca="false">Q45-N45</f>
+        <v>435.25</v>
+      </c>
+      <c r="S45" s="0" t="n">
+        <f aca="false">R45-O45</f>
+        <v>420.25</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
@@ -1772,6 +2636,26 @@
         <f aca="false">IF(H46&lt;&gt;"",H46,IF(AND(I46&lt;&gt;"",J46&lt;&gt;""),(I46+J46)/2,0))</f>
         <v>5</v>
       </c>
+      <c r="O46" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D46,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E46,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F46,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G46,$A$2:$A$63,0)),0))</f>
+        <v>20</v>
+      </c>
+      <c r="P46" s="0" t="n">
+        <f aca="false">O46+N46</f>
+        <v>25</v>
+      </c>
+      <c r="Q46" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A46)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A46)),IF(COUNTIF($E$2:$E$63,$A46)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A46)),IF(COUNTIF($F$2:$F$63,$A46)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A46)),IF(COUNTIF($G$2:$G$63,$A46)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A46)))</f>
+        <v>55</v>
+      </c>
+      <c r="R46" s="0" t="n">
+        <f aca="false">Q46-N46</f>
+        <v>50</v>
+      </c>
+      <c r="S46" s="0" t="n">
+        <f aca="false">R46-O46</f>
+        <v>30</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
@@ -1796,6 +2680,26 @@
         <f aca="false">IF(H47&lt;&gt;"",H47,IF(AND(I47&lt;&gt;"",J47&lt;&gt;""),(I47+J47)/2,0))</f>
         <v>10</v>
       </c>
+      <c r="O47" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D47,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E47,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F47,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G47,$A$2:$A$63,0)),0))</f>
+        <v>25</v>
+      </c>
+      <c r="P47" s="0" t="n">
+        <f aca="false">O47+N47</f>
+        <v>35</v>
+      </c>
+      <c r="Q47" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A47)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A47)),IF(COUNTIF($E$2:$E$63,$A47)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A47)),IF(COUNTIF($F$2:$F$63,$A47)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A47)),IF(COUNTIF($G$2:$G$63,$A47)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A47)))</f>
+        <v>65</v>
+      </c>
+      <c r="R47" s="0" t="n">
+        <f aca="false">Q47-N47</f>
+        <v>55</v>
+      </c>
+      <c r="S47" s="0" t="n">
+        <f aca="false">R47-O47</f>
+        <v>30</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
@@ -1820,6 +2724,26 @@
         <f aca="false">IF(H48&lt;&gt;"",H48,IF(AND(I48&lt;&gt;"",J48&lt;&gt;""),(I48+J48)/2,0))</f>
         <v>10</v>
       </c>
+      <c r="O48" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D48,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E48,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F48,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G48,$A$2:$A$63,0)),0))</f>
+        <v>25</v>
+      </c>
+      <c r="P48" s="0" t="n">
+        <f aca="false">O48+N48</f>
+        <v>35</v>
+      </c>
+      <c r="Q48" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A48)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A48)),IF(COUNTIF($E$2:$E$63,$A48)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A48)),IF(COUNTIF($F$2:$F$63,$A48)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A48)),IF(COUNTIF($G$2:$G$63,$A48)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A48)))</f>
+        <v>65</v>
+      </c>
+      <c r="R48" s="0" t="n">
+        <f aca="false">Q48-N48</f>
+        <v>55</v>
+      </c>
+      <c r="S48" s="0" t="n">
+        <f aca="false">R48-O48</f>
+        <v>30</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
@@ -1838,6 +2762,26 @@
         <f aca="false">IF(H49&lt;&gt;"",H49,IF(AND(I49&lt;&gt;"",J49&lt;&gt;""),(I49+J49)/2,0))</f>
         <v>0</v>
       </c>
+      <c r="O49" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D49,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E49,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F49,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G49,$A$2:$A$63,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="P49" s="0" t="n">
+        <f aca="false">O49+N49</f>
+        <v>0</v>
+      </c>
+      <c r="Q49" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A49)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A49)),IF(COUNTIF($E$2:$E$63,$A49)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A49)),IF(COUNTIF($F$2:$F$63,$A49)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A49)),IF(COUNTIF($G$2:$G$63,$A49)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A49)))</f>
+        <v>0</v>
+      </c>
+      <c r="R49" s="0" t="n">
+        <f aca="false">Q49-N49</f>
+        <v>0</v>
+      </c>
+      <c r="S49" s="0" t="n">
+        <f aca="false">R49-O49</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
@@ -1859,6 +2803,26 @@
         <f aca="false">IF(H50&lt;&gt;"",H50,IF(AND(I50&lt;&gt;"",J50&lt;&gt;""),(I50+J50)/2,0))</f>
         <v>0</v>
       </c>
+      <c r="O50" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D50,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E50,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F50,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G50,$A$2:$A$63,0)),0))</f>
+        <v>65</v>
+      </c>
+      <c r="P50" s="0" t="n">
+        <f aca="false">O50+N50</f>
+        <v>65</v>
+      </c>
+      <c r="Q50" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A50)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A50)),IF(COUNTIF($E$2:$E$63,$A50)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A50)),IF(COUNTIF($F$2:$F$63,$A50)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A50)),IF(COUNTIF($G$2:$G$63,$A50)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A50)))</f>
+        <v>65</v>
+      </c>
+      <c r="R50" s="0" t="n">
+        <f aca="false">Q50-N50</f>
+        <v>65</v>
+      </c>
+      <c r="S50" s="0" t="n">
+        <f aca="false">R50-O50</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
@@ -1883,6 +2847,26 @@
         <f aca="false">IF(H51&lt;&gt;"",H51,IF(AND(I51&lt;&gt;"",J51&lt;&gt;""),(I51+J51)/2,0))</f>
         <v>7.5</v>
       </c>
+      <c r="O51" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D51,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E51,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F51,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G51,$A$2:$A$63,0)),0))</f>
+        <v>65</v>
+      </c>
+      <c r="P51" s="0" t="n">
+        <f aca="false">O51+N51</f>
+        <v>72.5</v>
+      </c>
+      <c r="Q51" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A51)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A51)),IF(COUNTIF($E$2:$E$63,$A51)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A51)),IF(COUNTIF($F$2:$F$63,$A51)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A51)),IF(COUNTIF($G$2:$G$63,$A51)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A51)))</f>
+        <v>72.5</v>
+      </c>
+      <c r="R51" s="0" t="n">
+        <f aca="false">Q51-N51</f>
+        <v>65</v>
+      </c>
+      <c r="S51" s="0" t="n">
+        <f aca="false">R51-O51</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
@@ -1901,6 +2885,26 @@
         <f aca="false">IF(H52&lt;&gt;"",H52,IF(AND(I52&lt;&gt;"",J52&lt;&gt;""),(I52+J52)/2,0))</f>
         <v>0</v>
       </c>
+      <c r="O52" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D52,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E52,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F52,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G52,$A$2:$A$63,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="P52" s="0" t="n">
+        <f aca="false">O52+N52</f>
+        <v>0</v>
+      </c>
+      <c r="Q52" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A52)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A52)),IF(COUNTIF($E$2:$E$63,$A52)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A52)),IF(COUNTIF($F$2:$F$63,$A52)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A52)),IF(COUNTIF($G$2:$G$63,$A52)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A52)))</f>
+        <v>413.25</v>
+      </c>
+      <c r="R52" s="0" t="n">
+        <f aca="false">Q52-N52</f>
+        <v>413.25</v>
+      </c>
+      <c r="S52" s="0" t="n">
+        <f aca="false">R52-O52</f>
+        <v>413.25</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
@@ -1925,6 +2929,26 @@
         <f aca="false">IF(H53&lt;&gt;"",H53,IF(AND(I53&lt;&gt;"",J53&lt;&gt;""),(I53+J53)/2,0))</f>
         <v>21</v>
       </c>
+      <c r="O53" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D53,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E53,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F53,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G53,$A$2:$A$63,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="P53" s="0" t="n">
+        <f aca="false">O53+N53</f>
+        <v>21</v>
+      </c>
+      <c r="Q53" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A53)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A53)),IF(COUNTIF($E$2:$E$63,$A53)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A53)),IF(COUNTIF($F$2:$F$63,$A53)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A53)),IF(COUNTIF($G$2:$G$63,$A53)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A53)))</f>
+        <v>434.25</v>
+      </c>
+      <c r="R53" s="0" t="n">
+        <f aca="false">Q53-N53</f>
+        <v>413.25</v>
+      </c>
+      <c r="S53" s="0" t="n">
+        <f aca="false">R53-O53</f>
+        <v>413.25</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
@@ -1946,6 +2970,26 @@
         <f aca="false">IF(H54&lt;&gt;"",H54,IF(AND(I54&lt;&gt;"",J54&lt;&gt;""),(I54+J54)/2,0))</f>
         <v>0</v>
       </c>
+      <c r="O54" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D54,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E54,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F54,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G54,$A$2:$A$63,0)),0))</f>
+        <v>72.5</v>
+      </c>
+      <c r="P54" s="0" t="n">
+        <f aca="false">O54+N54</f>
+        <v>72.5</v>
+      </c>
+      <c r="Q54" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A54)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A54)),IF(COUNTIF($E$2:$E$63,$A54)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A54)),IF(COUNTIF($F$2:$F$63,$A54)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A54)),IF(COUNTIF($G$2:$G$63,$A54)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A54)))</f>
+        <v>434.25</v>
+      </c>
+      <c r="R54" s="0" t="n">
+        <f aca="false">Q54-N54</f>
+        <v>434.25</v>
+      </c>
+      <c r="S54" s="0" t="n">
+        <f aca="false">R54-O54</f>
+        <v>361.75</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
@@ -1970,6 +3014,26 @@
         <f aca="false">IF(H55&lt;&gt;"",H55,IF(AND(I55&lt;&gt;"",J55&lt;&gt;""),(I55+J55)/2,0))</f>
         <v>0.75</v>
       </c>
+      <c r="O55" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D55,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E55,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F55,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G55,$A$2:$A$63,0)),0))</f>
+        <v>72.5</v>
+      </c>
+      <c r="P55" s="0" t="n">
+        <f aca="false">O55+N55</f>
+        <v>73.25</v>
+      </c>
+      <c r="Q55" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A55)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A55)),IF(COUNTIF($E$2:$E$63,$A55)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A55)),IF(COUNTIF($F$2:$F$63,$A55)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A55)),IF(COUNTIF($G$2:$G$63,$A55)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A55)))</f>
+        <v>73.25</v>
+      </c>
+      <c r="R55" s="0" t="n">
+        <f aca="false">Q55-N55</f>
+        <v>72.5</v>
+      </c>
+      <c r="S55" s="0" t="n">
+        <f aca="false">R55-O55</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
@@ -1988,6 +3052,26 @@
         <f aca="false">IF(H56&lt;&gt;"",H56,IF(AND(I56&lt;&gt;"",J56&lt;&gt;""),(I56+J56)/2,0))</f>
         <v>0</v>
       </c>
+      <c r="O56" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D56,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E56,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F56,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G56,$A$2:$A$63,0)),0))</f>
+        <v>72.5</v>
+      </c>
+      <c r="P56" s="0" t="n">
+        <f aca="false">O56+N56</f>
+        <v>72.5</v>
+      </c>
+      <c r="Q56" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A56)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A56)),IF(COUNTIF($E$2:$E$63,$A56)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A56)),IF(COUNTIF($F$2:$F$63,$A56)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A56)),IF(COUNTIF($G$2:$G$63,$A56)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A56)))</f>
+        <v>438.25</v>
+      </c>
+      <c r="R56" s="0" t="n">
+        <f aca="false">Q56-N56</f>
+        <v>438.25</v>
+      </c>
+      <c r="S56" s="0" t="n">
+        <f aca="false">R56-O56</f>
+        <v>365.75</v>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
@@ -2009,6 +3093,26 @@
         <f aca="false">IF(H57&lt;&gt;"",H57,IF(AND(I57&lt;&gt;"",J57&lt;&gt;""),(I57+J57)/2,0))</f>
         <v>365</v>
       </c>
+      <c r="O57" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D57,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E57,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F57,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G57,$A$2:$A$63,0)),0))</f>
+        <v>73.25</v>
+      </c>
+      <c r="P57" s="0" t="n">
+        <f aca="false">O57+N57</f>
+        <v>438.25</v>
+      </c>
+      <c r="Q57" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A57)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A57)),IF(COUNTIF($E$2:$E$63,$A57)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A57)),IF(COUNTIF($F$2:$F$63,$A57)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A57)),IF(COUNTIF($G$2:$G$63,$A57)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A57)))</f>
+        <v>438.25</v>
+      </c>
+      <c r="R57" s="0" t="n">
+        <f aca="false">Q57-N57</f>
+        <v>73.25</v>
+      </c>
+      <c r="S57" s="0" t="n">
+        <f aca="false">R57-O57</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
@@ -2030,6 +3134,26 @@
         <f aca="false">IF(H58&lt;&gt;"",H58,IF(AND(I58&lt;&gt;"",J58&lt;&gt;""),(I58+J58)/2,0))</f>
         <v>4</v>
       </c>
+      <c r="O58" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D58,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E58,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F58,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G58,$A$2:$A$63,0)),0))</f>
+        <v>72.5</v>
+      </c>
+      <c r="P58" s="0" t="n">
+        <f aca="false">O58+N58</f>
+        <v>76.5</v>
+      </c>
+      <c r="Q58" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A58)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A58)),IF(COUNTIF($E$2:$E$63,$A58)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A58)),IF(COUNTIF($F$2:$F$63,$A58)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A58)),IF(COUNTIF($G$2:$G$63,$A58)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A58)))</f>
+        <v>438.25</v>
+      </c>
+      <c r="R58" s="0" t="n">
+        <f aca="false">Q58-N58</f>
+        <v>434.25</v>
+      </c>
+      <c r="S58" s="0" t="n">
+        <f aca="false">R58-O58</f>
+        <v>361.75</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
@@ -2054,6 +3178,26 @@
         <f aca="false">IF(H59&lt;&gt;"",H59,IF(AND(I59&lt;&gt;"",J59&lt;&gt;""),(I59+J59)/2,0))</f>
         <v>0</v>
       </c>
+      <c r="O59" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D59,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E59,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F59,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G59,$A$2:$A$63,0)),0))</f>
+        <v>38.5</v>
+      </c>
+      <c r="P59" s="0" t="n">
+        <f aca="false">O59+N59</f>
+        <v>38.5</v>
+      </c>
+      <c r="Q59" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A59)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A59)),IF(COUNTIF($E$2:$E$63,$A59)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A59)),IF(COUNTIF($F$2:$F$63,$A59)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A59)),IF(COUNTIF($G$2:$G$63,$A59)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A59)))</f>
+        <v>65</v>
+      </c>
+      <c r="R59" s="0" t="n">
+        <f aca="false">Q59-N59</f>
+        <v>65</v>
+      </c>
+      <c r="S59" s="0" t="n">
+        <f aca="false">R59-O59</f>
+        <v>26.5</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
@@ -2081,6 +3225,26 @@
         <f aca="false">IF(H60&lt;&gt;"",H60,IF(AND(I60&lt;&gt;"",J60&lt;&gt;""),(I60+J60)/2,0))</f>
         <v>0</v>
       </c>
+      <c r="O60" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D60,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E60,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F60,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G60,$A$2:$A$63,0)),0))</f>
+        <v>62</v>
+      </c>
+      <c r="P60" s="0" t="n">
+        <f aca="false">O60+N60</f>
+        <v>62</v>
+      </c>
+      <c r="Q60" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A60)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A60)),IF(COUNTIF($E$2:$E$63,$A60)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A60)),IF(COUNTIF($F$2:$F$63,$A60)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A60)),IF(COUNTIF($G$2:$G$63,$A60)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A60)))</f>
+        <v>65</v>
+      </c>
+      <c r="R60" s="0" t="n">
+        <f aca="false">Q60-N60</f>
+        <v>65</v>
+      </c>
+      <c r="S60" s="0" t="n">
+        <f aca="false">R60-O60</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
@@ -2099,6 +3263,26 @@
         <f aca="false">IF(H61&lt;&gt;"",H61,IF(AND(I61&lt;&gt;"",J61&lt;&gt;""),(I61+J61)/2,0))</f>
         <v>0</v>
       </c>
+      <c r="O61" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D61,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E61,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F61,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G61,$A$2:$A$63,0)),0))</f>
+        <v>45.5</v>
+      </c>
+      <c r="P61" s="0" t="n">
+        <f aca="false">O61+N61</f>
+        <v>45.5</v>
+      </c>
+      <c r="Q61" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A61)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A61)),IF(COUNTIF($E$2:$E$63,$A61)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A61)),IF(COUNTIF($F$2:$F$63,$A61)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A61)),IF(COUNTIF($G$2:$G$63,$A61)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A61)))</f>
+        <v>65</v>
+      </c>
+      <c r="R61" s="0" t="n">
+        <f aca="false">Q61-N61</f>
+        <v>65</v>
+      </c>
+      <c r="S61" s="0" t="n">
+        <f aca="false">R61-O61</f>
+        <v>19.5</v>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
@@ -2120,6 +3304,26 @@
         <f aca="false">IF(H62&lt;&gt;"",H62,IF(AND(I62&lt;&gt;"",J62&lt;&gt;""),(I62+J62)/2,0))</f>
         <v>0</v>
       </c>
+      <c r="O62" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D62,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E62,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F62,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G62,$A$2:$A$63,0)),0))</f>
+        <v>65</v>
+      </c>
+      <c r="P62" s="0" t="n">
+        <f aca="false">O62+N62</f>
+        <v>65</v>
+      </c>
+      <c r="Q62" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A62)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A62)),IF(COUNTIF($E$2:$E$63,$A62)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A62)),IF(COUNTIF($F$2:$F$63,$A62)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A62)),IF(COUNTIF($G$2:$G$63,$A62)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A62)))</f>
+        <v>65</v>
+      </c>
+      <c r="R62" s="0" t="n">
+        <f aca="false">Q62-N62</f>
+        <v>65</v>
+      </c>
+      <c r="S62" s="0" t="n">
+        <f aca="false">R62-O62</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
@@ -2147,10 +3351,34 @@
         <f aca="false">IF(H63&lt;&gt;"",H63,IF(AND(I63&lt;&gt;"",J63&lt;&gt;""),(I63+J63)/2,0))</f>
         <v>0</v>
       </c>
+      <c r="O63" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D63,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E63,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F63,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G63,$A$2:$A$63,0)),0))</f>
+        <v>65</v>
+      </c>
+      <c r="P63" s="0" t="n">
+        <f aca="false">O63+N63</f>
+        <v>65</v>
+      </c>
+      <c r="Q63" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A63)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A63)),IF(COUNTIF($E$2:$E$63,$A63)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A63)),IF(COUNTIF($F$2:$F$63,$A63)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A63)),IF(COUNTIF($G$2:$G$63,$A63)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A63)))</f>
+        <v>65</v>
+      </c>
+      <c r="R63" s="0" t="n">
+        <f aca="false">Q63-N63</f>
+        <v>65</v>
+      </c>
+      <c r="S63" s="0" t="n">
+        <f aca="false">R63-O63</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="M65" s="0" t="s">
         <v>144</v>
+      </c>
+      <c r="N65" s="0" t="n">
+        <f aca="false">MAX(P2:P63)</f>
+        <v>438.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix reading comprehension errors in task dependencies
</commit_message>
<xml_diff>
--- a/AC Tasks.xlsx
+++ b/AC Tasks.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="145">
   <si>
     <t xml:space="preserve">Id</t>
   </si>
@@ -140,7 +140,7 @@
     <t xml:space="preserve">B0</t>
   </si>
   <si>
-    <t xml:space="preserve">b/c/k</t>
+    <t xml:space="preserve">bookstore</t>
   </si>
   <si>
     <t xml:space="preserve">bookstore start</t>
@@ -371,61 +371,49 @@
     <t xml:space="preserve">Now</t>
   </si>
   <si>
-    <t xml:space="preserve">P1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nominal finish date</t>
+    <t xml:space="preserve">P2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Architect’s punch list tasks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inform architect of close out responsibilities</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Items completed by architecture firm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fire marshal’s inspection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sign general guarantee and warranty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sign final release of lien</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cleanup and ACI punch list</t>
   </si>
   <si>
     <t xml:space="preserve">P15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Architect’s punch list tasks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inform architect of close out responsibilities</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Items completed by architecture firm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fire marshal’s inspection</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sign general guarantee and warranty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sign final release of lien</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ACL relinquished of responsibilities</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cleanup and ACL internal punch list</t>
   </si>
   <si>
     <t xml:space="preserve">P10</t>
@@ -682,7 +670,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S65"/>
+  <dimension ref="A1:S63"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.21"/>
@@ -773,7 +761,7 @@
         <v>0</v>
       </c>
       <c r="O2" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D2,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E2,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F2,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G2,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D2,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E2,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F2,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G2,$A$2:$A$61,0)),0))</f>
         <v>0</v>
       </c>
       <c r="P2" s="0" t="n">
@@ -781,7 +769,7 @@
         <v>0</v>
       </c>
       <c r="Q2" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A2)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A2)),IF(COUNTIF($E$2:$E$63,$A2)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A2)),IF(COUNTIF($F$2:$F$63,$A2)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A2)),IF(COUNTIF($G$2:$G$63,$A2)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A2)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A2)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A2)),IF(COUNTIF($E$2:$E$61,$A2)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A2)),IF(COUNTIF($F$2:$F$61,$A2)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A2)),IF(COUNTIF($G$2:$G$61,$A2)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A2)))</f>
         <v>19.5</v>
       </c>
       <c r="R2" s="0" t="n">
@@ -814,7 +802,7 @@
         <v>8</v>
       </c>
       <c r="O3" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D3,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E3,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F3,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G3,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D3,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E3,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F3,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G3,$A$2:$A$61,0)),0))</f>
         <v>0</v>
       </c>
       <c r="P3" s="0" t="n">
@@ -822,7 +810,7 @@
         <v>8</v>
       </c>
       <c r="Q3" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A3)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A3)),IF(COUNTIF($E$2:$E$63,$A3)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A3)),IF(COUNTIF($F$2:$F$63,$A3)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A3)),IF(COUNTIF($G$2:$G$63,$A3)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A3)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A3)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A3)),IF(COUNTIF($E$2:$E$61,$A3)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A3)),IF(COUNTIF($F$2:$F$61,$A3)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A3)),IF(COUNTIF($G$2:$G$61,$A3)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A3)))</f>
         <v>27.5</v>
       </c>
       <c r="R3" s="0" t="n">
@@ -855,7 +843,7 @@
         <v>7</v>
       </c>
       <c r="O4" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D4,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E4,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F4,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G4,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D4,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E4,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F4,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G4,$A$2:$A$61,0)),0))</f>
         <v>8</v>
       </c>
       <c r="P4" s="0" t="n">
@@ -863,7 +851,7 @@
         <v>15</v>
       </c>
       <c r="Q4" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A4)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A4)),IF(COUNTIF($E$2:$E$63,$A4)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A4)),IF(COUNTIF($F$2:$F$63,$A4)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A4)),IF(COUNTIF($G$2:$G$63,$A4)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A4)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A4)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A4)),IF(COUNTIF($E$2:$E$61,$A4)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A4)),IF(COUNTIF($F$2:$F$61,$A4)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A4)),IF(COUNTIF($G$2:$G$61,$A4)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A4)))</f>
         <v>34.5</v>
       </c>
       <c r="R4" s="0" t="n">
@@ -896,7 +884,7 @@
         <v>3</v>
       </c>
       <c r="O5" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D5,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E5,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F5,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G5,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D5,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E5,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F5,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G5,$A$2:$A$61,0)),0))</f>
         <v>15</v>
       </c>
       <c r="P5" s="0" t="n">
@@ -904,7 +892,7 @@
         <v>18</v>
       </c>
       <c r="Q5" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A5)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A5)),IF(COUNTIF($E$2:$E$63,$A5)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A5)),IF(COUNTIF($F$2:$F$63,$A5)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A5)),IF(COUNTIF($G$2:$G$63,$A5)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A5)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A5)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A5)),IF(COUNTIF($E$2:$E$61,$A5)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A5)),IF(COUNTIF($F$2:$F$61,$A5)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A5)),IF(COUNTIF($G$2:$G$61,$A5)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A5)))</f>
         <v>37.5</v>
       </c>
       <c r="R5" s="0" t="n">
@@ -943,7 +931,7 @@
         <v>7.5</v>
       </c>
       <c r="O6" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D6,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E6,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F6,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G6,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D6,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E6,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F6,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G6,$A$2:$A$61,0)),0))</f>
         <v>18</v>
       </c>
       <c r="P6" s="0" t="n">
@@ -951,7 +939,7 @@
         <v>25.5</v>
       </c>
       <c r="Q6" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A6)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A6)),IF(COUNTIF($E$2:$E$63,$A6)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A6)),IF(COUNTIF($F$2:$F$63,$A6)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A6)),IF(COUNTIF($G$2:$G$63,$A6)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A6)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A6)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A6)),IF(COUNTIF($E$2:$E$61,$A6)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A6)),IF(COUNTIF($F$2:$F$61,$A6)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A6)),IF(COUNTIF($G$2:$G$61,$A6)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A6)))</f>
         <v>45</v>
       </c>
       <c r="R6" s="0" t="n">
@@ -987,7 +975,7 @@
         <v>10</v>
       </c>
       <c r="O7" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D7,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E7,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F7,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G7,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D7,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E7,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F7,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G7,$A$2:$A$61,0)),0))</f>
         <v>25.5</v>
       </c>
       <c r="P7" s="0" t="n">
@@ -995,7 +983,7 @@
         <v>35.5</v>
       </c>
       <c r="Q7" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A7)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A7)),IF(COUNTIF($E$2:$E$63,$A7)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A7)),IF(COUNTIF($F$2:$F$63,$A7)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A7)),IF(COUNTIF($G$2:$G$63,$A7)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A7)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A7)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A7)),IF(COUNTIF($E$2:$E$61,$A7)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A7)),IF(COUNTIF($F$2:$F$61,$A7)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A7)),IF(COUNTIF($G$2:$G$61,$A7)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A7)))</f>
         <v>55</v>
       </c>
       <c r="R7" s="0" t="n">
@@ -1028,7 +1016,7 @@
         <v>5</v>
       </c>
       <c r="O8" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D8,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E8,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F8,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G8,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D8,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E8,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F8,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G8,$A$2:$A$61,0)),0))</f>
         <v>25.5</v>
       </c>
       <c r="P8" s="0" t="n">
@@ -1036,7 +1024,7 @@
         <v>30.5</v>
       </c>
       <c r="Q8" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A8)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A8)),IF(COUNTIF($E$2:$E$63,$A8)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A8)),IF(COUNTIF($F$2:$F$63,$A8)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A8)),IF(COUNTIF($G$2:$G$63,$A8)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A8)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A8)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A8)),IF(COUNTIF($E$2:$E$61,$A8)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A8)),IF(COUNTIF($F$2:$F$61,$A8)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A8)),IF(COUNTIF($G$2:$G$61,$A8)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A8)))</f>
         <v>55</v>
       </c>
       <c r="R8" s="0" t="n">
@@ -1072,7 +1060,7 @@
         <v>10</v>
       </c>
       <c r="O9" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D9,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E9,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F9,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G9,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D9,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E9,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F9,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G9,$A$2:$A$61,0)),0))</f>
         <v>35.5</v>
       </c>
       <c r="P9" s="0" t="n">
@@ -1080,7 +1068,7 @@
         <v>45.5</v>
       </c>
       <c r="Q9" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A9)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A9)),IF(COUNTIF($E$2:$E$63,$A9)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A9)),IF(COUNTIF($F$2:$F$63,$A9)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A9)),IF(COUNTIF($G$2:$G$63,$A9)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A9)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A9)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A9)),IF(COUNTIF($E$2:$E$61,$A9)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A9)),IF(COUNTIF($F$2:$F$61,$A9)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A9)),IF(COUNTIF($G$2:$G$61,$A9)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A9)))</f>
         <v>65</v>
       </c>
       <c r="R9" s="0" t="n">
@@ -1110,7 +1098,7 @@
         <v>0</v>
       </c>
       <c r="O10" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D10,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E10,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F10,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G10,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D10,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E10,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F10,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G10,$A$2:$A$61,0)),0))</f>
         <v>0</v>
       </c>
       <c r="P10" s="0" t="n">
@@ -1118,7 +1106,7 @@
         <v>0</v>
       </c>
       <c r="Q10" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A10)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A10)),IF(COUNTIF($E$2:$E$63,$A10)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A10)),IF(COUNTIF($F$2:$F$63,$A10)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A10)),IF(COUNTIF($G$2:$G$63,$A10)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A10)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A10)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A10)),IF(COUNTIF($E$2:$E$61,$A10)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A10)),IF(COUNTIF($F$2:$F$61,$A10)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A10)),IF(COUNTIF($G$2:$G$61,$A10)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A10)))</f>
         <v>0</v>
       </c>
       <c r="R10" s="0" t="n">
@@ -1154,7 +1142,7 @@
         <v>22</v>
       </c>
       <c r="O11" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D11,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E11,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F11,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G11,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D11,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E11,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F11,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G11,$A$2:$A$61,0)),0))</f>
         <v>0</v>
       </c>
       <c r="P11" s="0" t="n">
@@ -1162,7 +1150,7 @@
         <v>22</v>
       </c>
       <c r="Q11" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A11)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A11)),IF(COUNTIF($E$2:$E$63,$A11)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A11)),IF(COUNTIF($F$2:$F$63,$A11)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A11)),IF(COUNTIF($G$2:$G$63,$A11)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A11)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A11)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A11)),IF(COUNTIF($E$2:$E$61,$A11)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A11)),IF(COUNTIF($F$2:$F$61,$A11)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A11)),IF(COUNTIF($G$2:$G$61,$A11)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A11)))</f>
         <v>22</v>
       </c>
       <c r="R11" s="0" t="n">
@@ -1195,7 +1183,7 @@
         <v>10</v>
       </c>
       <c r="O12" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D12,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E12,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F12,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G12,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D12,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E12,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F12,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G12,$A$2:$A$61,0)),0))</f>
         <v>22</v>
       </c>
       <c r="P12" s="0" t="n">
@@ -1203,7 +1191,7 @@
         <v>32</v>
       </c>
       <c r="Q12" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A12)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A12)),IF(COUNTIF($E$2:$E$63,$A12)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A12)),IF(COUNTIF($F$2:$F$63,$A12)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A12)),IF(COUNTIF($G$2:$G$63,$A12)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A12)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A12)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A12)),IF(COUNTIF($E$2:$E$61,$A12)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A12)),IF(COUNTIF($F$2:$F$61,$A12)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A12)),IF(COUNTIF($G$2:$G$61,$A12)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A12)))</f>
         <v>42</v>
       </c>
       <c r="R12" s="0" t="n">
@@ -1236,7 +1224,7 @@
         <v>5</v>
       </c>
       <c r="O13" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D13,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E13,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F13,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G13,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D13,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E13,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F13,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G13,$A$2:$A$61,0)),0))</f>
         <v>22</v>
       </c>
       <c r="P13" s="0" t="n">
@@ -1244,7 +1232,7 @@
         <v>27</v>
       </c>
       <c r="Q13" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A13)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A13)),IF(COUNTIF($E$2:$E$63,$A13)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A13)),IF(COUNTIF($F$2:$F$63,$A13)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A13)),IF(COUNTIF($G$2:$G$63,$A13)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A13)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A13)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A13)),IF(COUNTIF($E$2:$E$61,$A13)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A13)),IF(COUNTIF($F$2:$F$61,$A13)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A13)),IF(COUNTIF($G$2:$G$61,$A13)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A13)))</f>
         <v>42</v>
       </c>
       <c r="R13" s="0" t="n">
@@ -1283,7 +1271,7 @@
         <v>18</v>
       </c>
       <c r="O14" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D14,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E14,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F14,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G14,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D14,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E14,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F14,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G14,$A$2:$A$61,0)),0))</f>
         <v>22</v>
       </c>
       <c r="P14" s="0" t="n">
@@ -1291,7 +1279,7 @@
         <v>40</v>
       </c>
       <c r="Q14" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A14)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A14)),IF(COUNTIF($E$2:$E$63,$A14)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A14)),IF(COUNTIF($F$2:$F$63,$A14)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A14)),IF(COUNTIF($G$2:$G$63,$A14)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A14)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A14)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A14)),IF(COUNTIF($E$2:$E$61,$A14)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A14)),IF(COUNTIF($F$2:$F$61,$A14)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A14)),IF(COUNTIF($G$2:$G$61,$A14)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A14)))</f>
         <v>40</v>
       </c>
       <c r="R14" s="0" t="n">
@@ -1324,7 +1312,7 @@
         <v>5</v>
       </c>
       <c r="O15" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D15,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E15,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F15,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G15,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D15,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E15,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F15,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G15,$A$2:$A$61,0)),0))</f>
         <v>40</v>
       </c>
       <c r="P15" s="0" t="n">
@@ -1332,7 +1320,7 @@
         <v>45</v>
       </c>
       <c r="Q15" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A15)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A15)),IF(COUNTIF($E$2:$E$63,$A15)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A15)),IF(COUNTIF($F$2:$F$63,$A15)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A15)),IF(COUNTIF($G$2:$G$63,$A15)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A15)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A15)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A15)),IF(COUNTIF($E$2:$E$61,$A15)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A15)),IF(COUNTIF($F$2:$F$61,$A15)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A15)),IF(COUNTIF($G$2:$G$61,$A15)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A15)))</f>
         <v>45</v>
       </c>
       <c r="R15" s="0" t="n">
@@ -1365,7 +1353,7 @@
         <v>10</v>
       </c>
       <c r="O16" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D16,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E16,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F16,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G16,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D16,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E16,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F16,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G16,$A$2:$A$61,0)),0))</f>
         <v>45</v>
       </c>
       <c r="P16" s="0" t="n">
@@ -1373,7 +1361,7 @@
         <v>55</v>
       </c>
       <c r="Q16" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A16)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A16)),IF(COUNTIF($E$2:$E$63,$A16)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A16)),IF(COUNTIF($F$2:$F$63,$A16)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A16)),IF(COUNTIF($G$2:$G$63,$A16)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A16)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A16)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A16)),IF(COUNTIF($E$2:$E$61,$A16)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A16)),IF(COUNTIF($F$2:$F$61,$A16)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A16)),IF(COUNTIF($G$2:$G$61,$A16)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A16)))</f>
         <v>55</v>
       </c>
       <c r="R16" s="0" t="n">
@@ -1409,7 +1397,7 @@
         <v>3</v>
       </c>
       <c r="O17" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D17,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E17,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F17,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G17,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D17,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E17,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F17,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G17,$A$2:$A$61,0)),0))</f>
         <v>32</v>
       </c>
       <c r="P17" s="0" t="n">
@@ -1417,7 +1405,7 @@
         <v>35</v>
       </c>
       <c r="Q17" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A17)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A17)),IF(COUNTIF($E$2:$E$63,$A17)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A17)),IF(COUNTIF($F$2:$F$63,$A17)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A17)),IF(COUNTIF($G$2:$G$63,$A17)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A17)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A17)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A17)),IF(COUNTIF($E$2:$E$61,$A17)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A17)),IF(COUNTIF($F$2:$F$61,$A17)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A17)),IF(COUNTIF($G$2:$G$61,$A17)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A17)))</f>
         <v>45</v>
       </c>
       <c r="R17" s="0" t="n">
@@ -1450,7 +1438,7 @@
         <v>10</v>
       </c>
       <c r="O18" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D18,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E18,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F18,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G18,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D18,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E18,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F18,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G18,$A$2:$A$61,0)),0))</f>
         <v>35</v>
       </c>
       <c r="P18" s="0" t="n">
@@ -1458,7 +1446,7 @@
         <v>45</v>
       </c>
       <c r="Q18" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A18)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A18)),IF(COUNTIF($E$2:$E$63,$A18)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A18)),IF(COUNTIF($F$2:$F$63,$A18)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A18)),IF(COUNTIF($G$2:$G$63,$A18)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A18)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A18)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A18)),IF(COUNTIF($E$2:$E$61,$A18)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A18)),IF(COUNTIF($F$2:$F$61,$A18)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A18)),IF(COUNTIF($G$2:$G$61,$A18)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A18)))</f>
         <v>55</v>
       </c>
       <c r="R18" s="0" t="n">
@@ -1497,7 +1485,7 @@
         <v>6.5</v>
       </c>
       <c r="O19" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D19,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E19,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F19,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G19,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D19,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E19,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F19,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G19,$A$2:$A$61,0)),0))</f>
         <v>55</v>
       </c>
       <c r="P19" s="0" t="n">
@@ -1505,7 +1493,7 @@
         <v>61.5</v>
       </c>
       <c r="Q19" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A19)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A19)),IF(COUNTIF($E$2:$E$63,$A19)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A19)),IF(COUNTIF($F$2:$F$63,$A19)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A19)),IF(COUNTIF($G$2:$G$63,$A19)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A19)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A19)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A19)),IF(COUNTIF($E$2:$E$61,$A19)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A19)),IF(COUNTIF($F$2:$F$61,$A19)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A19)),IF(COUNTIF($G$2:$G$61,$A19)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A19)))</f>
         <v>65</v>
       </c>
       <c r="R19" s="0" t="n">
@@ -1541,7 +1529,7 @@
         <v>10</v>
       </c>
       <c r="O20" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D20,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E20,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F20,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G20,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D20,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E20,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F20,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G20,$A$2:$A$61,0)),0))</f>
         <v>55</v>
       </c>
       <c r="P20" s="0" t="n">
@@ -1549,7 +1537,7 @@
         <v>65</v>
       </c>
       <c r="Q20" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A20)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A20)),IF(COUNTIF($E$2:$E$63,$A20)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A20)),IF(COUNTIF($F$2:$F$63,$A20)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A20)),IF(COUNTIF($G$2:$G$63,$A20)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A20)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A20)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A20)),IF(COUNTIF($E$2:$E$61,$A20)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A20)),IF(COUNTIF($F$2:$F$61,$A20)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A20)),IF(COUNTIF($G$2:$G$61,$A20)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A20)))</f>
         <v>65</v>
       </c>
       <c r="R20" s="0" t="n">
@@ -1579,7 +1567,7 @@
         <v>0</v>
       </c>
       <c r="O21" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D21,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E21,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F21,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G21,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D21,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E21,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F21,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G21,$A$2:$A$61,0)),0))</f>
         <v>0</v>
       </c>
       <c r="P21" s="0" t="n">
@@ -1587,7 +1575,7 @@
         <v>0</v>
       </c>
       <c r="Q21" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A21)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A21)),IF(COUNTIF($E$2:$E$63,$A21)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A21)),IF(COUNTIF($F$2:$F$63,$A21)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A21)),IF(COUNTIF($G$2:$G$63,$A21)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A21)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A21)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A21)),IF(COUNTIF($E$2:$E$61,$A21)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A21)),IF(COUNTIF($F$2:$F$61,$A21)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A21)),IF(COUNTIF($G$2:$G$61,$A21)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A21)))</f>
         <v>3</v>
       </c>
       <c r="R21" s="0" t="n">
@@ -1620,7 +1608,7 @@
         <v>16</v>
       </c>
       <c r="O22" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D22,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E22,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F22,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G22,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D22,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E22,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F22,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G22,$A$2:$A$61,0)),0))</f>
         <v>0</v>
       </c>
       <c r="P22" s="0" t="n">
@@ -1628,7 +1616,7 @@
         <v>16</v>
       </c>
       <c r="Q22" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A22)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A22)),IF(COUNTIF($E$2:$E$63,$A22)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A22)),IF(COUNTIF($F$2:$F$63,$A22)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A22)),IF(COUNTIF($G$2:$G$63,$A22)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A22)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A22)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A22)),IF(COUNTIF($E$2:$E$61,$A22)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A22)),IF(COUNTIF($F$2:$F$61,$A22)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A22)),IF(COUNTIF($G$2:$G$61,$A22)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A22)))</f>
         <v>45</v>
       </c>
       <c r="R22" s="0" t="n">
@@ -1661,7 +1649,7 @@
         <v>2</v>
       </c>
       <c r="O23" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D23,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E23,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F23,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G23,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D23,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E23,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F23,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G23,$A$2:$A$61,0)),0))</f>
         <v>0</v>
       </c>
       <c r="P23" s="0" t="n">
@@ -1669,7 +1657,7 @@
         <v>2</v>
       </c>
       <c r="Q23" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A23)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A23)),IF(COUNTIF($E$2:$E$63,$A23)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A23)),IF(COUNTIF($F$2:$F$63,$A23)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A23)),IF(COUNTIF($G$2:$G$63,$A23)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A23)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A23)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A23)),IF(COUNTIF($E$2:$E$61,$A23)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A23)),IF(COUNTIF($F$2:$F$61,$A23)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A23)),IF(COUNTIF($G$2:$G$61,$A23)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A23)))</f>
         <v>5</v>
       </c>
       <c r="R23" s="0" t="n">
@@ -1702,7 +1690,7 @@
         <v>5</v>
       </c>
       <c r="O24" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D24,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E24,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F24,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G24,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D24,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E24,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F24,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G24,$A$2:$A$61,0)),0))</f>
         <v>2</v>
       </c>
       <c r="P24" s="0" t="n">
@@ -1710,7 +1698,7 @@
         <v>7</v>
       </c>
       <c r="Q24" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A24)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A24)),IF(COUNTIF($E$2:$E$63,$A24)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A24)),IF(COUNTIF($F$2:$F$63,$A24)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A24)),IF(COUNTIF($G$2:$G$63,$A24)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A24)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A24)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A24)),IF(COUNTIF($E$2:$E$61,$A24)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A24)),IF(COUNTIF($F$2:$F$61,$A24)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A24)),IF(COUNTIF($G$2:$G$61,$A24)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A24)))</f>
         <v>60</v>
       </c>
       <c r="R24" s="0" t="n">
@@ -1743,7 +1731,7 @@
         <v>15</v>
       </c>
       <c r="O25" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D25,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E25,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F25,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G25,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D25,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E25,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F25,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G25,$A$2:$A$61,0)),0))</f>
         <v>2</v>
       </c>
       <c r="P25" s="0" t="n">
@@ -1751,7 +1739,7 @@
         <v>17</v>
       </c>
       <c r="Q25" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A25)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A25)),IF(COUNTIF($E$2:$E$63,$A25)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A25)),IF(COUNTIF($F$2:$F$63,$A25)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A25)),IF(COUNTIF($G$2:$G$63,$A25)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A25)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A25)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A25)),IF(COUNTIF($E$2:$E$61,$A25)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A25)),IF(COUNTIF($F$2:$F$61,$A25)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A25)),IF(COUNTIF($G$2:$G$61,$A25)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A25)))</f>
         <v>20</v>
       </c>
       <c r="R25" s="0" t="n">
@@ -1784,7 +1772,7 @@
         <v>5</v>
       </c>
       <c r="O26" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D26,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E26,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F26,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G26,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D26,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E26,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F26,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G26,$A$2:$A$61,0)),0))</f>
         <v>7</v>
       </c>
       <c r="P26" s="0" t="n">
@@ -1792,7 +1780,7 @@
         <v>12</v>
       </c>
       <c r="Q26" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A26)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A26)),IF(COUNTIF($E$2:$E$63,$A26)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A26)),IF(COUNTIF($F$2:$F$63,$A26)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A26)),IF(COUNTIF($G$2:$G$63,$A26)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A26)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A26)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A26)),IF(COUNTIF($E$2:$E$61,$A26)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A26)),IF(COUNTIF($F$2:$F$61,$A26)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A26)),IF(COUNTIF($G$2:$G$61,$A26)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A26)))</f>
         <v>65</v>
       </c>
       <c r="R26" s="0" t="n">
@@ -1825,7 +1813,7 @@
         <v>25</v>
       </c>
       <c r="O27" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D27,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E27,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F27,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G27,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D27,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E27,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F27,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G27,$A$2:$A$61,0)),0))</f>
         <v>17</v>
       </c>
       <c r="P27" s="0" t="n">
@@ -1833,7 +1821,7 @@
         <v>42</v>
       </c>
       <c r="Q27" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A27)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A27)),IF(COUNTIF($E$2:$E$63,$A27)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A27)),IF(COUNTIF($F$2:$F$63,$A27)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A27)),IF(COUNTIF($G$2:$G$63,$A27)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A27)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A27)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A27)),IF(COUNTIF($E$2:$E$61,$A27)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A27)),IF(COUNTIF($F$2:$F$61,$A27)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A27)),IF(COUNTIF($G$2:$G$61,$A27)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A27)))</f>
         <v>45</v>
       </c>
       <c r="R27" s="0" t="n">
@@ -1872,7 +1860,7 @@
         <v>20</v>
       </c>
       <c r="O28" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D28,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E28,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F28,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G28,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D28,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E28,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F28,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G28,$A$2:$A$61,0)),0))</f>
         <v>17</v>
       </c>
       <c r="P28" s="0" t="n">
@@ -1880,7 +1868,7 @@
         <v>37</v>
       </c>
       <c r="Q28" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A28)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A28)),IF(COUNTIF($E$2:$E$63,$A28)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A28)),IF(COUNTIF($F$2:$F$63,$A28)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A28)),IF(COUNTIF($G$2:$G$63,$A28)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A28)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A28)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A28)),IF(COUNTIF($E$2:$E$61,$A28)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A28)),IF(COUNTIF($F$2:$F$61,$A28)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A28)),IF(COUNTIF($G$2:$G$61,$A28)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A28)))</f>
         <v>58.5</v>
       </c>
       <c r="R28" s="0" t="n">
@@ -1913,7 +1901,7 @@
         <v>5</v>
       </c>
       <c r="O29" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D29,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E29,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F29,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G29,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D29,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E29,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F29,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G29,$A$2:$A$61,0)),0))</f>
         <v>7</v>
       </c>
       <c r="P29" s="0" t="n">
@@ -1921,7 +1909,7 @@
         <v>12</v>
       </c>
       <c r="Q29" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A29)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A29)),IF(COUNTIF($E$2:$E$63,$A29)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A29)),IF(COUNTIF($F$2:$F$63,$A29)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A29)),IF(COUNTIF($G$2:$G$63,$A29)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A29)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A29)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A29)),IF(COUNTIF($E$2:$E$61,$A29)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A29)),IF(COUNTIF($F$2:$F$61,$A29)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A29)),IF(COUNTIF($G$2:$G$61,$A29)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A29)))</f>
         <v>38.5</v>
       </c>
       <c r="R29" s="0" t="n">
@@ -1957,7 +1945,7 @@
         <v>20</v>
       </c>
       <c r="O30" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D30,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E30,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F30,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G30,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D30,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E30,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F30,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G30,$A$2:$A$61,0)),0))</f>
         <v>42</v>
       </c>
       <c r="P30" s="0" t="n">
@@ -1965,7 +1953,7 @@
         <v>62</v>
       </c>
       <c r="Q30" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A30)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A30)),IF(COUNTIF($E$2:$E$63,$A30)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A30)),IF(COUNTIF($F$2:$F$63,$A30)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A30)),IF(COUNTIF($G$2:$G$63,$A30)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A30)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A30)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A30)),IF(COUNTIF($E$2:$E$61,$A30)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A30)),IF(COUNTIF($F$2:$F$61,$A30)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A30)),IF(COUNTIF($G$2:$G$61,$A30)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A30)))</f>
         <v>65</v>
       </c>
       <c r="R30" s="0" t="n">
@@ -1998,7 +1986,7 @@
         <v>5</v>
       </c>
       <c r="O31" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D31,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E31,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F31,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G31,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D31,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E31,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F31,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G31,$A$2:$A$61,0)),0))</f>
         <v>2</v>
       </c>
       <c r="P31" s="0" t="n">
@@ -2006,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="Q31" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A31)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A31)),IF(COUNTIF($E$2:$E$63,$A31)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A31)),IF(COUNTIF($F$2:$F$63,$A31)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A31)),IF(COUNTIF($G$2:$G$63,$A31)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A31)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A31)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A31)),IF(COUNTIF($E$2:$E$61,$A31)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A31)),IF(COUNTIF($F$2:$F$61,$A31)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A31)),IF(COUNTIF($G$2:$G$61,$A31)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A31)))</f>
         <v>33.5</v>
       </c>
       <c r="R31" s="0" t="n">
@@ -2039,7 +2027,7 @@
         <v>5</v>
       </c>
       <c r="O32" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D32,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E32,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F32,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G32,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D32,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E32,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F32,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G32,$A$2:$A$61,0)),0))</f>
         <v>7</v>
       </c>
       <c r="P32" s="0" t="n">
@@ -2047,7 +2035,7 @@
         <v>12</v>
       </c>
       <c r="Q32" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A32)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A32)),IF(COUNTIF($E$2:$E$63,$A32)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A32)),IF(COUNTIF($F$2:$F$63,$A32)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A32)),IF(COUNTIF($G$2:$G$63,$A32)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A32)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A32)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A32)),IF(COUNTIF($E$2:$E$61,$A32)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A32)),IF(COUNTIF($F$2:$F$61,$A32)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A32)),IF(COUNTIF($G$2:$G$61,$A32)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A32)))</f>
         <v>65</v>
       </c>
       <c r="R32" s="0" t="n">
@@ -2086,7 +2074,7 @@
         <v>6.5</v>
       </c>
       <c r="O33" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D33,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E33,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F33,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G33,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D33,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E33,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F33,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G33,$A$2:$A$61,0)),0))</f>
         <v>42</v>
       </c>
       <c r="P33" s="0" t="n">
@@ -2094,7 +2082,7 @@
         <v>48.5</v>
       </c>
       <c r="Q33" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A33)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A33)),IF(COUNTIF($E$2:$E$63,$A33)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A33)),IF(COUNTIF($F$2:$F$63,$A33)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A33)),IF(COUNTIF($G$2:$G$63,$A33)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A33)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A33)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A33)),IF(COUNTIF($E$2:$E$61,$A33)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A33)),IF(COUNTIF($F$2:$F$61,$A33)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A33)),IF(COUNTIF($G$2:$G$61,$A33)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A33)))</f>
         <v>65</v>
       </c>
       <c r="R33" s="0" t="n">
@@ -2124,7 +2112,7 @@
         <v>0</v>
       </c>
       <c r="O34" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D34,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E34,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F34,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G34,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D34,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E34,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F34,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G34,$A$2:$A$61,0)),0))</f>
         <v>0</v>
       </c>
       <c r="P34" s="0" t="n">
@@ -2132,7 +2120,7 @@
         <v>0</v>
       </c>
       <c r="Q34" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A34)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A34)),IF(COUNTIF($E$2:$E$63,$A34)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A34)),IF(COUNTIF($F$2:$F$63,$A34)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A34)),IF(COUNTIF($G$2:$G$63,$A34)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A34)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A34)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A34)),IF(COUNTIF($E$2:$E$61,$A34)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A34)),IF(COUNTIF($F$2:$F$61,$A34)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A34)),IF(COUNTIF($G$2:$G$61,$A34)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A34)))</f>
         <v>26.5</v>
       </c>
       <c r="R34" s="0" t="n">
@@ -2165,7 +2153,7 @@
         <v>3</v>
       </c>
       <c r="O35" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D35,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E35,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F35,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G35,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D35,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E35,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F35,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G35,$A$2:$A$61,0)),0))</f>
         <v>0</v>
       </c>
       <c r="P35" s="0" t="n">
@@ -2173,7 +2161,7 @@
         <v>3</v>
       </c>
       <c r="Q35" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A35)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A35)),IF(COUNTIF($E$2:$E$63,$A35)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A35)),IF(COUNTIF($F$2:$F$63,$A35)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A35)),IF(COUNTIF($G$2:$G$63,$A35)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A35)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A35)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A35)),IF(COUNTIF($E$2:$E$61,$A35)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A35)),IF(COUNTIF($F$2:$F$61,$A35)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A35)),IF(COUNTIF($G$2:$G$61,$A35)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A35)))</f>
         <v>29.5</v>
       </c>
       <c r="R35" s="0" t="n">
@@ -2206,7 +2194,7 @@
         <v>10</v>
       </c>
       <c r="O36" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D36,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E36,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F36,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G36,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D36,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E36,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F36,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G36,$A$2:$A$61,0)),0))</f>
         <v>0</v>
       </c>
       <c r="P36" s="0" t="n">
@@ -2214,7 +2202,7 @@
         <v>10</v>
       </c>
       <c r="Q36" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A36)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A36)),IF(COUNTIF($E$2:$E$63,$A36)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A36)),IF(COUNTIF($F$2:$F$63,$A36)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A36)),IF(COUNTIF($G$2:$G$63,$A36)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A36)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A36)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A36)),IF(COUNTIF($E$2:$E$61,$A36)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A36)),IF(COUNTIF($F$2:$F$61,$A36)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A36)),IF(COUNTIF($G$2:$G$61,$A36)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A36)))</f>
         <v>45</v>
       </c>
       <c r="R36" s="0" t="n">
@@ -2247,7 +2235,7 @@
         <v>15</v>
       </c>
       <c r="O37" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D37,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E37,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F37,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G37,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D37,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E37,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F37,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G37,$A$2:$A$61,0)),0))</f>
         <v>0</v>
       </c>
       <c r="P37" s="0" t="n">
@@ -2255,7 +2243,7 @@
         <v>15</v>
       </c>
       <c r="Q37" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A37)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A37)),IF(COUNTIF($E$2:$E$63,$A37)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A37)),IF(COUNTIF($F$2:$F$63,$A37)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A37)),IF(COUNTIF($G$2:$G$63,$A37)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A37)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A37)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A37)),IF(COUNTIF($E$2:$E$61,$A37)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A37)),IF(COUNTIF($F$2:$F$61,$A37)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A37)),IF(COUNTIF($G$2:$G$61,$A37)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A37)))</f>
         <v>45</v>
       </c>
       <c r="R37" s="0" t="n">
@@ -2288,7 +2276,7 @@
         <v>15</v>
       </c>
       <c r="O38" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D38,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E38,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F38,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G38,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D38,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E38,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F38,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G38,$A$2:$A$61,0)),0))</f>
         <v>0</v>
       </c>
       <c r="P38" s="0" t="n">
@@ -2296,7 +2284,7 @@
         <v>15</v>
       </c>
       <c r="Q38" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A38)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A38)),IF(COUNTIF($E$2:$E$63,$A38)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A38)),IF(COUNTIF($F$2:$F$63,$A38)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A38)),IF(COUNTIF($G$2:$G$63,$A38)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A38)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A38)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A38)),IF(COUNTIF($E$2:$E$61,$A38)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A38)),IF(COUNTIF($F$2:$F$61,$A38)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A38)),IF(COUNTIF($G$2:$G$61,$A38)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A38)))</f>
         <v>45</v>
       </c>
       <c r="R38" s="0" t="n">
@@ -2335,7 +2323,7 @@
         <v>5</v>
       </c>
       <c r="O39" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D39,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E39,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F39,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G39,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D39,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E39,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F39,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G39,$A$2:$A$61,0)),0))</f>
         <v>15</v>
       </c>
       <c r="P39" s="0" t="n">
@@ -2343,7 +2331,7 @@
         <v>20</v>
       </c>
       <c r="Q39" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A39)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A39)),IF(COUNTIF($E$2:$E$63,$A39)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A39)),IF(COUNTIF($F$2:$F$63,$A39)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A39)),IF(COUNTIF($G$2:$G$63,$A39)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A39)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A39)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A39)),IF(COUNTIF($E$2:$E$61,$A39)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A39)),IF(COUNTIF($F$2:$F$61,$A39)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A39)),IF(COUNTIF($G$2:$G$61,$A39)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A39)))</f>
         <v>50</v>
       </c>
       <c r="R39" s="0" t="n">
@@ -2379,7 +2367,7 @@
         <v>6.5</v>
       </c>
       <c r="O40" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D40,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E40,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F40,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G40,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D40,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E40,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F40,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G40,$A$2:$A$61,0)),0))</f>
         <v>3</v>
       </c>
       <c r="P40" s="0" t="n">
@@ -2387,7 +2375,7 @@
         <v>9.5</v>
       </c>
       <c r="Q40" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A40)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A40)),IF(COUNTIF($E$2:$E$63,$A40)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A40)),IF(COUNTIF($F$2:$F$63,$A40)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A40)),IF(COUNTIF($G$2:$G$63,$A40)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A40)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A40)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A40)),IF(COUNTIF($E$2:$E$61,$A40)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A40)),IF(COUNTIF($F$2:$F$61,$A40)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A40)),IF(COUNTIF($G$2:$G$61,$A40)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A40)))</f>
         <v>36</v>
       </c>
       <c r="R40" s="0" t="n">
@@ -2420,7 +2408,7 @@
         <v>5</v>
       </c>
       <c r="O41" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D41,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E41,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F41,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G41,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D41,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E41,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F41,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G41,$A$2:$A$61,0)),0))</f>
         <v>15</v>
       </c>
       <c r="P41" s="0" t="n">
@@ -2428,16 +2416,16 @@
         <v>20</v>
       </c>
       <c r="Q41" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A41)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A41)),IF(COUNTIF($E$2:$E$63,$A41)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A41)),IF(COUNTIF($F$2:$F$63,$A41)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A41)),IF(COUNTIF($G$2:$G$63,$A41)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A41)))</f>
-        <v>438.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A41)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A41)),IF(COUNTIF($E$2:$E$61,$A41)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A41)),IF(COUNTIF($F$2:$F$61,$A41)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A41)),IF(COUNTIF($G$2:$G$61,$A41)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A41)))</f>
+        <v>82.25</v>
       </c>
       <c r="R41" s="0" t="n">
         <f aca="false">Q41-N41</f>
-        <v>433.25</v>
+        <v>77.25</v>
       </c>
       <c r="S41" s="0" t="n">
         <f aca="false">R41-O41</f>
-        <v>418.25</v>
+        <v>62.25</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2467,7 +2455,7 @@
         <v>24</v>
       </c>
       <c r="O42" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D42,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E42,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F42,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G42,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D42,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E42,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F42,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G42,$A$2:$A$61,0)),0))</f>
         <v>9.5</v>
       </c>
       <c r="P42" s="0" t="n">
@@ -2475,7 +2463,7 @@
         <v>33.5</v>
       </c>
       <c r="Q42" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A42)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A42)),IF(COUNTIF($E$2:$E$63,$A42)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A42)),IF(COUNTIF($F$2:$F$63,$A42)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A42)),IF(COUNTIF($G$2:$G$63,$A42)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A42)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A42)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A42)),IF(COUNTIF($E$2:$E$61,$A42)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A42)),IF(COUNTIF($F$2:$F$61,$A42)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A42)),IF(COUNTIF($G$2:$G$61,$A42)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A42)))</f>
         <v>60</v>
       </c>
       <c r="R42" s="0" t="n">
@@ -2508,7 +2496,7 @@
         <v>5</v>
       </c>
       <c r="O43" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D43,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E43,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F43,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G43,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D43,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E43,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F43,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G43,$A$2:$A$61,0)),0))</f>
         <v>33.5</v>
       </c>
       <c r="P43" s="0" t="n">
@@ -2516,7 +2504,7 @@
         <v>38.5</v>
       </c>
       <c r="Q43" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A43)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A43)),IF(COUNTIF($E$2:$E$63,$A43)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A43)),IF(COUNTIF($F$2:$F$63,$A43)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A43)),IF(COUNTIF($G$2:$G$63,$A43)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A43)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A43)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A43)),IF(COUNTIF($E$2:$E$61,$A43)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A43)),IF(COUNTIF($F$2:$F$61,$A43)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A43)),IF(COUNTIF($G$2:$G$61,$A43)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A43)))</f>
         <v>65</v>
       </c>
       <c r="R43" s="0" t="n">
@@ -2552,7 +2540,7 @@
         <v>9</v>
       </c>
       <c r="O44" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D44,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E44,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F44,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G44,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D44,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E44,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F44,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G44,$A$2:$A$61,0)),0))</f>
         <v>15</v>
       </c>
       <c r="P44" s="0" t="n">
@@ -2560,7 +2548,7 @@
         <v>24</v>
       </c>
       <c r="Q44" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A44)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A44)),IF(COUNTIF($E$2:$E$63,$A44)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A44)),IF(COUNTIF($F$2:$F$63,$A44)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A44)),IF(COUNTIF($G$2:$G$63,$A44)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A44)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A44)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A44)),IF(COUNTIF($E$2:$E$61,$A44)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A44)),IF(COUNTIF($F$2:$F$61,$A44)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A44)),IF(COUNTIF($G$2:$G$61,$A44)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A44)))</f>
         <v>55</v>
       </c>
       <c r="R44" s="0" t="n">
@@ -2596,7 +2584,7 @@
         <v>3</v>
       </c>
       <c r="O45" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D45,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E45,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F45,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G45,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D45,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E45,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F45,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G45,$A$2:$A$61,0)),0))</f>
         <v>15</v>
       </c>
       <c r="P45" s="0" t="n">
@@ -2604,16 +2592,16 @@
         <v>18</v>
       </c>
       <c r="Q45" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A45)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A45)),IF(COUNTIF($E$2:$E$63,$A45)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A45)),IF(COUNTIF($F$2:$F$63,$A45)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A45)),IF(COUNTIF($G$2:$G$63,$A45)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A45)))</f>
-        <v>438.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A45)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A45)),IF(COUNTIF($E$2:$E$61,$A45)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A45)),IF(COUNTIF($F$2:$F$61,$A45)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A45)),IF(COUNTIF($G$2:$G$61,$A45)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A45)))</f>
+        <v>82.25</v>
       </c>
       <c r="R45" s="0" t="n">
         <f aca="false">Q45-N45</f>
-        <v>435.25</v>
+        <v>79.25</v>
       </c>
       <c r="S45" s="0" t="n">
         <f aca="false">R45-O45</f>
-        <v>420.25</v>
+        <v>64.25</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2637,7 +2625,7 @@
         <v>5</v>
       </c>
       <c r="O46" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D46,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E46,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F46,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G46,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D46,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E46,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F46,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G46,$A$2:$A$61,0)),0))</f>
         <v>20</v>
       </c>
       <c r="P46" s="0" t="n">
@@ -2645,7 +2633,7 @@
         <v>25</v>
       </c>
       <c r="Q46" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A46)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A46)),IF(COUNTIF($E$2:$E$63,$A46)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A46)),IF(COUNTIF($F$2:$F$63,$A46)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A46)),IF(COUNTIF($G$2:$G$63,$A46)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A46)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A46)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A46)),IF(COUNTIF($E$2:$E$61,$A46)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A46)),IF(COUNTIF($F$2:$F$61,$A46)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A46)),IF(COUNTIF($G$2:$G$61,$A46)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A46)))</f>
         <v>55</v>
       </c>
       <c r="R46" s="0" t="n">
@@ -2681,7 +2669,7 @@
         <v>10</v>
       </c>
       <c r="O47" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D47,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E47,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F47,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G47,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D47,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E47,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F47,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G47,$A$2:$A$61,0)),0))</f>
         <v>25</v>
       </c>
       <c r="P47" s="0" t="n">
@@ -2689,7 +2677,7 @@
         <v>35</v>
       </c>
       <c r="Q47" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A47)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A47)),IF(COUNTIF($E$2:$E$63,$A47)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A47)),IF(COUNTIF($F$2:$F$63,$A47)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A47)),IF(COUNTIF($G$2:$G$63,$A47)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A47)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A47)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A47)),IF(COUNTIF($E$2:$E$61,$A47)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A47)),IF(COUNTIF($F$2:$F$61,$A47)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A47)),IF(COUNTIF($G$2:$G$61,$A47)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A47)))</f>
         <v>65</v>
       </c>
       <c r="R47" s="0" t="n">
@@ -2725,7 +2713,7 @@
         <v>10</v>
       </c>
       <c r="O48" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D48,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E48,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F48,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G48,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D48,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E48,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F48,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G48,$A$2:$A$61,0)),0))</f>
         <v>25</v>
       </c>
       <c r="P48" s="0" t="n">
@@ -2733,7 +2721,7 @@
         <v>35</v>
       </c>
       <c r="Q48" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A48)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A48)),IF(COUNTIF($E$2:$E$63,$A48)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A48)),IF(COUNTIF($F$2:$F$63,$A48)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A48)),IF(COUNTIF($G$2:$G$63,$A48)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A48)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A48)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A48)),IF(COUNTIF($E$2:$E$61,$A48)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A48)),IF(COUNTIF($F$2:$F$61,$A48)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A48)),IF(COUNTIF($G$2:$G$61,$A48)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A48)))</f>
         <v>65</v>
       </c>
       <c r="R48" s="0" t="n">
@@ -2763,7 +2751,7 @@
         <v>0</v>
       </c>
       <c r="O49" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D49,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E49,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F49,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G49,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D49,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E49,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F49,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G49,$A$2:$A$61,0)),0))</f>
         <v>0</v>
       </c>
       <c r="P49" s="0" t="n">
@@ -2771,7 +2759,7 @@
         <v>0</v>
       </c>
       <c r="Q49" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A49)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A49)),IF(COUNTIF($E$2:$E$63,$A49)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A49)),IF(COUNTIF($F$2:$F$63,$A49)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A49)),IF(COUNTIF($G$2:$G$63,$A49)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A49)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A49)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A49)),IF(COUNTIF($E$2:$E$61,$A49)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A49)),IF(COUNTIF($F$2:$F$61,$A49)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A49)),IF(COUNTIF($G$2:$G$61,$A49)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A49)))</f>
         <v>0</v>
       </c>
       <c r="R49" s="0" t="n">
@@ -2796,28 +2784,31 @@
       <c r="D50" s="0" t="s">
         <v>118</v>
       </c>
-      <c r="M50" s="2" t="n">
-        <v>40161</v>
+      <c r="I50" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="J50" s="0" t="n">
+        <v>10</v>
       </c>
       <c r="N50" s="0" t="n">
         <f aca="false">IF(H50&lt;&gt;"",H50,IF(AND(I50&lt;&gt;"",J50&lt;&gt;""),(I50+J50)/2,0))</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="O50" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D50,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E50,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F50,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G50,$A$2:$A$63,0)),0))</f>
-        <v>65</v>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D50,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E50,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F50,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G50,$A$2:$A$61,0)),0))</f>
+        <v>74</v>
       </c>
       <c r="P50" s="0" t="n">
         <f aca="false">O50+N50</f>
-        <v>65</v>
+        <v>81.5</v>
       </c>
       <c r="Q50" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A50)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A50)),IF(COUNTIF($E$2:$E$63,$A50)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A50)),IF(COUNTIF($F$2:$F$63,$A50)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A50)),IF(COUNTIF($G$2:$G$63,$A50)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A50)))</f>
-        <v>65</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A50)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A50)),IF(COUNTIF($E$2:$E$61,$A50)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A50)),IF(COUNTIF($F$2:$F$61,$A50)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A50)),IF(COUNTIF($G$2:$G$61,$A50)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A50)))</f>
+        <v>81.5</v>
       </c>
       <c r="R50" s="0" t="n">
         <f aca="false">Q50-N50</f>
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="S50" s="0" t="n">
         <f aca="false">R50-O50</f>
@@ -2835,37 +2826,31 @@
         <v>120</v>
       </c>
       <c r="D51" s="0" t="s">
-        <v>116</v>
-      </c>
-      <c r="I51" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="J51" s="0" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="N51" s="0" t="n">
         <f aca="false">IF(H51&lt;&gt;"",H51,IF(AND(I51&lt;&gt;"",J51&lt;&gt;""),(I51+J51)/2,0))</f>
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="O51" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D51,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E51,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F51,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G51,$A$2:$A$63,0)),0))</f>
-        <v>65</v>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D51,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E51,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F51,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G51,$A$2:$A$61,0)),0))</f>
+        <v>0</v>
       </c>
       <c r="P51" s="0" t="n">
         <f aca="false">O51+N51</f>
-        <v>72.5</v>
+        <v>0</v>
       </c>
       <c r="Q51" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A51)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A51)),IF(COUNTIF($E$2:$E$63,$A51)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A51)),IF(COUNTIF($F$2:$F$63,$A51)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A51)),IF(COUNTIF($G$2:$G$63,$A51)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A51)))</f>
-        <v>72.5</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A51)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A51)),IF(COUNTIF($E$2:$E$61,$A51)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A51)),IF(COUNTIF($F$2:$F$61,$A51)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A51)),IF(COUNTIF($G$2:$G$61,$A51)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A51)))</f>
+        <v>48</v>
       </c>
       <c r="R51" s="0" t="n">
         <f aca="false">Q51-N51</f>
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="S51" s="0" t="n">
         <f aca="false">R51-O51</f>
-        <v>0</v>
+        <v>48</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2879,75 +2864,81 @@
         <v>122</v>
       </c>
       <c r="D52" s="0" t="s">
-        <v>22</v>
+        <v>119</v>
+      </c>
+      <c r="I52" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="J52" s="0" t="n">
+        <v>28</v>
       </c>
       <c r="N52" s="0" t="n">
         <f aca="false">IF(H52&lt;&gt;"",H52,IF(AND(I52&lt;&gt;"",J52&lt;&gt;""),(I52+J52)/2,0))</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="O52" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D52,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E52,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F52,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G52,$A$2:$A$63,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D52,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E52,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F52,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G52,$A$2:$A$61,0)),0))</f>
         <v>0</v>
       </c>
       <c r="P52" s="0" t="n">
         <f aca="false">O52+N52</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="Q52" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A52)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A52)),IF(COUNTIF($E$2:$E$63,$A52)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A52)),IF(COUNTIF($F$2:$F$63,$A52)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A52)),IF(COUNTIF($G$2:$G$63,$A52)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A52)))</f>
-        <v>413.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A52)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A52)),IF(COUNTIF($E$2:$E$61,$A52)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A52)),IF(COUNTIF($F$2:$F$61,$A52)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A52)),IF(COUNTIF($G$2:$G$61,$A52)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A52)))</f>
+        <v>69</v>
       </c>
       <c r="R52" s="0" t="n">
         <f aca="false">Q52-N52</f>
-        <v>413.25</v>
+        <v>48</v>
       </c>
       <c r="S52" s="0" t="n">
         <f aca="false">R52-O52</f>
-        <v>413.25</v>
+        <v>48</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B53" s="0" t="s">
         <v>114</v>
       </c>
       <c r="C53" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="D53" s="0" t="s">
         <v>124</v>
       </c>
-      <c r="D53" s="0" t="s">
+      <c r="E53" s="0" t="s">
         <v>121</v>
       </c>
-      <c r="I53" s="0" t="n">
-        <v>14</v>
-      </c>
-      <c r="J53" s="0" t="n">
-        <v>28</v>
+      <c r="H53" s="0" t="n">
+        <v>5</v>
       </c>
       <c r="N53" s="0" t="n">
         <f aca="false">IF(H53&lt;&gt;"",H53,IF(AND(I53&lt;&gt;"",J53&lt;&gt;""),(I53+J53)/2,0))</f>
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="O53" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D53,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E53,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F53,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G53,$A$2:$A$63,0)),0))</f>
-        <v>0</v>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D53,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E53,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F53,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G53,$A$2:$A$61,0)),0))</f>
+        <v>69</v>
       </c>
       <c r="P53" s="0" t="n">
         <f aca="false">O53+N53</f>
-        <v>21</v>
+        <v>74</v>
       </c>
       <c r="Q53" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A53)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A53)),IF(COUNTIF($E$2:$E$63,$A53)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A53)),IF(COUNTIF($F$2:$F$63,$A53)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A53)),IF(COUNTIF($G$2:$G$63,$A53)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A53)))</f>
-        <v>434.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A53)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A53)),IF(COUNTIF($E$2:$E$61,$A53)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A53)),IF(COUNTIF($F$2:$F$61,$A53)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A53)),IF(COUNTIF($G$2:$G$61,$A53)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A53)))</f>
+        <v>74</v>
       </c>
       <c r="R53" s="0" t="n">
         <f aca="false">Q53-N53</f>
-        <v>413.25</v>
+        <v>69</v>
       </c>
       <c r="S53" s="0" t="n">
         <f aca="false">R53-O53</f>
-        <v>413.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2961,34 +2952,37 @@
         <v>126</v>
       </c>
       <c r="D54" s="0" t="s">
-        <v>119</v>
-      </c>
-      <c r="E54" s="0" t="s">
-        <v>123</v>
+        <v>116</v>
+      </c>
+      <c r="I54" s="0" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J54" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="N54" s="0" t="n">
         <f aca="false">IF(H54&lt;&gt;"",H54,IF(AND(I54&lt;&gt;"",J54&lt;&gt;""),(I54+J54)/2,0))</f>
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="O54" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D54,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E54,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F54,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G54,$A$2:$A$63,0)),0))</f>
-        <v>72.5</v>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D54,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E54,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F54,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G54,$A$2:$A$61,0)),0))</f>
+        <v>81.5</v>
       </c>
       <c r="P54" s="0" t="n">
         <f aca="false">O54+N54</f>
-        <v>72.5</v>
+        <v>82.25</v>
       </c>
       <c r="Q54" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A54)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A54)),IF(COUNTIF($E$2:$E$63,$A54)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A54)),IF(COUNTIF($F$2:$F$63,$A54)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A54)),IF(COUNTIF($G$2:$G$63,$A54)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A54)))</f>
-        <v>434.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A54)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A54)),IF(COUNTIF($E$2:$E$61,$A54)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A54)),IF(COUNTIF($F$2:$F$61,$A54)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A54)),IF(COUNTIF($G$2:$G$61,$A54)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A54)))</f>
+        <v>82.25</v>
       </c>
       <c r="R54" s="0" t="n">
         <f aca="false">Q54-N54</f>
-        <v>434.25</v>
+        <v>81.5</v>
       </c>
       <c r="S54" s="0" t="n">
         <f aca="false">R54-O54</f>
-        <v>361.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3002,75 +2996,72 @@
         <v>128</v>
       </c>
       <c r="D55" s="0" t="s">
-        <v>119</v>
-      </c>
-      <c r="I55" s="0" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J55" s="0" t="n">
-        <v>1</v>
+        <v>116</v>
       </c>
       <c r="N55" s="0" t="n">
         <f aca="false">IF(H55&lt;&gt;"",H55,IF(AND(I55&lt;&gt;"",J55&lt;&gt;""),(I55+J55)/2,0))</f>
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="O55" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D55,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E55,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F55,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G55,$A$2:$A$63,0)),0))</f>
-        <v>72.5</v>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D55,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E55,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F55,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G55,$A$2:$A$61,0)),0))</f>
+        <v>81.5</v>
       </c>
       <c r="P55" s="0" t="n">
         <f aca="false">O55+N55</f>
-        <v>73.25</v>
+        <v>81.5</v>
       </c>
       <c r="Q55" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A55)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A55)),IF(COUNTIF($E$2:$E$63,$A55)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A55)),IF(COUNTIF($F$2:$F$63,$A55)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A55)),IF(COUNTIF($G$2:$G$63,$A55)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A55)))</f>
-        <v>73.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A55)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A55)),IF(COUNTIF($E$2:$E$61,$A55)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A55)),IF(COUNTIF($F$2:$F$61,$A55)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A55)),IF(COUNTIF($G$2:$G$61,$A55)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A55)))</f>
+        <v>82.25</v>
       </c>
       <c r="R55" s="0" t="n">
         <f aca="false">Q55-N55</f>
-        <v>72.5</v>
+        <v>82.25</v>
       </c>
       <c r="S55" s="0" t="n">
         <f aca="false">R55-O55</f>
-        <v>0</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B56" s="0" t="s">
         <v>114</v>
       </c>
       <c r="C56" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="D56" s="0" t="s">
         <v>130</v>
       </c>
-      <c r="D56" s="0" t="s">
-        <v>119</v>
+      <c r="H56" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="N56" s="0" t="n">
         <f aca="false">IF(H56&lt;&gt;"",H56,IF(AND(I56&lt;&gt;"",J56&lt;&gt;""),(I56+J56)/2,0))</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O56" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D56,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E56,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F56,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G56,$A$2:$A$63,0)),0))</f>
-        <v>72.5</v>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D56,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E56,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F56,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G56,$A$2:$A$61,0)),0))</f>
+        <v>65</v>
       </c>
       <c r="P56" s="0" t="n">
         <f aca="false">O56+N56</f>
-        <v>72.5</v>
+        <v>69</v>
       </c>
       <c r="Q56" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A56)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A56)),IF(COUNTIF($E$2:$E$63,$A56)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A56)),IF(COUNTIF($F$2:$F$63,$A56)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A56)),IF(COUNTIF($G$2:$G$63,$A56)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A56)))</f>
-        <v>438.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A56)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A56)),IF(COUNTIF($E$2:$E$61,$A56)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A56)),IF(COUNTIF($F$2:$F$61,$A56)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A56)),IF(COUNTIF($G$2:$G$61,$A56)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A56)))</f>
+        <v>69</v>
       </c>
       <c r="R56" s="0" t="n">
         <f aca="false">Q56-N56</f>
-        <v>438.25</v>
+        <v>65</v>
       </c>
       <c r="S56" s="0" t="n">
         <f aca="false">R56-O56</f>
-        <v>365.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3084,34 +3075,37 @@
         <v>132</v>
       </c>
       <c r="D57" s="0" t="s">
-        <v>127</v>
-      </c>
-      <c r="H57" s="0" t="n">
-        <v>365</v>
+        <v>113</v>
+      </c>
+      <c r="E57" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="F57" s="0" t="s">
+        <v>104</v>
       </c>
       <c r="N57" s="0" t="n">
         <f aca="false">IF(H57&lt;&gt;"",H57,IF(AND(I57&lt;&gt;"",J57&lt;&gt;""),(I57+J57)/2,0))</f>
-        <v>365</v>
+        <v>0</v>
       </c>
       <c r="O57" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D57,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E57,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F57,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G57,$A$2:$A$63,0)),0))</f>
-        <v>73.25</v>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D57,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E57,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F57,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G57,$A$2:$A$61,0)),0))</f>
+        <v>38.5</v>
       </c>
       <c r="P57" s="0" t="n">
         <f aca="false">O57+N57</f>
-        <v>438.25</v>
+        <v>38.5</v>
       </c>
       <c r="Q57" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A57)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A57)),IF(COUNTIF($E$2:$E$63,$A57)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A57)),IF(COUNTIF($F$2:$F$63,$A57)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A57)),IF(COUNTIF($G$2:$G$63,$A57)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A57)))</f>
-        <v>438.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A57)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A57)),IF(COUNTIF($E$2:$E$61,$A57)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A57)),IF(COUNTIF($F$2:$F$61,$A57)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A57)),IF(COUNTIF($G$2:$G$61,$A57)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A57)))</f>
+        <v>65</v>
       </c>
       <c r="R57" s="0" t="n">
         <f aca="false">Q57-N57</f>
-        <v>73.25</v>
+        <v>65</v>
       </c>
       <c r="S57" s="0" t="n">
         <f aca="false">R57-O57</f>
-        <v>0</v>
+        <v>26.5</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3125,34 +3119,40 @@
         <v>134</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>125</v>
-      </c>
-      <c r="H58" s="0" t="n">
-        <v>4</v>
+        <v>82</v>
+      </c>
+      <c r="E58" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F58" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="G58" s="0" t="s">
+        <v>71</v>
       </c>
       <c r="N58" s="0" t="n">
         <f aca="false">IF(H58&lt;&gt;"",H58,IF(AND(I58&lt;&gt;"",J58&lt;&gt;""),(I58+J58)/2,0))</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O58" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D58,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E58,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F58,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G58,$A$2:$A$63,0)),0))</f>
-        <v>72.5</v>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D58,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E58,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F58,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G58,$A$2:$A$61,0)),0))</f>
+        <v>62</v>
       </c>
       <c r="P58" s="0" t="n">
         <f aca="false">O58+N58</f>
-        <v>76.5</v>
+        <v>62</v>
       </c>
       <c r="Q58" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A58)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A58)),IF(COUNTIF($E$2:$E$63,$A58)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A58)),IF(COUNTIF($F$2:$F$63,$A58)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A58)),IF(COUNTIF($G$2:$G$63,$A58)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A58)))</f>
-        <v>438.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A58)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A58)),IF(COUNTIF($E$2:$E$61,$A58)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A58)),IF(COUNTIF($F$2:$F$61,$A58)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A58)),IF(COUNTIF($G$2:$G$61,$A58)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A58)))</f>
+        <v>65</v>
       </c>
       <c r="R58" s="0" t="n">
         <f aca="false">Q58-N58</f>
-        <v>434.25</v>
+        <v>65</v>
       </c>
       <c r="S58" s="0" t="n">
         <f aca="false">R58-O58</f>
-        <v>361.75</v>
+        <v>3</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3166,28 +3166,22 @@
         <v>136</v>
       </c>
       <c r="D59" s="0" t="s">
-        <v>113</v>
-      </c>
-      <c r="E59" s="0" t="s">
-        <v>112</v>
-      </c>
-      <c r="F59" s="0" t="s">
-        <v>104</v>
+        <v>36</v>
       </c>
       <c r="N59" s="0" t="n">
         <f aca="false">IF(H59&lt;&gt;"",H59,IF(AND(I59&lt;&gt;"",J59&lt;&gt;""),(I59+J59)/2,0))</f>
         <v>0</v>
       </c>
       <c r="O59" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D59,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E59,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F59,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G59,$A$2:$A$63,0)),0))</f>
-        <v>38.5</v>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D59,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E59,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F59,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G59,$A$2:$A$61,0)),0))</f>
+        <v>45.5</v>
       </c>
       <c r="P59" s="0" t="n">
         <f aca="false">O59+N59</f>
-        <v>38.5</v>
+        <v>45.5</v>
       </c>
       <c r="Q59" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A59)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A59)),IF(COUNTIF($E$2:$E$63,$A59)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A59)),IF(COUNTIF($F$2:$F$63,$A59)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A59)),IF(COUNTIF($G$2:$G$63,$A59)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A59)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A59)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A59)),IF(COUNTIF($E$2:$E$61,$A59)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A59)),IF(COUNTIF($F$2:$F$61,$A59)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A59)),IF(COUNTIF($G$2:$G$61,$A59)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A59)))</f>
         <v>65</v>
       </c>
       <c r="R59" s="0" t="n">
@@ -3196,7 +3190,7 @@
       </c>
       <c r="S59" s="0" t="n">
         <f aca="false">R59-O59</f>
-        <v>26.5</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3210,31 +3204,25 @@
         <v>138</v>
       </c>
       <c r="D60" s="0" t="s">
-        <v>82</v>
+        <v>57</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>84</v>
-      </c>
-      <c r="F60" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="G60" s="0" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="N60" s="0" t="n">
         <f aca="false">IF(H60&lt;&gt;"",H60,IF(AND(I60&lt;&gt;"",J60&lt;&gt;""),(I60+J60)/2,0))</f>
         <v>0</v>
       </c>
       <c r="O60" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D60,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E60,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F60,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G60,$A$2:$A$63,0)),0))</f>
-        <v>62</v>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D60,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E60,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F60,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G60,$A$2:$A$61,0)),0))</f>
+        <v>65</v>
       </c>
       <c r="P60" s="0" t="n">
         <f aca="false">O60+N60</f>
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="Q60" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A60)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A60)),IF(COUNTIF($E$2:$E$63,$A60)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A60)),IF(COUNTIF($F$2:$F$63,$A60)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A60)),IF(COUNTIF($G$2:$G$63,$A60)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A60)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A60)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A60)),IF(COUNTIF($E$2:$E$61,$A60)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A60)),IF(COUNTIF($F$2:$F$61,$A60)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A60)),IF(COUNTIF($G$2:$G$61,$A60)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A60)))</f>
         <v>65</v>
       </c>
       <c r="R60" s="0" t="n">
@@ -3243,36 +3231,45 @@
       </c>
       <c r="S60" s="0" t="n">
         <f aca="false">R60-O60</f>
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="1" t="s">
-        <v>139</v>
+      <c r="A61" s="0" t="s">
+        <v>130</v>
       </c>
       <c r="B61" s="0" t="s">
         <v>114</v>
       </c>
       <c r="C61" s="0" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>36</v>
+        <v>137</v>
+      </c>
+      <c r="E61" s="0" t="s">
+        <v>133</v>
+      </c>
+      <c r="F61" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="G61" s="0" t="s">
+        <v>135</v>
       </c>
       <c r="N61" s="0" t="n">
         <f aca="false">IF(H61&lt;&gt;"",H61,IF(AND(I61&lt;&gt;"",J61&lt;&gt;""),(I61+J61)/2,0))</f>
         <v>0</v>
       </c>
       <c r="O61" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D61,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E61,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F61,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G61,$A$2:$A$63,0)),0))</f>
-        <v>45.5</v>
+        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D61,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E61,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F61,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G61,$A$2:$A$61,0)),0))</f>
+        <v>65</v>
       </c>
       <c r="P61" s="0" t="n">
         <f aca="false">O61+N61</f>
-        <v>45.5</v>
+        <v>65</v>
       </c>
       <c r="Q61" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A61)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A61)),IF(COUNTIF($E$2:$E$63,$A61)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A61)),IF(COUNTIF($F$2:$F$63,$A61)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A61)),IF(COUNTIF($G$2:$G$63,$A61)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A61)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A61)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A61)),IF(COUNTIF($E$2:$E$61,$A61)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A61)),IF(COUNTIF($F$2:$F$61,$A61)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A61)),IF(COUNTIF($G$2:$G$61,$A61)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A61)))</f>
         <v>65</v>
       </c>
       <c r="R61" s="0" t="n">
@@ -3281,104 +3278,16 @@
       </c>
       <c r="S61" s="0" t="n">
         <f aca="false">R61-O61</f>
-        <v>19.5</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="B62" s="0" t="s">
-        <v>114</v>
-      </c>
-      <c r="C62" s="0" t="s">
-        <v>142</v>
-      </c>
-      <c r="D62" s="0" t="s">
-        <v>57</v>
-      </c>
-      <c r="E62" s="0" t="s">
-        <v>59</v>
-      </c>
-      <c r="N62" s="0" t="n">
-        <f aca="false">IF(H62&lt;&gt;"",H62,IF(AND(I62&lt;&gt;"",J62&lt;&gt;""),(I62+J62)/2,0))</f>
-        <v>0</v>
-      </c>
-      <c r="O62" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D62,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E62,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F62,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G62,$A$2:$A$63,0)),0))</f>
-        <v>65</v>
-      </c>
-      <c r="P62" s="0" t="n">
-        <f aca="false">O62+N62</f>
-        <v>65</v>
-      </c>
-      <c r="Q62" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A62)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A62)),IF(COUNTIF($E$2:$E$63,$A62)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A62)),IF(COUNTIF($F$2:$F$63,$A62)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A62)),IF(COUNTIF($G$2:$G$63,$A62)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A62)))</f>
-        <v>65</v>
-      </c>
-      <c r="R62" s="0" t="n">
-        <f aca="false">Q62-N62</f>
-        <v>65</v>
-      </c>
-      <c r="S62" s="0" t="n">
-        <f aca="false">R62-O62</f>
         <v>0</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="0" t="s">
-        <v>118</v>
-      </c>
-      <c r="B63" s="0" t="s">
-        <v>114</v>
-      </c>
-      <c r="C63" s="0" t="s">
-        <v>143</v>
-      </c>
-      <c r="D63" s="0" t="s">
-        <v>141</v>
-      </c>
-      <c r="E63" s="0" t="s">
-        <v>137</v>
-      </c>
-      <c r="F63" s="0" t="s">
-        <v>135</v>
-      </c>
-      <c r="G63" s="0" t="s">
-        <v>139</v>
+      <c r="M63" s="0" t="s">
+        <v>140</v>
       </c>
       <c r="N63" s="0" t="n">
-        <f aca="false">IF(H63&lt;&gt;"",H63,IF(AND(I63&lt;&gt;"",J63&lt;&gt;""),(I63+J63)/2,0))</f>
-        <v>0</v>
-      </c>
-      <c r="O63" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$63,MATCH(D63,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(E63,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(F63,$A$2:$A$63,0)),0),IFERROR(INDEX($P$2:$P$63,MATCH(G63,$A$2:$A$63,0)),0))</f>
-        <v>65</v>
-      </c>
-      <c r="P63" s="0" t="n">
-        <f aca="false">O63+N63</f>
-        <v>65</v>
-      </c>
-      <c r="Q63" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$63,$A63)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$D$2:$D$63,$A63)),IF(COUNTIF($E$2:$E$63,$A63)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$E$2:$E$63,$A63)),IF(COUNTIF($F$2:$F$63,$A63)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$F$2:$F$63,$A63)),IF(COUNTIF($G$2:$G$63,$A63)=0,$N$65,_xlfn.MINIFS($R$2:$R$63,$G$2:$G$63,$A63)))</f>
-        <v>65</v>
-      </c>
-      <c r="R63" s="0" t="n">
-        <f aca="false">Q63-N63</f>
-        <v>65</v>
-      </c>
-      <c r="S63" s="0" t="n">
-        <f aca="false">R63-O63</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M65" s="0" t="s">
-        <v>144</v>
-      </c>
-      <c r="N65" s="0" t="n">
-        <f aca="false">MAX(P2:P63)</f>
-        <v>438.25</v>
+        <f aca="false">MAX(P2:P61)</f>
+        <v>82.25</v>
       </c>
     </row>
   </sheetData>
@@ -3405,22 +3314,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="39.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="35.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="42.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="50.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="40.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Set occupancy milestone as end of critical path
</commit_message>
<xml_diff>
--- a/AC Tasks.xlsx
+++ b/AC Tasks.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="148">
   <si>
     <t xml:space="preserve">Id</t>
   </si>
@@ -53,6 +53,9 @@
     <t xml:space="preserve">High Estimate</t>
   </si>
   <si>
+    <t xml:space="preserve">Effective End</t>
+  </si>
+  <si>
     <t xml:space="preserve">Weather-dependent</t>
   </si>
   <si>
@@ -441,6 +444,12 @@
   </si>
   <si>
     <t xml:space="preserve">all sections done</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">occupancy permitted</t>
   </si>
   <si>
     <t xml:space="preserve">Project Finish</t>
@@ -670,7 +679,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S63"/>
+  <dimension ref="A1:T64"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.21"/>
@@ -680,8 +689,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="0" width="12.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="12.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="17.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="17.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="12.37"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -742,180 +751,183 @@
       <c r="S1" s="0" t="s">
         <v>18</v>
       </c>
+      <c r="T1" s="0" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="N2" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="O2" s="0" t="n">
         <f aca="false">IF(H2&lt;&gt;"",H2,IF(AND(I2&lt;&gt;"",J2&lt;&gt;""),(I2+J2)/2,0))</f>
         <v>0</v>
       </c>
-      <c r="O2" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D2,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E2,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F2,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G2,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
-      </c>
       <c r="P2" s="0" t="n">
-        <f aca="false">O2+N2</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D2,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E2,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F2,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G2,$A$2:$A$61,0)),0))</f>
         <v>0</v>
       </c>
       <c r="Q2" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A2)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A2)),IF(COUNTIF($E$2:$E$61,$A2)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A2)),IF(COUNTIF($F$2:$F$61,$A2)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A2)),IF(COUNTIF($G$2:$G$61,$A2)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A2)))</f>
-        <v>19.5</v>
+        <f aca="false">P2+O2</f>
+        <v>0</v>
       </c>
       <c r="R2" s="0" t="n">
-        <f aca="false">Q2-N2</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A2)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A2)),IF(COUNTIF($E$2:$E$61,$A2)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A2)),IF(COUNTIF($F$2:$F$61,$A2)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A2)),IF(COUNTIF($G$2:$G$61,$A2)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A2)))</f>
         <v>19.5</v>
       </c>
       <c r="S2" s="0" t="n">
         <f aca="false">R2-O2</f>
         <v>19.5</v>
       </c>
+      <c r="T2" s="0" t="n">
+        <f aca="false">S2-P2</f>
+        <v>19.5</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="H3" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="N3" s="0" t="n">
+      <c r="O3" s="0" t="n">
         <f aca="false">IF(H3&lt;&gt;"",H3,IF(AND(I3&lt;&gt;"",J3&lt;&gt;""),(I3+J3)/2,0))</f>
         <v>8</v>
       </c>
-      <c r="O3" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D3,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E3,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F3,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G3,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
-      </c>
       <c r="P3" s="0" t="n">
-        <f aca="false">O3+N3</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D3,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E3,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F3,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G3,$A$2:$A$61,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="Q3" s="0" t="n">
+        <f aca="false">P3+O3</f>
         <v>8</v>
       </c>
-      <c r="Q3" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A3)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A3)),IF(COUNTIF($E$2:$E$61,$A3)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A3)),IF(COUNTIF($F$2:$F$61,$A3)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A3)),IF(COUNTIF($G$2:$G$61,$A3)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A3)))</f>
+      <c r="R3" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A3)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A3)),IF(COUNTIF($E$2:$E$61,$A3)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A3)),IF(COUNTIF($F$2:$F$61,$A3)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A3)),IF(COUNTIF($G$2:$G$61,$A3)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A3)))</f>
         <v>27.5</v>
-      </c>
-      <c r="R3" s="0" t="n">
-        <f aca="false">Q3-N3</f>
-        <v>19.5</v>
       </c>
       <c r="S3" s="0" t="n">
         <f aca="false">R3-O3</f>
         <v>19.5</v>
       </c>
+      <c r="T3" s="0" t="n">
+        <f aca="false">S3-P3</f>
+        <v>19.5</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H4" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="N4" s="0" t="n">
+      <c r="O4" s="0" t="n">
         <f aca="false">IF(H4&lt;&gt;"",H4,IF(AND(I4&lt;&gt;"",J4&lt;&gt;""),(I4+J4)/2,0))</f>
         <v>7</v>
       </c>
-      <c r="O4" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D4,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E4,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F4,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G4,$A$2:$A$61,0)),0))</f>
+      <c r="P4" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D4,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E4,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F4,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G4,$A$2:$A$61,0)),0))</f>
         <v>8</v>
       </c>
-      <c r="P4" s="0" t="n">
-        <f aca="false">O4+N4</f>
+      <c r="Q4" s="0" t="n">
+        <f aca="false">P4+O4</f>
         <v>15</v>
       </c>
-      <c r="Q4" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A4)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A4)),IF(COUNTIF($E$2:$E$61,$A4)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A4)),IF(COUNTIF($F$2:$F$61,$A4)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A4)),IF(COUNTIF($G$2:$G$61,$A4)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A4)))</f>
+      <c r="R4" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A4)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A4)),IF(COUNTIF($E$2:$E$61,$A4)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A4)),IF(COUNTIF($F$2:$F$61,$A4)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A4)),IF(COUNTIF($G$2:$G$61,$A4)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A4)))</f>
         <v>34.5</v>
-      </c>
-      <c r="R4" s="0" t="n">
-        <f aca="false">Q4-N4</f>
-        <v>27.5</v>
       </c>
       <c r="S4" s="0" t="n">
         <f aca="false">R4-O4</f>
+        <v>27.5</v>
+      </c>
+      <c r="T4" s="0" t="n">
+        <f aca="false">S4-P4</f>
         <v>19.5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H5" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="N5" s="0" t="n">
+      <c r="O5" s="0" t="n">
         <f aca="false">IF(H5&lt;&gt;"",H5,IF(AND(I5&lt;&gt;"",J5&lt;&gt;""),(I5+J5)/2,0))</f>
         <v>3</v>
       </c>
-      <c r="O5" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D5,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E5,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F5,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G5,$A$2:$A$61,0)),0))</f>
+      <c r="P5" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D5,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E5,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F5,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G5,$A$2:$A$61,0)),0))</f>
         <v>15</v>
       </c>
-      <c r="P5" s="0" t="n">
-        <f aca="false">O5+N5</f>
+      <c r="Q5" s="0" t="n">
+        <f aca="false">P5+O5</f>
         <v>18</v>
       </c>
-      <c r="Q5" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A5)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A5)),IF(COUNTIF($E$2:$E$61,$A5)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A5)),IF(COUNTIF($F$2:$F$61,$A5)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A5)),IF(COUNTIF($G$2:$G$61,$A5)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A5)))</f>
+      <c r="R5" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A5)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A5)),IF(COUNTIF($E$2:$E$61,$A5)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A5)),IF(COUNTIF($F$2:$F$61,$A5)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A5)),IF(COUNTIF($G$2:$G$61,$A5)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A5)))</f>
         <v>37.5</v>
-      </c>
-      <c r="R5" s="0" t="n">
-        <f aca="false">Q5-N5</f>
-        <v>34.5</v>
       </c>
       <c r="S5" s="0" t="n">
         <f aca="false">R5-O5</f>
+        <v>34.5</v>
+      </c>
+      <c r="T5" s="0" t="n">
+        <f aca="false">S5-P5</f>
         <v>19.5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I6" s="0" t="n">
         <v>5</v>
@@ -923,213 +935,213 @@
       <c r="J6" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="K6" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="N6" s="0" t="n">
+      <c r="L6" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="O6" s="0" t="n">
         <f aca="false">IF(H6&lt;&gt;"",H6,IF(AND(I6&lt;&gt;"",J6&lt;&gt;""),(I6+J6)/2,0))</f>
         <v>7.5</v>
       </c>
-      <c r="O6" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D6,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E6,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F6,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G6,$A$2:$A$61,0)),0))</f>
+      <c r="P6" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D6,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E6,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F6,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G6,$A$2:$A$61,0)),0))</f>
         <v>18</v>
       </c>
-      <c r="P6" s="0" t="n">
-        <f aca="false">O6+N6</f>
+      <c r="Q6" s="0" t="n">
+        <f aca="false">P6+O6</f>
         <v>25.5</v>
       </c>
-      <c r="Q6" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A6)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A6)),IF(COUNTIF($E$2:$E$61,$A6)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A6)),IF(COUNTIF($F$2:$F$61,$A6)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A6)),IF(COUNTIF($G$2:$G$61,$A6)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A6)))</f>
+      <c r="R6" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A6)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A6)),IF(COUNTIF($E$2:$E$61,$A6)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A6)),IF(COUNTIF($F$2:$F$61,$A6)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A6)),IF(COUNTIF($G$2:$G$61,$A6)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A6)))</f>
         <v>45</v>
-      </c>
-      <c r="R6" s="0" t="n">
-        <f aca="false">Q6-N6</f>
-        <v>37.5</v>
       </c>
       <c r="S6" s="0" t="n">
         <f aca="false">R6-O6</f>
+        <v>37.5</v>
+      </c>
+      <c r="T6" s="0" t="n">
+        <f aca="false">S6-P6</f>
         <v>19.5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H7" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="L7" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="N7" s="0" t="n">
+      <c r="M7" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="O7" s="0" t="n">
         <f aca="false">IF(H7&lt;&gt;"",H7,IF(AND(I7&lt;&gt;"",J7&lt;&gt;""),(I7+J7)/2,0))</f>
         <v>10</v>
       </c>
-      <c r="O7" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D7,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E7,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F7,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G7,$A$2:$A$61,0)),0))</f>
+      <c r="P7" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D7,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E7,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F7,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G7,$A$2:$A$61,0)),0))</f>
         <v>25.5</v>
       </c>
-      <c r="P7" s="0" t="n">
-        <f aca="false">O7+N7</f>
+      <c r="Q7" s="0" t="n">
+        <f aca="false">P7+O7</f>
         <v>35.5</v>
       </c>
-      <c r="Q7" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A7)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A7)),IF(COUNTIF($E$2:$E$61,$A7)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A7)),IF(COUNTIF($F$2:$F$61,$A7)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A7)),IF(COUNTIF($G$2:$G$61,$A7)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A7)))</f>
+      <c r="R7" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A7)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A7)),IF(COUNTIF($E$2:$E$61,$A7)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A7)),IF(COUNTIF($F$2:$F$61,$A7)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A7)),IF(COUNTIF($G$2:$G$61,$A7)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A7)))</f>
         <v>55</v>
-      </c>
-      <c r="R7" s="0" t="n">
-        <f aca="false">Q7-N7</f>
-        <v>45</v>
       </c>
       <c r="S7" s="0" t="n">
         <f aca="false">R7-O7</f>
+        <v>45</v>
+      </c>
+      <c r="T7" s="0" t="n">
+        <f aca="false">S7-P7</f>
         <v>19.5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H8" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="N8" s="0" t="n">
+      <c r="O8" s="0" t="n">
         <f aca="false">IF(H8&lt;&gt;"",H8,IF(AND(I8&lt;&gt;"",J8&lt;&gt;""),(I8+J8)/2,0))</f>
         <v>5</v>
       </c>
-      <c r="O8" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D8,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E8,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F8,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G8,$A$2:$A$61,0)),0))</f>
+      <c r="P8" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D8,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E8,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F8,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G8,$A$2:$A$61,0)),0))</f>
         <v>25.5</v>
       </c>
-      <c r="P8" s="0" t="n">
-        <f aca="false">O8+N8</f>
+      <c r="Q8" s="0" t="n">
+        <f aca="false">P8+O8</f>
         <v>30.5</v>
       </c>
-      <c r="Q8" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A8)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A8)),IF(COUNTIF($E$2:$E$61,$A8)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A8)),IF(COUNTIF($F$2:$F$61,$A8)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A8)),IF(COUNTIF($G$2:$G$61,$A8)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A8)))</f>
+      <c r="R8" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A8)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A8)),IF(COUNTIF($E$2:$E$61,$A8)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A8)),IF(COUNTIF($F$2:$F$61,$A8)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A8)),IF(COUNTIF($G$2:$G$61,$A8)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A8)))</f>
         <v>55</v>
-      </c>
-      <c r="R8" s="0" t="n">
-        <f aca="false">Q8-N8</f>
-        <v>50</v>
       </c>
       <c r="S8" s="0" t="n">
         <f aca="false">R8-O8</f>
+        <v>50</v>
+      </c>
+      <c r="T8" s="0" t="n">
+        <f aca="false">S8-P8</f>
         <v>24.5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H9" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="N9" s="0" t="n">
+      <c r="O9" s="0" t="n">
         <f aca="false">IF(H9&lt;&gt;"",H9,IF(AND(I9&lt;&gt;"",J9&lt;&gt;""),(I9+J9)/2,0))</f>
         <v>10</v>
       </c>
-      <c r="O9" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D9,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E9,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F9,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G9,$A$2:$A$61,0)),0))</f>
+      <c r="P9" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D9,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E9,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F9,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G9,$A$2:$A$61,0)),0))</f>
         <v>35.5</v>
       </c>
-      <c r="P9" s="0" t="n">
-        <f aca="false">O9+N9</f>
+      <c r="Q9" s="0" t="n">
+        <f aca="false">P9+O9</f>
         <v>45.5</v>
       </c>
-      <c r="Q9" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A9)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A9)),IF(COUNTIF($E$2:$E$61,$A9)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A9)),IF(COUNTIF($F$2:$F$61,$A9)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A9)),IF(COUNTIF($G$2:$G$61,$A9)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A9)))</f>
+      <c r="R9" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A9)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A9)),IF(COUNTIF($E$2:$E$61,$A9)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A9)),IF(COUNTIF($F$2:$F$61,$A9)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A9)),IF(COUNTIF($G$2:$G$61,$A9)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A9)))</f>
         <v>65</v>
-      </c>
-      <c r="R9" s="0" t="n">
-        <f aca="false">Q9-N9</f>
-        <v>55</v>
       </c>
       <c r="S9" s="0" t="n">
         <f aca="false">R9-O9</f>
+        <v>55</v>
+      </c>
+      <c r="T9" s="0" t="n">
+        <f aca="false">S9-P9</f>
         <v>19.5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="N10" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="O10" s="0" t="n">
         <f aca="false">IF(H10&lt;&gt;"",H10,IF(AND(I10&lt;&gt;"",J10&lt;&gt;""),(I10+J10)/2,0))</f>
         <v>0</v>
       </c>
-      <c r="O10" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D10,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E10,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F10,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G10,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
-      </c>
       <c r="P10" s="0" t="n">
-        <f aca="false">O10+N10</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D10,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E10,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F10,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G10,$A$2:$A$61,0)),0))</f>
         <v>0</v>
       </c>
       <c r="Q10" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A10)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A10)),IF(COUNTIF($E$2:$E$61,$A10)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A10)),IF(COUNTIF($F$2:$F$61,$A10)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A10)),IF(COUNTIF($G$2:$G$61,$A10)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A10)))</f>
+        <f aca="false">P10+O10</f>
         <v>0</v>
       </c>
       <c r="R10" s="0" t="n">
-        <f aca="false">Q10-N10</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A10)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A10)),IF(COUNTIF($E$2:$E$61,$A10)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A10)),IF(COUNTIF($F$2:$F$61,$A10)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A10)),IF(COUNTIF($G$2:$G$61,$A10)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A10)))</f>
         <v>0</v>
       </c>
       <c r="S10" s="0" t="n">
         <f aca="false">R10-O10</f>
         <v>0</v>
       </c>
+      <c r="T10" s="0" t="n">
+        <f aca="false">S10-P10</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B11" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="0" t="s">
         <v>39</v>
-      </c>
-      <c r="C11" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="D11" s="0" t="s">
-        <v>38</v>
       </c>
       <c r="I11" s="0" t="n">
         <v>21</v>
@@ -1137,125 +1149,125 @@
       <c r="J11" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="N11" s="0" t="n">
+      <c r="O11" s="0" t="n">
         <f aca="false">IF(H11&lt;&gt;"",H11,IF(AND(I11&lt;&gt;"",J11&lt;&gt;""),(I11+J11)/2,0))</f>
         <v>22</v>
       </c>
-      <c r="O11" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D11,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E11,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F11,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G11,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
-      </c>
       <c r="P11" s="0" t="n">
-        <f aca="false">O11+N11</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D11,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E11,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F11,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G11,$A$2:$A$61,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="Q11" s="0" t="n">
+        <f aca="false">P11+O11</f>
         <v>22</v>
       </c>
-      <c r="Q11" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A11)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A11)),IF(COUNTIF($E$2:$E$61,$A11)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A11)),IF(COUNTIF($F$2:$F$61,$A11)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A11)),IF(COUNTIF($G$2:$G$61,$A11)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A11)))</f>
+      <c r="R11" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A11)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A11)),IF(COUNTIF($E$2:$E$61,$A11)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A11)),IF(COUNTIF($F$2:$F$61,$A11)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A11)),IF(COUNTIF($G$2:$G$61,$A11)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A11)))</f>
         <v>22</v>
-      </c>
-      <c r="R11" s="0" t="n">
-        <f aca="false">Q11-N11</f>
-        <v>0</v>
       </c>
       <c r="S11" s="0" t="n">
         <f aca="false">R11-O11</f>
         <v>0</v>
       </c>
+      <c r="T11" s="0" t="n">
+        <f aca="false">S11-P11</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H12" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="N12" s="0" t="n">
+      <c r="O12" s="0" t="n">
         <f aca="false">IF(H12&lt;&gt;"",H12,IF(AND(I12&lt;&gt;"",J12&lt;&gt;""),(I12+J12)/2,0))</f>
         <v>10</v>
       </c>
-      <c r="O12" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D12,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E12,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F12,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G12,$A$2:$A$61,0)),0))</f>
+      <c r="P12" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D12,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E12,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F12,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G12,$A$2:$A$61,0)),0))</f>
         <v>22</v>
       </c>
-      <c r="P12" s="0" t="n">
-        <f aca="false">O12+N12</f>
+      <c r="Q12" s="0" t="n">
+        <f aca="false">P12+O12</f>
         <v>32</v>
       </c>
-      <c r="Q12" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A12)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A12)),IF(COUNTIF($E$2:$E$61,$A12)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A12)),IF(COUNTIF($F$2:$F$61,$A12)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A12)),IF(COUNTIF($G$2:$G$61,$A12)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A12)))</f>
+      <c r="R12" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A12)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A12)),IF(COUNTIF($E$2:$E$61,$A12)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A12)),IF(COUNTIF($F$2:$F$61,$A12)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A12)),IF(COUNTIF($G$2:$G$61,$A12)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A12)))</f>
         <v>42</v>
-      </c>
-      <c r="R12" s="0" t="n">
-        <f aca="false">Q12-N12</f>
-        <v>32</v>
       </c>
       <c r="S12" s="0" t="n">
         <f aca="false">R12-O12</f>
+        <v>32</v>
+      </c>
+      <c r="T12" s="0" t="n">
+        <f aca="false">S12-P12</f>
         <v>10</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H13" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="N13" s="0" t="n">
+      <c r="O13" s="0" t="n">
         <f aca="false">IF(H13&lt;&gt;"",H13,IF(AND(I13&lt;&gt;"",J13&lt;&gt;""),(I13+J13)/2,0))</f>
         <v>5</v>
       </c>
-      <c r="O13" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D13,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E13,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F13,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G13,$A$2:$A$61,0)),0))</f>
+      <c r="P13" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D13,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E13,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F13,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G13,$A$2:$A$61,0)),0))</f>
         <v>22</v>
       </c>
-      <c r="P13" s="0" t="n">
-        <f aca="false">O13+N13</f>
+      <c r="Q13" s="0" t="n">
+        <f aca="false">P13+O13</f>
         <v>27</v>
       </c>
-      <c r="Q13" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A13)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A13)),IF(COUNTIF($E$2:$E$61,$A13)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A13)),IF(COUNTIF($F$2:$F$61,$A13)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A13)),IF(COUNTIF($G$2:$G$61,$A13)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A13)))</f>
+      <c r="R13" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A13)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A13)),IF(COUNTIF($E$2:$E$61,$A13)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A13)),IF(COUNTIF($F$2:$F$61,$A13)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A13)),IF(COUNTIF($G$2:$G$61,$A13)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A13)))</f>
         <v>42</v>
-      </c>
-      <c r="R13" s="0" t="n">
-        <f aca="false">Q13-N13</f>
-        <v>37</v>
       </c>
       <c r="S13" s="0" t="n">
         <f aca="false">R13-O13</f>
+        <v>37</v>
+      </c>
+      <c r="T13" s="0" t="n">
+        <f aca="false">S13-P13</f>
         <v>15</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I14" s="0" t="n">
         <v>15</v>
@@ -1263,216 +1275,216 @@
       <c r="J14" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="L14" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="N14" s="0" t="n">
+      <c r="M14" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="O14" s="0" t="n">
         <f aca="false">IF(H14&lt;&gt;"",H14,IF(AND(I14&lt;&gt;"",J14&lt;&gt;""),(I14+J14)/2,0))</f>
         <v>18</v>
       </c>
-      <c r="O14" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D14,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E14,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F14,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G14,$A$2:$A$61,0)),0))</f>
+      <c r="P14" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D14,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E14,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F14,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G14,$A$2:$A$61,0)),0))</f>
         <v>22</v>
       </c>
-      <c r="P14" s="0" t="n">
-        <f aca="false">O14+N14</f>
+      <c r="Q14" s="0" t="n">
+        <f aca="false">P14+O14</f>
         <v>40</v>
       </c>
-      <c r="Q14" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A14)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A14)),IF(COUNTIF($E$2:$E$61,$A14)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A14)),IF(COUNTIF($F$2:$F$61,$A14)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A14)),IF(COUNTIF($G$2:$G$61,$A14)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A14)))</f>
+      <c r="R14" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A14)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A14)),IF(COUNTIF($E$2:$E$61,$A14)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A14)),IF(COUNTIF($F$2:$F$61,$A14)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A14)),IF(COUNTIF($G$2:$G$61,$A14)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A14)))</f>
         <v>40</v>
-      </c>
-      <c r="R14" s="0" t="n">
-        <f aca="false">Q14-N14</f>
-        <v>22</v>
       </c>
       <c r="S14" s="0" t="n">
         <f aca="false">R14-O14</f>
+        <v>22</v>
+      </c>
+      <c r="T14" s="0" t="n">
+        <f aca="false">S14-P14</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H15" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="N15" s="0" t="n">
+      <c r="O15" s="0" t="n">
         <f aca="false">IF(H15&lt;&gt;"",H15,IF(AND(I15&lt;&gt;"",J15&lt;&gt;""),(I15+J15)/2,0))</f>
         <v>5</v>
       </c>
-      <c r="O15" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D15,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E15,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F15,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G15,$A$2:$A$61,0)),0))</f>
+      <c r="P15" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D15,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E15,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F15,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G15,$A$2:$A$61,0)),0))</f>
         <v>40</v>
       </c>
-      <c r="P15" s="0" t="n">
-        <f aca="false">O15+N15</f>
+      <c r="Q15" s="0" t="n">
+        <f aca="false">P15+O15</f>
         <v>45</v>
       </c>
-      <c r="Q15" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A15)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A15)),IF(COUNTIF($E$2:$E$61,$A15)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A15)),IF(COUNTIF($F$2:$F$61,$A15)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A15)),IF(COUNTIF($G$2:$G$61,$A15)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A15)))</f>
+      <c r="R15" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A15)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A15)),IF(COUNTIF($E$2:$E$61,$A15)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A15)),IF(COUNTIF($F$2:$F$61,$A15)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A15)),IF(COUNTIF($G$2:$G$61,$A15)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A15)))</f>
         <v>45</v>
-      </c>
-      <c r="R15" s="0" t="n">
-        <f aca="false">Q15-N15</f>
-        <v>40</v>
       </c>
       <c r="S15" s="0" t="n">
         <f aca="false">R15-O15</f>
+        <v>40</v>
+      </c>
+      <c r="T15" s="0" t="n">
+        <f aca="false">S15-P15</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H16" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="N16" s="0" t="n">
+      <c r="O16" s="0" t="n">
         <f aca="false">IF(H16&lt;&gt;"",H16,IF(AND(I16&lt;&gt;"",J16&lt;&gt;""),(I16+J16)/2,0))</f>
         <v>10</v>
       </c>
-      <c r="O16" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D16,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E16,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F16,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G16,$A$2:$A$61,0)),0))</f>
+      <c r="P16" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D16,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E16,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F16,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G16,$A$2:$A$61,0)),0))</f>
         <v>45</v>
       </c>
-      <c r="P16" s="0" t="n">
-        <f aca="false">O16+N16</f>
+      <c r="Q16" s="0" t="n">
+        <f aca="false">P16+O16</f>
         <v>55</v>
       </c>
-      <c r="Q16" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A16)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A16)),IF(COUNTIF($E$2:$E$61,$A16)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A16)),IF(COUNTIF($F$2:$F$61,$A16)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A16)),IF(COUNTIF($G$2:$G$61,$A16)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A16)))</f>
+      <c r="R16" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A16)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A16)),IF(COUNTIF($E$2:$E$61,$A16)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A16)),IF(COUNTIF($F$2:$F$61,$A16)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A16)),IF(COUNTIF($G$2:$G$61,$A16)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A16)))</f>
         <v>55</v>
-      </c>
-      <c r="R16" s="0" t="n">
-        <f aca="false">Q16-N16</f>
-        <v>45</v>
       </c>
       <c r="S16" s="0" t="n">
         <f aca="false">R16-O16</f>
+        <v>45</v>
+      </c>
+      <c r="T16" s="0" t="n">
+        <f aca="false">S16-P16</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H17" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="N17" s="0" t="n">
+      <c r="O17" s="0" t="n">
         <f aca="false">IF(H17&lt;&gt;"",H17,IF(AND(I17&lt;&gt;"",J17&lt;&gt;""),(I17+J17)/2,0))</f>
         <v>3</v>
       </c>
-      <c r="O17" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D17,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E17,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F17,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G17,$A$2:$A$61,0)),0))</f>
+      <c r="P17" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D17,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E17,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F17,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G17,$A$2:$A$61,0)),0))</f>
         <v>32</v>
       </c>
-      <c r="P17" s="0" t="n">
-        <f aca="false">O17+N17</f>
+      <c r="Q17" s="0" t="n">
+        <f aca="false">P17+O17</f>
         <v>35</v>
       </c>
-      <c r="Q17" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A17)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A17)),IF(COUNTIF($E$2:$E$61,$A17)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A17)),IF(COUNTIF($F$2:$F$61,$A17)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A17)),IF(COUNTIF($G$2:$G$61,$A17)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A17)))</f>
+      <c r="R17" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A17)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A17)),IF(COUNTIF($E$2:$E$61,$A17)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A17)),IF(COUNTIF($F$2:$F$61,$A17)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A17)),IF(COUNTIF($G$2:$G$61,$A17)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A17)))</f>
         <v>45</v>
-      </c>
-      <c r="R17" s="0" t="n">
-        <f aca="false">Q17-N17</f>
-        <v>42</v>
       </c>
       <c r="S17" s="0" t="n">
         <f aca="false">R17-O17</f>
+        <v>42</v>
+      </c>
+      <c r="T17" s="0" t="n">
+        <f aca="false">S17-P17</f>
         <v>10</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H18" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="N18" s="0" t="n">
+      <c r="O18" s="0" t="n">
         <f aca="false">IF(H18&lt;&gt;"",H18,IF(AND(I18&lt;&gt;"",J18&lt;&gt;""),(I18+J18)/2,0))</f>
         <v>10</v>
       </c>
-      <c r="O18" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D18,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E18,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F18,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G18,$A$2:$A$61,0)),0))</f>
+      <c r="P18" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D18,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E18,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F18,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G18,$A$2:$A$61,0)),0))</f>
         <v>35</v>
       </c>
-      <c r="P18" s="0" t="n">
-        <f aca="false">O18+N18</f>
+      <c r="Q18" s="0" t="n">
+        <f aca="false">P18+O18</f>
         <v>45</v>
       </c>
-      <c r="Q18" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A18)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A18)),IF(COUNTIF($E$2:$E$61,$A18)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A18)),IF(COUNTIF($F$2:$F$61,$A18)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A18)),IF(COUNTIF($G$2:$G$61,$A18)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A18)))</f>
+      <c r="R18" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A18)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A18)),IF(COUNTIF($E$2:$E$61,$A18)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A18)),IF(COUNTIF($F$2:$F$61,$A18)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A18)),IF(COUNTIF($G$2:$G$61,$A18)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A18)))</f>
         <v>55</v>
-      </c>
-      <c r="R18" s="0" t="n">
-        <f aca="false">Q18-N18</f>
-        <v>45</v>
       </c>
       <c r="S18" s="0" t="n">
         <f aca="false">R18-O18</f>
+        <v>45</v>
+      </c>
+      <c r="T18" s="0" t="n">
+        <f aca="false">S18-P18</f>
         <v>10</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I19" s="0" t="n">
         <v>5</v>
@@ -1480,588 +1492,588 @@
       <c r="J19" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="N19" s="0" t="n">
+      <c r="O19" s="0" t="n">
         <f aca="false">IF(H19&lt;&gt;"",H19,IF(AND(I19&lt;&gt;"",J19&lt;&gt;""),(I19+J19)/2,0))</f>
         <v>6.5</v>
       </c>
-      <c r="O19" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D19,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E19,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F19,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G19,$A$2:$A$61,0)),0))</f>
+      <c r="P19" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D19,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E19,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F19,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G19,$A$2:$A$61,0)),0))</f>
         <v>55</v>
       </c>
-      <c r="P19" s="0" t="n">
-        <f aca="false">O19+N19</f>
+      <c r="Q19" s="0" t="n">
+        <f aca="false">P19+O19</f>
         <v>61.5</v>
       </c>
-      <c r="Q19" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A19)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A19)),IF(COUNTIF($E$2:$E$61,$A19)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A19)),IF(COUNTIF($F$2:$F$61,$A19)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A19)),IF(COUNTIF($G$2:$G$61,$A19)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A19)))</f>
+      <c r="R19" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A19)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A19)),IF(COUNTIF($E$2:$E$61,$A19)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A19)),IF(COUNTIF($F$2:$F$61,$A19)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A19)),IF(COUNTIF($G$2:$G$61,$A19)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A19)))</f>
         <v>65</v>
-      </c>
-      <c r="R19" s="0" t="n">
-        <f aca="false">Q19-N19</f>
-        <v>58.5</v>
       </c>
       <c r="S19" s="0" t="n">
         <f aca="false">R19-O19</f>
+        <v>58.5</v>
+      </c>
+      <c r="T19" s="0" t="n">
+        <f aca="false">S19-P19</f>
         <v>3.5</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D20" s="0" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H20" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="N20" s="0" t="n">
+      <c r="O20" s="0" t="n">
         <f aca="false">IF(H20&lt;&gt;"",H20,IF(AND(I20&lt;&gt;"",J20&lt;&gt;""),(I20+J20)/2,0))</f>
         <v>10</v>
       </c>
-      <c r="O20" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D20,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E20,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F20,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G20,$A$2:$A$61,0)),0))</f>
+      <c r="P20" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D20,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E20,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F20,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G20,$A$2:$A$61,0)),0))</f>
         <v>55</v>
       </c>
-      <c r="P20" s="0" t="n">
-        <f aca="false">O20+N20</f>
+      <c r="Q20" s="0" t="n">
+        <f aca="false">P20+O20</f>
         <v>65</v>
       </c>
-      <c r="Q20" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A20)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A20)),IF(COUNTIF($E$2:$E$61,$A20)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A20)),IF(COUNTIF($F$2:$F$61,$A20)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A20)),IF(COUNTIF($G$2:$G$61,$A20)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A20)))</f>
+      <c r="R20" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A20)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A20)),IF(COUNTIF($E$2:$E$61,$A20)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A20)),IF(COUNTIF($F$2:$F$61,$A20)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A20)),IF(COUNTIF($G$2:$G$61,$A20)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A20)))</f>
         <v>65</v>
-      </c>
-      <c r="R20" s="0" t="n">
-        <f aca="false">Q20-N20</f>
-        <v>55</v>
       </c>
       <c r="S20" s="0" t="n">
         <f aca="false">R20-O20</f>
+        <v>55</v>
+      </c>
+      <c r="T20" s="0" t="n">
+        <f aca="false">S20-P20</f>
         <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C21" s="0" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D21" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="N21" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="O21" s="0" t="n">
         <f aca="false">IF(H21&lt;&gt;"",H21,IF(AND(I21&lt;&gt;"",J21&lt;&gt;""),(I21+J21)/2,0))</f>
         <v>0</v>
       </c>
-      <c r="O21" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D21,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E21,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F21,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G21,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
-      </c>
       <c r="P21" s="0" t="n">
-        <f aca="false">O21+N21</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D21,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E21,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F21,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G21,$A$2:$A$61,0)),0))</f>
         <v>0</v>
       </c>
       <c r="Q21" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A21)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A21)),IF(COUNTIF($E$2:$E$61,$A21)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A21)),IF(COUNTIF($F$2:$F$61,$A21)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A21)),IF(COUNTIF($G$2:$G$61,$A21)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A21)))</f>
-        <v>3</v>
+        <f aca="false">P21+O21</f>
+        <v>0</v>
       </c>
       <c r="R21" s="0" t="n">
-        <f aca="false">Q21-N21</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A21)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A21)),IF(COUNTIF($E$2:$E$61,$A21)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A21)),IF(COUNTIF($F$2:$F$61,$A21)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A21)),IF(COUNTIF($G$2:$G$61,$A21)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A21)))</f>
         <v>3</v>
       </c>
       <c r="S21" s="0" t="n">
         <f aca="false">R21-O21</f>
         <v>3</v>
       </c>
+      <c r="T21" s="0" t="n">
+        <f aca="false">S21-P21</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B22" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="C22" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="D22" s="0" t="s">
         <v>62</v>
-      </c>
-      <c r="C22" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="D22" s="0" t="s">
-        <v>61</v>
       </c>
       <c r="H22" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="N22" s="0" t="n">
+      <c r="O22" s="0" t="n">
         <f aca="false">IF(H22&lt;&gt;"",H22,IF(AND(I22&lt;&gt;"",J22&lt;&gt;""),(I22+J22)/2,0))</f>
         <v>16</v>
       </c>
-      <c r="O22" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D22,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E22,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F22,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G22,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
-      </c>
       <c r="P22" s="0" t="n">
-        <f aca="false">O22+N22</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D22,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E22,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F22,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G22,$A$2:$A$61,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="Q22" s="0" t="n">
+        <f aca="false">P22+O22</f>
         <v>16</v>
       </c>
-      <c r="Q22" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A22)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A22)),IF(COUNTIF($E$2:$E$61,$A22)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A22)),IF(COUNTIF($F$2:$F$61,$A22)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A22)),IF(COUNTIF($G$2:$G$61,$A22)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A22)))</f>
+      <c r="R22" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A22)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A22)),IF(COUNTIF($E$2:$E$61,$A22)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A22)),IF(COUNTIF($F$2:$F$61,$A22)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A22)),IF(COUNTIF($G$2:$G$61,$A22)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A22)))</f>
         <v>45</v>
-      </c>
-      <c r="R22" s="0" t="n">
-        <f aca="false">Q22-N22</f>
-        <v>29</v>
       </c>
       <c r="S22" s="0" t="n">
         <f aca="false">R22-O22</f>
         <v>29</v>
       </c>
+      <c r="T22" s="0" t="n">
+        <f aca="false">S22-P22</f>
+        <v>29</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B23" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="C23" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="D23" s="0" t="s">
         <v>62</v>
-      </c>
-      <c r="C23" s="0" t="s">
-        <v>66</v>
-      </c>
-      <c r="D23" s="0" t="s">
-        <v>61</v>
       </c>
       <c r="H23" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="N23" s="0" t="n">
+      <c r="O23" s="0" t="n">
         <f aca="false">IF(H23&lt;&gt;"",H23,IF(AND(I23&lt;&gt;"",J23&lt;&gt;""),(I23+J23)/2,0))</f>
         <v>2</v>
       </c>
-      <c r="O23" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D23,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E23,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F23,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G23,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
-      </c>
       <c r="P23" s="0" t="n">
-        <f aca="false">O23+N23</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D23,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E23,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F23,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G23,$A$2:$A$61,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="Q23" s="0" t="n">
+        <f aca="false">P23+O23</f>
         <v>2</v>
       </c>
-      <c r="Q23" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A23)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A23)),IF(COUNTIF($E$2:$E$61,$A23)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A23)),IF(COUNTIF($F$2:$F$61,$A23)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A23)),IF(COUNTIF($G$2:$G$61,$A23)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A23)))</f>
+      <c r="R23" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A23)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A23)),IF(COUNTIF($E$2:$E$61,$A23)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A23)),IF(COUNTIF($F$2:$F$61,$A23)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A23)),IF(COUNTIF($G$2:$G$61,$A23)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A23)))</f>
         <v>5</v>
-      </c>
-      <c r="R23" s="0" t="n">
-        <f aca="false">Q23-N23</f>
-        <v>3</v>
       </c>
       <c r="S23" s="0" t="n">
         <f aca="false">R23-O23</f>
         <v>3</v>
       </c>
+      <c r="T23" s="0" t="n">
+        <f aca="false">S23-P23</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D24" s="0" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H24" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="N24" s="0" t="n">
+      <c r="O24" s="0" t="n">
         <f aca="false">IF(H24&lt;&gt;"",H24,IF(AND(I24&lt;&gt;"",J24&lt;&gt;""),(I24+J24)/2,0))</f>
         <v>5</v>
       </c>
-      <c r="O24" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D24,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E24,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F24,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G24,$A$2:$A$61,0)),0))</f>
+      <c r="P24" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D24,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E24,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F24,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G24,$A$2:$A$61,0)),0))</f>
         <v>2</v>
       </c>
-      <c r="P24" s="0" t="n">
-        <f aca="false">O24+N24</f>
+      <c r="Q24" s="0" t="n">
+        <f aca="false">P24+O24</f>
         <v>7</v>
       </c>
-      <c r="Q24" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A24)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A24)),IF(COUNTIF($E$2:$E$61,$A24)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A24)),IF(COUNTIF($F$2:$F$61,$A24)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A24)),IF(COUNTIF($G$2:$G$61,$A24)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A24)))</f>
+      <c r="R24" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A24)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A24)),IF(COUNTIF($E$2:$E$61,$A24)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A24)),IF(COUNTIF($F$2:$F$61,$A24)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A24)),IF(COUNTIF($G$2:$G$61,$A24)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A24)))</f>
         <v>60</v>
-      </c>
-      <c r="R24" s="0" t="n">
-        <f aca="false">Q24-N24</f>
-        <v>55</v>
       </c>
       <c r="S24" s="0" t="n">
         <f aca="false">R24-O24</f>
+        <v>55</v>
+      </c>
+      <c r="T24" s="0" t="n">
+        <f aca="false">S24-P24</f>
         <v>53</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D25" s="0" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H25" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="N25" s="0" t="n">
+      <c r="O25" s="0" t="n">
         <f aca="false">IF(H25&lt;&gt;"",H25,IF(AND(I25&lt;&gt;"",J25&lt;&gt;""),(I25+J25)/2,0))</f>
         <v>15</v>
       </c>
-      <c r="O25" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D25,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E25,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F25,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G25,$A$2:$A$61,0)),0))</f>
+      <c r="P25" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D25,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E25,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F25,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G25,$A$2:$A$61,0)),0))</f>
         <v>2</v>
       </c>
-      <c r="P25" s="0" t="n">
-        <f aca="false">O25+N25</f>
+      <c r="Q25" s="0" t="n">
+        <f aca="false">P25+O25</f>
         <v>17</v>
       </c>
-      <c r="Q25" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A25)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A25)),IF(COUNTIF($E$2:$E$61,$A25)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A25)),IF(COUNTIF($F$2:$F$61,$A25)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A25)),IF(COUNTIF($G$2:$G$61,$A25)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A25)))</f>
+      <c r="R25" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A25)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A25)),IF(COUNTIF($E$2:$E$61,$A25)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A25)),IF(COUNTIF($F$2:$F$61,$A25)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A25)),IF(COUNTIF($G$2:$G$61,$A25)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A25)))</f>
         <v>20</v>
-      </c>
-      <c r="R25" s="0" t="n">
-        <f aca="false">Q25-N25</f>
-        <v>5</v>
       </c>
       <c r="S25" s="0" t="n">
         <f aca="false">R25-O25</f>
+        <v>5</v>
+      </c>
+      <c r="T25" s="0" t="n">
+        <f aca="false">S25-P25</f>
         <v>3</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D26" s="0" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H26" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="N26" s="0" t="n">
+      <c r="O26" s="0" t="n">
         <f aca="false">IF(H26&lt;&gt;"",H26,IF(AND(I26&lt;&gt;"",J26&lt;&gt;""),(I26+J26)/2,0))</f>
         <v>5</v>
       </c>
-      <c r="O26" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D26,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E26,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F26,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G26,$A$2:$A$61,0)),0))</f>
+      <c r="P26" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D26,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E26,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F26,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G26,$A$2:$A$61,0)),0))</f>
         <v>7</v>
       </c>
-      <c r="P26" s="0" t="n">
-        <f aca="false">O26+N26</f>
+      <c r="Q26" s="0" t="n">
+        <f aca="false">P26+O26</f>
         <v>12</v>
       </c>
-      <c r="Q26" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A26)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A26)),IF(COUNTIF($E$2:$E$61,$A26)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A26)),IF(COUNTIF($F$2:$F$61,$A26)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A26)),IF(COUNTIF($G$2:$G$61,$A26)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A26)))</f>
+      <c r="R26" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A26)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A26)),IF(COUNTIF($E$2:$E$61,$A26)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A26)),IF(COUNTIF($F$2:$F$61,$A26)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A26)),IF(COUNTIF($G$2:$G$61,$A26)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A26)))</f>
         <v>65</v>
-      </c>
-      <c r="R26" s="0" t="n">
-        <f aca="false">Q26-N26</f>
-        <v>60</v>
       </c>
       <c r="S26" s="0" t="n">
         <f aca="false">R26-O26</f>
+        <v>60</v>
+      </c>
+      <c r="T26" s="0" t="n">
+        <f aca="false">S26-P26</f>
         <v>53</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H27" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="N27" s="0" t="n">
+      <c r="O27" s="0" t="n">
         <f aca="false">IF(H27&lt;&gt;"",H27,IF(AND(I27&lt;&gt;"",J27&lt;&gt;""),(I27+J27)/2,0))</f>
         <v>25</v>
       </c>
-      <c r="O27" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D27,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E27,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F27,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G27,$A$2:$A$61,0)),0))</f>
+      <c r="P27" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D27,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E27,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F27,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G27,$A$2:$A$61,0)),0))</f>
         <v>17</v>
       </c>
-      <c r="P27" s="0" t="n">
-        <f aca="false">O27+N27</f>
+      <c r="Q27" s="0" t="n">
+        <f aca="false">P27+O27</f>
         <v>42</v>
       </c>
-      <c r="Q27" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A27)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A27)),IF(COUNTIF($E$2:$E$61,$A27)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A27)),IF(COUNTIF($F$2:$F$61,$A27)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A27)),IF(COUNTIF($G$2:$G$61,$A27)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A27)))</f>
+      <c r="R27" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A27)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A27)),IF(COUNTIF($E$2:$E$61,$A27)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A27)),IF(COUNTIF($F$2:$F$61,$A27)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A27)),IF(COUNTIF($G$2:$G$61,$A27)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A27)))</f>
         <v>45</v>
-      </c>
-      <c r="R27" s="0" t="n">
-        <f aca="false">Q27-N27</f>
-        <v>20</v>
       </c>
       <c r="S27" s="0" t="n">
         <f aca="false">R27-O27</f>
+        <v>20</v>
+      </c>
+      <c r="T27" s="0" t="n">
+        <f aca="false">S27-P27</f>
         <v>3</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D28" s="0" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E28" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H28" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="N28" s="0" t="n">
+      <c r="O28" s="0" t="n">
         <f aca="false">IF(H28&lt;&gt;"",H28,IF(AND(I28&lt;&gt;"",J28&lt;&gt;""),(I28+J28)/2,0))</f>
         <v>20</v>
       </c>
-      <c r="O28" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D28,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E28,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F28,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G28,$A$2:$A$61,0)),0))</f>
+      <c r="P28" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D28,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E28,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F28,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G28,$A$2:$A$61,0)),0))</f>
         <v>17</v>
       </c>
-      <c r="P28" s="0" t="n">
-        <f aca="false">O28+N28</f>
+      <c r="Q28" s="0" t="n">
+        <f aca="false">P28+O28</f>
         <v>37</v>
       </c>
-      <c r="Q28" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A28)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A28)),IF(COUNTIF($E$2:$E$61,$A28)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A28)),IF(COUNTIF($F$2:$F$61,$A28)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A28)),IF(COUNTIF($G$2:$G$61,$A28)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A28)))</f>
+      <c r="R28" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A28)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A28)),IF(COUNTIF($E$2:$E$61,$A28)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A28)),IF(COUNTIF($F$2:$F$61,$A28)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A28)),IF(COUNTIF($G$2:$G$61,$A28)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A28)))</f>
         <v>58.5</v>
-      </c>
-      <c r="R28" s="0" t="n">
-        <f aca="false">Q28-N28</f>
-        <v>38.5</v>
       </c>
       <c r="S28" s="0" t="n">
         <f aca="false">R28-O28</f>
+        <v>38.5</v>
+      </c>
+      <c r="T28" s="0" t="n">
+        <f aca="false">S28-P28</f>
         <v>21.5</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B29" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="C29" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="D29" s="0" t="s">
         <v>77</v>
-      </c>
-      <c r="B29" s="0" t="s">
-        <v>62</v>
-      </c>
-      <c r="C29" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="D29" s="0" t="s">
-        <v>76</v>
       </c>
       <c r="H29" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="N29" s="0" t="n">
+      <c r="O29" s="0" t="n">
         <f aca="false">IF(H29&lt;&gt;"",H29,IF(AND(I29&lt;&gt;"",J29&lt;&gt;""),(I29+J29)/2,0))</f>
         <v>5</v>
       </c>
-      <c r="O29" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D29,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E29,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F29,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G29,$A$2:$A$61,0)),0))</f>
+      <c r="P29" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D29,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E29,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F29,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G29,$A$2:$A$61,0)),0))</f>
         <v>7</v>
       </c>
-      <c r="P29" s="0" t="n">
-        <f aca="false">O29+N29</f>
+      <c r="Q29" s="0" t="n">
+        <f aca="false">P29+O29</f>
         <v>12</v>
       </c>
-      <c r="Q29" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A29)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A29)),IF(COUNTIF($E$2:$E$61,$A29)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A29)),IF(COUNTIF($F$2:$F$61,$A29)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A29)),IF(COUNTIF($G$2:$G$61,$A29)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A29)))</f>
+      <c r="R29" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A29)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A29)),IF(COUNTIF($E$2:$E$61,$A29)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A29)),IF(COUNTIF($F$2:$F$61,$A29)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A29)),IF(COUNTIF($G$2:$G$61,$A29)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A29)))</f>
         <v>38.5</v>
-      </c>
-      <c r="R29" s="0" t="n">
-        <f aca="false">Q29-N29</f>
-        <v>33.5</v>
       </c>
       <c r="S29" s="0" t="n">
         <f aca="false">R29-O29</f>
+        <v>33.5</v>
+      </c>
+      <c r="T29" s="0" t="n">
+        <f aca="false">S29-P29</f>
         <v>26.5</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C30" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D30" s="0" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E30" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H30" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="N30" s="0" t="n">
+      <c r="O30" s="0" t="n">
         <f aca="false">IF(H30&lt;&gt;"",H30,IF(AND(I30&lt;&gt;"",J30&lt;&gt;""),(I30+J30)/2,0))</f>
         <v>20</v>
       </c>
-      <c r="O30" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D30,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E30,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F30,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G30,$A$2:$A$61,0)),0))</f>
+      <c r="P30" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D30,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E30,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F30,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G30,$A$2:$A$61,0)),0))</f>
         <v>42</v>
       </c>
-      <c r="P30" s="0" t="n">
-        <f aca="false">O30+N30</f>
+      <c r="Q30" s="0" t="n">
+        <f aca="false">P30+O30</f>
         <v>62</v>
       </c>
-      <c r="Q30" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A30)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A30)),IF(COUNTIF($E$2:$E$61,$A30)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A30)),IF(COUNTIF($F$2:$F$61,$A30)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A30)),IF(COUNTIF($G$2:$G$61,$A30)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A30)))</f>
+      <c r="R30" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A30)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A30)),IF(COUNTIF($E$2:$E$61,$A30)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A30)),IF(COUNTIF($F$2:$F$61,$A30)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A30)),IF(COUNTIF($G$2:$G$61,$A30)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A30)))</f>
         <v>65</v>
-      </c>
-      <c r="R30" s="0" t="n">
-        <f aca="false">Q30-N30</f>
-        <v>45</v>
       </c>
       <c r="S30" s="0" t="n">
         <f aca="false">R30-O30</f>
+        <v>45</v>
+      </c>
+      <c r="T30" s="0" t="n">
+        <f aca="false">S30-P30</f>
         <v>3</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C31" s="0" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D31" s="0" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H31" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="N31" s="0" t="n">
+      <c r="O31" s="0" t="n">
         <f aca="false">IF(H31&lt;&gt;"",H31,IF(AND(I31&lt;&gt;"",J31&lt;&gt;""),(I31+J31)/2,0))</f>
         <v>5</v>
       </c>
-      <c r="O31" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D31,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E31,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F31,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G31,$A$2:$A$61,0)),0))</f>
+      <c r="P31" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D31,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E31,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F31,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G31,$A$2:$A$61,0)),0))</f>
         <v>2</v>
       </c>
-      <c r="P31" s="0" t="n">
-        <f aca="false">O31+N31</f>
+      <c r="Q31" s="0" t="n">
+        <f aca="false">P31+O31</f>
         <v>7</v>
       </c>
-      <c r="Q31" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A31)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A31)),IF(COUNTIF($E$2:$E$61,$A31)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A31)),IF(COUNTIF($F$2:$F$61,$A31)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A31)),IF(COUNTIF($G$2:$G$61,$A31)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A31)))</f>
+      <c r="R31" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A31)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A31)),IF(COUNTIF($E$2:$E$61,$A31)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A31)),IF(COUNTIF($F$2:$F$61,$A31)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A31)),IF(COUNTIF($G$2:$G$61,$A31)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A31)))</f>
         <v>33.5</v>
-      </c>
-      <c r="R31" s="0" t="n">
-        <f aca="false">Q31-N31</f>
-        <v>28.5</v>
       </c>
       <c r="S31" s="0" t="n">
         <f aca="false">R31-O31</f>
+        <v>28.5</v>
+      </c>
+      <c r="T31" s="0" t="n">
+        <f aca="false">S31-P31</f>
         <v>26.5</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C32" s="0" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D32" s="0" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H32" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="N32" s="0" t="n">
+      <c r="O32" s="0" t="n">
         <f aca="false">IF(H32&lt;&gt;"",H32,IF(AND(I32&lt;&gt;"",J32&lt;&gt;""),(I32+J32)/2,0))</f>
         <v>5</v>
       </c>
-      <c r="O32" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D32,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E32,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F32,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G32,$A$2:$A$61,0)),0))</f>
+      <c r="P32" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D32,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E32,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F32,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G32,$A$2:$A$61,0)),0))</f>
         <v>7</v>
       </c>
-      <c r="P32" s="0" t="n">
-        <f aca="false">O32+N32</f>
+      <c r="Q32" s="0" t="n">
+        <f aca="false">P32+O32</f>
         <v>12</v>
       </c>
-      <c r="Q32" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A32)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A32)),IF(COUNTIF($E$2:$E$61,$A32)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A32)),IF(COUNTIF($F$2:$F$61,$A32)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A32)),IF(COUNTIF($G$2:$G$61,$A32)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A32)))</f>
+      <c r="R32" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A32)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A32)),IF(COUNTIF($E$2:$E$61,$A32)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A32)),IF(COUNTIF($F$2:$F$61,$A32)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A32)),IF(COUNTIF($G$2:$G$61,$A32)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A32)))</f>
         <v>65</v>
-      </c>
-      <c r="R32" s="0" t="n">
-        <f aca="false">Q32-N32</f>
-        <v>60</v>
       </c>
       <c r="S32" s="0" t="n">
         <f aca="false">R32-O32</f>
+        <v>60</v>
+      </c>
+      <c r="T32" s="0" t="n">
+        <f aca="false">S32-P32</f>
         <v>53</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C33" s="0" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D33" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I33" s="0" t="n">
         <v>5</v>
@@ -2069,292 +2081,292 @@
       <c r="J33" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="N33" s="0" t="n">
+      <c r="O33" s="0" t="n">
         <f aca="false">IF(H33&lt;&gt;"",H33,IF(AND(I33&lt;&gt;"",J33&lt;&gt;""),(I33+J33)/2,0))</f>
         <v>6.5</v>
       </c>
-      <c r="O33" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D33,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E33,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F33,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G33,$A$2:$A$61,0)),0))</f>
+      <c r="P33" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D33,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E33,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F33,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G33,$A$2:$A$61,0)),0))</f>
         <v>42</v>
       </c>
-      <c r="P33" s="0" t="n">
-        <f aca="false">O33+N33</f>
+      <c r="Q33" s="0" t="n">
+        <f aca="false">P33+O33</f>
         <v>48.5</v>
       </c>
-      <c r="Q33" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A33)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A33)),IF(COUNTIF($E$2:$E$61,$A33)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A33)),IF(COUNTIF($F$2:$F$61,$A33)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A33)),IF(COUNTIF($G$2:$G$61,$A33)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A33)))</f>
+      <c r="R33" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A33)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A33)),IF(COUNTIF($E$2:$E$61,$A33)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A33)),IF(COUNTIF($F$2:$F$61,$A33)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A33)),IF(COUNTIF($G$2:$G$61,$A33)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A33)))</f>
         <v>65</v>
-      </c>
-      <c r="R33" s="0" t="n">
-        <f aca="false">Q33-N33</f>
-        <v>58.5</v>
       </c>
       <c r="S33" s="0" t="n">
         <f aca="false">R33-O33</f>
+        <v>58.5</v>
+      </c>
+      <c r="T33" s="0" t="n">
+        <f aca="false">S33-P33</f>
         <v>16.5</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C34" s="0" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D34" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="N34" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="O34" s="0" t="n">
         <f aca="false">IF(H34&lt;&gt;"",H34,IF(AND(I34&lt;&gt;"",J34&lt;&gt;""),(I34+J34)/2,0))</f>
         <v>0</v>
       </c>
-      <c r="O34" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D34,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E34,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F34,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G34,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
-      </c>
       <c r="P34" s="0" t="n">
-        <f aca="false">O34+N34</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D34,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E34,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F34,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G34,$A$2:$A$61,0)),0))</f>
         <v>0</v>
       </c>
       <c r="Q34" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A34)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A34)),IF(COUNTIF($E$2:$E$61,$A34)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A34)),IF(COUNTIF($F$2:$F$61,$A34)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A34)),IF(COUNTIF($G$2:$G$61,$A34)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A34)))</f>
-        <v>26.5</v>
+        <f aca="false">P34+O34</f>
+        <v>0</v>
       </c>
       <c r="R34" s="0" t="n">
-        <f aca="false">Q34-N34</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A34)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A34)),IF(COUNTIF($E$2:$E$61,$A34)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A34)),IF(COUNTIF($F$2:$F$61,$A34)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A34)),IF(COUNTIF($G$2:$G$61,$A34)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A34)))</f>
         <v>26.5</v>
       </c>
       <c r="S34" s="0" t="n">
         <f aca="false">R34-O34</f>
         <v>26.5</v>
       </c>
+      <c r="T34" s="0" t="n">
+        <f aca="false">S34-P34</f>
+        <v>26.5</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B35" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="C35" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="D35" s="0" t="s">
         <v>87</v>
-      </c>
-      <c r="C35" s="0" t="s">
-        <v>90</v>
-      </c>
-      <c r="D35" s="0" t="s">
-        <v>86</v>
       </c>
       <c r="H35" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="N35" s="0" t="n">
+      <c r="O35" s="0" t="n">
         <f aca="false">IF(H35&lt;&gt;"",H35,IF(AND(I35&lt;&gt;"",J35&lt;&gt;""),(I35+J35)/2,0))</f>
         <v>3</v>
       </c>
-      <c r="O35" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D35,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E35,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F35,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G35,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
-      </c>
       <c r="P35" s="0" t="n">
-        <f aca="false">O35+N35</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D35,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E35,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F35,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G35,$A$2:$A$61,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="Q35" s="0" t="n">
+        <f aca="false">P35+O35</f>
         <v>3</v>
       </c>
-      <c r="Q35" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A35)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A35)),IF(COUNTIF($E$2:$E$61,$A35)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A35)),IF(COUNTIF($F$2:$F$61,$A35)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A35)),IF(COUNTIF($G$2:$G$61,$A35)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A35)))</f>
+      <c r="R35" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A35)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A35)),IF(COUNTIF($E$2:$E$61,$A35)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A35)),IF(COUNTIF($F$2:$F$61,$A35)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A35)),IF(COUNTIF($G$2:$G$61,$A35)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A35)))</f>
         <v>29.5</v>
-      </c>
-      <c r="R35" s="0" t="n">
-        <f aca="false">Q35-N35</f>
-        <v>26.5</v>
       </c>
       <c r="S35" s="0" t="n">
         <f aca="false">R35-O35</f>
         <v>26.5</v>
       </c>
+      <c r="T35" s="0" t="n">
+        <f aca="false">S35-P35</f>
+        <v>26.5</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B36" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="C36" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="D36" s="0" t="s">
         <v>87</v>
-      </c>
-      <c r="C36" s="0" t="s">
-        <v>92</v>
-      </c>
-      <c r="D36" s="0" t="s">
-        <v>86</v>
       </c>
       <c r="H36" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="N36" s="0" t="n">
+      <c r="O36" s="0" t="n">
         <f aca="false">IF(H36&lt;&gt;"",H36,IF(AND(I36&lt;&gt;"",J36&lt;&gt;""),(I36+J36)/2,0))</f>
         <v>10</v>
       </c>
-      <c r="O36" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D36,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E36,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F36,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G36,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
-      </c>
       <c r="P36" s="0" t="n">
-        <f aca="false">O36+N36</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D36,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E36,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F36,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G36,$A$2:$A$61,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="Q36" s="0" t="n">
+        <f aca="false">P36+O36</f>
         <v>10</v>
       </c>
-      <c r="Q36" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A36)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A36)),IF(COUNTIF($E$2:$E$61,$A36)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A36)),IF(COUNTIF($F$2:$F$61,$A36)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A36)),IF(COUNTIF($G$2:$G$61,$A36)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A36)))</f>
+      <c r="R36" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A36)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A36)),IF(COUNTIF($E$2:$E$61,$A36)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A36)),IF(COUNTIF($F$2:$F$61,$A36)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A36)),IF(COUNTIF($G$2:$G$61,$A36)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A36)))</f>
         <v>45</v>
-      </c>
-      <c r="R36" s="0" t="n">
-        <f aca="false">Q36-N36</f>
-        <v>35</v>
       </c>
       <c r="S36" s="0" t="n">
         <f aca="false">R36-O36</f>
         <v>35</v>
       </c>
+      <c r="T36" s="0" t="n">
+        <f aca="false">S36-P36</f>
+        <v>35</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B37" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="C37" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="D37" s="0" t="s">
         <v>87</v>
-      </c>
-      <c r="C37" s="0" t="s">
-        <v>94</v>
-      </c>
-      <c r="D37" s="0" t="s">
-        <v>86</v>
       </c>
       <c r="H37" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="N37" s="0" t="n">
+      <c r="O37" s="0" t="n">
         <f aca="false">IF(H37&lt;&gt;"",H37,IF(AND(I37&lt;&gt;"",J37&lt;&gt;""),(I37+J37)/2,0))</f>
         <v>15</v>
       </c>
-      <c r="O37" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D37,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E37,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F37,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G37,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
-      </c>
       <c r="P37" s="0" t="n">
-        <f aca="false">O37+N37</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D37,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E37,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F37,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G37,$A$2:$A$61,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="Q37" s="0" t="n">
+        <f aca="false">P37+O37</f>
         <v>15</v>
       </c>
-      <c r="Q37" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A37)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A37)),IF(COUNTIF($E$2:$E$61,$A37)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A37)),IF(COUNTIF($F$2:$F$61,$A37)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A37)),IF(COUNTIF($G$2:$G$61,$A37)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A37)))</f>
+      <c r="R37" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A37)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A37)),IF(COUNTIF($E$2:$E$61,$A37)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A37)),IF(COUNTIF($F$2:$F$61,$A37)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A37)),IF(COUNTIF($G$2:$G$61,$A37)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A37)))</f>
         <v>45</v>
-      </c>
-      <c r="R37" s="0" t="n">
-        <f aca="false">Q37-N37</f>
-        <v>30</v>
       </c>
       <c r="S37" s="0" t="n">
         <f aca="false">R37-O37</f>
         <v>30</v>
       </c>
+      <c r="T37" s="0" t="n">
+        <f aca="false">S37-P37</f>
+        <v>30</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B38" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="C38" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="D38" s="0" t="s">
         <v>87</v>
-      </c>
-      <c r="C38" s="0" t="s">
-        <v>96</v>
-      </c>
-      <c r="D38" s="0" t="s">
-        <v>86</v>
       </c>
       <c r="H38" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="N38" s="0" t="n">
+      <c r="O38" s="0" t="n">
         <f aca="false">IF(H38&lt;&gt;"",H38,IF(AND(I38&lt;&gt;"",J38&lt;&gt;""),(I38+J38)/2,0))</f>
         <v>15</v>
       </c>
-      <c r="O38" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D38,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E38,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F38,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G38,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
-      </c>
       <c r="P38" s="0" t="n">
-        <f aca="false">O38+N38</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D38,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E38,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F38,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G38,$A$2:$A$61,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="Q38" s="0" t="n">
+        <f aca="false">P38+O38</f>
         <v>15</v>
       </c>
-      <c r="Q38" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A38)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A38)),IF(COUNTIF($E$2:$E$61,$A38)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A38)),IF(COUNTIF($F$2:$F$61,$A38)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A38)),IF(COUNTIF($G$2:$G$61,$A38)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A38)))</f>
+      <c r="R38" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A38)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A38)),IF(COUNTIF($E$2:$E$61,$A38)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A38)),IF(COUNTIF($F$2:$F$61,$A38)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A38)),IF(COUNTIF($G$2:$G$61,$A38)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A38)))</f>
         <v>45</v>
-      </c>
-      <c r="R38" s="0" t="n">
-        <f aca="false">Q38-N38</f>
-        <v>30</v>
       </c>
       <c r="S38" s="0" t="n">
         <f aca="false">R38-O38</f>
         <v>30</v>
       </c>
+      <c r="T38" s="0" t="n">
+        <f aca="false">S38-P38</f>
+        <v>30</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C39" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D39" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E39" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F39" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H39" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="N39" s="0" t="n">
+      <c r="O39" s="0" t="n">
         <f aca="false">IF(H39&lt;&gt;"",H39,IF(AND(I39&lt;&gt;"",J39&lt;&gt;""),(I39+J39)/2,0))</f>
         <v>5</v>
       </c>
-      <c r="O39" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D39,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E39,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F39,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G39,$A$2:$A$61,0)),0))</f>
+      <c r="P39" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D39,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E39,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F39,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G39,$A$2:$A$61,0)),0))</f>
         <v>15</v>
       </c>
-      <c r="P39" s="0" t="n">
-        <f aca="false">O39+N39</f>
+      <c r="Q39" s="0" t="n">
+        <f aca="false">P39+O39</f>
         <v>20</v>
       </c>
-      <c r="Q39" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A39)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A39)),IF(COUNTIF($E$2:$E$61,$A39)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A39)),IF(COUNTIF($F$2:$F$61,$A39)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A39)),IF(COUNTIF($G$2:$G$61,$A39)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A39)))</f>
+      <c r="R39" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A39)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A39)),IF(COUNTIF($E$2:$E$61,$A39)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A39)),IF(COUNTIF($F$2:$F$61,$A39)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A39)),IF(COUNTIF($G$2:$G$61,$A39)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A39)))</f>
         <v>50</v>
-      </c>
-      <c r="R39" s="0" t="n">
-        <f aca="false">Q39-N39</f>
-        <v>45</v>
       </c>
       <c r="S39" s="0" t="n">
         <f aca="false">R39-O39</f>
+        <v>45</v>
+      </c>
+      <c r="T39" s="0" t="n">
+        <f aca="false">S39-P39</f>
         <v>30</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C40" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D40" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I40" s="0" t="n">
         <v>5</v>
@@ -2362,84 +2374,84 @@
       <c r="J40" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="N40" s="0" t="n">
+      <c r="O40" s="0" t="n">
         <f aca="false">IF(H40&lt;&gt;"",H40,IF(AND(I40&lt;&gt;"",J40&lt;&gt;""),(I40+J40)/2,0))</f>
         <v>6.5</v>
       </c>
-      <c r="O40" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D40,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E40,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F40,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G40,$A$2:$A$61,0)),0))</f>
+      <c r="P40" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D40,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E40,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F40,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G40,$A$2:$A$61,0)),0))</f>
         <v>3</v>
       </c>
-      <c r="P40" s="0" t="n">
-        <f aca="false">O40+N40</f>
+      <c r="Q40" s="0" t="n">
+        <f aca="false">P40+O40</f>
         <v>9.5</v>
       </c>
-      <c r="Q40" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A40)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A40)),IF(COUNTIF($E$2:$E$61,$A40)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A40)),IF(COUNTIF($F$2:$F$61,$A40)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A40)),IF(COUNTIF($G$2:$G$61,$A40)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A40)))</f>
+      <c r="R40" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A40)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A40)),IF(COUNTIF($E$2:$E$61,$A40)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A40)),IF(COUNTIF($F$2:$F$61,$A40)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A40)),IF(COUNTIF($G$2:$G$61,$A40)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A40)))</f>
         <v>36</v>
-      </c>
-      <c r="R40" s="0" t="n">
-        <f aca="false">Q40-N40</f>
-        <v>29.5</v>
       </c>
       <c r="S40" s="0" t="n">
         <f aca="false">R40-O40</f>
+        <v>29.5</v>
+      </c>
+      <c r="T40" s="0" t="n">
+        <f aca="false">S40-P40</f>
         <v>26.5</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C41" s="0" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D41" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H41" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="N41" s="0" t="n">
+      <c r="O41" s="0" t="n">
         <f aca="false">IF(H41&lt;&gt;"",H41,IF(AND(I41&lt;&gt;"",J41&lt;&gt;""),(I41+J41)/2,0))</f>
         <v>5</v>
       </c>
-      <c r="O41" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D41,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E41,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F41,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G41,$A$2:$A$61,0)),0))</f>
+      <c r="P41" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D41,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E41,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F41,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G41,$A$2:$A$61,0)),0))</f>
         <v>15</v>
       </c>
-      <c r="P41" s="0" t="n">
-        <f aca="false">O41+N41</f>
+      <c r="Q41" s="0" t="n">
+        <f aca="false">P41+O41</f>
         <v>20</v>
       </c>
-      <c r="Q41" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A41)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A41)),IF(COUNTIF($E$2:$E$61,$A41)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A41)),IF(COUNTIF($F$2:$F$61,$A41)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A41)),IF(COUNTIF($G$2:$G$61,$A41)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A41)))</f>
+      <c r="R41" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A41)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A41)),IF(COUNTIF($E$2:$E$61,$A41)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A41)),IF(COUNTIF($F$2:$F$61,$A41)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A41)),IF(COUNTIF($G$2:$G$61,$A41)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A41)))</f>
         <v>82.25</v>
-      </c>
-      <c r="R41" s="0" t="n">
-        <f aca="false">Q41-N41</f>
-        <v>77.25</v>
       </c>
       <c r="S41" s="0" t="n">
         <f aca="false">R41-O41</f>
+        <v>77.25</v>
+      </c>
+      <c r="T41" s="0" t="n">
+        <f aca="false">S41-P41</f>
         <v>62.25</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C42" s="0" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D42" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I42" s="0" t="n">
         <v>20</v>
@@ -2447,342 +2459,342 @@
       <c r="J42" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="L42" s="0" t="s">
-        <v>103</v>
-      </c>
-      <c r="N42" s="0" t="n">
+      <c r="M42" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="O42" s="0" t="n">
         <f aca="false">IF(H42&lt;&gt;"",H42,IF(AND(I42&lt;&gt;"",J42&lt;&gt;""),(I42+J42)/2,0))</f>
         <v>24</v>
       </c>
-      <c r="O42" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D42,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E42,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F42,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G42,$A$2:$A$61,0)),0))</f>
+      <c r="P42" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D42,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E42,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F42,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G42,$A$2:$A$61,0)),0))</f>
         <v>9.5</v>
       </c>
-      <c r="P42" s="0" t="n">
-        <f aca="false">O42+N42</f>
+      <c r="Q42" s="0" t="n">
+        <f aca="false">P42+O42</f>
         <v>33.5</v>
       </c>
-      <c r="Q42" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A42)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A42)),IF(COUNTIF($E$2:$E$61,$A42)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A42)),IF(COUNTIF($F$2:$F$61,$A42)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A42)),IF(COUNTIF($G$2:$G$61,$A42)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A42)))</f>
+      <c r="R42" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A42)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A42)),IF(COUNTIF($E$2:$E$61,$A42)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A42)),IF(COUNTIF($F$2:$F$61,$A42)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A42)),IF(COUNTIF($G$2:$G$61,$A42)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A42)))</f>
         <v>60</v>
-      </c>
-      <c r="R42" s="0" t="n">
-        <f aca="false">Q42-N42</f>
-        <v>36</v>
       </c>
       <c r="S42" s="0" t="n">
         <f aca="false">R42-O42</f>
+        <v>36</v>
+      </c>
+      <c r="T42" s="0" t="n">
+        <f aca="false">S42-P42</f>
         <v>26.5</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C43" s="0" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D43" s="0" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H43" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="N43" s="0" t="n">
+      <c r="O43" s="0" t="n">
         <f aca="false">IF(H43&lt;&gt;"",H43,IF(AND(I43&lt;&gt;"",J43&lt;&gt;""),(I43+J43)/2,0))</f>
         <v>5</v>
       </c>
-      <c r="O43" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D43,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E43,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F43,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G43,$A$2:$A$61,0)),0))</f>
+      <c r="P43" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D43,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E43,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F43,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G43,$A$2:$A$61,0)),0))</f>
         <v>33.5</v>
       </c>
-      <c r="P43" s="0" t="n">
-        <f aca="false">O43+N43</f>
+      <c r="Q43" s="0" t="n">
+        <f aca="false">P43+O43</f>
         <v>38.5</v>
       </c>
-      <c r="Q43" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A43)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A43)),IF(COUNTIF($E$2:$E$61,$A43)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A43)),IF(COUNTIF($F$2:$F$61,$A43)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A43)),IF(COUNTIF($G$2:$G$61,$A43)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A43)))</f>
+      <c r="R43" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A43)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A43)),IF(COUNTIF($E$2:$E$61,$A43)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A43)),IF(COUNTIF($F$2:$F$61,$A43)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A43)),IF(COUNTIF($G$2:$G$61,$A43)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A43)))</f>
         <v>65</v>
-      </c>
-      <c r="R43" s="0" t="n">
-        <f aca="false">Q43-N43</f>
-        <v>60</v>
       </c>
       <c r="S43" s="0" t="n">
         <f aca="false">R43-O43</f>
+        <v>60</v>
+      </c>
+      <c r="T43" s="0" t="n">
+        <f aca="false">S43-P43</f>
         <v>26.5</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C44" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D44" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E44" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H44" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="N44" s="0" t="n">
+      <c r="O44" s="0" t="n">
         <f aca="false">IF(H44&lt;&gt;"",H44,IF(AND(I44&lt;&gt;"",J44&lt;&gt;""),(I44+J44)/2,0))</f>
         <v>9</v>
       </c>
-      <c r="O44" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D44,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E44,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F44,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G44,$A$2:$A$61,0)),0))</f>
+      <c r="P44" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D44,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E44,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F44,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G44,$A$2:$A$61,0)),0))</f>
         <v>15</v>
       </c>
-      <c r="P44" s="0" t="n">
-        <f aca="false">O44+N44</f>
+      <c r="Q44" s="0" t="n">
+        <f aca="false">P44+O44</f>
         <v>24</v>
       </c>
-      <c r="Q44" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A44)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A44)),IF(COUNTIF($E$2:$E$61,$A44)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A44)),IF(COUNTIF($F$2:$F$61,$A44)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A44)),IF(COUNTIF($G$2:$G$61,$A44)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A44)))</f>
+      <c r="R44" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A44)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A44)),IF(COUNTIF($E$2:$E$61,$A44)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A44)),IF(COUNTIF($F$2:$F$61,$A44)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A44)),IF(COUNTIF($G$2:$G$61,$A44)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A44)))</f>
         <v>55</v>
-      </c>
-      <c r="R44" s="0" t="n">
-        <f aca="false">Q44-N44</f>
-        <v>46</v>
       </c>
       <c r="S44" s="0" t="n">
         <f aca="false">R44-O44</f>
+        <v>46</v>
+      </c>
+      <c r="T44" s="0" t="n">
+        <f aca="false">S44-P44</f>
         <v>31</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C45" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D45" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H45" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="N45" s="0" t="n">
+      <c r="O45" s="0" t="n">
         <f aca="false">IF(H45&lt;&gt;"",H45,IF(AND(I45&lt;&gt;"",J45&lt;&gt;""),(I45+J45)/2,0))</f>
         <v>3</v>
       </c>
-      <c r="O45" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D45,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E45,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F45,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G45,$A$2:$A$61,0)),0))</f>
+      <c r="P45" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D45,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E45,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F45,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G45,$A$2:$A$61,0)),0))</f>
         <v>15</v>
       </c>
-      <c r="P45" s="0" t="n">
-        <f aca="false">O45+N45</f>
+      <c r="Q45" s="0" t="n">
+        <f aca="false">P45+O45</f>
         <v>18</v>
       </c>
-      <c r="Q45" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A45)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A45)),IF(COUNTIF($E$2:$E$61,$A45)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A45)),IF(COUNTIF($F$2:$F$61,$A45)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A45)),IF(COUNTIF($G$2:$G$61,$A45)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A45)))</f>
+      <c r="R45" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A45)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A45)),IF(COUNTIF($E$2:$E$61,$A45)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A45)),IF(COUNTIF($F$2:$F$61,$A45)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A45)),IF(COUNTIF($G$2:$G$61,$A45)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A45)))</f>
         <v>82.25</v>
-      </c>
-      <c r="R45" s="0" t="n">
-        <f aca="false">Q45-N45</f>
-        <v>79.25</v>
       </c>
       <c r="S45" s="0" t="n">
         <f aca="false">R45-O45</f>
+        <v>79.25</v>
+      </c>
+      <c r="T45" s="0" t="n">
+        <f aca="false">S45-P45</f>
         <v>64.25</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C46" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H46" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="N46" s="0" t="n">
+      <c r="O46" s="0" t="n">
         <f aca="false">IF(H46&lt;&gt;"",H46,IF(AND(I46&lt;&gt;"",J46&lt;&gt;""),(I46+J46)/2,0))</f>
         <v>5</v>
       </c>
-      <c r="O46" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D46,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E46,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F46,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G46,$A$2:$A$61,0)),0))</f>
+      <c r="P46" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D46,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E46,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F46,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G46,$A$2:$A$61,0)),0))</f>
         <v>20</v>
       </c>
-      <c r="P46" s="0" t="n">
-        <f aca="false">O46+N46</f>
+      <c r="Q46" s="0" t="n">
+        <f aca="false">P46+O46</f>
         <v>25</v>
       </c>
-      <c r="Q46" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A46)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A46)),IF(COUNTIF($E$2:$E$61,$A46)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A46)),IF(COUNTIF($F$2:$F$61,$A46)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A46)),IF(COUNTIF($G$2:$G$61,$A46)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A46)))</f>
+      <c r="R46" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A46)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A46)),IF(COUNTIF($E$2:$E$61,$A46)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A46)),IF(COUNTIF($F$2:$F$61,$A46)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A46)),IF(COUNTIF($G$2:$G$61,$A46)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A46)))</f>
         <v>55</v>
-      </c>
-      <c r="R46" s="0" t="n">
-        <f aca="false">Q46-N46</f>
-        <v>50</v>
       </c>
       <c r="S46" s="0" t="n">
         <f aca="false">R46-O46</f>
+        <v>50</v>
+      </c>
+      <c r="T46" s="0" t="n">
+        <f aca="false">S46-P46</f>
         <v>30</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C47" s="0" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D47" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H47" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="N47" s="0" t="n">
+      <c r="O47" s="0" t="n">
         <f aca="false">IF(H47&lt;&gt;"",H47,IF(AND(I47&lt;&gt;"",J47&lt;&gt;""),(I47+J47)/2,0))</f>
         <v>10</v>
       </c>
-      <c r="O47" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D47,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E47,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F47,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G47,$A$2:$A$61,0)),0))</f>
+      <c r="P47" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D47,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E47,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F47,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G47,$A$2:$A$61,0)),0))</f>
         <v>25</v>
       </c>
-      <c r="P47" s="0" t="n">
-        <f aca="false">O47+N47</f>
+      <c r="Q47" s="0" t="n">
+        <f aca="false">P47+O47</f>
         <v>35</v>
       </c>
-      <c r="Q47" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A47)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A47)),IF(COUNTIF($E$2:$E$61,$A47)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A47)),IF(COUNTIF($F$2:$F$61,$A47)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A47)),IF(COUNTIF($G$2:$G$61,$A47)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A47)))</f>
+      <c r="R47" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A47)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A47)),IF(COUNTIF($E$2:$E$61,$A47)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A47)),IF(COUNTIF($F$2:$F$61,$A47)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A47)),IF(COUNTIF($G$2:$G$61,$A47)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A47)))</f>
         <v>65</v>
-      </c>
-      <c r="R47" s="0" t="n">
-        <f aca="false">Q47-N47</f>
-        <v>55</v>
       </c>
       <c r="S47" s="0" t="n">
         <f aca="false">R47-O47</f>
+        <v>55</v>
+      </c>
+      <c r="T47" s="0" t="n">
+        <f aca="false">S47-P47</f>
         <v>30</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B48" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C48" s="0" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D48" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H48" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="N48" s="0" t="n">
+      <c r="O48" s="0" t="n">
         <f aca="false">IF(H48&lt;&gt;"",H48,IF(AND(I48&lt;&gt;"",J48&lt;&gt;""),(I48+J48)/2,0))</f>
         <v>10</v>
       </c>
-      <c r="O48" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D48,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E48,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F48,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G48,$A$2:$A$61,0)),0))</f>
+      <c r="P48" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D48,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E48,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F48,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G48,$A$2:$A$61,0)),0))</f>
         <v>25</v>
       </c>
-      <c r="P48" s="0" t="n">
-        <f aca="false">O48+N48</f>
+      <c r="Q48" s="0" t="n">
+        <f aca="false">P48+O48</f>
         <v>35</v>
       </c>
-      <c r="Q48" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A48)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A48)),IF(COUNTIF($E$2:$E$61,$A48)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A48)),IF(COUNTIF($F$2:$F$61,$A48)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A48)),IF(COUNTIF($G$2:$G$61,$A48)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A48)))</f>
+      <c r="R48" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A48)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A48)),IF(COUNTIF($E$2:$E$61,$A48)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A48)),IF(COUNTIF($F$2:$F$61,$A48)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A48)),IF(COUNTIF($G$2:$G$61,$A48)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A48)))</f>
         <v>65</v>
-      </c>
-      <c r="R48" s="0" t="n">
-        <f aca="false">Q48-N48</f>
-        <v>55</v>
       </c>
       <c r="S48" s="0" t="n">
         <f aca="false">R48-O48</f>
+        <v>55</v>
+      </c>
+      <c r="T48" s="0" t="n">
+        <f aca="false">S48-P48</f>
         <v>30</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B49" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C49" s="0" t="s">
-        <v>115</v>
-      </c>
-      <c r="M49" s="2" t="n">
+        <v>116</v>
+      </c>
+      <c r="N49" s="2" t="n">
         <v>40080</v>
       </c>
-      <c r="N49" s="0" t="n">
+      <c r="O49" s="0" t="n">
         <f aca="false">IF(H49&lt;&gt;"",H49,IF(AND(I49&lt;&gt;"",J49&lt;&gt;""),(I49+J49)/2,0))</f>
         <v>0</v>
       </c>
-      <c r="O49" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D49,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E49,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F49,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G49,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
-      </c>
       <c r="P49" s="0" t="n">
-        <f aca="false">O49+N49</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D49,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E49,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F49,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G49,$A$2:$A$61,0)),0))</f>
         <v>0</v>
       </c>
       <c r="Q49" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A49)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A49)),IF(COUNTIF($E$2:$E$61,$A49)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A49)),IF(COUNTIF($F$2:$F$61,$A49)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A49)),IF(COUNTIF($G$2:$G$61,$A49)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A49)))</f>
+        <f aca="false">P49+O49</f>
         <v>0</v>
       </c>
       <c r="R49" s="0" t="n">
-        <f aca="false">Q49-N49</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A49)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A49)),IF(COUNTIF($E$2:$E$61,$A49)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A49)),IF(COUNTIF($F$2:$F$61,$A49)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A49)),IF(COUNTIF($G$2:$G$61,$A49)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A49)))</f>
         <v>0</v>
       </c>
       <c r="S49" s="0" t="n">
         <f aca="false">R49-O49</f>
         <v>0</v>
       </c>
+      <c r="T49" s="0" t="n">
+        <f aca="false">S49-P49</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C50" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D50" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I50" s="0" t="n">
         <v>5</v>
@@ -2790,81 +2802,81 @@
       <c r="J50" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="N50" s="0" t="n">
+      <c r="O50" s="0" t="n">
         <f aca="false">IF(H50&lt;&gt;"",H50,IF(AND(I50&lt;&gt;"",J50&lt;&gt;""),(I50+J50)/2,0))</f>
         <v>7.5</v>
       </c>
-      <c r="O50" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D50,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E50,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F50,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G50,$A$2:$A$61,0)),0))</f>
+      <c r="P50" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D50,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E50,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F50,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G50,$A$2:$A$61,0)),0))</f>
         <v>74</v>
       </c>
-      <c r="P50" s="0" t="n">
-        <f aca="false">O50+N50</f>
+      <c r="Q50" s="0" t="n">
+        <f aca="false">P50+O50</f>
         <v>81.5</v>
       </c>
-      <c r="Q50" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A50)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A50)),IF(COUNTIF($E$2:$E$61,$A50)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A50)),IF(COUNTIF($F$2:$F$61,$A50)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A50)),IF(COUNTIF($G$2:$G$61,$A50)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A50)))</f>
+      <c r="R50" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A50)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A50)),IF(COUNTIF($E$2:$E$61,$A50)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A50)),IF(COUNTIF($F$2:$F$61,$A50)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A50)),IF(COUNTIF($G$2:$G$61,$A50)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A50)))</f>
         <v>81.5</v>
-      </c>
-      <c r="R50" s="0" t="n">
-        <f aca="false">Q50-N50</f>
-        <v>74</v>
       </c>
       <c r="S50" s="0" t="n">
         <f aca="false">R50-O50</f>
+        <v>74</v>
+      </c>
+      <c r="T50" s="0" t="n">
+        <f aca="false">S50-P50</f>
         <v>0</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B51" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C51" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D51" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="N51" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="O51" s="0" t="n">
         <f aca="false">IF(H51&lt;&gt;"",H51,IF(AND(I51&lt;&gt;"",J51&lt;&gt;""),(I51+J51)/2,0))</f>
         <v>0</v>
       </c>
-      <c r="O51" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D51,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E51,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F51,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G51,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
-      </c>
       <c r="P51" s="0" t="n">
-        <f aca="false">O51+N51</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D51,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E51,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F51,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G51,$A$2:$A$61,0)),0))</f>
         <v>0</v>
       </c>
       <c r="Q51" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A51)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A51)),IF(COUNTIF($E$2:$E$61,$A51)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A51)),IF(COUNTIF($F$2:$F$61,$A51)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A51)),IF(COUNTIF($G$2:$G$61,$A51)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A51)))</f>
-        <v>48</v>
+        <f aca="false">P51+O51</f>
+        <v>0</v>
       </c>
       <c r="R51" s="0" t="n">
-        <f aca="false">Q51-N51</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A51)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A51)),IF(COUNTIF($E$2:$E$61,$A51)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A51)),IF(COUNTIF($F$2:$F$61,$A51)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A51)),IF(COUNTIF($G$2:$G$61,$A51)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A51)))</f>
         <v>48</v>
       </c>
       <c r="S51" s="0" t="n">
         <f aca="false">R51-O51</f>
         <v>48</v>
       </c>
+      <c r="T51" s="0" t="n">
+        <f aca="false">S51-P51</f>
+        <v>48</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B52" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C52" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D52" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I52" s="0" t="n">
         <v>14</v>
@@ -2872,87 +2884,87 @@
       <c r="J52" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="N52" s="0" t="n">
+      <c r="O52" s="0" t="n">
         <f aca="false">IF(H52&lt;&gt;"",H52,IF(AND(I52&lt;&gt;"",J52&lt;&gt;""),(I52+J52)/2,0))</f>
         <v>21</v>
       </c>
-      <c r="O52" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D52,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E52,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F52,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G52,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
-      </c>
       <c r="P52" s="0" t="n">
-        <f aca="false">O52+N52</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D52,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E52,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F52,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G52,$A$2:$A$61,0)),0))</f>
+        <v>0</v>
+      </c>
+      <c r="Q52" s="0" t="n">
+        <f aca="false">P52+O52</f>
         <v>21</v>
       </c>
-      <c r="Q52" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A52)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A52)),IF(COUNTIF($E$2:$E$61,$A52)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A52)),IF(COUNTIF($F$2:$F$61,$A52)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A52)),IF(COUNTIF($G$2:$G$61,$A52)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A52)))</f>
+      <c r="R52" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A52)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A52)),IF(COUNTIF($E$2:$E$61,$A52)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A52)),IF(COUNTIF($F$2:$F$61,$A52)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A52)),IF(COUNTIF($G$2:$G$61,$A52)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A52)))</f>
         <v>69</v>
-      </c>
-      <c r="R52" s="0" t="n">
-        <f aca="false">Q52-N52</f>
-        <v>48</v>
       </c>
       <c r="S52" s="0" t="n">
         <f aca="false">R52-O52</f>
         <v>48</v>
       </c>
+      <c r="T52" s="0" t="n">
+        <f aca="false">S52-P52</f>
+        <v>48</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B53" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C53" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D53" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E53" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H53" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="N53" s="0" t="n">
+      <c r="O53" s="0" t="n">
         <f aca="false">IF(H53&lt;&gt;"",H53,IF(AND(I53&lt;&gt;"",J53&lt;&gt;""),(I53+J53)/2,0))</f>
         <v>5</v>
       </c>
-      <c r="O53" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D53,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E53,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F53,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G53,$A$2:$A$61,0)),0))</f>
+      <c r="P53" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D53,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E53,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F53,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G53,$A$2:$A$61,0)),0))</f>
         <v>69</v>
       </c>
-      <c r="P53" s="0" t="n">
-        <f aca="false">O53+N53</f>
+      <c r="Q53" s="0" t="n">
+        <f aca="false">P53+O53</f>
         <v>74</v>
       </c>
-      <c r="Q53" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A53)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A53)),IF(COUNTIF($E$2:$E$61,$A53)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A53)),IF(COUNTIF($F$2:$F$61,$A53)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A53)),IF(COUNTIF($G$2:$G$61,$A53)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A53)))</f>
+      <c r="R53" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A53)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A53)),IF(COUNTIF($E$2:$E$61,$A53)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A53)),IF(COUNTIF($F$2:$F$61,$A53)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A53)),IF(COUNTIF($G$2:$G$61,$A53)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A53)))</f>
         <v>74</v>
-      </c>
-      <c r="R53" s="0" t="n">
-        <f aca="false">Q53-N53</f>
-        <v>69</v>
       </c>
       <c r="S53" s="0" t="n">
         <f aca="false">R53-O53</f>
+        <v>69</v>
+      </c>
+      <c r="T53" s="0" t="n">
+        <f aca="false">S53-P53</f>
         <v>0</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B54" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C54" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D54" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I54" s="0" t="n">
         <v>0.5</v>
@@ -2960,333 +2972,374 @@
       <c r="J54" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="N54" s="0" t="n">
+      <c r="O54" s="0" t="n">
         <f aca="false">IF(H54&lt;&gt;"",H54,IF(AND(I54&lt;&gt;"",J54&lt;&gt;""),(I54+J54)/2,0))</f>
         <v>0.75</v>
       </c>
-      <c r="O54" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D54,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E54,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F54,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G54,$A$2:$A$61,0)),0))</f>
+      <c r="P54" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D54,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E54,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F54,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G54,$A$2:$A$61,0)),0))</f>
         <v>81.5</v>
       </c>
-      <c r="P54" s="0" t="n">
-        <f aca="false">O54+N54</f>
+      <c r="Q54" s="0" t="n">
+        <f aca="false">P54+O54</f>
         <v>82.25</v>
       </c>
-      <c r="Q54" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A54)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A54)),IF(COUNTIF($E$2:$E$61,$A54)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A54)),IF(COUNTIF($F$2:$F$61,$A54)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A54)),IF(COUNTIF($G$2:$G$61,$A54)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A54)))</f>
+      <c r="R54" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A54)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A54)),IF(COUNTIF($E$2:$E$61,$A54)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A54)),IF(COUNTIF($F$2:$F$61,$A54)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A54)),IF(COUNTIF($G$2:$G$61,$A54)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A54)))</f>
         <v>82.25</v>
-      </c>
-      <c r="R54" s="0" t="n">
-        <f aca="false">Q54-N54</f>
-        <v>81.5</v>
       </c>
       <c r="S54" s="0" t="n">
         <f aca="false">R54-O54</f>
+        <v>81.5</v>
+      </c>
+      <c r="T54" s="0" t="n">
+        <f aca="false">S54-P54</f>
         <v>0</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B55" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C55" s="0" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D55" s="0" t="s">
-        <v>116</v>
-      </c>
-      <c r="N55" s="0" t="n">
+        <v>117</v>
+      </c>
+      <c r="O55" s="0" t="n">
         <f aca="false">IF(H55&lt;&gt;"",H55,IF(AND(I55&lt;&gt;"",J55&lt;&gt;""),(I55+J55)/2,0))</f>
         <v>0</v>
       </c>
-      <c r="O55" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D55,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E55,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F55,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G55,$A$2:$A$61,0)),0))</f>
+      <c r="P55" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D55,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E55,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F55,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G55,$A$2:$A$61,0)),0))</f>
         <v>81.5</v>
       </c>
-      <c r="P55" s="0" t="n">
-        <f aca="false">O55+N55</f>
+      <c r="Q55" s="0" t="n">
+        <f aca="false">P55+O55</f>
         <v>81.5</v>
       </c>
-      <c r="Q55" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A55)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A55)),IF(COUNTIF($E$2:$E$61,$A55)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A55)),IF(COUNTIF($F$2:$F$61,$A55)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A55)),IF(COUNTIF($G$2:$G$61,$A55)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A55)))</f>
-        <v>82.25</v>
-      </c>
       <c r="R55" s="0" t="n">
-        <f aca="false">Q55-N55</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A55)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A55)),IF(COUNTIF($E$2:$E$61,$A55)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A55)),IF(COUNTIF($F$2:$F$61,$A55)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A55)),IF(COUNTIF($G$2:$G$61,$A55)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A55)))</f>
         <v>82.25</v>
       </c>
       <c r="S55" s="0" t="n">
         <f aca="false">R55-O55</f>
+        <v>82.25</v>
+      </c>
+      <c r="T55" s="0" t="n">
+        <f aca="false">S55-P55</f>
         <v>0.75</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B56" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C56" s="0" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H56" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="N56" s="0" t="n">
+      <c r="O56" s="0" t="n">
         <f aca="false">IF(H56&lt;&gt;"",H56,IF(AND(I56&lt;&gt;"",J56&lt;&gt;""),(I56+J56)/2,0))</f>
         <v>4</v>
       </c>
-      <c r="O56" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D56,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E56,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F56,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G56,$A$2:$A$61,0)),0))</f>
+      <c r="P56" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D56,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E56,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F56,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G56,$A$2:$A$61,0)),0))</f>
         <v>65</v>
       </c>
-      <c r="P56" s="0" t="n">
-        <f aca="false">O56+N56</f>
+      <c r="Q56" s="0" t="n">
+        <f aca="false">P56+O56</f>
         <v>69</v>
       </c>
-      <c r="Q56" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A56)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A56)),IF(COUNTIF($E$2:$E$61,$A56)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A56)),IF(COUNTIF($F$2:$F$61,$A56)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A56)),IF(COUNTIF($G$2:$G$61,$A56)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A56)))</f>
+      <c r="R56" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A56)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A56)),IF(COUNTIF($E$2:$E$61,$A56)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A56)),IF(COUNTIF($F$2:$F$61,$A56)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A56)),IF(COUNTIF($G$2:$G$61,$A56)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A56)))</f>
         <v>69</v>
-      </c>
-      <c r="R56" s="0" t="n">
-        <f aca="false">Q56-N56</f>
-        <v>65</v>
       </c>
       <c r="S56" s="0" t="n">
         <f aca="false">R56-O56</f>
+        <v>65</v>
+      </c>
+      <c r="T56" s="0" t="n">
+        <f aca="false">S56-P56</f>
         <v>0</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B57" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="C57" s="0" t="s">
+        <v>133</v>
+      </c>
+      <c r="D57" s="0" t="s">
         <v>114</v>
       </c>
-      <c r="C57" s="0" t="s">
-        <v>132</v>
-      </c>
-      <c r="D57" s="0" t="s">
+      <c r="E57" s="0" t="s">
         <v>113</v>
       </c>
-      <c r="E57" s="0" t="s">
-        <v>112</v>
-      </c>
       <c r="F57" s="0" t="s">
-        <v>104</v>
-      </c>
-      <c r="N57" s="0" t="n">
+        <v>105</v>
+      </c>
+      <c r="O57" s="0" t="n">
         <f aca="false">IF(H57&lt;&gt;"",H57,IF(AND(I57&lt;&gt;"",J57&lt;&gt;""),(I57+J57)/2,0))</f>
         <v>0</v>
       </c>
-      <c r="O57" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D57,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E57,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F57,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G57,$A$2:$A$61,0)),0))</f>
+      <c r="P57" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D57,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E57,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F57,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G57,$A$2:$A$61,0)),0))</f>
         <v>38.5</v>
       </c>
-      <c r="P57" s="0" t="n">
-        <f aca="false">O57+N57</f>
+      <c r="Q57" s="0" t="n">
+        <f aca="false">P57+O57</f>
         <v>38.5</v>
       </c>
-      <c r="Q57" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A57)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A57)),IF(COUNTIF($E$2:$E$61,$A57)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A57)),IF(COUNTIF($F$2:$F$61,$A57)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A57)),IF(COUNTIF($G$2:$G$61,$A57)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A57)))</f>
-        <v>65</v>
-      </c>
       <c r="R57" s="0" t="n">
-        <f aca="false">Q57-N57</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A57)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A57)),IF(COUNTIF($E$2:$E$61,$A57)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A57)),IF(COUNTIF($F$2:$F$61,$A57)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A57)),IF(COUNTIF($G$2:$G$61,$A57)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A57)))</f>
         <v>65</v>
       </c>
       <c r="S57" s="0" t="n">
         <f aca="false">R57-O57</f>
+        <v>65</v>
+      </c>
+      <c r="T57" s="0" t="n">
+        <f aca="false">S57-P57</f>
         <v>26.5</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B58" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C58" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E58" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F58" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G58" s="0" t="s">
-        <v>71</v>
-      </c>
-      <c r="N58" s="0" t="n">
+        <v>72</v>
+      </c>
+      <c r="O58" s="0" t="n">
         <f aca="false">IF(H58&lt;&gt;"",H58,IF(AND(I58&lt;&gt;"",J58&lt;&gt;""),(I58+J58)/2,0))</f>
         <v>0</v>
       </c>
-      <c r="O58" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D58,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E58,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F58,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G58,$A$2:$A$61,0)),0))</f>
+      <c r="P58" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D58,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E58,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F58,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G58,$A$2:$A$61,0)),0))</f>
         <v>62</v>
       </c>
-      <c r="P58" s="0" t="n">
-        <f aca="false">O58+N58</f>
+      <c r="Q58" s="0" t="n">
+        <f aca="false">P58+O58</f>
         <v>62</v>
       </c>
-      <c r="Q58" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A58)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A58)),IF(COUNTIF($E$2:$E$61,$A58)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A58)),IF(COUNTIF($F$2:$F$61,$A58)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A58)),IF(COUNTIF($G$2:$G$61,$A58)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A58)))</f>
-        <v>65</v>
-      </c>
       <c r="R58" s="0" t="n">
-        <f aca="false">Q58-N58</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A58)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A58)),IF(COUNTIF($E$2:$E$61,$A58)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A58)),IF(COUNTIF($F$2:$F$61,$A58)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A58)),IF(COUNTIF($G$2:$G$61,$A58)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A58)))</f>
         <v>65</v>
       </c>
       <c r="S58" s="0" t="n">
         <f aca="false">R58-O58</f>
+        <v>65</v>
+      </c>
+      <c r="T58" s="0" t="n">
+        <f aca="false">S58-P58</f>
         <v>3</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B59" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C59" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D59" s="0" t="s">
-        <v>36</v>
-      </c>
-      <c r="N59" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="O59" s="0" t="n">
         <f aca="false">IF(H59&lt;&gt;"",H59,IF(AND(I59&lt;&gt;"",J59&lt;&gt;""),(I59+J59)/2,0))</f>
         <v>0</v>
       </c>
-      <c r="O59" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D59,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E59,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F59,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G59,$A$2:$A$61,0)),0))</f>
+      <c r="P59" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D59,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E59,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F59,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G59,$A$2:$A$61,0)),0))</f>
         <v>45.5</v>
       </c>
-      <c r="P59" s="0" t="n">
-        <f aca="false">O59+N59</f>
+      <c r="Q59" s="0" t="n">
+        <f aca="false">P59+O59</f>
         <v>45.5</v>
       </c>
-      <c r="Q59" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A59)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A59)),IF(COUNTIF($E$2:$E$61,$A59)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A59)),IF(COUNTIF($F$2:$F$61,$A59)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A59)),IF(COUNTIF($G$2:$G$61,$A59)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A59)))</f>
-        <v>65</v>
-      </c>
       <c r="R59" s="0" t="n">
-        <f aca="false">Q59-N59</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A59)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A59)),IF(COUNTIF($E$2:$E$61,$A59)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A59)),IF(COUNTIF($F$2:$F$61,$A59)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A59)),IF(COUNTIF($G$2:$G$61,$A59)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A59)))</f>
         <v>65</v>
       </c>
       <c r="S59" s="0" t="n">
         <f aca="false">R59-O59</f>
+        <v>65</v>
+      </c>
+      <c r="T59" s="0" t="n">
+        <f aca="false">S59-P59</f>
         <v>19.5</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B60" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C60" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D60" s="0" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>59</v>
-      </c>
-      <c r="N60" s="0" t="n">
+        <v>60</v>
+      </c>
+      <c r="O60" s="0" t="n">
         <f aca="false">IF(H60&lt;&gt;"",H60,IF(AND(I60&lt;&gt;"",J60&lt;&gt;""),(I60+J60)/2,0))</f>
         <v>0</v>
       </c>
-      <c r="O60" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D60,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E60,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F60,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G60,$A$2:$A$61,0)),0))</f>
+      <c r="P60" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D60,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E60,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F60,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G60,$A$2:$A$61,0)),0))</f>
         <v>65</v>
       </c>
-      <c r="P60" s="0" t="n">
-        <f aca="false">O60+N60</f>
+      <c r="Q60" s="0" t="n">
+        <f aca="false">P60+O60</f>
         <v>65</v>
       </c>
-      <c r="Q60" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A60)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A60)),IF(COUNTIF($E$2:$E$61,$A60)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A60)),IF(COUNTIF($F$2:$F$61,$A60)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A60)),IF(COUNTIF($G$2:$G$61,$A60)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A60)))</f>
-        <v>65</v>
-      </c>
       <c r="R60" s="0" t="n">
-        <f aca="false">Q60-N60</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A60)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A60)),IF(COUNTIF($E$2:$E$61,$A60)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A60)),IF(COUNTIF($F$2:$F$61,$A60)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A60)),IF(COUNTIF($G$2:$G$61,$A60)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A60)))</f>
         <v>65</v>
       </c>
       <c r="S60" s="0" t="n">
         <f aca="false">R60-O60</f>
+        <v>65</v>
+      </c>
+      <c r="T60" s="0" t="n">
+        <f aca="false">S60-P60</f>
         <v>0</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B61" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C61" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F61" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G61" s="0" t="s">
-        <v>135</v>
-      </c>
-      <c r="N61" s="0" t="n">
+        <v>136</v>
+      </c>
+      <c r="O61" s="0" t="n">
         <f aca="false">IF(H61&lt;&gt;"",H61,IF(AND(I61&lt;&gt;"",J61&lt;&gt;""),(I61+J61)/2,0))</f>
         <v>0</v>
       </c>
-      <c r="O61" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($P$2:$P$61,MATCH(D61,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(E61,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(F61,$A$2:$A$61,0)),0),IFERROR(INDEX($P$2:$P$61,MATCH(G61,$A$2:$A$61,0)),0))</f>
+      <c r="P61" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D61,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E61,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F61,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G61,$A$2:$A$61,0)),0))</f>
         <v>65</v>
       </c>
-      <c r="P61" s="0" t="n">
-        <f aca="false">O61+N61</f>
+      <c r="Q61" s="0" t="n">
+        <f aca="false">P61+O61</f>
         <v>65</v>
       </c>
-      <c r="Q61" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A61)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$D$2:$D$61,$A61)),IF(COUNTIF($E$2:$E$61,$A61)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$E$2:$E$61,$A61)),IF(COUNTIF($F$2:$F$61,$A61)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$F$2:$F$61,$A61)),IF(COUNTIF($G$2:$G$61,$A61)=0,$N$63,_xlfn.MINIFS($R$2:$R$61,$G$2:$G$61,$A61)))</f>
-        <v>65</v>
-      </c>
       <c r="R61" s="0" t="n">
-        <f aca="false">Q61-N61</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A61)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A61)),IF(COUNTIF($E$2:$E$61,$A61)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A61)),IF(COUNTIF($F$2:$F$61,$A61)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A61)),IF(COUNTIF($G$2:$G$61,$A61)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A61)))</f>
         <v>65</v>
       </c>
       <c r="S61" s="0" t="n">
         <f aca="false">R61-O61</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M63" s="0" t="s">
-        <v>140</v>
-      </c>
-      <c r="N63" s="0" t="n">
-        <f aca="false">MAX(P2:P61)</f>
+        <v>65</v>
+      </c>
+      <c r="T61" s="0" t="n">
+        <f aca="false">S61-P61</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B62" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="C62" s="0" t="s">
+        <v>142</v>
+      </c>
+      <c r="D62" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="K62" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="O62" s="0" t="n">
+        <f aca="false">IF(H62&lt;&gt;"",H62,IF(AND(I62&lt;&gt;"",J62&lt;&gt;""),(I62+J62)/2,0))</f>
+        <v>0</v>
+      </c>
+      <c r="P62" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D62,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E62,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F62,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G62,$A$2:$A$61,0)),0))</f>
+        <v>74</v>
+      </c>
+      <c r="Q62" s="0" t="n">
+        <f aca="false">P62+O62</f>
+        <v>74</v>
+      </c>
+      <c r="R62" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A62)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A62)),IF(COUNTIF($E$2:$E$61,$A62)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A62)),IF(COUNTIF($F$2:$F$61,$A62)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A62)),IF(COUNTIF($G$2:$G$61,$A62)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A62)))</f>
+        <v>82.25</v>
+      </c>
+      <c r="S62" s="0" t="n">
+        <f aca="false">R62-O62</f>
+        <v>82.25</v>
+      </c>
+      <c r="T62" s="0" t="n">
+        <f aca="false">S62-P62</f>
+        <v>8.25</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N64" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="O64" s="0" t="n">
+        <f aca="false">MAX(Q2:Q61)</f>
         <v>82.25</v>
       </c>
     </row>
@@ -3314,22 +3367,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="39.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="35.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="42.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="50.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="40.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Crash bookstore drywall, split up cleanup and ACI punch list
</commit_message>
<xml_diff>
--- a/AC Tasks.xlsx
+++ b/AC Tasks.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="152">
   <si>
     <t xml:space="preserve">Id</t>
   </si>
@@ -140,6 +140,15 @@
     <t xml:space="preserve">masonry</t>
   </si>
   <si>
+    <t xml:space="preserve">T8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cleanup and ACI punch list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P12</t>
+  </si>
+  <si>
     <t xml:space="preserve">B0</t>
   </si>
   <si>
@@ -197,6 +206,12 @@
     <t xml:space="preserve">painting</t>
   </si>
   <si>
+    <t xml:space="preserve">B11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P14</t>
+  </si>
+  <si>
     <t xml:space="preserve">B9</t>
   </si>
   <si>
@@ -284,6 +299,12 @@
     <t xml:space="preserve">install doors and hardware</t>
   </si>
   <si>
+    <t xml:space="preserve">S13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P11</t>
+  </si>
+  <si>
     <t xml:space="preserve">L0</t>
   </si>
   <si>
@@ -368,6 +389,9 @@
     <t xml:space="preserve">L14</t>
   </si>
   <si>
+    <t xml:space="preserve">L15</t>
+  </si>
+  <si>
     <t xml:space="preserve">overall</t>
   </si>
   <si>
@@ -413,34 +437,22 @@
     <t xml:space="preserve">sign final release of lien</t>
   </si>
   <si>
-    <t xml:space="preserve">cleanup and ACI punch list</t>
-  </si>
-  <si>
     <t xml:space="preserve">P15</t>
   </si>
   <si>
     <t xml:space="preserve">P10</t>
   </si>
   <si>
-    <t xml:space="preserve">lobby done</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sanctuary done</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">terrace done</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bookstore done</t>
+    <t xml:space="preserve">lobby done except cleanup and ACI punch list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sanctuary done except cleanup and ACI punch list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">terrace done except cleanup and ACI punch list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bookstore done except cleanup and ACI punch list</t>
   </si>
   <si>
     <t xml:space="preserve">all sections done</t>
@@ -679,7 +691,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T64"/>
+  <dimension ref="A1:T68"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.21"/>
@@ -773,7 +785,7 @@
         <v>0</v>
       </c>
       <c r="P2" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D2,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E2,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F2,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G2,$A$2:$A$61,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D2,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E2,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F2,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G2,$A$2:$A$65,0)),0))</f>
         <v>0</v>
       </c>
       <c r="Q2" s="0" t="n">
@@ -781,16 +793,16 @@
         <v>0</v>
       </c>
       <c r="R2" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A2)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A2)),IF(COUNTIF($E$2:$E$61,$A2)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A2)),IF(COUNTIF($F$2:$F$61,$A2)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A2)),IF(COUNTIF($G$2:$G$61,$A2)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A2)))</f>
-        <v>19.5</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A2)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A2)),IF(COUNTIF($E$2:$E$65,$A2)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A2)),IF(COUNTIF($F$2:$F$65,$A2)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A2)),IF(COUNTIF($G$2:$G$65,$A2)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A2)))</f>
+        <v>16.5</v>
       </c>
       <c r="S2" s="0" t="n">
         <f aca="false">R2-O2</f>
-        <v>19.5</v>
+        <v>16.5</v>
       </c>
       <c r="T2" s="0" t="n">
         <f aca="false">S2-P2</f>
-        <v>19.5</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -814,7 +826,7 @@
         <v>8</v>
       </c>
       <c r="P3" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D3,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E3,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F3,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G3,$A$2:$A$61,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D3,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E3,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F3,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G3,$A$2:$A$65,0)),0))</f>
         <v>0</v>
       </c>
       <c r="Q3" s="0" t="n">
@@ -822,16 +834,16 @@
         <v>8</v>
       </c>
       <c r="R3" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A3)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A3)),IF(COUNTIF($E$2:$E$61,$A3)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A3)),IF(COUNTIF($F$2:$F$61,$A3)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A3)),IF(COUNTIF($G$2:$G$61,$A3)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A3)))</f>
-        <v>27.5</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A3)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A3)),IF(COUNTIF($E$2:$E$65,$A3)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A3)),IF(COUNTIF($F$2:$F$65,$A3)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A3)),IF(COUNTIF($G$2:$G$65,$A3)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A3)))</f>
+        <v>24.5</v>
       </c>
       <c r="S3" s="0" t="n">
         <f aca="false">R3-O3</f>
-        <v>19.5</v>
+        <v>16.5</v>
       </c>
       <c r="T3" s="0" t="n">
         <f aca="false">S3-P3</f>
-        <v>19.5</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -855,7 +867,7 @@
         <v>7</v>
       </c>
       <c r="P4" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D4,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E4,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F4,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G4,$A$2:$A$61,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D4,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E4,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F4,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G4,$A$2:$A$65,0)),0))</f>
         <v>8</v>
       </c>
       <c r="Q4" s="0" t="n">
@@ -863,16 +875,16 @@
         <v>15</v>
       </c>
       <c r="R4" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A4)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A4)),IF(COUNTIF($E$2:$E$61,$A4)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A4)),IF(COUNTIF($F$2:$F$61,$A4)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A4)),IF(COUNTIF($G$2:$G$61,$A4)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A4)))</f>
-        <v>34.5</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A4)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A4)),IF(COUNTIF($E$2:$E$65,$A4)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A4)),IF(COUNTIF($F$2:$F$65,$A4)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A4)),IF(COUNTIF($G$2:$G$65,$A4)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A4)))</f>
+        <v>31.5</v>
       </c>
       <c r="S4" s="0" t="n">
         <f aca="false">R4-O4</f>
-        <v>27.5</v>
+        <v>24.5</v>
       </c>
       <c r="T4" s="0" t="n">
         <f aca="false">S4-P4</f>
-        <v>19.5</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -896,7 +908,7 @@
         <v>3</v>
       </c>
       <c r="P5" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D5,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E5,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F5,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G5,$A$2:$A$61,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D5,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E5,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F5,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G5,$A$2:$A$65,0)),0))</f>
         <v>15</v>
       </c>
       <c r="Q5" s="0" t="n">
@@ -904,16 +916,16 @@
         <v>18</v>
       </c>
       <c r="R5" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A5)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A5)),IF(COUNTIF($E$2:$E$61,$A5)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A5)),IF(COUNTIF($F$2:$F$61,$A5)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A5)),IF(COUNTIF($G$2:$G$61,$A5)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A5)))</f>
-        <v>37.5</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A5)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A5)),IF(COUNTIF($E$2:$E$65,$A5)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A5)),IF(COUNTIF($F$2:$F$65,$A5)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A5)),IF(COUNTIF($G$2:$G$65,$A5)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A5)))</f>
+        <v>34.5</v>
       </c>
       <c r="S5" s="0" t="n">
         <f aca="false">R5-O5</f>
-        <v>34.5</v>
+        <v>31.5</v>
       </c>
       <c r="T5" s="0" t="n">
         <f aca="false">S5-P5</f>
-        <v>19.5</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -943,7 +955,7 @@
         <v>7.5</v>
       </c>
       <c r="P6" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D6,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E6,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F6,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G6,$A$2:$A$61,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D6,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E6,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F6,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G6,$A$2:$A$65,0)),0))</f>
         <v>18</v>
       </c>
       <c r="Q6" s="0" t="n">
@@ -951,16 +963,16 @@
         <v>25.5</v>
       </c>
       <c r="R6" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A6)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A6)),IF(COUNTIF($E$2:$E$61,$A6)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A6)),IF(COUNTIF($F$2:$F$61,$A6)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A6)),IF(COUNTIF($G$2:$G$61,$A6)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A6)))</f>
-        <v>45</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A6)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A6)),IF(COUNTIF($E$2:$E$65,$A6)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A6)),IF(COUNTIF($F$2:$F$65,$A6)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A6)),IF(COUNTIF($G$2:$G$65,$A6)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A6)))</f>
+        <v>42</v>
       </c>
       <c r="S6" s="0" t="n">
         <f aca="false">R6-O6</f>
-        <v>37.5</v>
+        <v>34.5</v>
       </c>
       <c r="T6" s="0" t="n">
         <f aca="false">S6-P6</f>
-        <v>19.5</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -987,7 +999,7 @@
         <v>10</v>
       </c>
       <c r="P7" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D7,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E7,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F7,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G7,$A$2:$A$61,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D7,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E7,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F7,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G7,$A$2:$A$65,0)),0))</f>
         <v>25.5</v>
       </c>
       <c r="Q7" s="0" t="n">
@@ -995,16 +1007,16 @@
         <v>35.5</v>
       </c>
       <c r="R7" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A7)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A7)),IF(COUNTIF($E$2:$E$61,$A7)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A7)),IF(COUNTIF($F$2:$F$61,$A7)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A7)),IF(COUNTIF($G$2:$G$61,$A7)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A7)))</f>
-        <v>55</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A7)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A7)),IF(COUNTIF($E$2:$E$65,$A7)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A7)),IF(COUNTIF($F$2:$F$65,$A7)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A7)),IF(COUNTIF($G$2:$G$65,$A7)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A7)))</f>
+        <v>52</v>
       </c>
       <c r="S7" s="0" t="n">
         <f aca="false">R7-O7</f>
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="T7" s="0" t="n">
         <f aca="false">S7-P7</f>
-        <v>19.5</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1028,7 +1040,7 @@
         <v>5</v>
       </c>
       <c r="P8" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D8,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E8,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F8,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G8,$A$2:$A$61,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D8,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E8,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F8,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G8,$A$2:$A$65,0)),0))</f>
         <v>25.5</v>
       </c>
       <c r="Q8" s="0" t="n">
@@ -1036,16 +1048,16 @@
         <v>30.5</v>
       </c>
       <c r="R8" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A8)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A8)),IF(COUNTIF($E$2:$E$61,$A8)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A8)),IF(COUNTIF($F$2:$F$61,$A8)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A8)),IF(COUNTIF($G$2:$G$61,$A8)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A8)))</f>
-        <v>55</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A8)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A8)),IF(COUNTIF($E$2:$E$65,$A8)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A8)),IF(COUNTIF($F$2:$F$65,$A8)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A8)),IF(COUNTIF($G$2:$G$65,$A8)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A8)))</f>
+        <v>52</v>
       </c>
       <c r="S8" s="0" t="n">
         <f aca="false">R8-O8</f>
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="T8" s="0" t="n">
         <f aca="false">S8-P8</f>
-        <v>24.5</v>
+        <v>21.5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1072,7 +1084,7 @@
         <v>10</v>
       </c>
       <c r="P9" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D9,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E9,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F9,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G9,$A$2:$A$61,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D9,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E9,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F9,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G9,$A$2:$A$65,0)),0))</f>
         <v>35.5</v>
       </c>
       <c r="Q9" s="0" t="n">
@@ -1080,16 +1092,16 @@
         <v>45.5</v>
       </c>
       <c r="R9" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A9)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A9)),IF(COUNTIF($E$2:$E$61,$A9)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A9)),IF(COUNTIF($F$2:$F$61,$A9)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A9)),IF(COUNTIF($G$2:$G$61,$A9)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A9)))</f>
-        <v>65</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A9)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A9)),IF(COUNTIF($E$2:$E$65,$A9)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A9)),IF(COUNTIF($F$2:$F$65,$A9)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A9)),IF(COUNTIF($G$2:$G$65,$A9)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A9)))</f>
+        <v>62</v>
       </c>
       <c r="S9" s="0" t="n">
         <f aca="false">R9-O9</f>
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="T9" s="0" t="n">
         <f aca="false">S9-P9</f>
-        <v>19.5</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1097,37 +1109,40 @@
         <v>39</v>
       </c>
       <c r="B10" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="0" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="D10" s="0" t="s">
         <v>41</v>
       </c>
-      <c r="D10" s="0" t="s">
-        <v>23</v>
+      <c r="H10" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="O10" s="0" t="n">
         <f aca="false">IF(H10&lt;&gt;"",H10,IF(AND(I10&lt;&gt;"",J10&lt;&gt;""),(I10+J10)/2,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P10" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D10,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E10,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F10,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G10,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D10,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E10,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F10,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G10,$A$2:$A$65,0)),0))</f>
+        <v>45.5</v>
       </c>
       <c r="Q10" s="0" t="n">
         <f aca="false">P10+O10</f>
-        <v>0</v>
+        <v>46.5</v>
       </c>
       <c r="R10" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A10)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A10)),IF(COUNTIF($E$2:$E$61,$A10)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A10)),IF(COUNTIF($F$2:$F$61,$A10)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A10)),IF(COUNTIF($G$2:$G$61,$A10)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A10)))</f>
-        <v>0</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A10)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A10)),IF(COUNTIF($E$2:$E$65,$A10)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A10)),IF(COUNTIF($F$2:$F$65,$A10)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A10)),IF(COUNTIF($G$2:$G$65,$A10)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A10)))</f>
+        <v>63</v>
       </c>
       <c r="S10" s="0" t="n">
         <f aca="false">R10-O10</f>
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="T10" s="0" t="n">
         <f aca="false">S10-P10</f>
-        <v>0</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1135,290 +1150,284 @@
         <v>42</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>39</v>
-      </c>
-      <c r="I11" s="0" t="n">
-        <v>21</v>
-      </c>
-      <c r="J11" s="0" t="n">
         <v>23</v>
       </c>
       <c r="O11" s="0" t="n">
         <f aca="false">IF(H11&lt;&gt;"",H11,IF(AND(I11&lt;&gt;"",J11&lt;&gt;""),(I11+J11)/2,0))</f>
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="P11" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D11,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E11,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F11,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G11,$A$2:$A$61,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D11,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E11,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F11,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G11,$A$2:$A$65,0)),0))</f>
         <v>0</v>
       </c>
       <c r="Q11" s="0" t="n">
         <f aca="false">P11+O11</f>
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="R11" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A11)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A11)),IF(COUNTIF($E$2:$E$61,$A11)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A11)),IF(COUNTIF($F$2:$F$61,$A11)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A11)),IF(COUNTIF($G$2:$G$61,$A11)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A11)))</f>
-        <v>22</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A11)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A11)),IF(COUNTIF($E$2:$E$65,$A11)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A11)),IF(COUNTIF($F$2:$F$65,$A11)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A11)),IF(COUNTIF($G$2:$G$65,$A11)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A11)))</f>
+        <v>2</v>
       </c>
       <c r="S11" s="0" t="n">
         <f aca="false">R11-O11</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T11" s="0" t="n">
         <f aca="false">S11-P11</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D12" s="0" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="0" t="n">
-        <v>10</v>
+      <c r="I12" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="J12" s="0" t="n">
+        <v>18</v>
       </c>
       <c r="O12" s="0" t="n">
         <f aca="false">IF(H12&lt;&gt;"",H12,IF(AND(I12&lt;&gt;"",J12&lt;&gt;""),(I12+J12)/2,0))</f>
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="P12" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D12,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E12,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F12,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G12,$A$2:$A$61,0)),0))</f>
-        <v>22</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D12,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E12,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F12,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G12,$A$2:$A$65,0)),0))</f>
+        <v>0</v>
       </c>
       <c r="Q12" s="0" t="n">
         <f aca="false">P12+O12</f>
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="R12" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A12)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A12)),IF(COUNTIF($E$2:$E$61,$A12)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A12)),IF(COUNTIF($F$2:$F$61,$A12)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A12)),IF(COUNTIF($G$2:$G$61,$A12)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A12)))</f>
-        <v>42</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A12)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A12)),IF(COUNTIF($E$2:$E$65,$A12)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A12)),IF(COUNTIF($F$2:$F$65,$A12)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A12)),IF(COUNTIF($G$2:$G$65,$A12)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A12)))</f>
+        <v>19</v>
       </c>
       <c r="S12" s="0" t="n">
         <f aca="false">R12-O12</f>
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="T12" s="0" t="n">
         <f aca="false">S12-P12</f>
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="H13" s="0" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="O13" s="0" t="n">
         <f aca="false">IF(H13&lt;&gt;"",H13,IF(AND(I13&lt;&gt;"",J13&lt;&gt;""),(I13+J13)/2,0))</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="P13" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D13,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E13,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F13,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G13,$A$2:$A$61,0)),0))</f>
-        <v>22</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D13,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E13,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F13,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G13,$A$2:$A$65,0)),0))</f>
+        <v>17</v>
       </c>
       <c r="Q13" s="0" t="n">
         <f aca="false">P13+O13</f>
         <v>27</v>
       </c>
       <c r="R13" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A13)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A13)),IF(COUNTIF($E$2:$E$61,$A13)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A13)),IF(COUNTIF($F$2:$F$61,$A13)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A13)),IF(COUNTIF($G$2:$G$61,$A13)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A13)))</f>
-        <v>42</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A13)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A13)),IF(COUNTIF($E$2:$E$65,$A13)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A13)),IF(COUNTIF($F$2:$F$65,$A13)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A13)),IF(COUNTIF($G$2:$G$65,$A13)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A13)))</f>
+        <v>39</v>
       </c>
       <c r="S13" s="0" t="n">
         <f aca="false">R13-O13</f>
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="T13" s="0" t="n">
         <f aca="false">S13-P13</f>
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="I14" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="J14" s="0" t="n">
-        <v>21</v>
-      </c>
-      <c r="M14" s="0" t="s">
-        <v>32</v>
+        <v>45</v>
+      </c>
+      <c r="H14" s="0" t="n">
+        <v>5</v>
       </c>
       <c r="O14" s="0" t="n">
         <f aca="false">IF(H14&lt;&gt;"",H14,IF(AND(I14&lt;&gt;"",J14&lt;&gt;""),(I14+J14)/2,0))</f>
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="P14" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D14,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E14,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F14,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G14,$A$2:$A$61,0)),0))</f>
-        <v>22</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D14,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E14,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F14,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G14,$A$2:$A$65,0)),0))</f>
+        <v>17</v>
       </c>
       <c r="Q14" s="0" t="n">
         <f aca="false">P14+O14</f>
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="R14" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A14)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A14)),IF(COUNTIF($E$2:$E$61,$A14)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A14)),IF(COUNTIF($F$2:$F$61,$A14)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A14)),IF(COUNTIF($G$2:$G$61,$A14)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A14)))</f>
-        <v>40</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A14)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A14)),IF(COUNTIF($E$2:$E$65,$A14)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A14)),IF(COUNTIF($F$2:$F$65,$A14)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A14)),IF(COUNTIF($G$2:$G$65,$A14)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A14)))</f>
+        <v>39</v>
       </c>
       <c r="S14" s="0" t="n">
         <f aca="false">R14-O14</f>
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="T14" s="0" t="n">
         <f aca="false">S14-P14</f>
-        <v>0</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="H15" s="0" t="n">
-        <v>5</v>
+        <v>45</v>
+      </c>
+      <c r="I15" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="J15" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="M15" s="0" t="s">
+        <v>32</v>
       </c>
       <c r="O15" s="0" t="n">
         <f aca="false">IF(H15&lt;&gt;"",H15,IF(AND(I15&lt;&gt;"",J15&lt;&gt;""),(I15+J15)/2,0))</f>
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="P15" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D15,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E15,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F15,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G15,$A$2:$A$61,0)),0))</f>
-        <v>40</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D15,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E15,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F15,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G15,$A$2:$A$65,0)),0))</f>
+        <v>17</v>
       </c>
       <c r="Q15" s="0" t="n">
         <f aca="false">P15+O15</f>
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="R15" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A15)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A15)),IF(COUNTIF($E$2:$E$61,$A15)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A15)),IF(COUNTIF($F$2:$F$61,$A15)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A15)),IF(COUNTIF($G$2:$G$61,$A15)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A15)))</f>
-        <v>45</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A15)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A15)),IF(COUNTIF($E$2:$E$65,$A15)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A15)),IF(COUNTIF($F$2:$F$65,$A15)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A15)),IF(COUNTIF($G$2:$G$65,$A15)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A15)))</f>
+        <v>37</v>
       </c>
       <c r="S15" s="0" t="n">
         <f aca="false">R15-O15</f>
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="T15" s="0" t="n">
         <f aca="false">S15-P15</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H16" s="0" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="O16" s="0" t="n">
         <f aca="false">IF(H16&lt;&gt;"",H16,IF(AND(I16&lt;&gt;"",J16&lt;&gt;""),(I16+J16)/2,0))</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="P16" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D16,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E16,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F16,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G16,$A$2:$A$61,0)),0))</f>
-        <v>45</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D16,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E16,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F16,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G16,$A$2:$A$65,0)),0))</f>
+        <v>35</v>
       </c>
       <c r="Q16" s="0" t="n">
         <f aca="false">P16+O16</f>
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="R16" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A16)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A16)),IF(COUNTIF($E$2:$E$61,$A16)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A16)),IF(COUNTIF($F$2:$F$61,$A16)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A16)),IF(COUNTIF($G$2:$G$61,$A16)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A16)))</f>
-        <v>55</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A16)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A16)),IF(COUNTIF($E$2:$E$65,$A16)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A16)),IF(COUNTIF($F$2:$F$65,$A16)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A16)),IF(COUNTIF($G$2:$G$65,$A16)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A16)))</f>
+        <v>42</v>
       </c>
       <c r="S16" s="0" t="n">
         <f aca="false">R16-O16</f>
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="T16" s="0" t="n">
         <f aca="false">S16-P16</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="E17" s="0" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="H17" s="0" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="O17" s="0" t="n">
         <f aca="false">IF(H17&lt;&gt;"",H17,IF(AND(I17&lt;&gt;"",J17&lt;&gt;""),(I17+J17)/2,0))</f>
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="P17" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D17,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E17,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F17,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G17,$A$2:$A$61,0)),0))</f>
-        <v>32</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D17,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E17,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F17,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G17,$A$2:$A$65,0)),0))</f>
+        <v>40</v>
       </c>
       <c r="Q17" s="0" t="n">
         <f aca="false">P17+O17</f>
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="R17" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A17)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A17)),IF(COUNTIF($E$2:$E$61,$A17)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A17)),IF(COUNTIF($F$2:$F$61,$A17)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A17)),IF(COUNTIF($G$2:$G$61,$A17)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A17)))</f>
-        <v>45</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A17)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A17)),IF(COUNTIF($E$2:$E$65,$A17)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A17)),IF(COUNTIF($F$2:$F$65,$A17)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A17)),IF(COUNTIF($G$2:$G$65,$A17)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A17)))</f>
+        <v>52</v>
       </c>
       <c r="S17" s="0" t="n">
         <f aca="false">R17-O17</f>
@@ -1426,177 +1435,180 @@
       </c>
       <c r="T17" s="0" t="n">
         <f aca="false">S17-P17</f>
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>54</v>
+        <v>49</v>
+      </c>
+      <c r="E18" s="0" t="s">
+        <v>47</v>
       </c>
       <c r="H18" s="0" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="O18" s="0" t="n">
         <f aca="false">IF(H18&lt;&gt;"",H18,IF(AND(I18&lt;&gt;"",J18&lt;&gt;""),(I18+J18)/2,0))</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="P18" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D18,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E18,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F18,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G18,$A$2:$A$61,0)),0))</f>
-        <v>35</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D18,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E18,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F18,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G18,$A$2:$A$65,0)),0))</f>
+        <v>27</v>
       </c>
       <c r="Q18" s="0" t="n">
         <f aca="false">P18+O18</f>
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="R18" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A18)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A18)),IF(COUNTIF($E$2:$E$61,$A18)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A18)),IF(COUNTIF($F$2:$F$61,$A18)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A18)),IF(COUNTIF($G$2:$G$61,$A18)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A18)))</f>
-        <v>55</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A18)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A18)),IF(COUNTIF($E$2:$E$65,$A18)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A18)),IF(COUNTIF($F$2:$F$65,$A18)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A18)),IF(COUNTIF($G$2:$G$65,$A18)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A18)))</f>
+        <v>42</v>
       </c>
       <c r="S18" s="0" t="n">
         <f aca="false">R18-O18</f>
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="T18" s="0" t="n">
         <f aca="false">S18-P18</f>
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="E19" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="I19" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="J19" s="0" t="n">
-        <v>8</v>
+        <v>57</v>
+      </c>
+      <c r="H19" s="0" t="n">
+        <v>10</v>
       </c>
       <c r="O19" s="0" t="n">
         <f aca="false">IF(H19&lt;&gt;"",H19,IF(AND(I19&lt;&gt;"",J19&lt;&gt;""),(I19+J19)/2,0))</f>
-        <v>6.5</v>
+        <v>10</v>
       </c>
       <c r="P19" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D19,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E19,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F19,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G19,$A$2:$A$61,0)),0))</f>
-        <v>55</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D19,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E19,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F19,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G19,$A$2:$A$65,0)),0))</f>
+        <v>30</v>
       </c>
       <c r="Q19" s="0" t="n">
         <f aca="false">P19+O19</f>
-        <v>61.5</v>
+        <v>40</v>
       </c>
       <c r="R19" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A19)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A19)),IF(COUNTIF($E$2:$E$61,$A19)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A19)),IF(COUNTIF($F$2:$F$61,$A19)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A19)),IF(COUNTIF($G$2:$G$61,$A19)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A19)))</f>
-        <v>65</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A19)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A19)),IF(COUNTIF($E$2:$E$65,$A19)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A19)),IF(COUNTIF($F$2:$F$65,$A19)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A19)),IF(COUNTIF($G$2:$G$65,$A19)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A19)))</f>
+        <v>52</v>
       </c>
       <c r="S19" s="0" t="n">
         <f aca="false">R19-O19</f>
-        <v>58.5</v>
+        <v>42</v>
       </c>
       <c r="T19" s="0" t="n">
         <f aca="false">S19-P19</f>
-        <v>3.5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B20" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" s="0" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="0" t="s">
-        <v>61</v>
-      </c>
       <c r="D20" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="E20" s="0" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H20" s="0" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O20" s="0" t="n">
         <f aca="false">IF(H20&lt;&gt;"",H20,IF(AND(I20&lt;&gt;"",J20&lt;&gt;""),(I20+J20)/2,0))</f>
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="P20" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D20,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E20,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F20,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G20,$A$2:$A$61,0)),0))</f>
-        <v>55</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D20,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E20,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F20,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G20,$A$2:$A$65,0)),0))</f>
+        <v>60</v>
       </c>
       <c r="Q20" s="0" t="n">
         <f aca="false">P20+O20</f>
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="R20" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A20)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A20)),IF(COUNTIF($E$2:$E$61,$A20)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A20)),IF(COUNTIF($F$2:$F$61,$A20)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A20)),IF(COUNTIF($G$2:$G$61,$A20)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A20)))</f>
-        <v>65</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A20)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A20)),IF(COUNTIF($E$2:$E$65,$A20)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A20)),IF(COUNTIF($F$2:$F$65,$A20)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A20)),IF(COUNTIF($G$2:$G$65,$A20)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A20)))</f>
+        <v>63</v>
       </c>
       <c r="S20" s="0" t="n">
         <f aca="false">R20-O20</f>
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="T20" s="0" t="n">
         <f aca="false">S20-P20</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>63</v>
+        <v>43</v>
       </c>
       <c r="C21" s="0" t="s">
         <v>64</v>
       </c>
       <c r="D21" s="0" t="s">
-        <v>23</v>
+        <v>59</v>
+      </c>
+      <c r="E21" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="I21" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="J21" s="0" t="n">
+        <v>8</v>
       </c>
       <c r="O21" s="0" t="n">
         <f aca="false">IF(H21&lt;&gt;"",H21,IF(AND(I21&lt;&gt;"",J21&lt;&gt;""),(I21+J21)/2,0))</f>
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="P21" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D21,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E21,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F21,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G21,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D21,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E21,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F21,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G21,$A$2:$A$65,0)),0))</f>
+        <v>50</v>
       </c>
       <c r="Q21" s="0" t="n">
         <f aca="false">P21+O21</f>
-        <v>0</v>
+        <v>56.5</v>
       </c>
       <c r="R21" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A21)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A21)),IF(COUNTIF($E$2:$E$61,$A21)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A21)),IF(COUNTIF($F$2:$F$61,$A21)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A21)),IF(COUNTIF($G$2:$G$61,$A21)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A21)))</f>
-        <v>3</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A21)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A21)),IF(COUNTIF($E$2:$E$65,$A21)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A21)),IF(COUNTIF($F$2:$F$65,$A21)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A21)),IF(COUNTIF($G$2:$G$65,$A21)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A21)))</f>
+        <v>62</v>
       </c>
       <c r="S21" s="0" t="n">
         <f aca="false">R21-O21</f>
-        <v>3</v>
+        <v>55.5</v>
       </c>
       <c r="T21" s="0" t="n">
         <f aca="false">S21-P21</f>
-        <v>3</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1604,177 +1616,177 @@
         <v>65</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>63</v>
+        <v>43</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>43</v>
+        <v>66</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>62</v>
+        <v>59</v>
+      </c>
+      <c r="E22" s="0" t="s">
+        <v>55</v>
       </c>
       <c r="H22" s="0" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="O22" s="0" t="n">
         <f aca="false">IF(H22&lt;&gt;"",H22,IF(AND(I22&lt;&gt;"",J22&lt;&gt;""),(I22+J22)/2,0))</f>
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="P22" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D22,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E22,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F22,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G22,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D22,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E22,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F22,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G22,$A$2:$A$65,0)),0))</f>
+        <v>50</v>
       </c>
       <c r="Q22" s="0" t="n">
         <f aca="false">P22+O22</f>
-        <v>16</v>
+        <v>60</v>
       </c>
       <c r="R22" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A22)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A22)),IF(COUNTIF($E$2:$E$61,$A22)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A22)),IF(COUNTIF($F$2:$F$61,$A22)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A22)),IF(COUNTIF($G$2:$G$61,$A22)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A22)))</f>
-        <v>45</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A22)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A22)),IF(COUNTIF($E$2:$E$65,$A22)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A22)),IF(COUNTIF($F$2:$F$65,$A22)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A22)),IF(COUNTIF($G$2:$G$65,$A22)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A22)))</f>
+        <v>62</v>
       </c>
       <c r="S22" s="0" t="n">
         <f aca="false">R22-O22</f>
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="T22" s="0" t="n">
         <f aca="false">S22-P22</f>
-        <v>29</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D23" s="0" t="s">
-        <v>62</v>
-      </c>
-      <c r="H23" s="0" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="O23" s="0" t="n">
         <f aca="false">IF(H23&lt;&gt;"",H23,IF(AND(I23&lt;&gt;"",J23&lt;&gt;""),(I23+J23)/2,0))</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P23" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D23,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E23,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F23,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G23,$A$2:$A$61,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D23,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E23,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F23,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G23,$A$2:$A$65,0)),0))</f>
         <v>0</v>
       </c>
       <c r="Q23" s="0" t="n">
         <f aca="false">P23+O23</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R23" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A23)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A23)),IF(COUNTIF($E$2:$E$61,$A23)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A23)),IF(COUNTIF($F$2:$F$61,$A23)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A23)),IF(COUNTIF($G$2:$G$61,$A23)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A23)))</f>
-        <v>5</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A23)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A23)),IF(COUNTIF($E$2:$E$65,$A23)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A23)),IF(COUNTIF($F$2:$F$65,$A23)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A23)),IF(COUNTIF($G$2:$G$65,$A23)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A23)))</f>
+        <v>0</v>
       </c>
       <c r="S23" s="0" t="n">
         <f aca="false">R23-O23</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="T23" s="0" t="n">
         <f aca="false">S23-P23</f>
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B24" s="0" t="s">
         <v>68</v>
       </c>
-      <c r="B24" s="0" t="s">
-        <v>63</v>
-      </c>
       <c r="C24" s="0" t="s">
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="D24" s="0" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H24" s="0" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="O24" s="0" t="n">
         <f aca="false">IF(H24&lt;&gt;"",H24,IF(AND(I24&lt;&gt;"",J24&lt;&gt;""),(I24+J24)/2,0))</f>
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="P24" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D24,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E24,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F24,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G24,$A$2:$A$61,0)),0))</f>
-        <v>2</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D24,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E24,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F24,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G24,$A$2:$A$65,0)),0))</f>
+        <v>0</v>
       </c>
       <c r="Q24" s="0" t="n">
         <f aca="false">P24+O24</f>
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="R24" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A24)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A24)),IF(COUNTIF($E$2:$E$61,$A24)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A24)),IF(COUNTIF($F$2:$F$61,$A24)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A24)),IF(COUNTIF($G$2:$G$61,$A24)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A24)))</f>
-        <v>60</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A24)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A24)),IF(COUNTIF($E$2:$E$65,$A24)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A24)),IF(COUNTIF($F$2:$F$65,$A24)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A24)),IF(COUNTIF($G$2:$G$65,$A24)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A24)))</f>
+        <v>42</v>
       </c>
       <c r="S24" s="0" t="n">
         <f aca="false">R24-O24</f>
-        <v>55</v>
+        <v>26</v>
       </c>
       <c r="T24" s="0" t="n">
         <f aca="false">S24-P24</f>
-        <v>53</v>
+        <v>26</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D25" s="0" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H25" s="0" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="O25" s="0" t="n">
         <f aca="false">IF(H25&lt;&gt;"",H25,IF(AND(I25&lt;&gt;"",J25&lt;&gt;""),(I25+J25)/2,0))</f>
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="P25" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D25,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E25,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F25,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G25,$A$2:$A$61,0)),0))</f>
-        <v>2</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D25,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E25,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F25,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G25,$A$2:$A$65,0)),0))</f>
+        <v>0</v>
       </c>
       <c r="Q25" s="0" t="n">
         <f aca="false">P25+O25</f>
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="R25" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A25)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A25)),IF(COUNTIF($E$2:$E$61,$A25)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A25)),IF(COUNTIF($F$2:$F$61,$A25)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A25)),IF(COUNTIF($G$2:$G$61,$A25)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A25)))</f>
-        <v>20</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A25)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A25)),IF(COUNTIF($E$2:$E$65,$A25)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A25)),IF(COUNTIF($F$2:$F$65,$A25)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A25)),IF(COUNTIF($G$2:$G$65,$A25)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A25)))</f>
+        <v>2</v>
       </c>
       <c r="S25" s="0" t="n">
         <f aca="false">R25-O25</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="T25" s="0" t="n">
         <f aca="false">S25-P25</f>
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D26" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="H26" s="0" t="n">
         <v>5</v>
@@ -1784,170 +1796,167 @@
         <v>5</v>
       </c>
       <c r="P26" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D26,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E26,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F26,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G26,$A$2:$A$61,0)),0))</f>
-        <v>7</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D26,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E26,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F26,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G26,$A$2:$A$65,0)),0))</f>
+        <v>2</v>
       </c>
       <c r="Q26" s="0" t="n">
         <f aca="false">P26+O26</f>
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="R26" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A26)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A26)),IF(COUNTIF($E$2:$E$61,$A26)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A26)),IF(COUNTIF($F$2:$F$61,$A26)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A26)),IF(COUNTIF($G$2:$G$61,$A26)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A26)))</f>
-        <v>65</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A26)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A26)),IF(COUNTIF($E$2:$E$65,$A26)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A26)),IF(COUNTIF($F$2:$F$65,$A26)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A26)),IF(COUNTIF($G$2:$G$65,$A26)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A26)))</f>
+        <v>57</v>
       </c>
       <c r="S26" s="0" t="n">
         <f aca="false">R26-O26</f>
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="T26" s="0" t="n">
         <f aca="false">S26-P26</f>
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H27" s="0" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="O27" s="0" t="n">
         <f aca="false">IF(H27&lt;&gt;"",H27,IF(AND(I27&lt;&gt;"",J27&lt;&gt;""),(I27+J27)/2,0))</f>
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="P27" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D27,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E27,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F27,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G27,$A$2:$A$61,0)),0))</f>
-        <v>17</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D27,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E27,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F27,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G27,$A$2:$A$65,0)),0))</f>
+        <v>2</v>
       </c>
       <c r="Q27" s="0" t="n">
         <f aca="false">P27+O27</f>
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="R27" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A27)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A27)),IF(COUNTIF($E$2:$E$61,$A27)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A27)),IF(COUNTIF($F$2:$F$61,$A27)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A27)),IF(COUNTIF($G$2:$G$61,$A27)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A27)))</f>
-        <v>45</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A27)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A27)),IF(COUNTIF($E$2:$E$65,$A27)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A27)),IF(COUNTIF($F$2:$F$65,$A27)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A27)),IF(COUNTIF($G$2:$G$65,$A27)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A27)))</f>
+        <v>17</v>
       </c>
       <c r="S27" s="0" t="n">
         <f aca="false">R27-O27</f>
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="T27" s="0" t="n">
         <f aca="false">S27-P27</f>
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="D28" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="E28" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="F28" s="0" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="H28" s="0" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="O28" s="0" t="n">
         <f aca="false">IF(H28&lt;&gt;"",H28,IF(AND(I28&lt;&gt;"",J28&lt;&gt;""),(I28+J28)/2,0))</f>
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="P28" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D28,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E28,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F28,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G28,$A$2:$A$61,0)),0))</f>
-        <v>17</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D28,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E28,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F28,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G28,$A$2:$A$65,0)),0))</f>
+        <v>7</v>
       </c>
       <c r="Q28" s="0" t="n">
         <f aca="false">P28+O28</f>
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="R28" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A28)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A28)),IF(COUNTIF($E$2:$E$61,$A28)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A28)),IF(COUNTIF($F$2:$F$61,$A28)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A28)),IF(COUNTIF($G$2:$G$61,$A28)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A28)))</f>
-        <v>58.5</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A28)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A28)),IF(COUNTIF($E$2:$E$65,$A28)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A28)),IF(COUNTIF($F$2:$F$65,$A28)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A28)),IF(COUNTIF($G$2:$G$65,$A28)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A28)))</f>
+        <v>62</v>
       </c>
       <c r="S28" s="0" t="n">
         <f aca="false">R28-O28</f>
-        <v>38.5</v>
+        <v>57</v>
       </c>
       <c r="T28" s="0" t="n">
         <f aca="false">S28-P28</f>
-        <v>21.5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H29" s="0" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="O29" s="0" t="n">
         <f aca="false">IF(H29&lt;&gt;"",H29,IF(AND(I29&lt;&gt;"",J29&lt;&gt;""),(I29+J29)/2,0))</f>
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="P29" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D29,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E29,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F29,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G29,$A$2:$A$61,0)),0))</f>
-        <v>7</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D29,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E29,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F29,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G29,$A$2:$A$65,0)),0))</f>
+        <v>17</v>
       </c>
       <c r="Q29" s="0" t="n">
         <f aca="false">P29+O29</f>
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="R29" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A29)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A29)),IF(COUNTIF($E$2:$E$61,$A29)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A29)),IF(COUNTIF($F$2:$F$61,$A29)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A29)),IF(COUNTIF($G$2:$G$61,$A29)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A29)))</f>
-        <v>38.5</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A29)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A29)),IF(COUNTIF($E$2:$E$65,$A29)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A29)),IF(COUNTIF($F$2:$F$65,$A29)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A29)),IF(COUNTIF($G$2:$G$65,$A29)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A29)))</f>
+        <v>42</v>
       </c>
       <c r="S29" s="0" t="n">
         <f aca="false">R29-O29</f>
-        <v>33.5</v>
+        <v>17</v>
       </c>
       <c r="T29" s="0" t="n">
         <f aca="false">S29-P29</f>
-        <v>26.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C30" s="0" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="D30" s="0" t="s">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="E30" s="0" t="s">
-        <v>74</v>
+        <v>83</v>
+      </c>
+      <c r="F30" s="0" t="s">
+        <v>75</v>
       </c>
       <c r="H30" s="0" t="n">
         <v>20</v>
@@ -1957,38 +1966,38 @@
         <v>20</v>
       </c>
       <c r="P30" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D30,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E30,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F30,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G30,$A$2:$A$61,0)),0))</f>
-        <v>42</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D30,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E30,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F30,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G30,$A$2:$A$65,0)),0))</f>
+        <v>17</v>
       </c>
       <c r="Q30" s="0" t="n">
         <f aca="false">P30+O30</f>
-        <v>62</v>
+        <v>37</v>
       </c>
       <c r="R30" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A30)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A30)),IF(COUNTIF($E$2:$E$61,$A30)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A30)),IF(COUNTIF($F$2:$F$61,$A30)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A30)),IF(COUNTIF($G$2:$G$61,$A30)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A30)))</f>
-        <v>65</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A30)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A30)),IF(COUNTIF($E$2:$E$65,$A30)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A30)),IF(COUNTIF($F$2:$F$65,$A30)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A30)),IF(COUNTIF($G$2:$G$65,$A30)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A30)))</f>
+        <v>55.5</v>
       </c>
       <c r="S30" s="0" t="n">
         <f aca="false">R30-O30</f>
-        <v>45</v>
+        <v>35.5</v>
       </c>
       <c r="T30" s="0" t="n">
         <f aca="false">S30-P30</f>
-        <v>3</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C31" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="D31" s="0" t="s">
         <v>82</v>
-      </c>
-      <c r="D31" s="0" t="s">
-        <v>66</v>
       </c>
       <c r="H31" s="0" t="n">
         <v>5</v>
@@ -1998,150 +2007,150 @@
         <v>5</v>
       </c>
       <c r="P31" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D31,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E31,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F31,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G31,$A$2:$A$61,0)),0))</f>
-        <v>2</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D31,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E31,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F31,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G31,$A$2:$A$65,0)),0))</f>
+        <v>7</v>
       </c>
       <c r="Q31" s="0" t="n">
         <f aca="false">P31+O31</f>
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="R31" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A31)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A31)),IF(COUNTIF($E$2:$E$61,$A31)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A31)),IF(COUNTIF($F$2:$F$61,$A31)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A31)),IF(COUNTIF($G$2:$G$61,$A31)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A31)))</f>
-        <v>33.5</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A31)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A31)),IF(COUNTIF($E$2:$E$65,$A31)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A31)),IF(COUNTIF($F$2:$F$65,$A31)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A31)),IF(COUNTIF($G$2:$G$65,$A31)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A31)))</f>
+        <v>35.5</v>
       </c>
       <c r="S31" s="0" t="n">
         <f aca="false">R31-O31</f>
-        <v>28.5</v>
+        <v>30.5</v>
       </c>
       <c r="T31" s="0" t="n">
         <f aca="false">S31-P31</f>
-        <v>26.5</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C32" s="0" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D32" s="0" t="s">
-        <v>77</v>
+        <v>70</v>
+      </c>
+      <c r="E32" s="0" t="s">
+        <v>79</v>
       </c>
       <c r="H32" s="0" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="O32" s="0" t="n">
         <f aca="false">IF(H32&lt;&gt;"",H32,IF(AND(I32&lt;&gt;"",J32&lt;&gt;""),(I32+J32)/2,0))</f>
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="P32" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D32,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E32,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F32,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G32,$A$2:$A$61,0)),0))</f>
-        <v>7</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D32,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E32,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F32,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G32,$A$2:$A$65,0)),0))</f>
+        <v>42</v>
       </c>
       <c r="Q32" s="0" t="n">
         <f aca="false">P32+O32</f>
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="R32" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A32)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A32)),IF(COUNTIF($E$2:$E$61,$A32)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A32)),IF(COUNTIF($F$2:$F$61,$A32)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A32)),IF(COUNTIF($G$2:$G$61,$A32)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A32)))</f>
-        <v>65</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A32)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A32)),IF(COUNTIF($E$2:$E$65,$A32)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A32)),IF(COUNTIF($F$2:$F$65,$A32)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A32)),IF(COUNTIF($G$2:$G$65,$A32)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A32)))</f>
+        <v>62</v>
       </c>
       <c r="S32" s="0" t="n">
         <f aca="false">R32-O32</f>
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="T32" s="0" t="n">
         <f aca="false">S32-P32</f>
-        <v>53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C33" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D33" s="0" t="s">
-        <v>76</v>
-      </c>
-      <c r="E33" s="0" t="s">
-        <v>74</v>
-      </c>
-      <c r="I33" s="0" t="n">
+        <v>71</v>
+      </c>
+      <c r="H33" s="0" t="n">
         <v>5</v>
-      </c>
-      <c r="J33" s="0" t="n">
-        <v>8</v>
       </c>
       <c r="O33" s="0" t="n">
         <f aca="false">IF(H33&lt;&gt;"",H33,IF(AND(I33&lt;&gt;"",J33&lt;&gt;""),(I33+J33)/2,0))</f>
-        <v>6.5</v>
+        <v>5</v>
       </c>
       <c r="P33" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D33,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E33,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F33,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G33,$A$2:$A$61,0)),0))</f>
-        <v>42</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D33,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E33,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F33,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G33,$A$2:$A$65,0)),0))</f>
+        <v>2</v>
       </c>
       <c r="Q33" s="0" t="n">
         <f aca="false">P33+O33</f>
-        <v>48.5</v>
+        <v>7</v>
       </c>
       <c r="R33" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A33)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A33)),IF(COUNTIF($E$2:$E$61,$A33)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A33)),IF(COUNTIF($F$2:$F$61,$A33)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A33)),IF(COUNTIF($G$2:$G$61,$A33)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A33)))</f>
-        <v>65</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A33)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A33)),IF(COUNTIF($E$2:$E$65,$A33)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A33)),IF(COUNTIF($F$2:$F$65,$A33)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A33)),IF(COUNTIF($G$2:$G$65,$A33)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A33)))</f>
+        <v>30.5</v>
       </c>
       <c r="S33" s="0" t="n">
         <f aca="false">R33-O33</f>
-        <v>58.5</v>
+        <v>25.5</v>
       </c>
       <c r="T33" s="0" t="n">
         <f aca="false">S33-P33</f>
-        <v>16.5</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="C34" s="0" t="s">
         <v>89</v>
       </c>
       <c r="D34" s="0" t="s">
-        <v>23</v>
+        <v>82</v>
+      </c>
+      <c r="H34" s="0" t="n">
+        <v>5</v>
       </c>
       <c r="O34" s="0" t="n">
         <f aca="false">IF(H34&lt;&gt;"",H34,IF(AND(I34&lt;&gt;"",J34&lt;&gt;""),(I34+J34)/2,0))</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P34" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D34,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E34,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F34,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G34,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D34,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E34,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F34,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G34,$A$2:$A$65,0)),0))</f>
+        <v>7</v>
       </c>
       <c r="Q34" s="0" t="n">
         <f aca="false">P34+O34</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="R34" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A34)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A34)),IF(COUNTIF($E$2:$E$61,$A34)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A34)),IF(COUNTIF($F$2:$F$61,$A34)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A34)),IF(COUNTIF($G$2:$G$61,$A34)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A34)))</f>
-        <v>26.5</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A34)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A34)),IF(COUNTIF($E$2:$E$65,$A34)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A34)),IF(COUNTIF($F$2:$F$65,$A34)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A34)),IF(COUNTIF($G$2:$G$65,$A34)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A34)))</f>
+        <v>62</v>
       </c>
       <c r="S34" s="0" t="n">
         <f aca="false">R34-O34</f>
-        <v>26.5</v>
+        <v>57</v>
       </c>
       <c r="T34" s="0" t="n">
         <f aca="false">S34-P34</f>
-        <v>26.5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2149,40 +2158,46 @@
         <v>90</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="C35" s="0" t="s">
         <v>91</v>
       </c>
       <c r="D35" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="H35" s="0" t="n">
-        <v>3</v>
+        <v>81</v>
+      </c>
+      <c r="E35" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="I35" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="J35" s="0" t="n">
+        <v>8</v>
       </c>
       <c r="O35" s="0" t="n">
         <f aca="false">IF(H35&lt;&gt;"",H35,IF(AND(I35&lt;&gt;"",J35&lt;&gt;""),(I35+J35)/2,0))</f>
-        <v>3</v>
+        <v>6.5</v>
       </c>
       <c r="P35" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D35,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E35,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F35,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G35,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D35,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E35,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F35,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G35,$A$2:$A$65,0)),0))</f>
+        <v>42</v>
       </c>
       <c r="Q35" s="0" t="n">
         <f aca="false">P35+O35</f>
-        <v>3</v>
+        <v>48.5</v>
       </c>
       <c r="R35" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A35)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A35)),IF(COUNTIF($E$2:$E$61,$A35)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A35)),IF(COUNTIF($F$2:$F$61,$A35)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A35)),IF(COUNTIF($G$2:$G$61,$A35)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A35)))</f>
-        <v>29.5</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A35)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A35)),IF(COUNTIF($E$2:$E$65,$A35)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A35)),IF(COUNTIF($F$2:$F$65,$A35)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A35)),IF(COUNTIF($G$2:$G$65,$A35)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A35)))</f>
+        <v>62</v>
       </c>
       <c r="S35" s="0" t="n">
         <f aca="false">R35-O35</f>
-        <v>26.5</v>
+        <v>55.5</v>
       </c>
       <c r="T35" s="0" t="n">
         <f aca="false">S35-P35</f>
-        <v>26.5</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2190,40 +2205,40 @@
         <v>92</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="C36" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="D36" s="0" t="s">
         <v>93</v>
       </c>
-      <c r="D36" s="0" t="s">
-        <v>87</v>
-      </c>
       <c r="H36" s="0" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O36" s="0" t="n">
         <f aca="false">IF(H36&lt;&gt;"",H36,IF(AND(I36&lt;&gt;"",J36&lt;&gt;""),(I36+J36)/2,0))</f>
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="P36" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D36,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E36,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F36,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G36,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D36,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E36,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F36,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G36,$A$2:$A$65,0)),0))</f>
+        <v>62</v>
       </c>
       <c r="Q36" s="0" t="n">
         <f aca="false">P36+O36</f>
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="R36" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A36)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A36)),IF(COUNTIF($E$2:$E$61,$A36)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A36)),IF(COUNTIF($F$2:$F$61,$A36)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A36)),IF(COUNTIF($G$2:$G$61,$A36)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A36)))</f>
-        <v>45</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A36)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A36)),IF(COUNTIF($E$2:$E$65,$A36)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A36)),IF(COUNTIF($F$2:$F$65,$A36)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A36)),IF(COUNTIF($G$2:$G$65,$A36)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A36)))</f>
+        <v>63</v>
       </c>
       <c r="S36" s="0" t="n">
         <f aca="false">R36-O36</f>
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="T36" s="0" t="n">
         <f aca="false">S36-P36</f>
-        <v>35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2231,345 +2246,333 @@
         <v>94</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C37" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D37" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="H37" s="0" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="O37" s="0" t="n">
         <f aca="false">IF(H37&lt;&gt;"",H37,IF(AND(I37&lt;&gt;"",J37&lt;&gt;""),(I37+J37)/2,0))</f>
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="P37" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D37,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E37,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F37,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G37,$A$2:$A$61,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D37,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E37,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F37,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G37,$A$2:$A$65,0)),0))</f>
         <v>0</v>
       </c>
       <c r="Q37" s="0" t="n">
         <f aca="false">P37+O37</f>
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="R37" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A37)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A37)),IF(COUNTIF($E$2:$E$61,$A37)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A37)),IF(COUNTIF($F$2:$F$61,$A37)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A37)),IF(COUNTIF($G$2:$G$61,$A37)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A37)))</f>
-        <v>45</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A37)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A37)),IF(COUNTIF($E$2:$E$65,$A37)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A37)),IF(COUNTIF($F$2:$F$65,$A37)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A37)),IF(COUNTIF($G$2:$G$65,$A37)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A37)))</f>
+        <v>41.75</v>
       </c>
       <c r="S37" s="0" t="n">
         <f aca="false">R37-O37</f>
-        <v>30</v>
+        <v>41.75</v>
       </c>
       <c r="T37" s="0" t="n">
         <f aca="false">S37-P37</f>
-        <v>30</v>
+        <v>41.75</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D38" s="0" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="H38" s="0" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="O38" s="0" t="n">
         <f aca="false">IF(H38&lt;&gt;"",H38,IF(AND(I38&lt;&gt;"",J38&lt;&gt;""),(I38+J38)/2,0))</f>
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="P38" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D38,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E38,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F38,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G38,$A$2:$A$61,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D38,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E38,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F38,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G38,$A$2:$A$65,0)),0))</f>
         <v>0</v>
       </c>
       <c r="Q38" s="0" t="n">
         <f aca="false">P38+O38</f>
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="R38" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A38)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A38)),IF(COUNTIF($E$2:$E$61,$A38)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A38)),IF(COUNTIF($F$2:$F$61,$A38)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A38)),IF(COUNTIF($G$2:$G$61,$A38)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A38)))</f>
-        <v>45</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A38)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A38)),IF(COUNTIF($E$2:$E$65,$A38)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A38)),IF(COUNTIF($F$2:$F$65,$A38)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A38)),IF(COUNTIF($G$2:$G$65,$A38)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A38)))</f>
+        <v>44.75</v>
       </c>
       <c r="S38" s="0" t="n">
         <f aca="false">R38-O38</f>
-        <v>30</v>
+        <v>41.75</v>
       </c>
       <c r="T38" s="0" t="n">
         <f aca="false">S38-P38</f>
-        <v>30</v>
+        <v>41.75</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C39" s="0" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="D39" s="0" t="s">
-        <v>96</v>
-      </c>
-      <c r="E39" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="F39" s="0" t="s">
-        <v>92</v>
-      </c>
       <c r="H39" s="0" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="O39" s="0" t="n">
         <f aca="false">IF(H39&lt;&gt;"",H39,IF(AND(I39&lt;&gt;"",J39&lt;&gt;""),(I39+J39)/2,0))</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="P39" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D39,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E39,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F39,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G39,$A$2:$A$61,0)),0))</f>
-        <v>15</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D39,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E39,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F39,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G39,$A$2:$A$65,0)),0))</f>
+        <v>0</v>
       </c>
       <c r="Q39" s="0" t="n">
         <f aca="false">P39+O39</f>
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="R39" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A39)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A39)),IF(COUNTIF($E$2:$E$61,$A39)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A39)),IF(COUNTIF($F$2:$F$61,$A39)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A39)),IF(COUNTIF($G$2:$G$61,$A39)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A39)))</f>
-        <v>50</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A39)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A39)),IF(COUNTIF($E$2:$E$65,$A39)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A39)),IF(COUNTIF($F$2:$F$65,$A39)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A39)),IF(COUNTIF($G$2:$G$65,$A39)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A39)))</f>
+        <v>60.25</v>
       </c>
       <c r="S39" s="0" t="n">
         <f aca="false">R39-O39</f>
-        <v>45</v>
+        <v>50.25</v>
       </c>
       <c r="T39" s="0" t="n">
         <f aca="false">S39-P39</f>
-        <v>30</v>
+        <v>50.25</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C40" s="0" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D40" s="0" t="s">
-        <v>90</v>
-      </c>
-      <c r="I40" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="J40" s="0" t="n">
-        <v>8</v>
+        <v>94</v>
+      </c>
+      <c r="H40" s="0" t="n">
+        <v>15</v>
       </c>
       <c r="O40" s="0" t="n">
         <f aca="false">IF(H40&lt;&gt;"",H40,IF(AND(I40&lt;&gt;"",J40&lt;&gt;""),(I40+J40)/2,0))</f>
-        <v>6.5</v>
+        <v>15</v>
       </c>
       <c r="P40" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D40,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E40,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F40,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G40,$A$2:$A$61,0)),0))</f>
-        <v>3</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D40,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E40,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F40,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G40,$A$2:$A$65,0)),0))</f>
+        <v>0</v>
       </c>
       <c r="Q40" s="0" t="n">
         <f aca="false">P40+O40</f>
-        <v>9.5</v>
+        <v>15</v>
       </c>
       <c r="R40" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A40)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A40)),IF(COUNTIF($E$2:$E$61,$A40)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A40)),IF(COUNTIF($F$2:$F$61,$A40)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A40)),IF(COUNTIF($G$2:$G$61,$A40)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A40)))</f>
-        <v>36</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A40)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A40)),IF(COUNTIF($E$2:$E$65,$A40)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A40)),IF(COUNTIF($F$2:$F$65,$A40)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A40)),IF(COUNTIF($G$2:$G$65,$A40)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A40)))</f>
+        <v>60.25</v>
       </c>
       <c r="S40" s="0" t="n">
         <f aca="false">R40-O40</f>
-        <v>29.5</v>
+        <v>45.25</v>
       </c>
       <c r="T40" s="0" t="n">
         <f aca="false">S40-P40</f>
-        <v>26.5</v>
+        <v>45.25</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C41" s="0" t="s">
-        <v>45</v>
+        <v>104</v>
       </c>
       <c r="D41" s="0" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="H41" s="0" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="O41" s="0" t="n">
         <f aca="false">IF(H41&lt;&gt;"",H41,IF(AND(I41&lt;&gt;"",J41&lt;&gt;""),(I41+J41)/2,0))</f>
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="P41" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D41,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E41,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F41,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G41,$A$2:$A$61,0)),0))</f>
-        <v>15</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D41,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E41,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F41,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G41,$A$2:$A$65,0)),0))</f>
+        <v>0</v>
       </c>
       <c r="Q41" s="0" t="n">
         <f aca="false">P41+O41</f>
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="R41" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A41)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A41)),IF(COUNTIF($E$2:$E$61,$A41)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A41)),IF(COUNTIF($F$2:$F$61,$A41)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A41)),IF(COUNTIF($G$2:$G$61,$A41)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A41)))</f>
-        <v>82.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A41)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A41)),IF(COUNTIF($E$2:$E$65,$A41)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A41)),IF(COUNTIF($F$2:$F$65,$A41)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A41)),IF(COUNTIF($G$2:$G$65,$A41)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A41)))</f>
+        <v>60.25</v>
       </c>
       <c r="S41" s="0" t="n">
         <f aca="false">R41-O41</f>
-        <v>77.25</v>
+        <v>45.25</v>
       </c>
       <c r="T41" s="0" t="n">
         <f aca="false">S41-P41</f>
-        <v>62.25</v>
+        <v>45.25</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C42" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="D42" s="0" t="s">
         <v>103</v>
       </c>
-      <c r="D42" s="0" t="s">
+      <c r="E42" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="F42" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="I42" s="0" t="n">
-        <v>20</v>
-      </c>
-      <c r="J42" s="0" t="n">
-        <v>28</v>
-      </c>
-      <c r="M42" s="0" t="s">
-        <v>104</v>
+      <c r="H42" s="0" t="n">
+        <v>5</v>
       </c>
       <c r="O42" s="0" t="n">
         <f aca="false">IF(H42&lt;&gt;"",H42,IF(AND(I42&lt;&gt;"",J42&lt;&gt;""),(I42+J42)/2,0))</f>
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="P42" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D42,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E42,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F42,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G42,$A$2:$A$61,0)),0))</f>
-        <v>9.5</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D42,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E42,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F42,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G42,$A$2:$A$65,0)),0))</f>
+        <v>15</v>
       </c>
       <c r="Q42" s="0" t="n">
         <f aca="false">P42+O42</f>
-        <v>33.5</v>
+        <v>20</v>
       </c>
       <c r="R42" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A42)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A42)),IF(COUNTIF($E$2:$E$61,$A42)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A42)),IF(COUNTIF($F$2:$F$61,$A42)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A42)),IF(COUNTIF($G$2:$G$61,$A42)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A42)))</f>
-        <v>60</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A42)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A42)),IF(COUNTIF($E$2:$E$65,$A42)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A42)),IF(COUNTIF($F$2:$F$65,$A42)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A42)),IF(COUNTIF($G$2:$G$65,$A42)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A42)))</f>
+        <v>65.25</v>
       </c>
       <c r="S42" s="0" t="n">
         <f aca="false">R42-O42</f>
-        <v>36</v>
+        <v>60.25</v>
       </c>
       <c r="T42" s="0" t="n">
         <f aca="false">S42-P42</f>
-        <v>26.5</v>
+        <v>45.25</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C43" s="0" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D43" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="H43" s="0" t="n">
+        <v>97</v>
+      </c>
+      <c r="I43" s="0" t="n">
         <v>5</v>
+      </c>
+      <c r="J43" s="0" t="n">
+        <v>8</v>
       </c>
       <c r="O43" s="0" t="n">
         <f aca="false">IF(H43&lt;&gt;"",H43,IF(AND(I43&lt;&gt;"",J43&lt;&gt;""),(I43+J43)/2,0))</f>
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="P43" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D43,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E43,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F43,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G43,$A$2:$A$61,0)),0))</f>
-        <v>33.5</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D43,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E43,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F43,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G43,$A$2:$A$65,0)),0))</f>
+        <v>3</v>
       </c>
       <c r="Q43" s="0" t="n">
         <f aca="false">P43+O43</f>
-        <v>38.5</v>
+        <v>9.5</v>
       </c>
       <c r="R43" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A43)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A43)),IF(COUNTIF($E$2:$E$61,$A43)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A43)),IF(COUNTIF($F$2:$F$61,$A43)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A43)),IF(COUNTIF($G$2:$G$61,$A43)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A43)))</f>
-        <v>65</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A43)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A43)),IF(COUNTIF($E$2:$E$65,$A43)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A43)),IF(COUNTIF($F$2:$F$65,$A43)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A43)),IF(COUNTIF($G$2:$G$65,$A43)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A43)))</f>
+        <v>51.25</v>
       </c>
       <c r="S43" s="0" t="n">
         <f aca="false">R43-O43</f>
-        <v>60</v>
+        <v>44.75</v>
       </c>
       <c r="T43" s="0" t="n">
         <f aca="false">S43-P43</f>
-        <v>26.5</v>
+        <v>41.75</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C44" s="0" t="s">
-        <v>108</v>
+        <v>48</v>
       </c>
       <c r="D44" s="0" t="s">
-        <v>94</v>
-      </c>
-      <c r="E44" s="0" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="H44" s="0" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="O44" s="0" t="n">
         <f aca="false">IF(H44&lt;&gt;"",H44,IF(AND(I44&lt;&gt;"",J44&lt;&gt;""),(I44+J44)/2,0))</f>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="P44" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D44,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E44,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F44,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G44,$A$2:$A$61,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D44,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E44,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F44,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G44,$A$2:$A$65,0)),0))</f>
         <v>15</v>
       </c>
       <c r="Q44" s="0" t="n">
         <f aca="false">P44+O44</f>
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="R44" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A44)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A44)),IF(COUNTIF($E$2:$E$61,$A44)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A44)),IF(COUNTIF($F$2:$F$61,$A44)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A44)),IF(COUNTIF($G$2:$G$61,$A44)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A44)))</f>
-        <v>55</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A44)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A44)),IF(COUNTIF($E$2:$E$65,$A44)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A44)),IF(COUNTIF($F$2:$F$65,$A44)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A44)),IF(COUNTIF($G$2:$G$65,$A44)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A44)))</f>
+        <v>80.25</v>
       </c>
       <c r="S44" s="0" t="n">
         <f aca="false">R44-O44</f>
-        <v>46</v>
+        <v>75.25</v>
       </c>
       <c r="T44" s="0" t="n">
         <f aca="false">S44-P44</f>
-        <v>31</v>
+        <v>60.25</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2577,57 +2580,60 @@
         <v>109</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C45" s="0" t="s">
         <v>110</v>
       </c>
       <c r="D45" s="0" t="s">
-        <v>94</v>
-      </c>
-      <c r="E45" s="0" t="s">
-        <v>96</v>
-      </c>
-      <c r="H45" s="0" t="n">
-        <v>3</v>
+        <v>106</v>
+      </c>
+      <c r="I45" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="J45" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="M45" s="0" t="s">
+        <v>111</v>
       </c>
       <c r="O45" s="0" t="n">
         <f aca="false">IF(H45&lt;&gt;"",H45,IF(AND(I45&lt;&gt;"",J45&lt;&gt;""),(I45+J45)/2,0))</f>
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="P45" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D45,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E45,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F45,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G45,$A$2:$A$61,0)),0))</f>
-        <v>15</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D45,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E45,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F45,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G45,$A$2:$A$65,0)),0))</f>
+        <v>9.5</v>
       </c>
       <c r="Q45" s="0" t="n">
         <f aca="false">P45+O45</f>
-        <v>18</v>
+        <v>33.5</v>
       </c>
       <c r="R45" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A45)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A45)),IF(COUNTIF($E$2:$E$61,$A45)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A45)),IF(COUNTIF($F$2:$F$61,$A45)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A45)),IF(COUNTIF($G$2:$G$61,$A45)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A45)))</f>
-        <v>82.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A45)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A45)),IF(COUNTIF($E$2:$E$65,$A45)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A45)),IF(COUNTIF($F$2:$F$65,$A45)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A45)),IF(COUNTIF($G$2:$G$65,$A45)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A45)))</f>
+        <v>75.25</v>
       </c>
       <c r="S45" s="0" t="n">
         <f aca="false">R45-O45</f>
-        <v>79.25</v>
+        <v>51.25</v>
       </c>
       <c r="T45" s="0" t="n">
         <f aca="false">S45-P45</f>
-        <v>64.25</v>
+        <v>41.75</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C46" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="H46" s="0" t="n">
         <v>5</v>
@@ -2637,232 +2643,241 @@
         <v>5</v>
       </c>
       <c r="P46" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D46,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E46,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F46,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G46,$A$2:$A$61,0)),0))</f>
-        <v>20</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D46,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E46,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F46,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G46,$A$2:$A$65,0)),0))</f>
+        <v>33.5</v>
       </c>
       <c r="Q46" s="0" t="n">
         <f aca="false">P46+O46</f>
-        <v>25</v>
+        <v>38.5</v>
       </c>
       <c r="R46" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A46)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A46)),IF(COUNTIF($E$2:$E$61,$A46)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A46)),IF(COUNTIF($F$2:$F$61,$A46)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A46)),IF(COUNTIF($G$2:$G$61,$A46)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A46)))</f>
-        <v>55</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A46)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A46)),IF(COUNTIF($E$2:$E$65,$A46)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A46)),IF(COUNTIF($F$2:$F$65,$A46)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A46)),IF(COUNTIF($G$2:$G$65,$A46)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A46)))</f>
+        <v>80.25</v>
       </c>
       <c r="S46" s="0" t="n">
         <f aca="false">R46-O46</f>
-        <v>50</v>
+        <v>75.25</v>
       </c>
       <c r="T46" s="0" t="n">
         <f aca="false">S46-P46</f>
-        <v>30</v>
+        <v>41.75</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C47" s="0" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
       <c r="D47" s="0" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="H47" s="0" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="O47" s="0" t="n">
         <f aca="false">IF(H47&lt;&gt;"",H47,IF(AND(I47&lt;&gt;"",J47&lt;&gt;""),(I47+J47)/2,0))</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="P47" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D47,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E47,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F47,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G47,$A$2:$A$61,0)),0))</f>
-        <v>25</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D47,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E47,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F47,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G47,$A$2:$A$65,0)),0))</f>
+        <v>15</v>
       </c>
       <c r="Q47" s="0" t="n">
         <f aca="false">P47+O47</f>
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="R47" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A47)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A47)),IF(COUNTIF($E$2:$E$61,$A47)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A47)),IF(COUNTIF($F$2:$F$61,$A47)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A47)),IF(COUNTIF($G$2:$G$61,$A47)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A47)))</f>
-        <v>65</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A47)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A47)),IF(COUNTIF($E$2:$E$65,$A47)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A47)),IF(COUNTIF($F$2:$F$65,$A47)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A47)),IF(COUNTIF($G$2:$G$65,$A47)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A47)))</f>
+        <v>70.25</v>
       </c>
       <c r="S47" s="0" t="n">
         <f aca="false">R47-O47</f>
-        <v>55</v>
+        <v>61.25</v>
       </c>
       <c r="T47" s="0" t="n">
         <f aca="false">S47-P47</f>
-        <v>30</v>
+        <v>46.25</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B48" s="0" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C48" s="0" t="s">
-        <v>61</v>
+        <v>117</v>
       </c>
       <c r="D48" s="0" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="H48" s="0" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="O48" s="0" t="n">
         <f aca="false">IF(H48&lt;&gt;"",H48,IF(AND(I48&lt;&gt;"",J48&lt;&gt;""),(I48+J48)/2,0))</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="P48" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D48,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E48,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F48,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G48,$A$2:$A$61,0)),0))</f>
-        <v>25</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D48,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E48,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F48,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G48,$A$2:$A$65,0)),0))</f>
+        <v>15</v>
       </c>
       <c r="Q48" s="0" t="n">
         <f aca="false">P48+O48</f>
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="R48" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A48)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A48)),IF(COUNTIF($E$2:$E$61,$A48)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A48)),IF(COUNTIF($F$2:$F$61,$A48)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A48)),IF(COUNTIF($G$2:$G$61,$A48)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A48)))</f>
-        <v>65</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A48)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A48)),IF(COUNTIF($E$2:$E$65,$A48)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A48)),IF(COUNTIF($F$2:$F$65,$A48)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A48)),IF(COUNTIF($G$2:$G$65,$A48)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A48)))</f>
+        <v>80.25</v>
       </c>
       <c r="S48" s="0" t="n">
         <f aca="false">R48-O48</f>
-        <v>55</v>
+        <v>77.25</v>
       </c>
       <c r="T48" s="0" t="n">
         <f aca="false">S48-P48</f>
-        <v>30</v>
+        <v>62.25</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>23</v>
+        <v>118</v>
       </c>
       <c r="B49" s="0" t="s">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="C49" s="0" t="s">
-        <v>116</v>
-      </c>
-      <c r="N49" s="2" t="n">
-        <v>40080</v>
+        <v>119</v>
+      </c>
+      <c r="D49" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="H49" s="0" t="n">
+        <v>5</v>
       </c>
       <c r="O49" s="0" t="n">
         <f aca="false">IF(H49&lt;&gt;"",H49,IF(AND(I49&lt;&gt;"",J49&lt;&gt;""),(I49+J49)/2,0))</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P49" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D49,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E49,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F49,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G49,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D49,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E49,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F49,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G49,$A$2:$A$65,0)),0))</f>
+        <v>20</v>
       </c>
       <c r="Q49" s="0" t="n">
         <f aca="false">P49+O49</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="R49" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A49)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A49)),IF(COUNTIF($E$2:$E$61,$A49)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A49)),IF(COUNTIF($F$2:$F$61,$A49)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A49)),IF(COUNTIF($G$2:$G$61,$A49)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A49)))</f>
-        <v>0</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A49)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A49)),IF(COUNTIF($E$2:$E$65,$A49)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A49)),IF(COUNTIF($F$2:$F$65,$A49)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A49)),IF(COUNTIF($G$2:$G$65,$A49)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A49)))</f>
+        <v>70.25</v>
       </c>
       <c r="S49" s="0" t="n">
         <f aca="false">R49-O49</f>
-        <v>0</v>
+        <v>65.25</v>
       </c>
       <c r="T49" s="0" t="n">
         <f aca="false">S49-P49</f>
-        <v>0</v>
+        <v>45.25</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="C50" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="D50" s="0" t="s">
         <v>118</v>
       </c>
-      <c r="D50" s="0" t="s">
-        <v>119</v>
-      </c>
-      <c r="I50" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="J50" s="0" t="n">
+      <c r="E50" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="H50" s="0" t="n">
         <v>10</v>
       </c>
       <c r="O50" s="0" t="n">
         <f aca="false">IF(H50&lt;&gt;"",H50,IF(AND(I50&lt;&gt;"",J50&lt;&gt;""),(I50+J50)/2,0))</f>
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="P50" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D50,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E50,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F50,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G50,$A$2:$A$61,0)),0))</f>
-        <v>74</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D50,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E50,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F50,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G50,$A$2:$A$65,0)),0))</f>
+        <v>25</v>
       </c>
       <c r="Q50" s="0" t="n">
         <f aca="false">P50+O50</f>
-        <v>81.5</v>
+        <v>35</v>
       </c>
       <c r="R50" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A50)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A50)),IF(COUNTIF($E$2:$E$61,$A50)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A50)),IF(COUNTIF($F$2:$F$61,$A50)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A50)),IF(COUNTIF($G$2:$G$61,$A50)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A50)))</f>
-        <v>81.5</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A50)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A50)),IF(COUNTIF($E$2:$E$65,$A50)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A50)),IF(COUNTIF($F$2:$F$65,$A50)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A50)),IF(COUNTIF($G$2:$G$65,$A50)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A50)))</f>
+        <v>80.25</v>
       </c>
       <c r="S50" s="0" t="n">
         <f aca="false">R50-O50</f>
-        <v>74</v>
+        <v>70.25</v>
       </c>
       <c r="T50" s="0" t="n">
         <f aca="false">S50-P50</f>
-        <v>0</v>
+        <v>45.25</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B51" s="0" t="s">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="C51" s="0" t="s">
-        <v>121</v>
+        <v>66</v>
       </c>
       <c r="D51" s="0" t="s">
-        <v>23</v>
+        <v>118</v>
+      </c>
+      <c r="E51" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="H51" s="0" t="n">
+        <v>10</v>
       </c>
       <c r="O51" s="0" t="n">
         <f aca="false">IF(H51&lt;&gt;"",H51,IF(AND(I51&lt;&gt;"",J51&lt;&gt;""),(I51+J51)/2,0))</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P51" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D51,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E51,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F51,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G51,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D51,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E51,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F51,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G51,$A$2:$A$65,0)),0))</f>
+        <v>25</v>
       </c>
       <c r="Q51" s="0" t="n">
         <f aca="false">P51+O51</f>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="R51" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A51)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A51)),IF(COUNTIF($E$2:$E$61,$A51)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A51)),IF(COUNTIF($F$2:$F$61,$A51)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A51)),IF(COUNTIF($G$2:$G$61,$A51)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A51)))</f>
-        <v>48</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A51)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A51)),IF(COUNTIF($E$2:$E$65,$A51)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A51)),IF(COUNTIF($F$2:$F$65,$A51)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A51)),IF(COUNTIF($G$2:$G$65,$A51)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A51)))</f>
+        <v>80.25</v>
       </c>
       <c r="S51" s="0" t="n">
         <f aca="false">R51-O51</f>
-        <v>48</v>
+        <v>70.25</v>
       </c>
       <c r="T51" s="0" t="n">
         <f aca="false">S51-P51</f>
-        <v>48</v>
+        <v>45.25</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2870,83 +2885,74 @@
         <v>122</v>
       </c>
       <c r="B52" s="0" t="s">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="C52" s="0" t="s">
-        <v>123</v>
+        <v>40</v>
       </c>
       <c r="D52" s="0" t="s">
-        <v>120</v>
-      </c>
-      <c r="I52" s="0" t="n">
-        <v>14</v>
-      </c>
-      <c r="J52" s="0" t="n">
-        <v>28</v>
+        <v>62</v>
+      </c>
+      <c r="H52" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="O52" s="0" t="n">
         <f aca="false">IF(H52&lt;&gt;"",H52,IF(AND(I52&lt;&gt;"",J52&lt;&gt;""),(I52+J52)/2,0))</f>
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="P52" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D52,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E52,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F52,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G52,$A$2:$A$61,0)),0))</f>
-        <v>0</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D52,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E52,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F52,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G52,$A$2:$A$65,0)),0))</f>
+        <v>60</v>
       </c>
       <c r="Q52" s="0" t="n">
         <f aca="false">P52+O52</f>
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="R52" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A52)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A52)),IF(COUNTIF($E$2:$E$61,$A52)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A52)),IF(COUNTIF($F$2:$F$61,$A52)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A52)),IF(COUNTIF($G$2:$G$61,$A52)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A52)))</f>
-        <v>69</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A52)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A52)),IF(COUNTIF($E$2:$E$65,$A52)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A52)),IF(COUNTIF($F$2:$F$65,$A52)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A52)),IF(COUNTIF($G$2:$G$65,$A52)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A52)))</f>
+        <v>63</v>
       </c>
       <c r="S52" s="0" t="n">
         <f aca="false">R52-O52</f>
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="T52" s="0" t="n">
         <f aca="false">S52-P52</f>
-        <v>48</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>119</v>
+        <v>23</v>
       </c>
       <c r="B53" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="C53" s="0" t="s">
         <v>124</v>
       </c>
-      <c r="D53" s="0" t="s">
-        <v>125</v>
-      </c>
-      <c r="E53" s="0" t="s">
-        <v>122</v>
-      </c>
-      <c r="H53" s="0" t="n">
-        <v>5</v>
+      <c r="N53" s="2" t="n">
+        <v>40080</v>
       </c>
       <c r="O53" s="0" t="n">
         <f aca="false">IF(H53&lt;&gt;"",H53,IF(AND(I53&lt;&gt;"",J53&lt;&gt;""),(I53+J53)/2,0))</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P53" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D53,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E53,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F53,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G53,$A$2:$A$61,0)),0))</f>
-        <v>69</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D53,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E53,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F53,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G53,$A$2:$A$65,0)),0))</f>
+        <v>0</v>
       </c>
       <c r="Q53" s="0" t="n">
         <f aca="false">P53+O53</f>
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="R53" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A53)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A53)),IF(COUNTIF($E$2:$E$61,$A53)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A53)),IF(COUNTIF($F$2:$F$61,$A53)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A53)),IF(COUNTIF($G$2:$G$61,$A53)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A53)))</f>
-        <v>74</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A53)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A53)),IF(COUNTIF($E$2:$E$65,$A53)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A53)),IF(COUNTIF($F$2:$F$65,$A53)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A53)),IF(COUNTIF($G$2:$G$65,$A53)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A53)))</f>
+        <v>0</v>
       </c>
       <c r="S53" s="0" t="n">
         <f aca="false">R53-O53</f>
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="T53" s="0" t="n">
         <f aca="false">S53-P53</f>
@@ -2955,42 +2961,42 @@
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B54" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="C54" s="0" t="s">
         <v>126</v>
       </c>
-      <c r="B54" s="0" t="s">
-        <v>115</v>
-      </c>
-      <c r="C54" s="0" t="s">
+      <c r="D54" s="0" t="s">
         <v>127</v>
       </c>
-      <c r="D54" s="0" t="s">
-        <v>117</v>
-      </c>
       <c r="I54" s="0" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="J54" s="0" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="O54" s="0" t="n">
         <f aca="false">IF(H54&lt;&gt;"",H54,IF(AND(I54&lt;&gt;"",J54&lt;&gt;""),(I54+J54)/2,0))</f>
-        <v>0.75</v>
+        <v>7.5</v>
       </c>
       <c r="P54" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D54,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E54,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F54,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G54,$A$2:$A$61,0)),0))</f>
-        <v>81.5</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D54,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E54,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F54,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G54,$A$2:$A$65,0)),0))</f>
+        <v>72</v>
       </c>
       <c r="Q54" s="0" t="n">
         <f aca="false">P54+O54</f>
-        <v>82.25</v>
+        <v>79.5</v>
       </c>
       <c r="R54" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A54)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A54)),IF(COUNTIF($E$2:$E$61,$A54)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A54)),IF(COUNTIF($F$2:$F$61,$A54)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A54)),IF(COUNTIF($G$2:$G$61,$A54)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A54)))</f>
-        <v>82.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A54)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A54)),IF(COUNTIF($E$2:$E$65,$A54)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A54)),IF(COUNTIF($F$2:$F$65,$A54)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A54)),IF(COUNTIF($G$2:$G$65,$A54)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A54)))</f>
+        <v>79.5</v>
       </c>
       <c r="S54" s="0" t="n">
         <f aca="false">R54-O54</f>
-        <v>81.5</v>
+        <v>72</v>
       </c>
       <c r="T54" s="0" t="n">
         <f aca="false">S54-P54</f>
@@ -3002,122 +3008,125 @@
         <v>128</v>
       </c>
       <c r="B55" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="C55" s="0" t="s">
         <v>129</v>
       </c>
       <c r="D55" s="0" t="s">
-        <v>117</v>
+        <v>23</v>
       </c>
       <c r="O55" s="0" t="n">
         <f aca="false">IF(H55&lt;&gt;"",H55,IF(AND(I55&lt;&gt;"",J55&lt;&gt;""),(I55+J55)/2,0))</f>
         <v>0</v>
       </c>
       <c r="P55" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D55,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E55,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F55,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G55,$A$2:$A$61,0)),0))</f>
-        <v>81.5</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D55,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E55,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F55,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G55,$A$2:$A$65,0)),0))</f>
+        <v>0</v>
       </c>
       <c r="Q55" s="0" t="n">
         <f aca="false">P55+O55</f>
-        <v>81.5</v>
+        <v>0</v>
       </c>
       <c r="R55" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A55)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A55)),IF(COUNTIF($E$2:$E$61,$A55)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A55)),IF(COUNTIF($F$2:$F$61,$A55)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A55)),IF(COUNTIF($G$2:$G$61,$A55)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A55)))</f>
-        <v>82.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A55)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A55)),IF(COUNTIF($E$2:$E$65,$A55)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A55)),IF(COUNTIF($F$2:$F$65,$A55)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A55)),IF(COUNTIF($G$2:$G$65,$A55)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A55)))</f>
+        <v>46</v>
       </c>
       <c r="S55" s="0" t="n">
         <f aca="false">R55-O55</f>
-        <v>82.25</v>
+        <v>46</v>
       </c>
       <c r="T55" s="0" t="n">
         <f aca="false">S55-P55</f>
-        <v>0.75</v>
+        <v>46</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B56" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="C56" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="H56" s="0" t="n">
-        <v>4</v>
+        <v>128</v>
+      </c>
+      <c r="I56" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="J56" s="0" t="n">
+        <v>28</v>
       </c>
       <c r="O56" s="0" t="n">
         <f aca="false">IF(H56&lt;&gt;"",H56,IF(AND(I56&lt;&gt;"",J56&lt;&gt;""),(I56+J56)/2,0))</f>
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="P56" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D56,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E56,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F56,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G56,$A$2:$A$61,0)),0))</f>
-        <v>65</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D56,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E56,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F56,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G56,$A$2:$A$65,0)),0))</f>
+        <v>0</v>
       </c>
       <c r="Q56" s="0" t="n">
         <f aca="false">P56+O56</f>
-        <v>69</v>
+        <v>21</v>
       </c>
       <c r="R56" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A56)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A56)),IF(COUNTIF($E$2:$E$61,$A56)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A56)),IF(COUNTIF($F$2:$F$61,$A56)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A56)),IF(COUNTIF($G$2:$G$61,$A56)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A56)))</f>
-        <v>69</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A56)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A56)),IF(COUNTIF($E$2:$E$65,$A56)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A56)),IF(COUNTIF($F$2:$F$65,$A56)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A56)),IF(COUNTIF($G$2:$G$65,$A56)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A56)))</f>
+        <v>67</v>
       </c>
       <c r="S56" s="0" t="n">
         <f aca="false">R56-O56</f>
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="T56" s="0" t="n">
         <f aca="false">S56-P56</f>
-        <v>0</v>
+        <v>46</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B57" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="C57" s="0" t="s">
         <v>132</v>
       </c>
-      <c r="B57" s="0" t="s">
-        <v>115</v>
-      </c>
-      <c r="C57" s="0" t="s">
+      <c r="D57" s="0" t="s">
         <v>133</v>
       </c>
-      <c r="D57" s="0" t="s">
-        <v>114</v>
-      </c>
       <c r="E57" s="0" t="s">
-        <v>113</v>
-      </c>
-      <c r="F57" s="0" t="s">
-        <v>105</v>
+        <v>130</v>
+      </c>
+      <c r="H57" s="0" t="n">
+        <v>5</v>
       </c>
       <c r="O57" s="0" t="n">
         <f aca="false">IF(H57&lt;&gt;"",H57,IF(AND(I57&lt;&gt;"",J57&lt;&gt;""),(I57+J57)/2,0))</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P57" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D57,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E57,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F57,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G57,$A$2:$A$61,0)),0))</f>
-        <v>38.5</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D57,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E57,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F57,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G57,$A$2:$A$65,0)),0))</f>
+        <v>67</v>
       </c>
       <c r="Q57" s="0" t="n">
         <f aca="false">P57+O57</f>
-        <v>38.5</v>
+        <v>72</v>
       </c>
       <c r="R57" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A57)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A57)),IF(COUNTIF($E$2:$E$61,$A57)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A57)),IF(COUNTIF($F$2:$F$61,$A57)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A57)),IF(COUNTIF($G$2:$G$61,$A57)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A57)))</f>
-        <v>65</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A57)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A57)),IF(COUNTIF($E$2:$E$65,$A57)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A57)),IF(COUNTIF($F$2:$F$65,$A57)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A57)),IF(COUNTIF($G$2:$G$65,$A57)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A57)))</f>
+        <v>72</v>
       </c>
       <c r="S57" s="0" t="n">
         <f aca="false">R57-O57</f>
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="T57" s="0" t="n">
         <f aca="false">S57-P57</f>
-        <v>26.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3125,46 +3134,43 @@
         <v>134</v>
       </c>
       <c r="B58" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="C58" s="0" t="s">
         <v>135</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>83</v>
-      </c>
-      <c r="E58" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="F58" s="0" t="s">
-        <v>80</v>
-      </c>
-      <c r="G58" s="0" t="s">
-        <v>72</v>
+        <v>125</v>
+      </c>
+      <c r="I58" s="0" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J58" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="O58" s="0" t="n">
         <f aca="false">IF(H58&lt;&gt;"",H58,IF(AND(I58&lt;&gt;"",J58&lt;&gt;""),(I58+J58)/2,0))</f>
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="P58" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D58,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E58,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F58,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G58,$A$2:$A$61,0)),0))</f>
-        <v>62</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D58,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E58,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F58,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G58,$A$2:$A$65,0)),0))</f>
+        <v>79.5</v>
       </c>
       <c r="Q58" s="0" t="n">
         <f aca="false">P58+O58</f>
-        <v>62</v>
+        <v>80.25</v>
       </c>
       <c r="R58" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A58)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A58)),IF(COUNTIF($E$2:$E$61,$A58)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A58)),IF(COUNTIF($F$2:$F$61,$A58)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A58)),IF(COUNTIF($G$2:$G$61,$A58)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A58)))</f>
-        <v>65</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A58)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A58)),IF(COUNTIF($E$2:$E$65,$A58)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A58)),IF(COUNTIF($F$2:$F$65,$A58)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A58)),IF(COUNTIF($G$2:$G$65,$A58)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A58)))</f>
+        <v>80.25</v>
       </c>
       <c r="S58" s="0" t="n">
         <f aca="false">R58-O58</f>
-        <v>65</v>
+        <v>79.5</v>
       </c>
       <c r="T58" s="0" t="n">
         <f aca="false">S58-P58</f>
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3172,74 +3178,74 @@
         <v>136</v>
       </c>
       <c r="B59" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="C59" s="0" t="s">
         <v>137</v>
       </c>
       <c r="D59" s="0" t="s">
-        <v>37</v>
+        <v>125</v>
       </c>
       <c r="O59" s="0" t="n">
         <f aca="false">IF(H59&lt;&gt;"",H59,IF(AND(I59&lt;&gt;"",J59&lt;&gt;""),(I59+J59)/2,0))</f>
         <v>0</v>
       </c>
       <c r="P59" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D59,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E59,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F59,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G59,$A$2:$A$61,0)),0))</f>
-        <v>45.5</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D59,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E59,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F59,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G59,$A$2:$A$65,0)),0))</f>
+        <v>79.5</v>
       </c>
       <c r="Q59" s="0" t="n">
         <f aca="false">P59+O59</f>
-        <v>45.5</v>
+        <v>79.5</v>
       </c>
       <c r="R59" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A59)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A59)),IF(COUNTIF($E$2:$E$61,$A59)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A59)),IF(COUNTIF($F$2:$F$61,$A59)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A59)),IF(COUNTIF($G$2:$G$61,$A59)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A59)))</f>
-        <v>65</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A59)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A59)),IF(COUNTIF($E$2:$E$65,$A59)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A59)),IF(COUNTIF($F$2:$F$65,$A59)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A59)),IF(COUNTIF($G$2:$G$65,$A59)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A59)))</f>
+        <v>80.25</v>
       </c>
       <c r="S59" s="0" t="n">
         <f aca="false">R59-O59</f>
-        <v>65</v>
+        <v>80.25</v>
       </c>
       <c r="T59" s="0" t="n">
         <f aca="false">S59-P59</f>
-        <v>19.5</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B60" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="C60" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="D60" s="0" t="s">
         <v>138</v>
       </c>
-      <c r="B60" s="0" t="s">
-        <v>115</v>
-      </c>
-      <c r="C60" s="0" t="s">
-        <v>139</v>
-      </c>
-      <c r="D60" s="0" t="s">
-        <v>58</v>
-      </c>
-      <c r="E60" s="0" t="s">
-        <v>60</v>
+      <c r="H60" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="O60" s="0" t="n">
         <f aca="false">IF(H60&lt;&gt;"",H60,IF(AND(I60&lt;&gt;"",J60&lt;&gt;""),(I60+J60)/2,0))</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P60" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D60,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E60,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F60,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G60,$A$2:$A$61,0)),0))</f>
-        <v>65</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D60,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E60,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F60,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G60,$A$2:$A$65,0)),0))</f>
+        <v>63</v>
       </c>
       <c r="Q60" s="0" t="n">
         <f aca="false">P60+O60</f>
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="R60" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A60)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A60)),IF(COUNTIF($E$2:$E$61,$A60)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A60)),IF(COUNTIF($F$2:$F$61,$A60)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A60)),IF(COUNTIF($G$2:$G$61,$A60)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A60)))</f>
-        <v>65</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A60)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A60)),IF(COUNTIF($E$2:$E$65,$A60)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A60)),IF(COUNTIF($F$2:$F$65,$A60)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A60)),IF(COUNTIF($G$2:$G$65,$A60)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A60)))</f>
+        <v>67</v>
       </c>
       <c r="S60" s="0" t="n">
         <f aca="false">R60-O60</f>
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="T60" s="0" t="n">
         <f aca="false">S60-P60</f>
@@ -3247,100 +3253,270 @@
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="0" t="s">
-        <v>131</v>
+      <c r="A61" s="1" t="s">
+        <v>139</v>
       </c>
       <c r="B61" s="0" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="C61" s="0" t="s">
         <v>140</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>138</v>
+        <v>121</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
       <c r="F61" s="0" t="s">
-        <v>132</v>
-      </c>
-      <c r="G61" s="0" t="s">
-        <v>136</v>
+        <v>112</v>
       </c>
       <c r="O61" s="0" t="n">
         <f aca="false">IF(H61&lt;&gt;"",H61,IF(AND(I61&lt;&gt;"",J61&lt;&gt;""),(I61+J61)/2,0))</f>
         <v>0</v>
       </c>
       <c r="P61" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D61,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E61,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F61,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G61,$A$2:$A$61,0)),0))</f>
-        <v>65</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D61,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E61,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F61,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G61,$A$2:$A$65,0)),0))</f>
+        <v>38.5</v>
       </c>
       <c r="Q61" s="0" t="n">
         <f aca="false">P61+O61</f>
-        <v>65</v>
+        <v>38.5</v>
       </c>
       <c r="R61" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A61)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A61)),IF(COUNTIF($E$2:$E$61,$A61)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A61)),IF(COUNTIF($F$2:$F$61,$A61)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A61)),IF(COUNTIF($G$2:$G$61,$A61)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A61)))</f>
-        <v>65</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A61)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A61)),IF(COUNTIF($E$2:$E$65,$A61)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A61)),IF(COUNTIF($F$2:$F$65,$A61)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A61)),IF(COUNTIF($G$2:$G$65,$A61)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A61)))</f>
+        <v>80.25</v>
       </c>
       <c r="S61" s="0" t="n">
         <f aca="false">R61-O61</f>
-        <v>65</v>
+        <v>80.25</v>
       </c>
       <c r="T61" s="0" t="n">
         <f aca="false">S61-P61</f>
-        <v>0</v>
+        <v>41.75</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B62" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="C62" s="0" t="s">
         <v>141</v>
       </c>
-      <c r="B62" s="0" t="s">
-        <v>115</v>
-      </c>
-      <c r="C62" s="0" t="s">
-        <v>142</v>
-      </c>
       <c r="D62" s="0" t="s">
-        <v>119</v>
-      </c>
-      <c r="K62" s="0" t="s">
-        <v>32</v>
+        <v>88</v>
+      </c>
+      <c r="E62" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="F62" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="G62" s="0" t="s">
+        <v>77</v>
       </c>
       <c r="O62" s="0" t="n">
         <f aca="false">IF(H62&lt;&gt;"",H62,IF(AND(I62&lt;&gt;"",J62&lt;&gt;""),(I62+J62)/2,0))</f>
         <v>0</v>
       </c>
       <c r="P62" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$61,MATCH(D62,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(E62,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(F62,$A$2:$A$61,0)),0),IFERROR(INDEX($Q$2:$Q$61,MATCH(G62,$A$2:$A$61,0)),0))</f>
-        <v>74</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D62,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E62,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F62,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G62,$A$2:$A$65,0)),0))</f>
+        <v>62</v>
       </c>
       <c r="Q62" s="0" t="n">
         <f aca="false">P62+O62</f>
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="R62" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$61,$A62)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$D$2:$D$61,$A62)),IF(COUNTIF($E$2:$E$61,$A62)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$E$2:$E$61,$A62)),IF(COUNTIF($F$2:$F$61,$A62)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$F$2:$F$61,$A62)),IF(COUNTIF($G$2:$G$61,$A62)=0,$O$64,_xlfn.MINIFS($S$2:$S$61,$G$2:$G$61,$A62)))</f>
-        <v>82.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A62)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A62)),IF(COUNTIF($E$2:$E$65,$A62)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A62)),IF(COUNTIF($F$2:$F$65,$A62)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A62)),IF(COUNTIF($G$2:$G$65,$A62)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A62)))</f>
+        <v>62</v>
       </c>
       <c r="S62" s="0" t="n">
         <f aca="false">R62-O62</f>
-        <v>82.25</v>
+        <v>62</v>
       </c>
       <c r="T62" s="0" t="n">
         <f aca="false">S62-P62</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B63" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="C63" s="0" t="s">
+        <v>142</v>
+      </c>
+      <c r="D63" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="O63" s="0" t="n">
+        <f aca="false">IF(H63&lt;&gt;"",H63,IF(AND(I63&lt;&gt;"",J63&lt;&gt;""),(I63+J63)/2,0))</f>
+        <v>0</v>
+      </c>
+      <c r="P63" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D63,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E63,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F63,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G63,$A$2:$A$65,0)),0))</f>
+        <v>45.5</v>
+      </c>
+      <c r="Q63" s="0" t="n">
+        <f aca="false">P63+O63</f>
+        <v>45.5</v>
+      </c>
+      <c r="R63" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A63)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A63)),IF(COUNTIF($E$2:$E$65,$A63)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A63)),IF(COUNTIF($F$2:$F$65,$A63)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A63)),IF(COUNTIF($G$2:$G$65,$A63)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A63)))</f>
+        <v>62</v>
+      </c>
+      <c r="S63" s="0" t="n">
+        <f aca="false">R63-O63</f>
+        <v>62</v>
+      </c>
+      <c r="T63" s="0" t="n">
+        <f aca="false">S63-P63</f>
+        <v>16.5</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B64" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="C64" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="D64" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="E64" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="O64" s="0" t="n">
+        <f aca="false">IF(H64&lt;&gt;"",H64,IF(AND(I64&lt;&gt;"",J64&lt;&gt;""),(I64+J64)/2,0))</f>
+        <v>0</v>
+      </c>
+      <c r="P64" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D64,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E64,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F64,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G64,$A$2:$A$65,0)),0))</f>
+        <v>60</v>
+      </c>
+      <c r="Q64" s="0" t="n">
+        <f aca="false">P64+O64</f>
+        <v>60</v>
+      </c>
+      <c r="R64" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A64)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A64)),IF(COUNTIF($E$2:$E$65,$A64)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A64)),IF(COUNTIF($F$2:$F$65,$A64)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A64)),IF(COUNTIF($G$2:$G$65,$A64)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A64)))</f>
+        <v>62</v>
+      </c>
+      <c r="S64" s="0" t="n">
+        <f aca="false">R64-O64</f>
+        <v>62</v>
+      </c>
+      <c r="T64" s="0" t="n">
+        <f aca="false">S64-P64</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="B65" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="C65" s="0" t="s">
+        <v>144</v>
+      </c>
+      <c r="D65" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E65" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="F65" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="G65" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="O65" s="0" t="n">
+        <f aca="false">IF(H65&lt;&gt;"",H65,IF(AND(I65&lt;&gt;"",J65&lt;&gt;""),(I65+J65)/2,0))</f>
+        <v>0</v>
+      </c>
+      <c r="P65" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D65,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E65,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F65,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G65,$A$2:$A$65,0)),0))</f>
+        <v>63</v>
+      </c>
+      <c r="Q65" s="0" t="n">
+        <f aca="false">P65+O65</f>
+        <v>63</v>
+      </c>
+      <c r="R65" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A65)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A65)),IF(COUNTIF($E$2:$E$65,$A65)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A65)),IF(COUNTIF($F$2:$F$65,$A65)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A65)),IF(COUNTIF($G$2:$G$65,$A65)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A65)))</f>
+        <v>63</v>
+      </c>
+      <c r="S65" s="0" t="n">
+        <f aca="false">R65-O65</f>
+        <v>63</v>
+      </c>
+      <c r="T65" s="0" t="n">
+        <f aca="false">S65-P65</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B66" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="C66" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="D66" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="K66" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="O66" s="0" t="n">
+        <f aca="false">IF(H66&lt;&gt;"",H66,IF(AND(I66&lt;&gt;"",J66&lt;&gt;""),(I66+J66)/2,0))</f>
+        <v>0</v>
+      </c>
+      <c r="P66" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D66,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E66,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F66,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G66,$A$2:$A$65,0)),0))</f>
+        <v>72</v>
+      </c>
+      <c r="Q66" s="0" t="n">
+        <f aca="false">P66+O66</f>
+        <v>72</v>
+      </c>
+      <c r="R66" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A66)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A66)),IF(COUNTIF($E$2:$E$65,$A66)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A66)),IF(COUNTIF($F$2:$F$65,$A66)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A66)),IF(COUNTIF($G$2:$G$65,$A66)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A66)))</f>
+        <v>80.25</v>
+      </c>
+      <c r="S66" s="0" t="n">
+        <f aca="false">R66-O66</f>
+        <v>80.25</v>
+      </c>
+      <c r="T66" s="0" t="n">
+        <f aca="false">S66-P66</f>
         <v>8.25</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N64" s="0" t="s">
-        <v>143</v>
-      </c>
-      <c r="O64" s="0" t="n">
-        <f aca="false">MAX(Q2:Q61)</f>
-        <v>82.25</v>
+    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N68" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="O68" s="0" t="n">
+        <f aca="false">MAX(Q2:Q65)</f>
+        <v>80.25</v>
       </c>
     </row>
   </sheetData>
@@ -3367,22 +3543,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="39.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="35.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="42.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="50.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="40.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Split sanctuary into left and right. Crash bookstore drywall down to 2-4 days
</commit_message>
<xml_diff>
--- a/AC Tasks.xlsx
+++ b/AC Tasks.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="162">
   <si>
     <t xml:space="preserve">Id</t>
   </si>
@@ -236,22 +236,40 @@
     <t xml:space="preserve">S1</t>
   </si>
   <si>
-    <t xml:space="preserve">S2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">core drill for rails</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">install rails</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">install carpeting at seats</t>
+    <t xml:space="preserve">S2.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">core drill for rails (left side)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S2.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">core drill for rails (right side)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S3.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">install rails (left side)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S3.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">install rails (right side)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S4.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">install carpeting at seats (left side)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S4.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">install carpeting at seats (right side)</t>
   </si>
   <si>
     <t xml:space="preserve">S5</t>
@@ -260,10 +278,16 @@
     <t xml:space="preserve">carpeting at rails</t>
   </si>
   <si>
-    <t xml:space="preserve">S6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wood paneling, trim and stage</t>
+    <t xml:space="preserve">S6.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wood paneling, trim and stage (left side)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S6.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wood paneling, trim and stage (right side)</t>
   </si>
   <si>
     <t xml:space="preserve">S7</t>
@@ -278,10 +302,16 @@
     <t xml:space="preserve">concrete floor staining</t>
   </si>
   <si>
-    <t xml:space="preserve">S9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">installation of seats</t>
+    <t xml:space="preserve">S9.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">installation of seats (left side)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S9.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">installation of seats (right side)</t>
   </si>
   <si>
     <t xml:space="preserve">wood stage steps</t>
@@ -392,6 +422,9 @@
     <t xml:space="preserve">L15</t>
   </si>
   <si>
+    <t xml:space="preserve">P10</t>
+  </si>
+  <si>
     <t xml:space="preserve">overall</t>
   </si>
   <si>
@@ -438,9 +471,6 @@
   </si>
   <si>
     <t xml:space="preserve">P15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P10</t>
   </si>
   <si>
     <t xml:space="preserve">lobby done except cleanup and ACI punch list</t>
@@ -691,7 +721,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T68"/>
+  <dimension ref="A1:T73"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.21"/>
@@ -785,7 +815,7 @@
         <v>0</v>
       </c>
       <c r="P2" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D2,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E2,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F2,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G2,$A$2:$A$65,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D2,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E2,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F2,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G2,$A$2:$A$70,0)),0))</f>
         <v>0</v>
       </c>
       <c r="Q2" s="0" t="n">
@@ -793,16 +823,16 @@
         <v>0</v>
       </c>
       <c r="R2" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A2)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A2)),IF(COUNTIF($E$2:$E$65,$A2)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A2)),IF(COUNTIF($F$2:$F$65,$A2)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A2)),IF(COUNTIF($G$2:$G$65,$A2)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A2)))</f>
-        <v>16.5</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A2)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A2)),IF(COUNTIF($E$2:$E$70,$A2)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A2)),IF(COUNTIF($F$2:$F$70,$A2)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A2)),IF(COUNTIF($G$2:$G$70,$A2)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A2)))</f>
+        <v>0.5</v>
       </c>
       <c r="S2" s="0" t="n">
         <f aca="false">R2-O2</f>
-        <v>16.5</v>
+        <v>0.5</v>
       </c>
       <c r="T2" s="0" t="n">
         <f aca="false">S2-P2</f>
-        <v>16.5</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -826,7 +856,7 @@
         <v>8</v>
       </c>
       <c r="P3" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D3,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E3,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F3,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G3,$A$2:$A$65,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D3,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E3,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F3,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G3,$A$2:$A$70,0)),0))</f>
         <v>0</v>
       </c>
       <c r="Q3" s="0" t="n">
@@ -834,16 +864,16 @@
         <v>8</v>
       </c>
       <c r="R3" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A3)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A3)),IF(COUNTIF($E$2:$E$65,$A3)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A3)),IF(COUNTIF($F$2:$F$65,$A3)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A3)),IF(COUNTIF($G$2:$G$65,$A3)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A3)))</f>
-        <v>24.5</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A3)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A3)),IF(COUNTIF($E$2:$E$70,$A3)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A3)),IF(COUNTIF($F$2:$F$70,$A3)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A3)),IF(COUNTIF($G$2:$G$70,$A3)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A3)))</f>
+        <v>8.5</v>
       </c>
       <c r="S3" s="0" t="n">
         <f aca="false">R3-O3</f>
-        <v>16.5</v>
+        <v>0.5</v>
       </c>
       <c r="T3" s="0" t="n">
         <f aca="false">S3-P3</f>
-        <v>16.5</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -867,7 +897,7 @@
         <v>7</v>
       </c>
       <c r="P4" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D4,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E4,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F4,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G4,$A$2:$A$65,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D4,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E4,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F4,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G4,$A$2:$A$70,0)),0))</f>
         <v>8</v>
       </c>
       <c r="Q4" s="0" t="n">
@@ -875,16 +905,16 @@
         <v>15</v>
       </c>
       <c r="R4" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A4)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A4)),IF(COUNTIF($E$2:$E$65,$A4)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A4)),IF(COUNTIF($F$2:$F$65,$A4)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A4)),IF(COUNTIF($G$2:$G$65,$A4)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A4)))</f>
-        <v>31.5</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A4)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A4)),IF(COUNTIF($E$2:$E$70,$A4)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A4)),IF(COUNTIF($F$2:$F$70,$A4)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A4)),IF(COUNTIF($G$2:$G$70,$A4)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A4)))</f>
+        <v>15.5</v>
       </c>
       <c r="S4" s="0" t="n">
         <f aca="false">R4-O4</f>
-        <v>24.5</v>
+        <v>8.5</v>
       </c>
       <c r="T4" s="0" t="n">
         <f aca="false">S4-P4</f>
-        <v>16.5</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -908,7 +938,7 @@
         <v>3</v>
       </c>
       <c r="P5" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D5,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E5,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F5,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G5,$A$2:$A$65,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D5,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E5,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F5,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G5,$A$2:$A$70,0)),0))</f>
         <v>15</v>
       </c>
       <c r="Q5" s="0" t="n">
@@ -916,16 +946,16 @@
         <v>18</v>
       </c>
       <c r="R5" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A5)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A5)),IF(COUNTIF($E$2:$E$65,$A5)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A5)),IF(COUNTIF($F$2:$F$65,$A5)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A5)),IF(COUNTIF($G$2:$G$65,$A5)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A5)))</f>
-        <v>34.5</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A5)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A5)),IF(COUNTIF($E$2:$E$70,$A5)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A5)),IF(COUNTIF($F$2:$F$70,$A5)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A5)),IF(COUNTIF($G$2:$G$70,$A5)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A5)))</f>
+        <v>18.5</v>
       </c>
       <c r="S5" s="0" t="n">
         <f aca="false">R5-O5</f>
-        <v>31.5</v>
+        <v>15.5</v>
       </c>
       <c r="T5" s="0" t="n">
         <f aca="false">S5-P5</f>
-        <v>16.5</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -955,7 +985,7 @@
         <v>7.5</v>
       </c>
       <c r="P6" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D6,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E6,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F6,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G6,$A$2:$A$65,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D6,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E6,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F6,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G6,$A$2:$A$70,0)),0))</f>
         <v>18</v>
       </c>
       <c r="Q6" s="0" t="n">
@@ -963,16 +993,16 @@
         <v>25.5</v>
       </c>
       <c r="R6" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A6)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A6)),IF(COUNTIF($E$2:$E$65,$A6)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A6)),IF(COUNTIF($F$2:$F$65,$A6)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A6)),IF(COUNTIF($G$2:$G$65,$A6)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A6)))</f>
-        <v>42</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A6)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A6)),IF(COUNTIF($E$2:$E$70,$A6)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A6)),IF(COUNTIF($F$2:$F$70,$A6)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A6)),IF(COUNTIF($G$2:$G$70,$A6)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A6)))</f>
+        <v>26</v>
       </c>
       <c r="S6" s="0" t="n">
         <f aca="false">R6-O6</f>
-        <v>34.5</v>
+        <v>18.5</v>
       </c>
       <c r="T6" s="0" t="n">
         <f aca="false">S6-P6</f>
-        <v>16.5</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -999,7 +1029,7 @@
         <v>10</v>
       </c>
       <c r="P7" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D7,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E7,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F7,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G7,$A$2:$A$65,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D7,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E7,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F7,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G7,$A$2:$A$70,0)),0))</f>
         <v>25.5</v>
       </c>
       <c r="Q7" s="0" t="n">
@@ -1007,16 +1037,16 @@
         <v>35.5</v>
       </c>
       <c r="R7" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A7)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A7)),IF(COUNTIF($E$2:$E$65,$A7)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A7)),IF(COUNTIF($F$2:$F$65,$A7)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A7)),IF(COUNTIF($G$2:$G$65,$A7)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A7)))</f>
-        <v>52</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A7)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A7)),IF(COUNTIF($E$2:$E$70,$A7)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A7)),IF(COUNTIF($F$2:$F$70,$A7)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A7)),IF(COUNTIF($G$2:$G$70,$A7)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A7)))</f>
+        <v>36</v>
       </c>
       <c r="S7" s="0" t="n">
         <f aca="false">R7-O7</f>
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="T7" s="0" t="n">
         <f aca="false">S7-P7</f>
-        <v>16.5</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1040,7 +1070,7 @@
         <v>5</v>
       </c>
       <c r="P8" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D8,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E8,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F8,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G8,$A$2:$A$65,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D8,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E8,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F8,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G8,$A$2:$A$70,0)),0))</f>
         <v>25.5</v>
       </c>
       <c r="Q8" s="0" t="n">
@@ -1048,16 +1078,16 @@
         <v>30.5</v>
       </c>
       <c r="R8" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A8)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A8)),IF(COUNTIF($E$2:$E$65,$A8)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A8)),IF(COUNTIF($F$2:$F$65,$A8)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A8)),IF(COUNTIF($G$2:$G$65,$A8)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A8)))</f>
-        <v>52</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A8)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A8)),IF(COUNTIF($E$2:$E$70,$A8)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A8)),IF(COUNTIF($F$2:$F$70,$A8)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A8)),IF(COUNTIF($G$2:$G$70,$A8)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A8)))</f>
+        <v>36</v>
       </c>
       <c r="S8" s="0" t="n">
         <f aca="false">R8-O8</f>
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="T8" s="0" t="n">
         <f aca="false">S8-P8</f>
-        <v>21.5</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1084,7 +1114,7 @@
         <v>10</v>
       </c>
       <c r="P9" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D9,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E9,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F9,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G9,$A$2:$A$65,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D9,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E9,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F9,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G9,$A$2:$A$70,0)),0))</f>
         <v>35.5</v>
       </c>
       <c r="Q9" s="0" t="n">
@@ -1092,16 +1122,16 @@
         <v>45.5</v>
       </c>
       <c r="R9" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A9)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A9)),IF(COUNTIF($E$2:$E$65,$A9)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A9)),IF(COUNTIF($F$2:$F$65,$A9)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A9)),IF(COUNTIF($G$2:$G$65,$A9)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A9)))</f>
-        <v>62</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A9)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A9)),IF(COUNTIF($E$2:$E$70,$A9)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A9)),IF(COUNTIF($F$2:$F$70,$A9)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A9)),IF(COUNTIF($G$2:$G$70,$A9)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A9)))</f>
+        <v>46</v>
       </c>
       <c r="S9" s="0" t="n">
         <f aca="false">R9-O9</f>
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="T9" s="0" t="n">
         <f aca="false">S9-P9</f>
-        <v>16.5</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1125,7 +1155,7 @@
         <v>1</v>
       </c>
       <c r="P10" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D10,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E10,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F10,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G10,$A$2:$A$65,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D10,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E10,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F10,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G10,$A$2:$A$70,0)),0))</f>
         <v>45.5</v>
       </c>
       <c r="Q10" s="0" t="n">
@@ -1133,16 +1163,16 @@
         <v>46.5</v>
       </c>
       <c r="R10" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A10)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A10)),IF(COUNTIF($E$2:$E$65,$A10)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A10)),IF(COUNTIF($F$2:$F$65,$A10)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A10)),IF(COUNTIF($G$2:$G$65,$A10)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A10)))</f>
-        <v>63</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A10)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A10)),IF(COUNTIF($E$2:$E$70,$A10)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A10)),IF(COUNTIF($F$2:$F$70,$A10)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A10)),IF(COUNTIF($G$2:$G$70,$A10)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A10)))</f>
+        <v>47</v>
       </c>
       <c r="S10" s="0" t="n">
         <f aca="false">R10-O10</f>
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="T10" s="0" t="n">
         <f aca="false">S10-P10</f>
-        <v>16.5</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1163,7 +1193,7 @@
         <v>0</v>
       </c>
       <c r="P11" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D11,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E11,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F11,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G11,$A$2:$A$65,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D11,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E11,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F11,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G11,$A$2:$A$70,0)),0))</f>
         <v>0</v>
       </c>
       <c r="Q11" s="0" t="n">
@@ -1171,16 +1201,16 @@
         <v>0</v>
       </c>
       <c r="R11" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A11)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A11)),IF(COUNTIF($E$2:$E$65,$A11)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A11)),IF(COUNTIF($F$2:$F$65,$A11)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A11)),IF(COUNTIF($G$2:$G$65,$A11)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A11)))</f>
-        <v>2</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A11)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A11)),IF(COUNTIF($E$2:$E$70,$A11)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A11)),IF(COUNTIF($F$2:$F$70,$A11)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A11)),IF(COUNTIF($G$2:$G$70,$A11)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A11)))</f>
+        <v>0</v>
       </c>
       <c r="S11" s="0" t="n">
         <f aca="false">R11-O11</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T11" s="0" t="n">
         <f aca="false">S11-P11</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1197,34 +1227,34 @@
         <v>42</v>
       </c>
       <c r="I12" s="0" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="J12" s="0" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="O12" s="0" t="n">
         <f aca="false">IF(H12&lt;&gt;"",H12,IF(AND(I12&lt;&gt;"",J12&lt;&gt;""),(I12+J12)/2,0))</f>
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="P12" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D12,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E12,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F12,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G12,$A$2:$A$65,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D12,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E12,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F12,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G12,$A$2:$A$70,0)),0))</f>
         <v>0</v>
       </c>
       <c r="Q12" s="0" t="n">
         <f aca="false">P12+O12</f>
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="R12" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A12)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A12)),IF(COUNTIF($E$2:$E$65,$A12)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A12)),IF(COUNTIF($F$2:$F$65,$A12)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A12)),IF(COUNTIF($G$2:$G$65,$A12)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A12)))</f>
-        <v>19</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A12)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A12)),IF(COUNTIF($E$2:$E$70,$A12)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A12)),IF(COUNTIF($F$2:$F$70,$A12)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A12)),IF(COUNTIF($G$2:$G$70,$A12)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A12)))</f>
+        <v>3</v>
       </c>
       <c r="S12" s="0" t="n">
         <f aca="false">R12-O12</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T12" s="0" t="n">
         <f aca="false">S12-P12</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1248,24 +1278,24 @@
         <v>10</v>
       </c>
       <c r="P13" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D13,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E13,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F13,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G13,$A$2:$A$65,0)),0))</f>
-        <v>17</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D13,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E13,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F13,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G13,$A$2:$A$70,0)),0))</f>
+        <v>3</v>
       </c>
       <c r="Q13" s="0" t="n">
         <f aca="false">P13+O13</f>
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="R13" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A13)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A13)),IF(COUNTIF($E$2:$E$65,$A13)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A13)),IF(COUNTIF($F$2:$F$65,$A13)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A13)),IF(COUNTIF($G$2:$G$65,$A13)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A13)))</f>
-        <v>39</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A13)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A13)),IF(COUNTIF($E$2:$E$70,$A13)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A13)),IF(COUNTIF($F$2:$F$70,$A13)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A13)),IF(COUNTIF($G$2:$G$70,$A13)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A13)))</f>
+        <v>23</v>
       </c>
       <c r="S13" s="0" t="n">
         <f aca="false">R13-O13</f>
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="T13" s="0" t="n">
         <f aca="false">S13-P13</f>
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1289,24 +1319,24 @@
         <v>5</v>
       </c>
       <c r="P14" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D14,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E14,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F14,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G14,$A$2:$A$65,0)),0))</f>
-        <v>17</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D14,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E14,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F14,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G14,$A$2:$A$70,0)),0))</f>
+        <v>3</v>
       </c>
       <c r="Q14" s="0" t="n">
         <f aca="false">P14+O14</f>
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="R14" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A14)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A14)),IF(COUNTIF($E$2:$E$65,$A14)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A14)),IF(COUNTIF($F$2:$F$65,$A14)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A14)),IF(COUNTIF($G$2:$G$65,$A14)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A14)))</f>
-        <v>39</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A14)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A14)),IF(COUNTIF($E$2:$E$70,$A14)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A14)),IF(COUNTIF($F$2:$F$70,$A14)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A14)),IF(COUNTIF($G$2:$G$70,$A14)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A14)))</f>
+        <v>23</v>
       </c>
       <c r="S14" s="0" t="n">
         <f aca="false">R14-O14</f>
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="T14" s="0" t="n">
         <f aca="false">S14-P14</f>
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1336,24 +1366,24 @@
         <v>18</v>
       </c>
       <c r="P15" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D15,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E15,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F15,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G15,$A$2:$A$65,0)),0))</f>
-        <v>17</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D15,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E15,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F15,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G15,$A$2:$A$70,0)),0))</f>
+        <v>3</v>
       </c>
       <c r="Q15" s="0" t="n">
         <f aca="false">P15+O15</f>
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="R15" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A15)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A15)),IF(COUNTIF($E$2:$E$65,$A15)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A15)),IF(COUNTIF($F$2:$F$65,$A15)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A15)),IF(COUNTIF($G$2:$G$65,$A15)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A15)))</f>
-        <v>37</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A15)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A15)),IF(COUNTIF($E$2:$E$70,$A15)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A15)),IF(COUNTIF($F$2:$F$70,$A15)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A15)),IF(COUNTIF($G$2:$G$70,$A15)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A15)))</f>
+        <v>21</v>
       </c>
       <c r="S15" s="0" t="n">
         <f aca="false">R15-O15</f>
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="T15" s="0" t="n">
         <f aca="false">S15-P15</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1377,24 +1407,24 @@
         <v>5</v>
       </c>
       <c r="P16" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D16,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E16,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F16,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G16,$A$2:$A$65,0)),0))</f>
-        <v>35</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D16,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E16,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F16,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G16,$A$2:$A$70,0)),0))</f>
+        <v>21</v>
       </c>
       <c r="Q16" s="0" t="n">
         <f aca="false">P16+O16</f>
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="R16" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A16)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A16)),IF(COUNTIF($E$2:$E$65,$A16)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A16)),IF(COUNTIF($F$2:$F$65,$A16)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A16)),IF(COUNTIF($G$2:$G$65,$A16)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A16)))</f>
-        <v>42</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A16)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A16)),IF(COUNTIF($E$2:$E$70,$A16)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A16)),IF(COUNTIF($F$2:$F$70,$A16)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A16)),IF(COUNTIF($G$2:$G$70,$A16)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A16)))</f>
+        <v>26</v>
       </c>
       <c r="S16" s="0" t="n">
         <f aca="false">R16-O16</f>
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="T16" s="0" t="n">
         <f aca="false">S16-P16</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1418,24 +1448,24 @@
         <v>10</v>
       </c>
       <c r="P17" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D17,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E17,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F17,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G17,$A$2:$A$65,0)),0))</f>
-        <v>40</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D17,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E17,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F17,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G17,$A$2:$A$70,0)),0))</f>
+        <v>26</v>
       </c>
       <c r="Q17" s="0" t="n">
         <f aca="false">P17+O17</f>
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="R17" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A17)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A17)),IF(COUNTIF($E$2:$E$65,$A17)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A17)),IF(COUNTIF($F$2:$F$65,$A17)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A17)),IF(COUNTIF($G$2:$G$65,$A17)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A17)))</f>
-        <v>52</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A17)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A17)),IF(COUNTIF($E$2:$E$70,$A17)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A17)),IF(COUNTIF($F$2:$F$70,$A17)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A17)),IF(COUNTIF($G$2:$G$70,$A17)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A17)))</f>
+        <v>36</v>
       </c>
       <c r="S17" s="0" t="n">
         <f aca="false">R17-O17</f>
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="T17" s="0" t="n">
         <f aca="false">S17-P17</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1462,24 +1492,24 @@
         <v>3</v>
       </c>
       <c r="P18" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D18,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E18,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F18,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G18,$A$2:$A$65,0)),0))</f>
-        <v>27</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D18,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E18,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F18,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G18,$A$2:$A$70,0)),0))</f>
+        <v>13</v>
       </c>
       <c r="Q18" s="0" t="n">
         <f aca="false">P18+O18</f>
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="R18" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A18)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A18)),IF(COUNTIF($E$2:$E$65,$A18)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A18)),IF(COUNTIF($F$2:$F$65,$A18)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A18)),IF(COUNTIF($G$2:$G$65,$A18)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A18)))</f>
-        <v>42</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A18)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A18)),IF(COUNTIF($E$2:$E$70,$A18)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A18)),IF(COUNTIF($F$2:$F$70,$A18)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A18)),IF(COUNTIF($G$2:$G$70,$A18)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A18)))</f>
+        <v>26</v>
       </c>
       <c r="S18" s="0" t="n">
         <f aca="false">R18-O18</f>
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="T18" s="0" t="n">
         <f aca="false">S18-P18</f>
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1503,24 +1533,24 @@
         <v>10</v>
       </c>
       <c r="P19" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D19,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E19,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F19,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G19,$A$2:$A$65,0)),0))</f>
-        <v>30</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D19,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E19,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F19,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G19,$A$2:$A$70,0)),0))</f>
+        <v>16</v>
       </c>
       <c r="Q19" s="0" t="n">
         <f aca="false">P19+O19</f>
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="R19" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A19)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A19)),IF(COUNTIF($E$2:$E$65,$A19)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A19)),IF(COUNTIF($F$2:$F$65,$A19)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A19)),IF(COUNTIF($G$2:$G$65,$A19)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A19)))</f>
-        <v>52</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A19)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A19)),IF(COUNTIF($E$2:$E$70,$A19)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A19)),IF(COUNTIF($F$2:$F$70,$A19)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A19)),IF(COUNTIF($G$2:$G$70,$A19)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A19)))</f>
+        <v>36</v>
       </c>
       <c r="S19" s="0" t="n">
         <f aca="false">R19-O19</f>
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="T19" s="0" t="n">
         <f aca="false">S19-P19</f>
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1544,24 +1574,24 @@
         <v>1</v>
       </c>
       <c r="P20" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D20,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E20,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F20,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G20,$A$2:$A$65,0)),0))</f>
-        <v>60</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D20,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E20,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F20,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G20,$A$2:$A$70,0)),0))</f>
+        <v>46</v>
       </c>
       <c r="Q20" s="0" t="n">
         <f aca="false">P20+O20</f>
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="R20" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A20)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A20)),IF(COUNTIF($E$2:$E$65,$A20)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A20)),IF(COUNTIF($F$2:$F$65,$A20)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A20)),IF(COUNTIF($G$2:$G$65,$A20)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A20)))</f>
-        <v>63</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A20)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A20)),IF(COUNTIF($E$2:$E$70,$A20)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A20)),IF(COUNTIF($F$2:$F$70,$A20)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A20)),IF(COUNTIF($G$2:$G$70,$A20)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A20)))</f>
+        <v>47</v>
       </c>
       <c r="S20" s="0" t="n">
         <f aca="false">R20-O20</f>
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="T20" s="0" t="n">
         <f aca="false">S20-P20</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1591,24 +1621,24 @@
         <v>6.5</v>
       </c>
       <c r="P21" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D21,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E21,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F21,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G21,$A$2:$A$65,0)),0))</f>
-        <v>50</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D21,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E21,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F21,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G21,$A$2:$A$70,0)),0))</f>
+        <v>36</v>
       </c>
       <c r="Q21" s="0" t="n">
         <f aca="false">P21+O21</f>
-        <v>56.5</v>
+        <v>42.5</v>
       </c>
       <c r="R21" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A21)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A21)),IF(COUNTIF($E$2:$E$65,$A21)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A21)),IF(COUNTIF($F$2:$F$65,$A21)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A21)),IF(COUNTIF($G$2:$G$65,$A21)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A21)))</f>
-        <v>62</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A21)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A21)),IF(COUNTIF($E$2:$E$70,$A21)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A21)),IF(COUNTIF($F$2:$F$70,$A21)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A21)),IF(COUNTIF($G$2:$G$70,$A21)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A21)))</f>
+        <v>46</v>
       </c>
       <c r="S21" s="0" t="n">
         <f aca="false">R21-O21</f>
-        <v>55.5</v>
+        <v>39.5</v>
       </c>
       <c r="T21" s="0" t="n">
         <f aca="false">S21-P21</f>
-        <v>5.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1635,24 +1665,24 @@
         <v>10</v>
       </c>
       <c r="P22" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D22,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E22,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F22,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G22,$A$2:$A$65,0)),0))</f>
-        <v>50</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D22,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E22,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F22,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G22,$A$2:$A$70,0)),0))</f>
+        <v>36</v>
       </c>
       <c r="Q22" s="0" t="n">
         <f aca="false">P22+O22</f>
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="R22" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A22)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A22)),IF(COUNTIF($E$2:$E$65,$A22)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A22)),IF(COUNTIF($F$2:$F$65,$A22)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A22)),IF(COUNTIF($G$2:$G$65,$A22)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A22)))</f>
-        <v>62</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A22)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A22)),IF(COUNTIF($E$2:$E$70,$A22)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A22)),IF(COUNTIF($F$2:$F$70,$A22)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A22)),IF(COUNTIF($G$2:$G$70,$A22)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A22)))</f>
+        <v>46</v>
       </c>
       <c r="S22" s="0" t="n">
         <f aca="false">R22-O22</f>
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="T22" s="0" t="n">
         <f aca="false">S22-P22</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1673,7 +1703,7 @@
         <v>0</v>
       </c>
       <c r="P23" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D23,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E23,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F23,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G23,$A$2:$A$65,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D23,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E23,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F23,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G23,$A$2:$A$70,0)),0))</f>
         <v>0</v>
       </c>
       <c r="Q23" s="0" t="n">
@@ -1681,16 +1711,16 @@
         <v>0</v>
       </c>
       <c r="R23" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A23)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A23)),IF(COUNTIF($E$2:$E$65,$A23)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A23)),IF(COUNTIF($F$2:$F$65,$A23)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A23)),IF(COUNTIF($G$2:$G$65,$A23)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A23)))</f>
-        <v>0</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A23)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A23)),IF(COUNTIF($E$2:$E$70,$A23)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A23)),IF(COUNTIF($F$2:$F$70,$A23)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A23)),IF(COUNTIF($G$2:$G$70,$A23)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A23)))</f>
+        <v>8.5</v>
       </c>
       <c r="S23" s="0" t="n">
         <f aca="false">R23-O23</f>
-        <v>0</v>
+        <v>8.5</v>
       </c>
       <c r="T23" s="0" t="n">
         <f aca="false">S23-P23</f>
-        <v>0</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1714,7 +1744,7 @@
         <v>16</v>
       </c>
       <c r="P24" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D24,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E24,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F24,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G24,$A$2:$A$65,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D24,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E24,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F24,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G24,$A$2:$A$70,0)),0))</f>
         <v>0</v>
       </c>
       <c r="Q24" s="0" t="n">
@@ -1722,16 +1752,16 @@
         <v>16</v>
       </c>
       <c r="R24" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A24)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A24)),IF(COUNTIF($E$2:$E$65,$A24)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A24)),IF(COUNTIF($F$2:$F$65,$A24)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A24)),IF(COUNTIF($G$2:$G$65,$A24)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A24)))</f>
-        <v>42</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A24)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A24)),IF(COUNTIF($E$2:$E$70,$A24)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A24)),IF(COUNTIF($F$2:$F$70,$A24)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A24)),IF(COUNTIF($G$2:$G$70,$A24)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A24)))</f>
+        <v>36</v>
       </c>
       <c r="S24" s="0" t="n">
         <f aca="false">R24-O24</f>
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="T24" s="0" t="n">
         <f aca="false">S24-P24</f>
-        <v>26</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1748,31 +1778,31 @@
         <v>67</v>
       </c>
       <c r="H25" s="0" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O25" s="0" t="n">
         <f aca="false">IF(H25&lt;&gt;"",H25,IF(AND(I25&lt;&gt;"",J25&lt;&gt;""),(I25+J25)/2,0))</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P25" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D25,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E25,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F25,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G25,$A$2:$A$65,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D25,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E25,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F25,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G25,$A$2:$A$70,0)),0))</f>
         <v>0</v>
       </c>
       <c r="Q25" s="0" t="n">
         <f aca="false">P25+O25</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R25" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A25)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A25)),IF(COUNTIF($E$2:$E$65,$A25)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A25)),IF(COUNTIF($F$2:$F$65,$A25)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A25)),IF(COUNTIF($G$2:$G$65,$A25)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A25)))</f>
-        <v>2</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A25)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A25)),IF(COUNTIF($E$2:$E$70,$A25)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A25)),IF(COUNTIF($F$2:$F$70,$A25)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A25)),IF(COUNTIF($G$2:$G$70,$A25)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A25)))</f>
+        <v>12</v>
       </c>
       <c r="S25" s="0" t="n">
         <f aca="false">R25-O25</f>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="T25" s="0" t="n">
         <f aca="false">S25-P25</f>
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1786,34 +1816,34 @@
         <v>74</v>
       </c>
       <c r="D26" s="0" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="H26" s="0" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O26" s="0" t="n">
         <f aca="false">IF(H26&lt;&gt;"",H26,IF(AND(I26&lt;&gt;"",J26&lt;&gt;""),(I26+J26)/2,0))</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="P26" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D26,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E26,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F26,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G26,$A$2:$A$65,0)),0))</f>
-        <v>2</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D26,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E26,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F26,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G26,$A$2:$A$70,0)),0))</f>
+        <v>0</v>
       </c>
       <c r="Q26" s="0" t="n">
         <f aca="false">P26+O26</f>
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="R26" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A26)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A26)),IF(COUNTIF($E$2:$E$65,$A26)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A26)),IF(COUNTIF($F$2:$F$65,$A26)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A26)),IF(COUNTIF($G$2:$G$65,$A26)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A26)))</f>
-        <v>57</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A26)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A26)),IF(COUNTIF($E$2:$E$70,$A26)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A26)),IF(COUNTIF($F$2:$F$70,$A26)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A26)),IF(COUNTIF($G$2:$G$70,$A26)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A26)))</f>
+        <v>9.5</v>
       </c>
       <c r="S26" s="0" t="n">
         <f aca="false">R26-O26</f>
-        <v>52</v>
+        <v>8.5</v>
       </c>
       <c r="T26" s="0" t="n">
         <f aca="false">S26-P26</f>
-        <v>50</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1830,31 +1860,31 @@
         <v>71</v>
       </c>
       <c r="H27" s="0" t="n">
-        <v>15</v>
+        <v>2.5</v>
       </c>
       <c r="O27" s="0" t="n">
         <f aca="false">IF(H27&lt;&gt;"",H27,IF(AND(I27&lt;&gt;"",J27&lt;&gt;""),(I27+J27)/2,0))</f>
-        <v>15</v>
+        <v>2.5</v>
       </c>
       <c r="P27" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D27,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E27,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F27,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G27,$A$2:$A$65,0)),0))</f>
-        <v>2</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D27,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E27,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F27,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G27,$A$2:$A$70,0)),0))</f>
+        <v>1</v>
       </c>
       <c r="Q27" s="0" t="n">
         <f aca="false">P27+O27</f>
-        <v>17</v>
+        <v>3.5</v>
       </c>
       <c r="R27" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A27)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A27)),IF(COUNTIF($E$2:$E$65,$A27)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A27)),IF(COUNTIF($F$2:$F$65,$A27)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A27)),IF(COUNTIF($G$2:$G$65,$A27)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A27)))</f>
-        <v>17</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A27)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A27)),IF(COUNTIF($E$2:$E$70,$A27)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A27)),IF(COUNTIF($F$2:$F$70,$A27)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A27)),IF(COUNTIF($G$2:$G$70,$A27)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A27)))</f>
+        <v>41</v>
       </c>
       <c r="S27" s="0" t="n">
         <f aca="false">R27-O27</f>
-        <v>2</v>
+        <v>38.5</v>
       </c>
       <c r="T27" s="0" t="n">
         <f aca="false">S27-P27</f>
-        <v>0</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1871,31 +1901,31 @@
         <v>73</v>
       </c>
       <c r="H28" s="0" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="O28" s="0" t="n">
         <f aca="false">IF(H28&lt;&gt;"",H28,IF(AND(I28&lt;&gt;"",J28&lt;&gt;""),(I28+J28)/2,0))</f>
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="P28" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D28,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E28,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F28,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G28,$A$2:$A$65,0)),0))</f>
-        <v>7</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D28,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E28,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F28,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G28,$A$2:$A$70,0)),0))</f>
+        <v>1</v>
       </c>
       <c r="Q28" s="0" t="n">
         <f aca="false">P28+O28</f>
-        <v>12</v>
+        <v>3.5</v>
       </c>
       <c r="R28" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A28)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A28)),IF(COUNTIF($E$2:$E$65,$A28)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A28)),IF(COUNTIF($F$2:$F$65,$A28)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A28)),IF(COUNTIF($G$2:$G$65,$A28)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A28)))</f>
-        <v>62</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A28)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A28)),IF(COUNTIF($E$2:$E$70,$A28)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A28)),IF(COUNTIF($F$2:$F$70,$A28)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A28)),IF(COUNTIF($G$2:$G$70,$A28)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A28)))</f>
+        <v>41</v>
       </c>
       <c r="S28" s="0" t="n">
         <f aca="false">R28-O28</f>
-        <v>57</v>
+        <v>38.5</v>
       </c>
       <c r="T28" s="0" t="n">
         <f aca="false">S28-P28</f>
-        <v>50</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1909,34 +1939,34 @@
         <v>80</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="H29" s="0" t="n">
-        <v>25</v>
+        <v>7.5</v>
       </c>
       <c r="O29" s="0" t="n">
         <f aca="false">IF(H29&lt;&gt;"",H29,IF(AND(I29&lt;&gt;"",J29&lt;&gt;""),(I29+J29)/2,0))</f>
-        <v>25</v>
+        <v>7.5</v>
       </c>
       <c r="P29" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D29,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E29,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F29,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G29,$A$2:$A$65,0)),0))</f>
-        <v>17</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D29,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E29,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F29,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G29,$A$2:$A$70,0)),0))</f>
+        <v>1</v>
       </c>
       <c r="Q29" s="0" t="n">
         <f aca="false">P29+O29</f>
-        <v>42</v>
+        <v>8.5</v>
       </c>
       <c r="R29" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A29)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A29)),IF(COUNTIF($E$2:$E$65,$A29)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A29)),IF(COUNTIF($F$2:$F$65,$A29)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A29)),IF(COUNTIF($G$2:$G$65,$A29)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A29)))</f>
-        <v>42</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A29)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A29)),IF(COUNTIF($E$2:$E$70,$A29)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A29)),IF(COUNTIF($F$2:$F$70,$A29)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A29)),IF(COUNTIF($G$2:$G$70,$A29)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A29)))</f>
+        <v>19.5</v>
       </c>
       <c r="S29" s="0" t="n">
         <f aca="false">R29-O29</f>
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="T29" s="0" t="n">
         <f aca="false">S29-P29</f>
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1947,43 +1977,37 @@
         <v>68</v>
       </c>
       <c r="C30" s="0" t="s">
-        <v>60</v>
+        <v>82</v>
       </c>
       <c r="D30" s="0" t="s">
-        <v>82</v>
-      </c>
-      <c r="E30" s="0" t="s">
-        <v>83</v>
-      </c>
-      <c r="F30" s="0" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H30" s="0" t="n">
-        <v>20</v>
+        <v>7.5</v>
       </c>
       <c r="O30" s="0" t="n">
         <f aca="false">IF(H30&lt;&gt;"",H30,IF(AND(I30&lt;&gt;"",J30&lt;&gt;""),(I30+J30)/2,0))</f>
-        <v>20</v>
+        <v>7.5</v>
       </c>
       <c r="P30" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D30,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E30,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F30,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G30,$A$2:$A$65,0)),0))</f>
-        <v>17</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D30,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E30,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F30,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G30,$A$2:$A$70,0)),0))</f>
+        <v>1</v>
       </c>
       <c r="Q30" s="0" t="n">
         <f aca="false">P30+O30</f>
-        <v>37</v>
+        <v>8.5</v>
       </c>
       <c r="R30" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A30)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A30)),IF(COUNTIF($E$2:$E$65,$A30)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A30)),IF(COUNTIF($F$2:$F$65,$A30)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A30)),IF(COUNTIF($G$2:$G$65,$A30)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A30)))</f>
-        <v>55.5</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A30)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A30)),IF(COUNTIF($E$2:$E$70,$A30)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A30)),IF(COUNTIF($F$2:$F$70,$A30)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A30)),IF(COUNTIF($G$2:$G$70,$A30)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A30)))</f>
+        <v>19.5</v>
       </c>
       <c r="S30" s="0" t="n">
         <f aca="false">R30-O30</f>
-        <v>35.5</v>
+        <v>12</v>
       </c>
       <c r="T30" s="0" t="n">
         <f aca="false">S30-P30</f>
-        <v>18.5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1997,7 +2021,10 @@
         <v>84</v>
       </c>
       <c r="D31" s="0" t="s">
-        <v>82</v>
+        <v>75</v>
+      </c>
+      <c r="E31" s="0" t="s">
+        <v>77</v>
       </c>
       <c r="H31" s="0" t="n">
         <v>5</v>
@@ -2007,24 +2034,24 @@
         <v>5</v>
       </c>
       <c r="P31" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D31,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E31,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F31,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G31,$A$2:$A$65,0)),0))</f>
-        <v>7</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(E31,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E31,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F31,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G31,$A$2:$A$70,0)),0))</f>
+        <v>3.5</v>
       </c>
       <c r="Q31" s="0" t="n">
         <f aca="false">P31+O31</f>
-        <v>12</v>
+        <v>8.5</v>
       </c>
       <c r="R31" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A31)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A31)),IF(COUNTIF($E$2:$E$65,$A31)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A31)),IF(COUNTIF($F$2:$F$65,$A31)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A31)),IF(COUNTIF($G$2:$G$65,$A31)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A31)))</f>
-        <v>35.5</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A31)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A31)),IF(COUNTIF($E$2:$E$70,$A31)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A31)),IF(COUNTIF($F$2:$F$70,$A31)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A31)),IF(COUNTIF($G$2:$G$70,$A31)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A31)))</f>
+        <v>46</v>
       </c>
       <c r="S31" s="0" t="n">
         <f aca="false">R31-O31</f>
-        <v>30.5</v>
+        <v>41</v>
       </c>
       <c r="T31" s="0" t="n">
         <f aca="false">S31-P31</f>
-        <v>23.5</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2038,673 +2065,673 @@
         <v>86</v>
       </c>
       <c r="D32" s="0" t="s">
-        <v>70</v>
-      </c>
-      <c r="E32" s="0" t="s">
         <v>79</v>
       </c>
       <c r="H32" s="0" t="n">
-        <v>20</v>
+        <v>12.5</v>
       </c>
       <c r="O32" s="0" t="n">
         <f aca="false">IF(H32&lt;&gt;"",H32,IF(AND(I32&lt;&gt;"",J32&lt;&gt;""),(I32+J32)/2,0))</f>
-        <v>20</v>
+        <v>12.5</v>
       </c>
       <c r="P32" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D32,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E32,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F32,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G32,$A$2:$A$65,0)),0))</f>
-        <v>42</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D32,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E32,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F32,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G32,$A$2:$A$70,0)),0))</f>
+        <v>8.5</v>
       </c>
       <c r="Q32" s="0" t="n">
         <f aca="false">P32+O32</f>
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="R32" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A32)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A32)),IF(COUNTIF($E$2:$E$65,$A32)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A32)),IF(COUNTIF($F$2:$F$65,$A32)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A32)),IF(COUNTIF($G$2:$G$65,$A32)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A32)))</f>
-        <v>62</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A32)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A32)),IF(COUNTIF($E$2:$E$70,$A32)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A32)),IF(COUNTIF($F$2:$F$70,$A32)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A32)),IF(COUNTIF($G$2:$G$70,$A32)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A32)))</f>
+        <v>54.25</v>
       </c>
       <c r="S32" s="0" t="n">
         <f aca="false">R32-O32</f>
-        <v>42</v>
+        <v>41.75</v>
       </c>
       <c r="T32" s="0" t="n">
         <f aca="false">S32-P32</f>
-        <v>0</v>
+        <v>33.25</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B33" s="0" t="s">
         <v>68</v>
       </c>
       <c r="C33" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D33" s="0" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="H33" s="0" t="n">
-        <v>5</v>
+        <v>12.5</v>
       </c>
       <c r="O33" s="0" t="n">
         <f aca="false">IF(H33&lt;&gt;"",H33,IF(AND(I33&lt;&gt;"",J33&lt;&gt;""),(I33+J33)/2,0))</f>
-        <v>5</v>
+        <v>12.5</v>
       </c>
       <c r="P33" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D33,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E33,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F33,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G33,$A$2:$A$65,0)),0))</f>
-        <v>2</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D33,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E33,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F33,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G33,$A$2:$A$70,0)),0))</f>
+        <v>8.5</v>
       </c>
       <c r="Q33" s="0" t="n">
         <f aca="false">P33+O33</f>
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="R33" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A33)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A33)),IF(COUNTIF($E$2:$E$65,$A33)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A33)),IF(COUNTIF($F$2:$F$65,$A33)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A33)),IF(COUNTIF($G$2:$G$65,$A33)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A33)))</f>
-        <v>30.5</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A33)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A33)),IF(COUNTIF($E$2:$E$70,$A33)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A33)),IF(COUNTIF($F$2:$F$70,$A33)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A33)),IF(COUNTIF($G$2:$G$70,$A33)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A33)))</f>
+        <v>36</v>
       </c>
       <c r="S33" s="0" t="n">
         <f aca="false">R33-O33</f>
-        <v>25.5</v>
+        <v>23.5</v>
       </c>
       <c r="T33" s="0" t="n">
         <f aca="false">S33-P33</f>
-        <v>23.5</v>
+        <v>15</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B34" s="0" t="s">
         <v>68</v>
       </c>
       <c r="C34" s="0" t="s">
-        <v>89</v>
+        <v>60</v>
       </c>
       <c r="D34" s="0" t="s">
-        <v>82</v>
+        <v>90</v>
+      </c>
+      <c r="E34" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="F34" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="G34" s="0" t="s">
+        <v>81</v>
       </c>
       <c r="H34" s="0" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="O34" s="0" t="n">
         <f aca="false">IF(H34&lt;&gt;"",H34,IF(AND(I34&lt;&gt;"",J34&lt;&gt;""),(I34+J34)/2,0))</f>
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="P34" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D34,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E34,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F34,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G34,$A$2:$A$65,0)),0))</f>
-        <v>7</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D34,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E34,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F34,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G34,$A$2:$A$70,0)),0))</f>
+        <v>11</v>
       </c>
       <c r="Q34" s="0" t="n">
         <f aca="false">P34+O34</f>
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="R34" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A34)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A34)),IF(COUNTIF($E$2:$E$65,$A34)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A34)),IF(COUNTIF($F$2:$F$65,$A34)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A34)),IF(COUNTIF($G$2:$G$65,$A34)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A34)))</f>
-        <v>62</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A34)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A34)),IF(COUNTIF($E$2:$E$70,$A34)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A34)),IF(COUNTIF($F$2:$F$70,$A34)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A34)),IF(COUNTIF($G$2:$G$70,$A34)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A34)))</f>
+        <v>39.5</v>
       </c>
       <c r="S34" s="0" t="n">
         <f aca="false">R34-O34</f>
-        <v>57</v>
+        <v>19.5</v>
       </c>
       <c r="T34" s="0" t="n">
         <f aca="false">S34-P34</f>
-        <v>50</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B35" s="0" t="s">
         <v>68</v>
       </c>
       <c r="C35" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D35" s="0" t="s">
-        <v>81</v>
-      </c>
-      <c r="E35" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="I35" s="0" t="n">
+        <v>90</v>
+      </c>
+      <c r="H35" s="0" t="n">
         <v>5</v>
-      </c>
-      <c r="J35" s="0" t="n">
-        <v>8</v>
       </c>
       <c r="O35" s="0" t="n">
         <f aca="false">IF(H35&lt;&gt;"",H35,IF(AND(I35&lt;&gt;"",J35&lt;&gt;""),(I35+J35)/2,0))</f>
-        <v>6.5</v>
+        <v>5</v>
       </c>
       <c r="P35" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D35,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E35,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F35,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G35,$A$2:$A$65,0)),0))</f>
-        <v>42</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D35,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E35,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F35,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G35,$A$2:$A$70,0)),0))</f>
+        <v>6</v>
       </c>
       <c r="Q35" s="0" t="n">
         <f aca="false">P35+O35</f>
-        <v>48.5</v>
+        <v>11</v>
       </c>
       <c r="R35" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A35)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A35)),IF(COUNTIF($E$2:$E$65,$A35)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A35)),IF(COUNTIF($F$2:$F$65,$A35)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A35)),IF(COUNTIF($G$2:$G$65,$A35)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A35)))</f>
-        <v>62</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A35)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A35)),IF(COUNTIF($E$2:$E$70,$A35)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A35)),IF(COUNTIF($F$2:$F$70,$A35)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A35)),IF(COUNTIF($G$2:$G$70,$A35)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A35)))</f>
+        <v>19.5</v>
       </c>
       <c r="S35" s="0" t="n">
         <f aca="false">R35-O35</f>
-        <v>55.5</v>
+        <v>14.5</v>
       </c>
       <c r="T35" s="0" t="n">
         <f aca="false">S35-P35</f>
-        <v>13.5</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B36" s="0" t="s">
         <v>68</v>
       </c>
       <c r="C36" s="0" t="s">
-        <v>40</v>
+        <v>94</v>
       </c>
       <c r="D36" s="0" t="s">
-        <v>93</v>
+        <v>70</v>
+      </c>
+      <c r="E36" s="0" t="s">
+        <v>85</v>
       </c>
       <c r="H36" s="0" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="O36" s="0" t="n">
         <f aca="false">IF(H36&lt;&gt;"",H36,IF(AND(I36&lt;&gt;"",J36&lt;&gt;""),(I36+J36)/2,0))</f>
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="P36" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D36,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E36,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F36,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G36,$A$2:$A$65,0)),0))</f>
-        <v>62</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D36,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E36,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F36,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G36,$A$2:$A$70,0)),0))</f>
+        <v>21</v>
       </c>
       <c r="Q36" s="0" t="n">
         <f aca="false">P36+O36</f>
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="R36" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A36)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A36)),IF(COUNTIF($E$2:$E$65,$A36)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A36)),IF(COUNTIF($F$2:$F$65,$A36)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A36)),IF(COUNTIF($G$2:$G$65,$A36)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A36)))</f>
-        <v>63</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A36)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A36)),IF(COUNTIF($E$2:$E$70,$A36)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A36)),IF(COUNTIF($F$2:$F$70,$A36)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A36)),IF(COUNTIF($G$2:$G$70,$A36)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A36)))</f>
+        <v>64.25</v>
       </c>
       <c r="S36" s="0" t="n">
         <f aca="false">R36-O36</f>
-        <v>62</v>
+        <v>54.25</v>
       </c>
       <c r="T36" s="0" t="n">
         <f aca="false">S36-P36</f>
-        <v>0</v>
+        <v>33.25</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>95</v>
+        <v>68</v>
       </c>
       <c r="C37" s="0" t="s">
         <v>96</v>
       </c>
       <c r="D37" s="0" t="s">
-        <v>23</v>
+        <v>70</v>
+      </c>
+      <c r="E37" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="H37" s="0" t="n">
+        <v>10</v>
       </c>
       <c r="O37" s="0" t="n">
         <f aca="false">IF(H37&lt;&gt;"",H37,IF(AND(I37&lt;&gt;"",J37&lt;&gt;""),(I37+J37)/2,0))</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P37" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D37,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E37,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F37,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G37,$A$2:$A$65,0)),0))</f>
-        <v>0</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D37,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E37,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F37,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G37,$A$2:$A$70,0)),0))</f>
+        <v>21</v>
       </c>
       <c r="Q37" s="0" t="n">
         <f aca="false">P37+O37</f>
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="R37" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A37)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A37)),IF(COUNTIF($E$2:$E$65,$A37)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A37)),IF(COUNTIF($F$2:$F$65,$A37)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A37)),IF(COUNTIF($G$2:$G$65,$A37)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A37)))</f>
-        <v>41.75</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A37)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A37)),IF(COUNTIF($E$2:$E$70,$A37)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A37)),IF(COUNTIF($F$2:$F$70,$A37)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A37)),IF(COUNTIF($G$2:$G$70,$A37)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A37)))</f>
+        <v>46</v>
       </c>
       <c r="S37" s="0" t="n">
         <f aca="false">R37-O37</f>
-        <v>41.75</v>
+        <v>36</v>
       </c>
       <c r="T37" s="0" t="n">
         <f aca="false">S37-P37</f>
-        <v>41.75</v>
+        <v>15</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B38" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="C38" s="0" t="s">
         <v>97</v>
       </c>
-      <c r="B38" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="C38" s="0" t="s">
-        <v>98</v>
-      </c>
       <c r="D38" s="0" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="H38" s="0" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O38" s="0" t="n">
         <f aca="false">IF(H38&lt;&gt;"",H38,IF(AND(I38&lt;&gt;"",J38&lt;&gt;""),(I38+J38)/2,0))</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P38" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D38,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E38,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F38,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G38,$A$2:$A$65,0)),0))</f>
-        <v>0</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D38,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E38,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F38,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G38,$A$2:$A$70,0)),0))</f>
+        <v>1</v>
       </c>
       <c r="Q38" s="0" t="n">
         <f aca="false">P38+O38</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="R38" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A38)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A38)),IF(COUNTIF($E$2:$E$65,$A38)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A38)),IF(COUNTIF($F$2:$F$65,$A38)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A38)),IF(COUNTIF($G$2:$G$65,$A38)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A38)))</f>
-        <v>44.75</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A38)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A38)),IF(COUNTIF($E$2:$E$70,$A38)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A38)),IF(COUNTIF($F$2:$F$70,$A38)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A38)),IF(COUNTIF($G$2:$G$70,$A38)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A38)))</f>
+        <v>14.5</v>
       </c>
       <c r="S38" s="0" t="n">
         <f aca="false">R38-O38</f>
-        <v>41.75</v>
+        <v>9.5</v>
       </c>
       <c r="T38" s="0" t="n">
         <f aca="false">S38-P38</f>
-        <v>41.75</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B39" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="C39" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="B39" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="C39" s="0" t="s">
-        <v>100</v>
-      </c>
       <c r="D39" s="0" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="H39" s="0" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="O39" s="0" t="n">
         <f aca="false">IF(H39&lt;&gt;"",H39,IF(AND(I39&lt;&gt;"",J39&lt;&gt;""),(I39+J39)/2,0))</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="P39" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D39,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E39,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F39,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G39,$A$2:$A$65,0)),0))</f>
-        <v>0</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D39,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E39,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F39,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G39,$A$2:$A$70,0)),0))</f>
+        <v>6</v>
       </c>
       <c r="Q39" s="0" t="n">
         <f aca="false">P39+O39</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R39" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A39)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A39)),IF(COUNTIF($E$2:$E$65,$A39)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A39)),IF(COUNTIF($F$2:$F$65,$A39)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A39)),IF(COUNTIF($G$2:$G$65,$A39)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A39)))</f>
-        <v>60.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A39)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A39)),IF(COUNTIF($E$2:$E$70,$A39)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A39)),IF(COUNTIF($F$2:$F$70,$A39)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A39)),IF(COUNTIF($G$2:$G$70,$A39)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A39)))</f>
+        <v>46</v>
       </c>
       <c r="S39" s="0" t="n">
         <f aca="false">R39-O39</f>
-        <v>50.25</v>
+        <v>41</v>
       </c>
       <c r="T39" s="0" t="n">
         <f aca="false">S39-P39</f>
-        <v>50.25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B40" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="C40" s="0" t="s">
         <v>101</v>
       </c>
-      <c r="B40" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="C40" s="0" t="s">
-        <v>102</v>
-      </c>
       <c r="D40" s="0" t="s">
-        <v>94</v>
-      </c>
-      <c r="H40" s="0" t="n">
-        <v>15</v>
+        <v>89</v>
+      </c>
+      <c r="E40" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="I40" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="J40" s="0" t="n">
+        <v>8</v>
       </c>
       <c r="O40" s="0" t="n">
         <f aca="false">IF(H40&lt;&gt;"",H40,IF(AND(I40&lt;&gt;"",J40&lt;&gt;""),(I40+J40)/2,0))</f>
-        <v>15</v>
+        <v>6.5</v>
       </c>
       <c r="P40" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D40,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E40,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F40,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G40,$A$2:$A$65,0)),0))</f>
-        <v>0</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D40,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E40,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F40,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G40,$A$2:$A$70,0)),0))</f>
+        <v>31</v>
       </c>
       <c r="Q40" s="0" t="n">
         <f aca="false">P40+O40</f>
-        <v>15</v>
+        <v>37.5</v>
       </c>
       <c r="R40" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A40)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A40)),IF(COUNTIF($E$2:$E$65,$A40)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A40)),IF(COUNTIF($F$2:$F$65,$A40)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A40)),IF(COUNTIF($G$2:$G$65,$A40)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A40)))</f>
-        <v>60.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A40)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A40)),IF(COUNTIF($E$2:$E$70,$A40)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A40)),IF(COUNTIF($F$2:$F$70,$A40)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A40)),IF(COUNTIF($G$2:$G$70,$A40)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A40)))</f>
+        <v>46</v>
       </c>
       <c r="S40" s="0" t="n">
         <f aca="false">R40-O40</f>
-        <v>45.25</v>
+        <v>39.5</v>
       </c>
       <c r="T40" s="0" t="n">
         <f aca="false">S40-P40</f>
-        <v>45.25</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B41" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="C41" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="D41" s="0" t="s">
         <v>103</v>
       </c>
-      <c r="B41" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="C41" s="0" t="s">
-        <v>104</v>
-      </c>
-      <c r="D41" s="0" t="s">
-        <v>94</v>
-      </c>
       <c r="H41" s="0" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="O41" s="0" t="n">
         <f aca="false">IF(H41&lt;&gt;"",H41,IF(AND(I41&lt;&gt;"",J41&lt;&gt;""),(I41+J41)/2,0))</f>
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="P41" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D41,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E41,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F41,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G41,$A$2:$A$65,0)),0))</f>
-        <v>0</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D41,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E41,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F41,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G41,$A$2:$A$70,0)),0))</f>
+        <v>37.5</v>
       </c>
       <c r="Q41" s="0" t="n">
         <f aca="false">P41+O41</f>
-        <v>15</v>
+        <v>38.5</v>
       </c>
       <c r="R41" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A41)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A41)),IF(COUNTIF($E$2:$E$65,$A41)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A41)),IF(COUNTIF($F$2:$F$65,$A41)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A41)),IF(COUNTIF($G$2:$G$65,$A41)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A41)))</f>
-        <v>60.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A41)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A41)),IF(COUNTIF($E$2:$E$70,$A41)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A41)),IF(COUNTIF($F$2:$F$70,$A41)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A41)),IF(COUNTIF($G$2:$G$70,$A41)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A41)))</f>
+        <v>47</v>
       </c>
       <c r="S41" s="0" t="n">
         <f aca="false">R41-O41</f>
-        <v>45.25</v>
+        <v>46</v>
       </c>
       <c r="T41" s="0" t="n">
         <f aca="false">S41-P41</f>
-        <v>45.25</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B42" s="0" t="s">
         <v>105</v>
       </c>
-      <c r="B42" s="0" t="s">
-        <v>95</v>
-      </c>
       <c r="C42" s="0" t="s">
-        <v>60</v>
+        <v>106</v>
       </c>
       <c r="D42" s="0" t="s">
-        <v>103</v>
-      </c>
-      <c r="E42" s="0" t="s">
-        <v>101</v>
-      </c>
-      <c r="F42" s="0" t="s">
-        <v>99</v>
-      </c>
-      <c r="H42" s="0" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="O42" s="0" t="n">
         <f aca="false">IF(H42&lt;&gt;"",H42,IF(AND(I42&lt;&gt;"",J42&lt;&gt;""),(I42+J42)/2,0))</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P42" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D42,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E42,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F42,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G42,$A$2:$A$65,0)),0))</f>
-        <v>15</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D42,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E42,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F42,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G42,$A$2:$A$70,0)),0))</f>
+        <v>0</v>
       </c>
       <c r="Q42" s="0" t="n">
         <f aca="false">P42+O42</f>
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="R42" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A42)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A42)),IF(COUNTIF($E$2:$E$65,$A42)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A42)),IF(COUNTIF($F$2:$F$65,$A42)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A42)),IF(COUNTIF($G$2:$G$65,$A42)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A42)))</f>
-        <v>65.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A42)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A42)),IF(COUNTIF($E$2:$E$70,$A42)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A42)),IF(COUNTIF($F$2:$F$70,$A42)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A42)),IF(COUNTIF($G$2:$G$70,$A42)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A42)))</f>
+        <v>7.5</v>
       </c>
       <c r="S42" s="0" t="n">
         <f aca="false">R42-O42</f>
-        <v>60.25</v>
+        <v>7.5</v>
       </c>
       <c r="T42" s="0" t="n">
         <f aca="false">S42-P42</f>
-        <v>45.25</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="C43" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D43" s="0" t="s">
-        <v>97</v>
-      </c>
-      <c r="I43" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="J43" s="0" t="n">
-        <v>8</v>
+        <v>104</v>
+      </c>
+      <c r="H43" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="O43" s="0" t="n">
         <f aca="false">IF(H43&lt;&gt;"",H43,IF(AND(I43&lt;&gt;"",J43&lt;&gt;""),(I43+J43)/2,0))</f>
-        <v>6.5</v>
+        <v>3</v>
       </c>
       <c r="P43" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D43,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E43,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F43,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G43,$A$2:$A$65,0)),0))</f>
-        <v>3</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D43,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E43,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F43,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G43,$A$2:$A$70,0)),0))</f>
+        <v>0</v>
       </c>
       <c r="Q43" s="0" t="n">
         <f aca="false">P43+O43</f>
-        <v>9.5</v>
+        <v>3</v>
       </c>
       <c r="R43" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A43)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A43)),IF(COUNTIF($E$2:$E$65,$A43)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A43)),IF(COUNTIF($F$2:$F$65,$A43)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A43)),IF(COUNTIF($G$2:$G$65,$A43)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A43)))</f>
-        <v>51.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A43)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A43)),IF(COUNTIF($E$2:$E$70,$A43)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A43)),IF(COUNTIF($F$2:$F$70,$A43)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A43)),IF(COUNTIF($G$2:$G$70,$A43)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A43)))</f>
+        <v>10.5</v>
       </c>
       <c r="S43" s="0" t="n">
         <f aca="false">R43-O43</f>
-        <v>44.75</v>
+        <v>7.5</v>
       </c>
       <c r="T43" s="0" t="n">
         <f aca="false">S43-P43</f>
-        <v>41.75</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="C44" s="0" t="s">
-        <v>48</v>
+        <v>110</v>
       </c>
       <c r="D44" s="0" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H44" s="0" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="O44" s="0" t="n">
         <f aca="false">IF(H44&lt;&gt;"",H44,IF(AND(I44&lt;&gt;"",J44&lt;&gt;""),(I44+J44)/2,0))</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="P44" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D44,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E44,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F44,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G44,$A$2:$A$65,0)),0))</f>
-        <v>15</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D44,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E44,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F44,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G44,$A$2:$A$70,0)),0))</f>
+        <v>0</v>
       </c>
       <c r="Q44" s="0" t="n">
         <f aca="false">P44+O44</f>
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="R44" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A44)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A44)),IF(COUNTIF($E$2:$E$65,$A44)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A44)),IF(COUNTIF($F$2:$F$65,$A44)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A44)),IF(COUNTIF($G$2:$G$65,$A44)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A44)))</f>
-        <v>80.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A44)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A44)),IF(COUNTIF($E$2:$E$70,$A44)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A44)),IF(COUNTIF($F$2:$F$70,$A44)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A44)),IF(COUNTIF($G$2:$G$70,$A44)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A44)))</f>
+        <v>26</v>
       </c>
       <c r="S44" s="0" t="n">
         <f aca="false">R44-O44</f>
-        <v>75.25</v>
+        <v>16</v>
       </c>
       <c r="T44" s="0" t="n">
         <f aca="false">S44-P44</f>
-        <v>60.25</v>
+        <v>16</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="C45" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D45" s="0" t="s">
-        <v>106</v>
-      </c>
-      <c r="I45" s="0" t="n">
-        <v>20</v>
-      </c>
-      <c r="J45" s="0" t="n">
-        <v>28</v>
-      </c>
-      <c r="M45" s="0" t="s">
-        <v>111</v>
+        <v>104</v>
+      </c>
+      <c r="H45" s="0" t="n">
+        <v>15</v>
       </c>
       <c r="O45" s="0" t="n">
         <f aca="false">IF(H45&lt;&gt;"",H45,IF(AND(I45&lt;&gt;"",J45&lt;&gt;""),(I45+J45)/2,0))</f>
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="P45" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D45,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E45,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F45,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G45,$A$2:$A$65,0)),0))</f>
-        <v>9.5</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D45,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E45,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F45,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G45,$A$2:$A$70,0)),0))</f>
+        <v>0</v>
       </c>
       <c r="Q45" s="0" t="n">
         <f aca="false">P45+O45</f>
-        <v>33.5</v>
+        <v>15</v>
       </c>
       <c r="R45" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A45)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A45)),IF(COUNTIF($E$2:$E$65,$A45)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A45)),IF(COUNTIF($F$2:$F$65,$A45)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A45)),IF(COUNTIF($G$2:$G$65,$A45)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A45)))</f>
-        <v>75.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A45)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A45)),IF(COUNTIF($E$2:$E$70,$A45)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A45)),IF(COUNTIF($F$2:$F$70,$A45)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A45)),IF(COUNTIF($G$2:$G$70,$A45)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A45)))</f>
+        <v>26</v>
       </c>
       <c r="S45" s="0" t="n">
         <f aca="false">R45-O45</f>
-        <v>51.25</v>
+        <v>11</v>
       </c>
       <c r="T45" s="0" t="n">
         <f aca="false">S45-P45</f>
-        <v>41.75</v>
+        <v>11</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="C46" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="H46" s="0" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="O46" s="0" t="n">
         <f aca="false">IF(H46&lt;&gt;"",H46,IF(AND(I46&lt;&gt;"",J46&lt;&gt;""),(I46+J46)/2,0))</f>
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="P46" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D46,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E46,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F46,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G46,$A$2:$A$65,0)),0))</f>
-        <v>33.5</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D46,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E46,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F46,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G46,$A$2:$A$70,0)),0))</f>
+        <v>0</v>
       </c>
       <c r="Q46" s="0" t="n">
         <f aca="false">P46+O46</f>
-        <v>38.5</v>
+        <v>15</v>
       </c>
       <c r="R46" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A46)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A46)),IF(COUNTIF($E$2:$E$65,$A46)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A46)),IF(COUNTIF($F$2:$F$65,$A46)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A46)),IF(COUNTIF($G$2:$G$65,$A46)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A46)))</f>
-        <v>80.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A46)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A46)),IF(COUNTIF($E$2:$E$70,$A46)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A46)),IF(COUNTIF($F$2:$F$70,$A46)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A46)),IF(COUNTIF($G$2:$G$70,$A46)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A46)))</f>
+        <v>26</v>
       </c>
       <c r="S46" s="0" t="n">
         <f aca="false">R46-O46</f>
-        <v>75.25</v>
+        <v>11</v>
       </c>
       <c r="T46" s="0" t="n">
         <f aca="false">S46-P46</f>
-        <v>41.75</v>
+        <v>11</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="C47" s="0" t="s">
-        <v>115</v>
+        <v>60</v>
       </c>
       <c r="D47" s="0" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>103</v>
+        <v>111</v>
+      </c>
+      <c r="F47" s="0" t="s">
+        <v>109</v>
       </c>
       <c r="H47" s="0" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="O47" s="0" t="n">
         <f aca="false">IF(H47&lt;&gt;"",H47,IF(AND(I47&lt;&gt;"",J47&lt;&gt;""),(I47+J47)/2,0))</f>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="P47" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D47,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E47,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F47,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G47,$A$2:$A$65,0)),0))</f>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D47,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E47,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F47,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G47,$A$2:$A$70,0)),0))</f>
         <v>15</v>
       </c>
       <c r="Q47" s="0" t="n">
         <f aca="false">P47+O47</f>
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="R47" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A47)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A47)),IF(COUNTIF($E$2:$E$65,$A47)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A47)),IF(COUNTIF($F$2:$F$65,$A47)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A47)),IF(COUNTIF($G$2:$G$65,$A47)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A47)))</f>
-        <v>70.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A47)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A47)),IF(COUNTIF($E$2:$E$70,$A47)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A47)),IF(COUNTIF($F$2:$F$70,$A47)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A47)),IF(COUNTIF($G$2:$G$70,$A47)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A47)))</f>
+        <v>31</v>
       </c>
       <c r="S47" s="0" t="n">
         <f aca="false">R47-O47</f>
-        <v>61.25</v>
+        <v>26</v>
       </c>
       <c r="T47" s="0" t="n">
         <f aca="false">S47-P47</f>
-        <v>46.25</v>
+        <v>11</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2712,43 +2739,43 @@
         <v>116</v>
       </c>
       <c r="B48" s="0" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="C48" s="0" t="s">
         <v>117</v>
       </c>
       <c r="D48" s="0" t="s">
-        <v>101</v>
-      </c>
-      <c r="E48" s="0" t="s">
-        <v>103</v>
-      </c>
-      <c r="H48" s="0" t="n">
-        <v>3</v>
+        <v>107</v>
+      </c>
+      <c r="I48" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="J48" s="0" t="n">
+        <v>8</v>
       </c>
       <c r="O48" s="0" t="n">
         <f aca="false">IF(H48&lt;&gt;"",H48,IF(AND(I48&lt;&gt;"",J48&lt;&gt;""),(I48+J48)/2,0))</f>
+        <v>6.5</v>
+      </c>
+      <c r="P48" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D48,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E48,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F48,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G48,$A$2:$A$70,0)),0))</f>
         <v>3</v>
-      </c>
-      <c r="P48" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D48,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E48,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F48,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G48,$A$2:$A$65,0)),0))</f>
-        <v>15</v>
       </c>
       <c r="Q48" s="0" t="n">
         <f aca="false">P48+O48</f>
-        <v>18</v>
+        <v>9.5</v>
       </c>
       <c r="R48" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A48)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A48)),IF(COUNTIF($E$2:$E$65,$A48)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A48)),IF(COUNTIF($F$2:$F$65,$A48)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A48)),IF(COUNTIF($G$2:$G$65,$A48)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A48)))</f>
-        <v>80.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A48)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A48)),IF(COUNTIF($E$2:$E$70,$A48)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A48)),IF(COUNTIF($F$2:$F$70,$A48)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A48)),IF(COUNTIF($G$2:$G$70,$A48)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A48)))</f>
+        <v>17</v>
       </c>
       <c r="S48" s="0" t="n">
         <f aca="false">R48-O48</f>
-        <v>77.25</v>
+        <v>10.5</v>
       </c>
       <c r="T48" s="0" t="n">
         <f aca="false">S48-P48</f>
-        <v>62.25</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2756,13 +2783,13 @@
         <v>118</v>
       </c>
       <c r="B49" s="0" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="C49" s="0" t="s">
-        <v>119</v>
+        <v>48</v>
       </c>
       <c r="D49" s="0" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="H49" s="0" t="n">
         <v>5</v>
@@ -2772,401 +2799,404 @@
         <v>5</v>
       </c>
       <c r="P49" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D49,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E49,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F49,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G49,$A$2:$A$65,0)),0))</f>
-        <v>20</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D49,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E49,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F49,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G49,$A$2:$A$70,0)),0))</f>
+        <v>15</v>
       </c>
       <c r="Q49" s="0" t="n">
         <f aca="false">P49+O49</f>
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="R49" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A49)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A49)),IF(COUNTIF($E$2:$E$65,$A49)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A49)),IF(COUNTIF($F$2:$F$65,$A49)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A49)),IF(COUNTIF($G$2:$G$65,$A49)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A49)))</f>
-        <v>70.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A49)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A49)),IF(COUNTIF($E$2:$E$70,$A49)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A49)),IF(COUNTIF($F$2:$F$70,$A49)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A49)),IF(COUNTIF($G$2:$G$70,$A49)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A49)))</f>
+        <v>64.25</v>
       </c>
       <c r="S49" s="0" t="n">
         <f aca="false">R49-O49</f>
-        <v>65.25</v>
+        <v>59.25</v>
       </c>
       <c r="T49" s="0" t="n">
         <f aca="false">S49-P49</f>
-        <v>45.25</v>
+        <v>44.25</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B50" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="C50" s="0" t="s">
         <v>120</v>
       </c>
-      <c r="B50" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="C50" s="0" t="s">
-        <v>64</v>
-      </c>
       <c r="D50" s="0" t="s">
-        <v>118</v>
-      </c>
-      <c r="E50" s="0" t="s">
-        <v>114</v>
-      </c>
-      <c r="H50" s="0" t="n">
-        <v>10</v>
+        <v>116</v>
+      </c>
+      <c r="I50" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="J50" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="M50" s="0" t="s">
+        <v>121</v>
       </c>
       <c r="O50" s="0" t="n">
         <f aca="false">IF(H50&lt;&gt;"",H50,IF(AND(I50&lt;&gt;"",J50&lt;&gt;""),(I50+J50)/2,0))</f>
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="P50" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D50,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E50,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F50,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G50,$A$2:$A$65,0)),0))</f>
-        <v>25</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D50,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E50,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F50,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G50,$A$2:$A$70,0)),0))</f>
+        <v>9.5</v>
       </c>
       <c r="Q50" s="0" t="n">
         <f aca="false">P50+O50</f>
-        <v>35</v>
+        <v>33.5</v>
       </c>
       <c r="R50" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A50)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A50)),IF(COUNTIF($E$2:$E$65,$A50)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A50)),IF(COUNTIF($F$2:$F$65,$A50)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A50)),IF(COUNTIF($G$2:$G$65,$A50)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A50)))</f>
-        <v>80.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A50)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A50)),IF(COUNTIF($E$2:$E$70,$A50)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A50)),IF(COUNTIF($F$2:$F$70,$A50)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A50)),IF(COUNTIF($G$2:$G$70,$A50)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A50)))</f>
+        <v>41</v>
       </c>
       <c r="S50" s="0" t="n">
         <f aca="false">R50-O50</f>
-        <v>70.25</v>
+        <v>17</v>
       </c>
       <c r="T50" s="0" t="n">
         <f aca="false">S50-P50</f>
-        <v>45.25</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B51" s="0" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="C51" s="0" t="s">
-        <v>66</v>
+        <v>123</v>
       </c>
       <c r="D51" s="0" t="s">
-        <v>118</v>
-      </c>
-      <c r="E51" s="0" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="H51" s="0" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="O51" s="0" t="n">
         <f aca="false">IF(H51&lt;&gt;"",H51,IF(AND(I51&lt;&gt;"",J51&lt;&gt;""),(I51+J51)/2,0))</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="P51" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D51,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E51,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F51,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G51,$A$2:$A$65,0)),0))</f>
-        <v>25</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D51,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E51,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F51,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G51,$A$2:$A$70,0)),0))</f>
+        <v>33.5</v>
       </c>
       <c r="Q51" s="0" t="n">
         <f aca="false">P51+O51</f>
-        <v>35</v>
+        <v>38.5</v>
       </c>
       <c r="R51" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A51)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A51)),IF(COUNTIF($E$2:$E$65,$A51)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A51)),IF(COUNTIF($F$2:$F$65,$A51)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A51)),IF(COUNTIF($G$2:$G$65,$A51)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A51)))</f>
-        <v>80.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A51)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A51)),IF(COUNTIF($E$2:$E$70,$A51)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A51)),IF(COUNTIF($F$2:$F$70,$A51)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A51)),IF(COUNTIF($G$2:$G$70,$A51)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A51)))</f>
+        <v>46</v>
       </c>
       <c r="S51" s="0" t="n">
         <f aca="false">R51-O51</f>
-        <v>70.25</v>
+        <v>41</v>
       </c>
       <c r="T51" s="0" t="n">
         <f aca="false">S51-P51</f>
-        <v>45.25</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B52" s="0" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="C52" s="0" t="s">
-        <v>40</v>
+        <v>125</v>
       </c>
       <c r="D52" s="0" t="s">
-        <v>62</v>
+        <v>111</v>
+      </c>
+      <c r="E52" s="0" t="s">
+        <v>113</v>
       </c>
       <c r="H52" s="0" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="O52" s="0" t="n">
         <f aca="false">IF(H52&lt;&gt;"",H52,IF(AND(I52&lt;&gt;"",J52&lt;&gt;""),(I52+J52)/2,0))</f>
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="P52" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D52,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E52,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F52,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G52,$A$2:$A$65,0)),0))</f>
-        <v>60</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D52,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E52,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F52,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G52,$A$2:$A$70,0)),0))</f>
+        <v>15</v>
       </c>
       <c r="Q52" s="0" t="n">
         <f aca="false">P52+O52</f>
-        <v>61</v>
+        <v>24</v>
       </c>
       <c r="R52" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A52)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A52)),IF(COUNTIF($E$2:$E$65,$A52)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A52)),IF(COUNTIF($F$2:$F$65,$A52)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A52)),IF(COUNTIF($G$2:$G$65,$A52)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A52)))</f>
-        <v>63</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A52)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A52)),IF(COUNTIF($E$2:$E$70,$A52)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A52)),IF(COUNTIF($F$2:$F$70,$A52)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A52)),IF(COUNTIF($G$2:$G$70,$A52)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A52)))</f>
+        <v>36</v>
       </c>
       <c r="S52" s="0" t="n">
         <f aca="false">R52-O52</f>
-        <v>62</v>
+        <v>27</v>
       </c>
       <c r="T52" s="0" t="n">
         <f aca="false">S52-P52</f>
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>23</v>
+        <v>126</v>
       </c>
       <c r="B53" s="0" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="C53" s="0" t="s">
-        <v>124</v>
-      </c>
-      <c r="N53" s="2" t="n">
-        <v>40080</v>
+        <v>127</v>
+      </c>
+      <c r="D53" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="E53" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="H53" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="O53" s="0" t="n">
         <f aca="false">IF(H53&lt;&gt;"",H53,IF(AND(I53&lt;&gt;"",J53&lt;&gt;""),(I53+J53)/2,0))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P53" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D53,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E53,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F53,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G53,$A$2:$A$65,0)),0))</f>
-        <v>0</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D53,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E53,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F53,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G53,$A$2:$A$70,0)),0))</f>
+        <v>15</v>
       </c>
       <c r="Q53" s="0" t="n">
         <f aca="false">P53+O53</f>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="R53" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A53)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A53)),IF(COUNTIF($E$2:$E$65,$A53)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A53)),IF(COUNTIF($F$2:$F$65,$A53)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A53)),IF(COUNTIF($G$2:$G$65,$A53)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A53)))</f>
-        <v>0</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A53)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A53)),IF(COUNTIF($E$2:$E$70,$A53)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A53)),IF(COUNTIF($F$2:$F$70,$A53)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A53)),IF(COUNTIF($G$2:$G$70,$A53)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A53)))</f>
+        <v>64.25</v>
       </c>
       <c r="S53" s="0" t="n">
         <f aca="false">R53-O53</f>
-        <v>0</v>
+        <v>61.25</v>
       </c>
       <c r="T53" s="0" t="n">
         <f aca="false">S53-P53</f>
-        <v>0</v>
+        <v>46.25</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B54" s="0" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="C54" s="0" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D54" s="0" t="s">
-        <v>127</v>
-      </c>
-      <c r="I54" s="0" t="n">
+        <v>115</v>
+      </c>
+      <c r="H54" s="0" t="n">
         <v>5</v>
-      </c>
-      <c r="J54" s="0" t="n">
-        <v>10</v>
       </c>
       <c r="O54" s="0" t="n">
         <f aca="false">IF(H54&lt;&gt;"",H54,IF(AND(I54&lt;&gt;"",J54&lt;&gt;""),(I54+J54)/2,0))</f>
-        <v>7.5</v>
+        <v>5</v>
       </c>
       <c r="P54" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D54,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E54,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F54,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G54,$A$2:$A$65,0)),0))</f>
-        <v>72</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D54,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E54,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F54,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G54,$A$2:$A$70,0)),0))</f>
+        <v>20</v>
       </c>
       <c r="Q54" s="0" t="n">
         <f aca="false">P54+O54</f>
-        <v>79.5</v>
+        <v>25</v>
       </c>
       <c r="R54" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A54)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A54)),IF(COUNTIF($E$2:$E$65,$A54)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A54)),IF(COUNTIF($F$2:$F$65,$A54)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A54)),IF(COUNTIF($G$2:$G$65,$A54)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A54)))</f>
-        <v>79.5</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A54)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A54)),IF(COUNTIF($E$2:$E$70,$A54)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A54)),IF(COUNTIF($F$2:$F$70,$A54)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A54)),IF(COUNTIF($G$2:$G$70,$A54)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A54)))</f>
+        <v>36</v>
       </c>
       <c r="S54" s="0" t="n">
         <f aca="false">R54-O54</f>
-        <v>72</v>
+        <v>31</v>
       </c>
       <c r="T54" s="0" t="n">
         <f aca="false">S54-P54</f>
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B55" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="C55" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="D55" s="0" t="s">
         <v>128</v>
       </c>
-      <c r="B55" s="0" t="s">
-        <v>123</v>
-      </c>
-      <c r="C55" s="0" t="s">
-        <v>129</v>
-      </c>
-      <c r="D55" s="0" t="s">
-        <v>23</v>
+      <c r="E55" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="H55" s="0" t="n">
+        <v>10</v>
       </c>
       <c r="O55" s="0" t="n">
         <f aca="false">IF(H55&lt;&gt;"",H55,IF(AND(I55&lt;&gt;"",J55&lt;&gt;""),(I55+J55)/2,0))</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P55" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D55,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E55,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F55,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G55,$A$2:$A$65,0)),0))</f>
-        <v>0</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D55,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E55,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F55,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G55,$A$2:$A$70,0)),0))</f>
+        <v>25</v>
       </c>
       <c r="Q55" s="0" t="n">
         <f aca="false">P55+O55</f>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="R55" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A55)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A55)),IF(COUNTIF($E$2:$E$65,$A55)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A55)),IF(COUNTIF($F$2:$F$65,$A55)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A55)),IF(COUNTIF($G$2:$G$65,$A55)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A55)))</f>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A55)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A55)),IF(COUNTIF($E$2:$E$70,$A55)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A55)),IF(COUNTIF($F$2:$F$70,$A55)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A55)),IF(COUNTIF($G$2:$G$70,$A55)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A55)))</f>
         <v>46</v>
       </c>
       <c r="S55" s="0" t="n">
         <f aca="false">R55-O55</f>
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="T55" s="0" t="n">
         <f aca="false">S55-P55</f>
-        <v>46</v>
+        <v>11</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B56" s="0" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="C56" s="0" t="s">
-        <v>131</v>
+        <v>66</v>
       </c>
       <c r="D56" s="0" t="s">
         <v>128</v>
       </c>
-      <c r="I56" s="0" t="n">
-        <v>14</v>
-      </c>
-      <c r="J56" s="0" t="n">
-        <v>28</v>
+      <c r="E56" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="H56" s="0" t="n">
+        <v>10</v>
       </c>
       <c r="O56" s="0" t="n">
         <f aca="false">IF(H56&lt;&gt;"",H56,IF(AND(I56&lt;&gt;"",J56&lt;&gt;""),(I56+J56)/2,0))</f>
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="P56" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D56,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E56,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F56,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G56,$A$2:$A$65,0)),0))</f>
-        <v>0</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D56,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E56,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F56,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G56,$A$2:$A$70,0)),0))</f>
+        <v>25</v>
       </c>
       <c r="Q56" s="0" t="n">
         <f aca="false">P56+O56</f>
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="R56" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A56)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A56)),IF(COUNTIF($E$2:$E$65,$A56)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A56)),IF(COUNTIF($F$2:$F$65,$A56)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A56)),IF(COUNTIF($G$2:$G$65,$A56)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A56)))</f>
-        <v>67</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A56)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A56)),IF(COUNTIF($E$2:$E$70,$A56)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A56)),IF(COUNTIF($F$2:$F$70,$A56)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A56)),IF(COUNTIF($G$2:$G$70,$A56)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A56)))</f>
+        <v>46</v>
       </c>
       <c r="S56" s="0" t="n">
         <f aca="false">R56-O56</f>
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="T56" s="0" t="n">
         <f aca="false">S56-P56</f>
-        <v>46</v>
+        <v>11</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="B57" s="0" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="C57" s="0" t="s">
-        <v>132</v>
+        <v>40</v>
       </c>
       <c r="D57" s="0" t="s">
         <v>133</v>
       </c>
-      <c r="E57" s="0" t="s">
-        <v>130</v>
-      </c>
       <c r="H57" s="0" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O57" s="0" t="n">
         <f aca="false">IF(H57&lt;&gt;"",H57,IF(AND(I57&lt;&gt;"",J57&lt;&gt;""),(I57+J57)/2,0))</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="P57" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D57,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E57,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F57,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G57,$A$2:$A$65,0)),0))</f>
-        <v>67</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D57,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E57,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F57,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G57,$A$2:$A$70,0)),0))</f>
+        <v>38.5</v>
       </c>
       <c r="Q57" s="0" t="n">
         <f aca="false">P57+O57</f>
-        <v>72</v>
+        <v>39.5</v>
       </c>
       <c r="R57" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A57)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A57)),IF(COUNTIF($E$2:$E$65,$A57)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A57)),IF(COUNTIF($F$2:$F$65,$A57)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A57)),IF(COUNTIF($G$2:$G$65,$A57)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A57)))</f>
-        <v>72</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A57)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A57)),IF(COUNTIF($E$2:$E$70,$A57)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A57)),IF(COUNTIF($F$2:$F$70,$A57)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A57)),IF(COUNTIF($G$2:$G$70,$A57)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A57)))</f>
+        <v>47</v>
       </c>
       <c r="S57" s="0" t="n">
         <f aca="false">R57-O57</f>
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="T57" s="0" t="n">
         <f aca="false">S57-P57</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B58" s="0" t="s">
         <v>134</v>
-      </c>
-      <c r="B58" s="0" t="s">
-        <v>123</v>
       </c>
       <c r="C58" s="0" t="s">
         <v>135</v>
       </c>
-      <c r="D58" s="0" t="s">
-        <v>125</v>
-      </c>
-      <c r="I58" s="0" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J58" s="0" t="n">
-        <v>1</v>
+      <c r="N58" s="2" t="n">
+        <v>40080</v>
       </c>
       <c r="O58" s="0" t="n">
         <f aca="false">IF(H58&lt;&gt;"",H58,IF(AND(I58&lt;&gt;"",J58&lt;&gt;""),(I58+J58)/2,0))</f>
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="P58" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D58,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E58,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F58,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G58,$A$2:$A$65,0)),0))</f>
-        <v>79.5</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D58,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E58,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F58,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G58,$A$2:$A$70,0)),0))</f>
+        <v>0</v>
       </c>
       <c r="Q58" s="0" t="n">
         <f aca="false">P58+O58</f>
-        <v>80.25</v>
+        <v>0</v>
       </c>
       <c r="R58" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A58)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A58)),IF(COUNTIF($E$2:$E$65,$A58)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A58)),IF(COUNTIF($F$2:$F$65,$A58)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A58)),IF(COUNTIF($G$2:$G$65,$A58)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A58)))</f>
-        <v>80.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A58)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A58)),IF(COUNTIF($E$2:$E$70,$A58)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A58)),IF(COUNTIF($F$2:$F$70,$A58)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A58)),IF(COUNTIF($G$2:$G$70,$A58)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A58)))</f>
+        <v>0</v>
       </c>
       <c r="S58" s="0" t="n">
         <f aca="false">R58-O58</f>
-        <v>79.5</v>
+        <v>0</v>
       </c>
       <c r="T58" s="0" t="n">
         <f aca="false">S58-P58</f>
@@ -3178,165 +3208,165 @@
         <v>136</v>
       </c>
       <c r="B59" s="0" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="C59" s="0" t="s">
         <v>137</v>
       </c>
       <c r="D59" s="0" t="s">
-        <v>125</v>
+        <v>138</v>
+      </c>
+      <c r="I59" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="J59" s="0" t="n">
+        <v>10</v>
       </c>
       <c r="O59" s="0" t="n">
         <f aca="false">IF(H59&lt;&gt;"",H59,IF(AND(I59&lt;&gt;"",J59&lt;&gt;""),(I59+J59)/2,0))</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="P59" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D59,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E59,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F59,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G59,$A$2:$A$65,0)),0))</f>
-        <v>79.5</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D59,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E59,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F59,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G59,$A$2:$A$70,0)),0))</f>
+        <v>56</v>
       </c>
       <c r="Q59" s="0" t="n">
         <f aca="false">P59+O59</f>
-        <v>79.5</v>
+        <v>63.5</v>
       </c>
       <c r="R59" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A59)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A59)),IF(COUNTIF($E$2:$E$65,$A59)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A59)),IF(COUNTIF($F$2:$F$65,$A59)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A59)),IF(COUNTIF($G$2:$G$65,$A59)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A59)))</f>
-        <v>80.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A59)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A59)),IF(COUNTIF($E$2:$E$70,$A59)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A59)),IF(COUNTIF($F$2:$F$70,$A59)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A59)),IF(COUNTIF($G$2:$G$70,$A59)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A59)))</f>
+        <v>63.5</v>
       </c>
       <c r="S59" s="0" t="n">
         <f aca="false">R59-O59</f>
-        <v>80.25</v>
+        <v>56</v>
       </c>
       <c r="T59" s="0" t="n">
         <f aca="false">S59-P59</f>
-        <v>0.75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B60" s="0" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="C60" s="0" t="s">
-        <v>40</v>
+        <v>140</v>
       </c>
       <c r="D60" s="0" t="s">
-        <v>138</v>
-      </c>
-      <c r="H60" s="0" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="O60" s="0" t="n">
         <f aca="false">IF(H60&lt;&gt;"",H60,IF(AND(I60&lt;&gt;"",J60&lt;&gt;""),(I60+J60)/2,0))</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P60" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D60,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E60,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F60,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G60,$A$2:$A$65,0)),0))</f>
-        <v>63</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D60,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E60,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F60,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G60,$A$2:$A$70,0)),0))</f>
+        <v>0</v>
       </c>
       <c r="Q60" s="0" t="n">
         <f aca="false">P60+O60</f>
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="R60" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A60)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A60)),IF(COUNTIF($E$2:$E$65,$A60)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A60)),IF(COUNTIF($F$2:$F$65,$A60)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A60)),IF(COUNTIF($G$2:$G$65,$A60)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A60)))</f>
-        <v>67</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A60)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A60)),IF(COUNTIF($E$2:$E$70,$A60)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A60)),IF(COUNTIF($F$2:$F$70,$A60)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A60)),IF(COUNTIF($G$2:$G$70,$A60)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A60)))</f>
+        <v>30</v>
       </c>
       <c r="S60" s="0" t="n">
         <f aca="false">R60-O60</f>
-        <v>63</v>
+        <v>30</v>
       </c>
       <c r="T60" s="0" t="n">
         <f aca="false">S60-P60</f>
-        <v>0</v>
+        <v>30</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B61" s="0" t="s">
+        <v>134</v>
+      </c>
+      <c r="C61" s="0" t="s">
+        <v>142</v>
+      </c>
+      <c r="D61" s="0" t="s">
         <v>139</v>
       </c>
-      <c r="B61" s="0" t="s">
-        <v>123</v>
-      </c>
-      <c r="C61" s="0" t="s">
-        <v>140</v>
-      </c>
-      <c r="D61" s="0" t="s">
-        <v>121</v>
-      </c>
-      <c r="E61" s="0" t="s">
-        <v>120</v>
-      </c>
-      <c r="F61" s="0" t="s">
-        <v>112</v>
+      <c r="I61" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="J61" s="0" t="n">
+        <v>28</v>
       </c>
       <c r="O61" s="0" t="n">
         <f aca="false">IF(H61&lt;&gt;"",H61,IF(AND(I61&lt;&gt;"",J61&lt;&gt;""),(I61+J61)/2,0))</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="P61" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D61,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E61,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F61,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G61,$A$2:$A$65,0)),0))</f>
-        <v>38.5</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D61,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E61,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F61,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G61,$A$2:$A$70,0)),0))</f>
+        <v>0</v>
       </c>
       <c r="Q61" s="0" t="n">
         <f aca="false">P61+O61</f>
-        <v>38.5</v>
+        <v>21</v>
       </c>
       <c r="R61" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A61)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A61)),IF(COUNTIF($E$2:$E$65,$A61)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A61)),IF(COUNTIF($F$2:$F$65,$A61)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A61)),IF(COUNTIF($G$2:$G$65,$A61)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A61)))</f>
-        <v>80.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A61)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A61)),IF(COUNTIF($E$2:$E$70,$A61)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A61)),IF(COUNTIF($F$2:$F$70,$A61)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A61)),IF(COUNTIF($G$2:$G$70,$A61)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A61)))</f>
+        <v>51</v>
       </c>
       <c r="S61" s="0" t="n">
         <f aca="false">R61-O61</f>
-        <v>80.25</v>
+        <v>30</v>
       </c>
       <c r="T61" s="0" t="n">
         <f aca="false">S61-P61</f>
-        <v>41.75</v>
+        <v>30</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>93</v>
+        <v>138</v>
       </c>
       <c r="B62" s="0" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="C62" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="D62" s="0" t="s">
+        <v>144</v>
+      </c>
+      <c r="E62" s="0" t="s">
         <v>141</v>
       </c>
-      <c r="D62" s="0" t="s">
-        <v>88</v>
-      </c>
-      <c r="E62" s="0" t="s">
-        <v>90</v>
-      </c>
-      <c r="F62" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="G62" s="0" t="s">
-        <v>77</v>
+      <c r="H62" s="0" t="n">
+        <v>5</v>
       </c>
       <c r="O62" s="0" t="n">
         <f aca="false">IF(H62&lt;&gt;"",H62,IF(AND(I62&lt;&gt;"",J62&lt;&gt;""),(I62+J62)/2,0))</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P62" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D62,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E62,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F62,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G62,$A$2:$A$65,0)),0))</f>
-        <v>62</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D62,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E62,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F62,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G62,$A$2:$A$70,0)),0))</f>
+        <v>51</v>
       </c>
       <c r="Q62" s="0" t="n">
         <f aca="false">P62+O62</f>
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="R62" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A62)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A62)),IF(COUNTIF($E$2:$E$65,$A62)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A62)),IF(COUNTIF($F$2:$F$65,$A62)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A62)),IF(COUNTIF($G$2:$G$65,$A62)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A62)))</f>
-        <v>62</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A62)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A62)),IF(COUNTIF($E$2:$E$70,$A62)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A62)),IF(COUNTIF($F$2:$F$70,$A62)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A62)),IF(COUNTIF($G$2:$G$70,$A62)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A62)))</f>
+        <v>56</v>
       </c>
       <c r="S62" s="0" t="n">
         <f aca="false">R62-O62</f>
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="T62" s="0" t="n">
         <f aca="false">S62-P62</f>
@@ -3345,124 +3375,121 @@
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>41</v>
+        <v>145</v>
       </c>
       <c r="B63" s="0" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="C63" s="0" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="D63" s="0" t="s">
-        <v>37</v>
+        <v>136</v>
+      </c>
+      <c r="I63" s="0" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J63" s="0" t="n">
+        <v>1</v>
       </c>
       <c r="O63" s="0" t="n">
         <f aca="false">IF(H63&lt;&gt;"",H63,IF(AND(I63&lt;&gt;"",J63&lt;&gt;""),(I63+J63)/2,0))</f>
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="P63" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D63,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E63,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F63,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G63,$A$2:$A$65,0)),0))</f>
-        <v>45.5</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D63,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E63,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F63,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G63,$A$2:$A$70,0)),0))</f>
+        <v>63.5</v>
       </c>
       <c r="Q63" s="0" t="n">
         <f aca="false">P63+O63</f>
-        <v>45.5</v>
+        <v>64.25</v>
       </c>
       <c r="R63" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A63)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A63)),IF(COUNTIF($E$2:$E$65,$A63)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A63)),IF(COUNTIF($F$2:$F$65,$A63)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A63)),IF(COUNTIF($G$2:$G$65,$A63)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A63)))</f>
-        <v>62</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A63)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A63)),IF(COUNTIF($E$2:$E$70,$A63)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A63)),IF(COUNTIF($F$2:$F$70,$A63)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A63)),IF(COUNTIF($G$2:$G$70,$A63)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A63)))</f>
+        <v>64.25</v>
       </c>
       <c r="S63" s="0" t="n">
         <f aca="false">R63-O63</f>
-        <v>62</v>
+        <v>63.5</v>
       </c>
       <c r="T63" s="0" t="n">
         <f aca="false">S63-P63</f>
-        <v>16.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
       <c r="B64" s="0" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="C64" s="0" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="D64" s="0" t="s">
-        <v>63</v>
-      </c>
-      <c r="E64" s="0" t="s">
-        <v>65</v>
+        <v>136</v>
       </c>
       <c r="O64" s="0" t="n">
         <f aca="false">IF(H64&lt;&gt;"",H64,IF(AND(I64&lt;&gt;"",J64&lt;&gt;""),(I64+J64)/2,0))</f>
         <v>0</v>
       </c>
       <c r="P64" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D64,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E64,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F64,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G64,$A$2:$A$65,0)),0))</f>
-        <v>60</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D64,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E64,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F64,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G64,$A$2:$A$70,0)),0))</f>
+        <v>63.5</v>
       </c>
       <c r="Q64" s="0" t="n">
         <f aca="false">P64+O64</f>
-        <v>60</v>
+        <v>63.5</v>
       </c>
       <c r="R64" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A64)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A64)),IF(COUNTIF($E$2:$E$65,$A64)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A64)),IF(COUNTIF($F$2:$F$65,$A64)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A64)),IF(COUNTIF($G$2:$G$65,$A64)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A64)))</f>
-        <v>62</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A64)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A64)),IF(COUNTIF($E$2:$E$70,$A64)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A64)),IF(COUNTIF($F$2:$F$70,$A64)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A64)),IF(COUNTIF($G$2:$G$70,$A64)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A64)))</f>
+        <v>64.25</v>
       </c>
       <c r="S64" s="0" t="n">
         <f aca="false">R64-O64</f>
-        <v>62</v>
+        <v>64.25</v>
       </c>
       <c r="T64" s="0" t="n">
         <f aca="false">S64-P64</f>
-        <v>2</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="0" t="s">
-        <v>138</v>
+      <c r="A65" s="1" t="s">
+        <v>144</v>
       </c>
       <c r="B65" s="0" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="C65" s="0" t="s">
-        <v>144</v>
+        <v>40</v>
       </c>
       <c r="D65" s="0" t="s">
-        <v>122</v>
-      </c>
-      <c r="E65" s="0" t="s">
-        <v>92</v>
-      </c>
-      <c r="F65" s="0" t="s">
-        <v>61</v>
-      </c>
-      <c r="G65" s="0" t="s">
-        <v>39</v>
+        <v>149</v>
+      </c>
+      <c r="H65" s="0" t="n">
+        <v>4</v>
       </c>
       <c r="O65" s="0" t="n">
         <f aca="false">IF(H65&lt;&gt;"",H65,IF(AND(I65&lt;&gt;"",J65&lt;&gt;""),(I65+J65)/2,0))</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P65" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D65,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E65,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F65,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G65,$A$2:$A$65,0)),0))</f>
-        <v>63</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D65,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E65,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F65,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G65,$A$2:$A$70,0)),0))</f>
+        <v>47</v>
       </c>
       <c r="Q65" s="0" t="n">
         <f aca="false">P65+O65</f>
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="R65" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A65)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A65)),IF(COUNTIF($E$2:$E$65,$A65)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A65)),IF(COUNTIF($F$2:$F$65,$A65)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A65)),IF(COUNTIF($G$2:$G$65,$A65)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A65)))</f>
-        <v>63</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A65)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A65)),IF(COUNTIF($E$2:$E$70,$A65)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A65)),IF(COUNTIF($F$2:$F$70,$A65)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A65)),IF(COUNTIF($G$2:$G$70,$A65)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A65)))</f>
+        <v>51</v>
       </c>
       <c r="S65" s="0" t="n">
         <f aca="false">R65-O65</f>
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="T65" s="0" t="n">
         <f aca="false">S65-P65</f>
@@ -3471,52 +3498,269 @@
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="B66" s="0" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="C66" s="0" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="D66" s="0" t="s">
-        <v>127</v>
-      </c>
-      <c r="K66" s="0" t="s">
-        <v>32</v>
+        <v>131</v>
+      </c>
+      <c r="E66" s="0" t="s">
+        <v>130</v>
+      </c>
+      <c r="F66" s="0" t="s">
+        <v>122</v>
       </c>
       <c r="O66" s="0" t="n">
         <f aca="false">IF(H66&lt;&gt;"",H66,IF(AND(I66&lt;&gt;"",J66&lt;&gt;""),(I66+J66)/2,0))</f>
         <v>0</v>
       </c>
       <c r="P66" s="0" t="n">
-        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$65,MATCH(D66,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(E66,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(F66,$A$2:$A$65,0)),0),IFERROR(INDEX($Q$2:$Q$65,MATCH(G66,$A$2:$A$65,0)),0))</f>
-        <v>72</v>
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D66,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E66,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F66,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G66,$A$2:$A$70,0)),0))</f>
+        <v>38.5</v>
       </c>
       <c r="Q66" s="0" t="n">
         <f aca="false">P66+O66</f>
-        <v>72</v>
+        <v>38.5</v>
       </c>
       <c r="R66" s="0" t="n">
-        <f aca="false">MIN(IF(COUNTIF($D$2:$D$65,$A66)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$D$2:$D$65,$A66)),IF(COUNTIF($E$2:$E$65,$A66)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$E$2:$E$65,$A66)),IF(COUNTIF($F$2:$F$65,$A66)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$F$2:$F$65,$A66)),IF(COUNTIF($G$2:$G$65,$A66)=0,$O$68,_xlfn.MINIFS($S$2:$S$65,$G$2:$G$65,$A66)))</f>
-        <v>80.25</v>
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A66)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A66)),IF(COUNTIF($E$2:$E$70,$A66)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A66)),IF(COUNTIF($F$2:$F$70,$A66)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A66)),IF(COUNTIF($G$2:$G$70,$A66)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A66)))</f>
+        <v>46</v>
       </c>
       <c r="S66" s="0" t="n">
         <f aca="false">R66-O66</f>
-        <v>80.25</v>
+        <v>46</v>
       </c>
       <c r="T66" s="0" t="n">
         <f aca="false">S66-P66</f>
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B67" s="0" t="s">
+        <v>134</v>
+      </c>
+      <c r="C67" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="D67" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="E67" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="F67" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="G67" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="O67" s="0" t="n">
+        <f aca="false">IF(H67&lt;&gt;"",H67,IF(AND(I67&lt;&gt;"",J67&lt;&gt;""),(I67+J67)/2,0))</f>
+        <v>0</v>
+      </c>
+      <c r="P67" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D67,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E67,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F67,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G67,$A$2:$A$70,0)),0))</f>
+        <v>37.5</v>
+      </c>
+      <c r="Q67" s="0" t="n">
+        <f aca="false">P67+O67</f>
+        <v>37.5</v>
+      </c>
+      <c r="R67" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A67)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A67)),IF(COUNTIF($E$2:$E$70,$A67)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A67)),IF(COUNTIF($F$2:$F$70,$A67)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A67)),IF(COUNTIF($G$2:$G$70,$A67)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A67)))</f>
+        <v>46</v>
+      </c>
+      <c r="S67" s="0" t="n">
+        <f aca="false">R67-O67</f>
+        <v>46</v>
+      </c>
+      <c r="T67" s="0" t="n">
+        <f aca="false">S67-P67</f>
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B68" s="0" t="s">
+        <v>134</v>
+      </c>
+      <c r="C68" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="D68" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="O68" s="0" t="n">
+        <f aca="false">IF(H68&lt;&gt;"",H68,IF(AND(I68&lt;&gt;"",J68&lt;&gt;""),(I68+J68)/2,0))</f>
+        <v>0</v>
+      </c>
+      <c r="P68" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D68,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E68,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F68,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G68,$A$2:$A$70,0)),0))</f>
+        <v>45.5</v>
+      </c>
+      <c r="Q68" s="0" t="n">
+        <f aca="false">P68+O68</f>
+        <v>45.5</v>
+      </c>
+      <c r="R68" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A68)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A68)),IF(COUNTIF($E$2:$E$70,$A68)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A68)),IF(COUNTIF($F$2:$F$70,$A68)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A68)),IF(COUNTIF($G$2:$G$70,$A68)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A68)))</f>
+        <v>46</v>
+      </c>
+      <c r="S68" s="0" t="n">
+        <f aca="false">R68-O68</f>
+        <v>46</v>
+      </c>
+      <c r="T68" s="0" t="n">
+        <f aca="false">S68-P68</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B69" s="0" t="s">
+        <v>134</v>
+      </c>
+      <c r="C69" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="D69" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="E69" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="O69" s="0" t="n">
+        <f aca="false">IF(H69&lt;&gt;"",H69,IF(AND(I69&lt;&gt;"",J69&lt;&gt;""),(I69+J69)/2,0))</f>
+        <v>0</v>
+      </c>
+      <c r="P69" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D69,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E69,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F69,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G69,$A$2:$A$70,0)),0))</f>
+        <v>46</v>
+      </c>
+      <c r="Q69" s="0" t="n">
+        <f aca="false">P69+O69</f>
+        <v>46</v>
+      </c>
+      <c r="R69" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A69)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A69)),IF(COUNTIF($E$2:$E$70,$A69)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A69)),IF(COUNTIF($F$2:$F$70,$A69)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A69)),IF(COUNTIF($G$2:$G$70,$A69)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A69)))</f>
+        <v>46</v>
+      </c>
+      <c r="S69" s="0" t="n">
+        <f aca="false">R69-O69</f>
+        <v>46</v>
+      </c>
+      <c r="T69" s="0" t="n">
+        <f aca="false">S69-P69</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="B70" s="0" t="s">
+        <v>134</v>
+      </c>
+      <c r="C70" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="D70" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="E70" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="F70" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="G70" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="O70" s="0" t="n">
+        <f aca="false">IF(H70&lt;&gt;"",H70,IF(AND(I70&lt;&gt;"",J70&lt;&gt;""),(I70+J70)/2,0))</f>
+        <v>0</v>
+      </c>
+      <c r="P70" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D70,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E70,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F70,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G70,$A$2:$A$70,0)),0))</f>
+        <v>47</v>
+      </c>
+      <c r="Q70" s="0" t="n">
+        <f aca="false">P70+O70</f>
+        <v>47</v>
+      </c>
+      <c r="R70" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A70)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A70)),IF(COUNTIF($E$2:$E$70,$A70)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A70)),IF(COUNTIF($F$2:$F$70,$A70)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A70)),IF(COUNTIF($G$2:$G$70,$A70)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A70)))</f>
+        <v>47</v>
+      </c>
+      <c r="S70" s="0" t="n">
+        <f aca="false">R70-O70</f>
+        <v>47</v>
+      </c>
+      <c r="T70" s="0" t="n">
+        <f aca="false">S70-P70</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B71" s="0" t="s">
+        <v>134</v>
+      </c>
+      <c r="C71" s="0" t="s">
+        <v>156</v>
+      </c>
+      <c r="D71" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="K71" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="O71" s="0" t="n">
+        <f aca="false">IF(H71&lt;&gt;"",H71,IF(AND(I71&lt;&gt;"",J71&lt;&gt;""),(I71+J71)/2,0))</f>
+        <v>0</v>
+      </c>
+      <c r="P71" s="0" t="n">
+        <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D71,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E71,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F71,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G71,$A$2:$A$70,0)),0))</f>
+        <v>56</v>
+      </c>
+      <c r="Q71" s="0" t="n">
+        <f aca="false">P71+O71</f>
+        <v>56</v>
+      </c>
+      <c r="R71" s="0" t="n">
+        <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A71)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A71)),IF(COUNTIF($E$2:$E$70,$A71)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A71)),IF(COUNTIF($F$2:$F$70,$A71)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A71)),IF(COUNTIF($G$2:$G$70,$A71)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A71)))</f>
+        <v>64.25</v>
+      </c>
+      <c r="S71" s="0" t="n">
+        <f aca="false">R71-O71</f>
+        <v>64.25</v>
+      </c>
+      <c r="T71" s="0" t="n">
+        <f aca="false">S71-P71</f>
         <v>8.25</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N68" s="0" t="s">
-        <v>147</v>
-      </c>
-      <c r="O68" s="0" t="n">
-        <f aca="false">MAX(Q2:Q65)</f>
-        <v>80.25</v>
+    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N73" s="0" t="s">
+        <v>157</v>
+      </c>
+      <c r="O73" s="0" t="n">
+        <f aca="false">MAX(Q2:Q70)</f>
+        <v>64.25</v>
       </c>
     </row>
   </sheetData>
@@ -3543,22 +3787,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="39.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="35.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="42.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="50.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="40.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Crash bookstore millwork by five days
</commit_message>
<xml_diff>
--- a/AC Tasks.xlsx
+++ b/AC Tasks.xlsx
@@ -824,15 +824,15 @@
       </c>
       <c r="R2" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A2)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A2)),IF(COUNTIF($E$2:$E$70,$A2)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A2)),IF(COUNTIF($F$2:$F$70,$A2)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A2)),IF(COUNTIF($G$2:$G$70,$A2)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A2)))</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="S2" s="0" t="n">
         <f aca="false">R2-O2</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="T2" s="0" t="n">
         <f aca="false">S2-P2</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -865,15 +865,15 @@
       </c>
       <c r="R3" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A3)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A3)),IF(COUNTIF($E$2:$E$70,$A3)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A3)),IF(COUNTIF($F$2:$F$70,$A3)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A3)),IF(COUNTIF($G$2:$G$70,$A3)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A3)))</f>
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="S3" s="0" t="n">
         <f aca="false">R3-O3</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="T3" s="0" t="n">
         <f aca="false">S3-P3</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -906,15 +906,15 @@
       </c>
       <c r="R4" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A4)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A4)),IF(COUNTIF($E$2:$E$70,$A4)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A4)),IF(COUNTIF($F$2:$F$70,$A4)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A4)),IF(COUNTIF($G$2:$G$70,$A4)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A4)))</f>
-        <v>15.5</v>
+        <v>15</v>
       </c>
       <c r="S4" s="0" t="n">
         <f aca="false">R4-O4</f>
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="T4" s="0" t="n">
         <f aca="false">S4-P4</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -947,15 +947,15 @@
       </c>
       <c r="R5" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A5)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A5)),IF(COUNTIF($E$2:$E$70,$A5)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A5)),IF(COUNTIF($F$2:$F$70,$A5)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A5)),IF(COUNTIF($G$2:$G$70,$A5)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A5)))</f>
-        <v>18.5</v>
+        <v>18</v>
       </c>
       <c r="S5" s="0" t="n">
         <f aca="false">R5-O5</f>
-        <v>15.5</v>
+        <v>15</v>
       </c>
       <c r="T5" s="0" t="n">
         <f aca="false">S5-P5</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -994,15 +994,15 @@
       </c>
       <c r="R6" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A6)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A6)),IF(COUNTIF($E$2:$E$70,$A6)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A6)),IF(COUNTIF($F$2:$F$70,$A6)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A6)),IF(COUNTIF($G$2:$G$70,$A6)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A6)))</f>
-        <v>26</v>
+        <v>25.5</v>
       </c>
       <c r="S6" s="0" t="n">
         <f aca="false">R6-O6</f>
-        <v>18.5</v>
+        <v>18</v>
       </c>
       <c r="T6" s="0" t="n">
         <f aca="false">S6-P6</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1038,15 +1038,15 @@
       </c>
       <c r="R7" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A7)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A7)),IF(COUNTIF($E$2:$E$70,$A7)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A7)),IF(COUNTIF($F$2:$F$70,$A7)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A7)),IF(COUNTIF($G$2:$G$70,$A7)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A7)))</f>
-        <v>36</v>
+        <v>35.5</v>
       </c>
       <c r="S7" s="0" t="n">
         <f aca="false">R7-O7</f>
-        <v>26</v>
+        <v>25.5</v>
       </c>
       <c r="T7" s="0" t="n">
         <f aca="false">S7-P7</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1079,15 +1079,15 @@
       </c>
       <c r="R8" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A8)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A8)),IF(COUNTIF($E$2:$E$70,$A8)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A8)),IF(COUNTIF($F$2:$F$70,$A8)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A8)),IF(COUNTIF($G$2:$G$70,$A8)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A8)))</f>
-        <v>36</v>
+        <v>35.5</v>
       </c>
       <c r="S8" s="0" t="n">
         <f aca="false">R8-O8</f>
-        <v>31</v>
+        <v>30.5</v>
       </c>
       <c r="T8" s="0" t="n">
         <f aca="false">S8-P8</f>
-        <v>5.5</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1123,15 +1123,15 @@
       </c>
       <c r="R9" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A9)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A9)),IF(COUNTIF($E$2:$E$70,$A9)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A9)),IF(COUNTIF($F$2:$F$70,$A9)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A9)),IF(COUNTIF($G$2:$G$70,$A9)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A9)))</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="S9" s="0" t="n">
         <f aca="false">R9-O9</f>
-        <v>36</v>
+        <v>35.5</v>
       </c>
       <c r="T9" s="0" t="n">
         <f aca="false">S9-P9</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1164,15 +1164,15 @@
       </c>
       <c r="R10" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A10)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A10)),IF(COUNTIF($E$2:$E$70,$A10)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A10)),IF(COUNTIF($F$2:$F$70,$A10)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A10)),IF(COUNTIF($G$2:$G$70,$A10)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A10)))</f>
-        <v>47</v>
+        <v>46.5</v>
       </c>
       <c r="S10" s="0" t="n">
         <f aca="false">R10-O10</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="T10" s="0" t="n">
         <f aca="false">S10-P10</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1202,15 +1202,15 @@
       </c>
       <c r="R11" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A11)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A11)),IF(COUNTIF($E$2:$E$70,$A11)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A11)),IF(COUNTIF($F$2:$F$70,$A11)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A11)),IF(COUNTIF($G$2:$G$70,$A11)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A11)))</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="S11" s="0" t="n">
         <f aca="false">R11-O11</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="T11" s="0" t="n">
         <f aca="false">S11-P11</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1246,15 +1246,15 @@
       </c>
       <c r="R12" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A12)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A12)),IF(COUNTIF($E$2:$E$70,$A12)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A12)),IF(COUNTIF($F$2:$F$70,$A12)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A12)),IF(COUNTIF($G$2:$G$70,$A12)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A12)))</f>
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="S12" s="0" t="n">
         <f aca="false">R12-O12</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="T12" s="0" t="n">
         <f aca="false">S12-P12</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1287,15 +1287,15 @@
       </c>
       <c r="R13" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A13)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A13)),IF(COUNTIF($E$2:$E$70,$A13)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A13)),IF(COUNTIF($F$2:$F$70,$A13)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A13)),IF(COUNTIF($G$2:$G$70,$A13)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A13)))</f>
-        <v>23</v>
+        <v>22.5</v>
       </c>
       <c r="S13" s="0" t="n">
         <f aca="false">R13-O13</f>
-        <v>13</v>
+        <v>12.5</v>
       </c>
       <c r="T13" s="0" t="n">
         <f aca="false">S13-P13</f>
-        <v>10</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1328,15 +1328,15 @@
       </c>
       <c r="R14" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A14)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A14)),IF(COUNTIF($E$2:$E$70,$A14)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A14)),IF(COUNTIF($F$2:$F$70,$A14)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A14)),IF(COUNTIF($G$2:$G$70,$A14)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A14)))</f>
-        <v>23</v>
+        <v>22.5</v>
       </c>
       <c r="S14" s="0" t="n">
         <f aca="false">R14-O14</f>
-        <v>18</v>
+        <v>17.5</v>
       </c>
       <c r="T14" s="0" t="n">
         <f aca="false">S14-P14</f>
-        <v>15</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1353,17 +1353,17 @@
         <v>45</v>
       </c>
       <c r="I15" s="0" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J15" s="0" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="M15" s="0" t="s">
         <v>32</v>
       </c>
       <c r="O15" s="0" t="n">
         <f aca="false">IF(H15&lt;&gt;"",H15,IF(AND(I15&lt;&gt;"",J15&lt;&gt;""),(I15+J15)/2,0))</f>
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="P15" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D15,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E15,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F15,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G15,$A$2:$A$70,0)),0))</f>
@@ -1371,19 +1371,19 @@
       </c>
       <c r="Q15" s="0" t="n">
         <f aca="false">P15+O15</f>
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="R15" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A15)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A15)),IF(COUNTIF($E$2:$E$70,$A15)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A15)),IF(COUNTIF($F$2:$F$70,$A15)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A15)),IF(COUNTIF($G$2:$G$70,$A15)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A15)))</f>
-        <v>21</v>
+        <v>20.5</v>
       </c>
       <c r="S15" s="0" t="n">
         <f aca="false">R15-O15</f>
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="T15" s="0" t="n">
         <f aca="false">S15-P15</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1408,23 +1408,23 @@
       </c>
       <c r="P16" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D16,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E16,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F16,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G16,$A$2:$A$70,0)),0))</f>
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="Q16" s="0" t="n">
         <f aca="false">P16+O16</f>
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="R16" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A16)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A16)),IF(COUNTIF($E$2:$E$70,$A16)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A16)),IF(COUNTIF($F$2:$F$70,$A16)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A16)),IF(COUNTIF($G$2:$G$70,$A16)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A16)))</f>
-        <v>26</v>
+        <v>25.5</v>
       </c>
       <c r="S16" s="0" t="n">
         <f aca="false">R16-O16</f>
-        <v>21</v>
+        <v>20.5</v>
       </c>
       <c r="T16" s="0" t="n">
         <f aca="false">S16-P16</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1449,23 +1449,23 @@
       </c>
       <c r="P17" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D17,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E17,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F17,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G17,$A$2:$A$70,0)),0))</f>
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="Q17" s="0" t="n">
         <f aca="false">P17+O17</f>
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="R17" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A17)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A17)),IF(COUNTIF($E$2:$E$70,$A17)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A17)),IF(COUNTIF($F$2:$F$70,$A17)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A17)),IF(COUNTIF($G$2:$G$70,$A17)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A17)))</f>
-        <v>36</v>
+        <v>35.5</v>
       </c>
       <c r="S17" s="0" t="n">
         <f aca="false">R17-O17</f>
-        <v>26</v>
+        <v>25.5</v>
       </c>
       <c r="T17" s="0" t="n">
         <f aca="false">S17-P17</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1501,15 +1501,15 @@
       </c>
       <c r="R18" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A18)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A18)),IF(COUNTIF($E$2:$E$70,$A18)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A18)),IF(COUNTIF($F$2:$F$70,$A18)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A18)),IF(COUNTIF($G$2:$G$70,$A18)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A18)))</f>
-        <v>26</v>
+        <v>25.5</v>
       </c>
       <c r="S18" s="0" t="n">
         <f aca="false">R18-O18</f>
-        <v>23</v>
+        <v>22.5</v>
       </c>
       <c r="T18" s="0" t="n">
         <f aca="false">S18-P18</f>
-        <v>10</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1542,15 +1542,15 @@
       </c>
       <c r="R19" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A19)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A19)),IF(COUNTIF($E$2:$E$70,$A19)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A19)),IF(COUNTIF($F$2:$F$70,$A19)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A19)),IF(COUNTIF($G$2:$G$70,$A19)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A19)))</f>
-        <v>36</v>
+        <v>35.5</v>
       </c>
       <c r="S19" s="0" t="n">
         <f aca="false">R19-O19</f>
-        <v>26</v>
+        <v>25.5</v>
       </c>
       <c r="T19" s="0" t="n">
         <f aca="false">S19-P19</f>
-        <v>10</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1575,23 +1575,23 @@
       </c>
       <c r="P20" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D20,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E20,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F20,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G20,$A$2:$A$70,0)),0))</f>
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="Q20" s="0" t="n">
         <f aca="false">P20+O20</f>
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="R20" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A20)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A20)),IF(COUNTIF($E$2:$E$70,$A20)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A20)),IF(COUNTIF($F$2:$F$70,$A20)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A20)),IF(COUNTIF($G$2:$G$70,$A20)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A20)))</f>
-        <v>47</v>
+        <v>46.5</v>
       </c>
       <c r="S20" s="0" t="n">
         <f aca="false">R20-O20</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="T20" s="0" t="n">
         <f aca="false">S20-P20</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1622,23 +1622,23 @@
       </c>
       <c r="P21" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D21,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E21,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F21,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G21,$A$2:$A$70,0)),0))</f>
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="Q21" s="0" t="n">
         <f aca="false">P21+O21</f>
-        <v>42.5</v>
+        <v>37.5</v>
       </c>
       <c r="R21" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A21)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A21)),IF(COUNTIF($E$2:$E$70,$A21)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A21)),IF(COUNTIF($F$2:$F$70,$A21)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A21)),IF(COUNTIF($G$2:$G$70,$A21)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A21)))</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="S21" s="0" t="n">
         <f aca="false">R21-O21</f>
-        <v>39.5</v>
+        <v>39</v>
       </c>
       <c r="T21" s="0" t="n">
         <f aca="false">S21-P21</f>
-        <v>3.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1666,23 +1666,23 @@
       </c>
       <c r="P22" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D22,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E22,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F22,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G22,$A$2:$A$70,0)),0))</f>
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="Q22" s="0" t="n">
         <f aca="false">P22+O22</f>
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="R22" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A22)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A22)),IF(COUNTIF($E$2:$E$70,$A22)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A22)),IF(COUNTIF($F$2:$F$70,$A22)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A22)),IF(COUNTIF($G$2:$G$70,$A22)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A22)))</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="S22" s="0" t="n">
         <f aca="false">R22-O22</f>
-        <v>36</v>
+        <v>35.5</v>
       </c>
       <c r="T22" s="0" t="n">
         <f aca="false">S22-P22</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1712,15 +1712,15 @@
       </c>
       <c r="R23" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A23)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A23)),IF(COUNTIF($E$2:$E$70,$A23)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A23)),IF(COUNTIF($F$2:$F$70,$A23)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A23)),IF(COUNTIF($G$2:$G$70,$A23)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A23)))</f>
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="S23" s="0" t="n">
         <f aca="false">R23-O23</f>
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="T23" s="0" t="n">
         <f aca="false">S23-P23</f>
-        <v>8.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1753,15 +1753,15 @@
       </c>
       <c r="R24" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A24)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A24)),IF(COUNTIF($E$2:$E$70,$A24)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A24)),IF(COUNTIF($F$2:$F$70,$A24)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A24)),IF(COUNTIF($G$2:$G$70,$A24)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A24)))</f>
-        <v>36</v>
+        <v>35.5</v>
       </c>
       <c r="S24" s="0" t="n">
         <f aca="false">R24-O24</f>
-        <v>20</v>
+        <v>19.5</v>
       </c>
       <c r="T24" s="0" t="n">
         <f aca="false">S24-P24</f>
-        <v>20</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1794,15 +1794,15 @@
       </c>
       <c r="R25" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A25)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A25)),IF(COUNTIF($E$2:$E$70,$A25)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A25)),IF(COUNTIF($F$2:$F$70,$A25)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A25)),IF(COUNTIF($G$2:$G$70,$A25)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A25)))</f>
-        <v>12</v>
+        <v>11.5</v>
       </c>
       <c r="S25" s="0" t="n">
         <f aca="false">R25-O25</f>
-        <v>11</v>
+        <v>10.5</v>
       </c>
       <c r="T25" s="0" t="n">
         <f aca="false">S25-P25</f>
-        <v>11</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1835,15 +1835,15 @@
       </c>
       <c r="R26" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A26)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A26)),IF(COUNTIF($E$2:$E$70,$A26)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A26)),IF(COUNTIF($F$2:$F$70,$A26)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A26)),IF(COUNTIF($G$2:$G$70,$A26)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A26)))</f>
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="S26" s="0" t="n">
         <f aca="false">R26-O26</f>
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="T26" s="0" t="n">
         <f aca="false">S26-P26</f>
-        <v>8.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1876,15 +1876,15 @@
       </c>
       <c r="R27" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A27)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A27)),IF(COUNTIF($E$2:$E$70,$A27)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A27)),IF(COUNTIF($F$2:$F$70,$A27)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A27)),IF(COUNTIF($G$2:$G$70,$A27)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A27)))</f>
-        <v>41</v>
+        <v>40.5</v>
       </c>
       <c r="S27" s="0" t="n">
         <f aca="false">R27-O27</f>
-        <v>38.5</v>
+        <v>38</v>
       </c>
       <c r="T27" s="0" t="n">
         <f aca="false">S27-P27</f>
-        <v>37.5</v>
+        <v>37</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1917,15 +1917,15 @@
       </c>
       <c r="R28" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A28)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A28)),IF(COUNTIF($E$2:$E$70,$A28)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A28)),IF(COUNTIF($F$2:$F$70,$A28)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A28)),IF(COUNTIF($G$2:$G$70,$A28)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A28)))</f>
-        <v>41</v>
+        <v>40.5</v>
       </c>
       <c r="S28" s="0" t="n">
         <f aca="false">R28-O28</f>
-        <v>38.5</v>
+        <v>38</v>
       </c>
       <c r="T28" s="0" t="n">
         <f aca="false">S28-P28</f>
-        <v>37.5</v>
+        <v>37</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1958,15 +1958,15 @@
       </c>
       <c r="R29" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A29)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A29)),IF(COUNTIF($E$2:$E$70,$A29)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A29)),IF(COUNTIF($F$2:$F$70,$A29)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A29)),IF(COUNTIF($G$2:$G$70,$A29)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A29)))</f>
-        <v>19.5</v>
+        <v>19</v>
       </c>
       <c r="S29" s="0" t="n">
         <f aca="false">R29-O29</f>
-        <v>12</v>
+        <v>11.5</v>
       </c>
       <c r="T29" s="0" t="n">
         <f aca="false">S29-P29</f>
-        <v>11</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1999,15 +1999,15 @@
       </c>
       <c r="R30" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A30)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A30)),IF(COUNTIF($E$2:$E$70,$A30)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A30)),IF(COUNTIF($F$2:$F$70,$A30)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A30)),IF(COUNTIF($G$2:$G$70,$A30)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A30)))</f>
-        <v>19.5</v>
+        <v>19</v>
       </c>
       <c r="S30" s="0" t="n">
         <f aca="false">R30-O30</f>
-        <v>12</v>
+        <v>11.5</v>
       </c>
       <c r="T30" s="0" t="n">
         <f aca="false">S30-P30</f>
-        <v>11</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2043,15 +2043,15 @@
       </c>
       <c r="R31" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A31)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A31)),IF(COUNTIF($E$2:$E$70,$A31)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A31)),IF(COUNTIF($F$2:$F$70,$A31)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A31)),IF(COUNTIF($G$2:$G$70,$A31)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A31)))</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="S31" s="0" t="n">
         <f aca="false">R31-O31</f>
-        <v>41</v>
+        <v>40.5</v>
       </c>
       <c r="T31" s="0" t="n">
         <f aca="false">S31-P31</f>
-        <v>37.5</v>
+        <v>37</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2084,15 +2084,15 @@
       </c>
       <c r="R32" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A32)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A32)),IF(COUNTIF($E$2:$E$70,$A32)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A32)),IF(COUNTIF($F$2:$F$70,$A32)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A32)),IF(COUNTIF($G$2:$G$70,$A32)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A32)))</f>
-        <v>54.25</v>
+        <v>53.75</v>
       </c>
       <c r="S32" s="0" t="n">
         <f aca="false">R32-O32</f>
-        <v>41.75</v>
+        <v>41.25</v>
       </c>
       <c r="T32" s="0" t="n">
         <f aca="false">S32-P32</f>
-        <v>33.25</v>
+        <v>32.75</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2125,15 +2125,15 @@
       </c>
       <c r="R33" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A33)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A33)),IF(COUNTIF($E$2:$E$70,$A33)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A33)),IF(COUNTIF($F$2:$F$70,$A33)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A33)),IF(COUNTIF($G$2:$G$70,$A33)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A33)))</f>
-        <v>36</v>
+        <v>35.5</v>
       </c>
       <c r="S33" s="0" t="n">
         <f aca="false">R33-O33</f>
-        <v>23.5</v>
+        <v>23</v>
       </c>
       <c r="T33" s="0" t="n">
         <f aca="false">S33-P33</f>
-        <v>15</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2175,15 +2175,15 @@
       </c>
       <c r="R34" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A34)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A34)),IF(COUNTIF($E$2:$E$70,$A34)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A34)),IF(COUNTIF($F$2:$F$70,$A34)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A34)),IF(COUNTIF($G$2:$G$70,$A34)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A34)))</f>
-        <v>39.5</v>
+        <v>39</v>
       </c>
       <c r="S34" s="0" t="n">
         <f aca="false">R34-O34</f>
-        <v>19.5</v>
+        <v>19</v>
       </c>
       <c r="T34" s="0" t="n">
         <f aca="false">S34-P34</f>
-        <v>8.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2216,15 +2216,15 @@
       </c>
       <c r="R35" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A35)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A35)),IF(COUNTIF($E$2:$E$70,$A35)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A35)),IF(COUNTIF($F$2:$F$70,$A35)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A35)),IF(COUNTIF($G$2:$G$70,$A35)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A35)))</f>
-        <v>19.5</v>
+        <v>19</v>
       </c>
       <c r="S35" s="0" t="n">
         <f aca="false">R35-O35</f>
-        <v>14.5</v>
+        <v>14</v>
       </c>
       <c r="T35" s="0" t="n">
         <f aca="false">S35-P35</f>
-        <v>8.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2260,15 +2260,15 @@
       </c>
       <c r="R36" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A36)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A36)),IF(COUNTIF($E$2:$E$70,$A36)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A36)),IF(COUNTIF($F$2:$F$70,$A36)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A36)),IF(COUNTIF($G$2:$G$70,$A36)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A36)))</f>
-        <v>64.25</v>
+        <v>63.75</v>
       </c>
       <c r="S36" s="0" t="n">
         <f aca="false">R36-O36</f>
-        <v>54.25</v>
+        <v>53.75</v>
       </c>
       <c r="T36" s="0" t="n">
         <f aca="false">S36-P36</f>
-        <v>33.25</v>
+        <v>32.75</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2304,15 +2304,15 @@
       </c>
       <c r="R37" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A37)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A37)),IF(COUNTIF($E$2:$E$70,$A37)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A37)),IF(COUNTIF($F$2:$F$70,$A37)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A37)),IF(COUNTIF($G$2:$G$70,$A37)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A37)))</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="S37" s="0" t="n">
         <f aca="false">R37-O37</f>
-        <v>36</v>
+        <v>35.5</v>
       </c>
       <c r="T37" s="0" t="n">
         <f aca="false">S37-P37</f>
-        <v>15</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2345,15 +2345,15 @@
       </c>
       <c r="R38" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A38)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A38)),IF(COUNTIF($E$2:$E$70,$A38)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A38)),IF(COUNTIF($F$2:$F$70,$A38)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A38)),IF(COUNTIF($G$2:$G$70,$A38)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A38)))</f>
-        <v>14.5</v>
+        <v>14</v>
       </c>
       <c r="S38" s="0" t="n">
         <f aca="false">R38-O38</f>
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="T38" s="0" t="n">
         <f aca="false">S38-P38</f>
-        <v>8.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2386,15 +2386,15 @@
       </c>
       <c r="R39" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A39)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A39)),IF(COUNTIF($E$2:$E$70,$A39)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A39)),IF(COUNTIF($F$2:$F$70,$A39)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A39)),IF(COUNTIF($G$2:$G$70,$A39)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A39)))</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="S39" s="0" t="n">
         <f aca="false">R39-O39</f>
-        <v>41</v>
+        <v>40.5</v>
       </c>
       <c r="T39" s="0" t="n">
         <f aca="false">S39-P39</f>
-        <v>35</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2433,15 +2433,15 @@
       </c>
       <c r="R40" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A40)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A40)),IF(COUNTIF($E$2:$E$70,$A40)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A40)),IF(COUNTIF($F$2:$F$70,$A40)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A40)),IF(COUNTIF($G$2:$G$70,$A40)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A40)))</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="S40" s="0" t="n">
         <f aca="false">R40-O40</f>
-        <v>39.5</v>
+        <v>39</v>
       </c>
       <c r="T40" s="0" t="n">
         <f aca="false">S40-P40</f>
-        <v>8.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2474,15 +2474,15 @@
       </c>
       <c r="R41" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A41)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A41)),IF(COUNTIF($E$2:$E$70,$A41)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A41)),IF(COUNTIF($F$2:$F$70,$A41)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A41)),IF(COUNTIF($G$2:$G$70,$A41)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A41)))</f>
-        <v>47</v>
+        <v>46.5</v>
       </c>
       <c r="S41" s="0" t="n">
         <f aca="false">R41-O41</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="T41" s="0" t="n">
         <f aca="false">S41-P41</f>
-        <v>8.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2512,15 +2512,15 @@
       </c>
       <c r="R42" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A42)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A42)),IF(COUNTIF($E$2:$E$70,$A42)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A42)),IF(COUNTIF($F$2:$F$70,$A42)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A42)),IF(COUNTIF($G$2:$G$70,$A42)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A42)))</f>
-        <v>7.5</v>
+        <v>7</v>
       </c>
       <c r="S42" s="0" t="n">
         <f aca="false">R42-O42</f>
-        <v>7.5</v>
+        <v>7</v>
       </c>
       <c r="T42" s="0" t="n">
         <f aca="false">S42-P42</f>
-        <v>7.5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2553,15 +2553,15 @@
       </c>
       <c r="R43" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A43)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A43)),IF(COUNTIF($E$2:$E$70,$A43)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A43)),IF(COUNTIF($F$2:$F$70,$A43)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A43)),IF(COUNTIF($G$2:$G$70,$A43)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A43)))</f>
-        <v>10.5</v>
+        <v>10</v>
       </c>
       <c r="S43" s="0" t="n">
         <f aca="false">R43-O43</f>
-        <v>7.5</v>
+        <v>7</v>
       </c>
       <c r="T43" s="0" t="n">
         <f aca="false">S43-P43</f>
-        <v>7.5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2594,15 +2594,15 @@
       </c>
       <c r="R44" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A44)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A44)),IF(COUNTIF($E$2:$E$70,$A44)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A44)),IF(COUNTIF($F$2:$F$70,$A44)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A44)),IF(COUNTIF($G$2:$G$70,$A44)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A44)))</f>
-        <v>26</v>
+        <v>25.5</v>
       </c>
       <c r="S44" s="0" t="n">
         <f aca="false">R44-O44</f>
-        <v>16</v>
+        <v>15.5</v>
       </c>
       <c r="T44" s="0" t="n">
         <f aca="false">S44-P44</f>
-        <v>16</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2635,15 +2635,15 @@
       </c>
       <c r="R45" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A45)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A45)),IF(COUNTIF($E$2:$E$70,$A45)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A45)),IF(COUNTIF($F$2:$F$70,$A45)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A45)),IF(COUNTIF($G$2:$G$70,$A45)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A45)))</f>
-        <v>26</v>
+        <v>25.5</v>
       </c>
       <c r="S45" s="0" t="n">
         <f aca="false">R45-O45</f>
-        <v>11</v>
+        <v>10.5</v>
       </c>
       <c r="T45" s="0" t="n">
         <f aca="false">S45-P45</f>
-        <v>11</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2676,15 +2676,15 @@
       </c>
       <c r="R46" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A46)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A46)),IF(COUNTIF($E$2:$E$70,$A46)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A46)),IF(COUNTIF($F$2:$F$70,$A46)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A46)),IF(COUNTIF($G$2:$G$70,$A46)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A46)))</f>
-        <v>26</v>
+        <v>25.5</v>
       </c>
       <c r="S46" s="0" t="n">
         <f aca="false">R46-O46</f>
-        <v>11</v>
+        <v>10.5</v>
       </c>
       <c r="T46" s="0" t="n">
         <f aca="false">S46-P46</f>
-        <v>11</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2723,15 +2723,15 @@
       </c>
       <c r="R47" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A47)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A47)),IF(COUNTIF($E$2:$E$70,$A47)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A47)),IF(COUNTIF($F$2:$F$70,$A47)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A47)),IF(COUNTIF($G$2:$G$70,$A47)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A47)))</f>
-        <v>31</v>
+        <v>30.5</v>
       </c>
       <c r="S47" s="0" t="n">
         <f aca="false">R47-O47</f>
-        <v>26</v>
+        <v>25.5</v>
       </c>
       <c r="T47" s="0" t="n">
         <f aca="false">S47-P47</f>
-        <v>11</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2767,15 +2767,15 @@
       </c>
       <c r="R48" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A48)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A48)),IF(COUNTIF($E$2:$E$70,$A48)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A48)),IF(COUNTIF($F$2:$F$70,$A48)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A48)),IF(COUNTIF($G$2:$G$70,$A48)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A48)))</f>
-        <v>17</v>
+        <v>16.5</v>
       </c>
       <c r="S48" s="0" t="n">
         <f aca="false">R48-O48</f>
-        <v>10.5</v>
+        <v>10</v>
       </c>
       <c r="T48" s="0" t="n">
         <f aca="false">S48-P48</f>
-        <v>7.5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2808,15 +2808,15 @@
       </c>
       <c r="R49" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A49)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A49)),IF(COUNTIF($E$2:$E$70,$A49)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A49)),IF(COUNTIF($F$2:$F$70,$A49)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A49)),IF(COUNTIF($G$2:$G$70,$A49)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A49)))</f>
-        <v>64.25</v>
+        <v>63.75</v>
       </c>
       <c r="S49" s="0" t="n">
         <f aca="false">R49-O49</f>
-        <v>59.25</v>
+        <v>58.75</v>
       </c>
       <c r="T49" s="0" t="n">
         <f aca="false">S49-P49</f>
-        <v>44.25</v>
+        <v>43.75</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2855,15 +2855,15 @@
       </c>
       <c r="R50" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A50)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A50)),IF(COUNTIF($E$2:$E$70,$A50)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A50)),IF(COUNTIF($F$2:$F$70,$A50)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A50)),IF(COUNTIF($G$2:$G$70,$A50)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A50)))</f>
-        <v>41</v>
+        <v>40.5</v>
       </c>
       <c r="S50" s="0" t="n">
         <f aca="false">R50-O50</f>
-        <v>17</v>
+        <v>16.5</v>
       </c>
       <c r="T50" s="0" t="n">
         <f aca="false">S50-P50</f>
-        <v>7.5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2896,15 +2896,15 @@
       </c>
       <c r="R51" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A51)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A51)),IF(COUNTIF($E$2:$E$70,$A51)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A51)),IF(COUNTIF($F$2:$F$70,$A51)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A51)),IF(COUNTIF($G$2:$G$70,$A51)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A51)))</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="S51" s="0" t="n">
         <f aca="false">R51-O51</f>
-        <v>41</v>
+        <v>40.5</v>
       </c>
       <c r="T51" s="0" t="n">
         <f aca="false">S51-P51</f>
-        <v>7.5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2940,15 +2940,15 @@
       </c>
       <c r="R52" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A52)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A52)),IF(COUNTIF($E$2:$E$70,$A52)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A52)),IF(COUNTIF($F$2:$F$70,$A52)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A52)),IF(COUNTIF($G$2:$G$70,$A52)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A52)))</f>
-        <v>36</v>
+        <v>35.5</v>
       </c>
       <c r="S52" s="0" t="n">
         <f aca="false">R52-O52</f>
-        <v>27</v>
+        <v>26.5</v>
       </c>
       <c r="T52" s="0" t="n">
         <f aca="false">S52-P52</f>
-        <v>12</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2984,15 +2984,15 @@
       </c>
       <c r="R53" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A53)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A53)),IF(COUNTIF($E$2:$E$70,$A53)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A53)),IF(COUNTIF($F$2:$F$70,$A53)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A53)),IF(COUNTIF($G$2:$G$70,$A53)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A53)))</f>
-        <v>64.25</v>
+        <v>63.75</v>
       </c>
       <c r="S53" s="0" t="n">
         <f aca="false">R53-O53</f>
-        <v>61.25</v>
+        <v>60.75</v>
       </c>
       <c r="T53" s="0" t="n">
         <f aca="false">S53-P53</f>
-        <v>46.25</v>
+        <v>45.75</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3025,15 +3025,15 @@
       </c>
       <c r="R54" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A54)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A54)),IF(COUNTIF($E$2:$E$70,$A54)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A54)),IF(COUNTIF($F$2:$F$70,$A54)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A54)),IF(COUNTIF($G$2:$G$70,$A54)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A54)))</f>
-        <v>36</v>
+        <v>35.5</v>
       </c>
       <c r="S54" s="0" t="n">
         <f aca="false">R54-O54</f>
-        <v>31</v>
+        <v>30.5</v>
       </c>
       <c r="T54" s="0" t="n">
         <f aca="false">S54-P54</f>
-        <v>11</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3069,15 +3069,15 @@
       </c>
       <c r="R55" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A55)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A55)),IF(COUNTIF($E$2:$E$70,$A55)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A55)),IF(COUNTIF($F$2:$F$70,$A55)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A55)),IF(COUNTIF($G$2:$G$70,$A55)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A55)))</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="S55" s="0" t="n">
         <f aca="false">R55-O55</f>
-        <v>36</v>
+        <v>35.5</v>
       </c>
       <c r="T55" s="0" t="n">
         <f aca="false">S55-P55</f>
-        <v>11</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3113,15 +3113,15 @@
       </c>
       <c r="R56" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A56)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A56)),IF(COUNTIF($E$2:$E$70,$A56)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A56)),IF(COUNTIF($F$2:$F$70,$A56)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A56)),IF(COUNTIF($G$2:$G$70,$A56)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A56)))</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="S56" s="0" t="n">
         <f aca="false">R56-O56</f>
-        <v>36</v>
+        <v>35.5</v>
       </c>
       <c r="T56" s="0" t="n">
         <f aca="false">S56-P56</f>
-        <v>11</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3154,15 +3154,15 @@
       </c>
       <c r="R57" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A57)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A57)),IF(COUNTIF($E$2:$E$70,$A57)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A57)),IF(COUNTIF($F$2:$F$70,$A57)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A57)),IF(COUNTIF($G$2:$G$70,$A57)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A57)))</f>
-        <v>47</v>
+        <v>46.5</v>
       </c>
       <c r="S57" s="0" t="n">
         <f aca="false">R57-O57</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="T57" s="0" t="n">
         <f aca="false">S57-P57</f>
-        <v>7.5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3228,19 +3228,19 @@
       </c>
       <c r="P59" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D59,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E59,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F59,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G59,$A$2:$A$70,0)),0))</f>
-        <v>56</v>
+        <v>55.5</v>
       </c>
       <c r="Q59" s="0" t="n">
         <f aca="false">P59+O59</f>
-        <v>63.5</v>
+        <v>63</v>
       </c>
       <c r="R59" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A59)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A59)),IF(COUNTIF($E$2:$E$70,$A59)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A59)),IF(COUNTIF($F$2:$F$70,$A59)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A59)),IF(COUNTIF($G$2:$G$70,$A59)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A59)))</f>
-        <v>63.5</v>
+        <v>63</v>
       </c>
       <c r="S59" s="0" t="n">
         <f aca="false">R59-O59</f>
-        <v>56</v>
+        <v>55.5</v>
       </c>
       <c r="T59" s="0" t="n">
         <f aca="false">S59-P59</f>
@@ -3274,15 +3274,15 @@
       </c>
       <c r="R60" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A60)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A60)),IF(COUNTIF($E$2:$E$70,$A60)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A60)),IF(COUNTIF($F$2:$F$70,$A60)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A60)),IF(COUNTIF($G$2:$G$70,$A60)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A60)))</f>
-        <v>30</v>
+        <v>29.5</v>
       </c>
       <c r="S60" s="0" t="n">
         <f aca="false">R60-O60</f>
-        <v>30</v>
+        <v>29.5</v>
       </c>
       <c r="T60" s="0" t="n">
         <f aca="false">S60-P60</f>
-        <v>30</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3318,15 +3318,15 @@
       </c>
       <c r="R61" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A61)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A61)),IF(COUNTIF($E$2:$E$70,$A61)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A61)),IF(COUNTIF($F$2:$F$70,$A61)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A61)),IF(COUNTIF($G$2:$G$70,$A61)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A61)))</f>
-        <v>51</v>
+        <v>50.5</v>
       </c>
       <c r="S61" s="0" t="n">
         <f aca="false">R61-O61</f>
-        <v>30</v>
+        <v>29.5</v>
       </c>
       <c r="T61" s="0" t="n">
         <f aca="false">S61-P61</f>
-        <v>30</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3354,19 +3354,19 @@
       </c>
       <c r="P62" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D62,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E62,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F62,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G62,$A$2:$A$70,0)),0))</f>
-        <v>51</v>
+        <v>50.5</v>
       </c>
       <c r="Q62" s="0" t="n">
         <f aca="false">P62+O62</f>
-        <v>56</v>
+        <v>55.5</v>
       </c>
       <c r="R62" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A62)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A62)),IF(COUNTIF($E$2:$E$70,$A62)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A62)),IF(COUNTIF($F$2:$F$70,$A62)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A62)),IF(COUNTIF($G$2:$G$70,$A62)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A62)))</f>
-        <v>56</v>
+        <v>55.5</v>
       </c>
       <c r="S62" s="0" t="n">
         <f aca="false">R62-O62</f>
-        <v>51</v>
+        <v>50.5</v>
       </c>
       <c r="T62" s="0" t="n">
         <f aca="false">S62-P62</f>
@@ -3398,19 +3398,19 @@
       </c>
       <c r="P63" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D63,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E63,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F63,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G63,$A$2:$A$70,0)),0))</f>
-        <v>63.5</v>
+        <v>63</v>
       </c>
       <c r="Q63" s="0" t="n">
         <f aca="false">P63+O63</f>
-        <v>64.25</v>
+        <v>63.75</v>
       </c>
       <c r="R63" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A63)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A63)),IF(COUNTIF($E$2:$E$70,$A63)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A63)),IF(COUNTIF($F$2:$F$70,$A63)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A63)),IF(COUNTIF($G$2:$G$70,$A63)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A63)))</f>
-        <v>64.25</v>
+        <v>63.75</v>
       </c>
       <c r="S63" s="0" t="n">
         <f aca="false">R63-O63</f>
-        <v>63.5</v>
+        <v>63</v>
       </c>
       <c r="T63" s="0" t="n">
         <f aca="false">S63-P63</f>
@@ -3436,19 +3436,19 @@
       </c>
       <c r="P64" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D64,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E64,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F64,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G64,$A$2:$A$70,0)),0))</f>
-        <v>63.5</v>
+        <v>63</v>
       </c>
       <c r="Q64" s="0" t="n">
         <f aca="false">P64+O64</f>
-        <v>63.5</v>
+        <v>63</v>
       </c>
       <c r="R64" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A64)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A64)),IF(COUNTIF($E$2:$E$70,$A64)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A64)),IF(COUNTIF($F$2:$F$70,$A64)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A64)),IF(COUNTIF($G$2:$G$70,$A64)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A64)))</f>
-        <v>64.25</v>
+        <v>63.75</v>
       </c>
       <c r="S64" s="0" t="n">
         <f aca="false">R64-O64</f>
-        <v>64.25</v>
+        <v>63.75</v>
       </c>
       <c r="T64" s="0" t="n">
         <f aca="false">S64-P64</f>
@@ -3477,19 +3477,19 @@
       </c>
       <c r="P65" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D65,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E65,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F65,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G65,$A$2:$A$70,0)),0))</f>
-        <v>47</v>
+        <v>46.5</v>
       </c>
       <c r="Q65" s="0" t="n">
         <f aca="false">P65+O65</f>
-        <v>51</v>
+        <v>50.5</v>
       </c>
       <c r="R65" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A65)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A65)),IF(COUNTIF($E$2:$E$70,$A65)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A65)),IF(COUNTIF($F$2:$F$70,$A65)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A65)),IF(COUNTIF($G$2:$G$70,$A65)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A65)))</f>
-        <v>51</v>
+        <v>50.5</v>
       </c>
       <c r="S65" s="0" t="n">
         <f aca="false">R65-O65</f>
-        <v>47</v>
+        <v>46.5</v>
       </c>
       <c r="T65" s="0" t="n">
         <f aca="false">S65-P65</f>
@@ -3529,15 +3529,15 @@
       </c>
       <c r="R66" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A66)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A66)),IF(COUNTIF($E$2:$E$70,$A66)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A66)),IF(COUNTIF($F$2:$F$70,$A66)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A66)),IF(COUNTIF($G$2:$G$70,$A66)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A66)))</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="S66" s="0" t="n">
         <f aca="false">R66-O66</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="T66" s="0" t="n">
         <f aca="false">S66-P66</f>
-        <v>7.5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3576,15 +3576,15 @@
       </c>
       <c r="R67" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A67)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A67)),IF(COUNTIF($E$2:$E$70,$A67)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A67)),IF(COUNTIF($F$2:$F$70,$A67)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A67)),IF(COUNTIF($G$2:$G$70,$A67)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A67)))</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="S67" s="0" t="n">
         <f aca="false">R67-O67</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="T67" s="0" t="n">
         <f aca="false">S67-P67</f>
-        <v>8.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3614,15 +3614,15 @@
       </c>
       <c r="R68" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A68)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A68)),IF(COUNTIF($E$2:$E$70,$A68)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A68)),IF(COUNTIF($F$2:$F$70,$A68)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A68)),IF(COUNTIF($G$2:$G$70,$A68)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A68)))</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="S68" s="0" t="n">
         <f aca="false">R68-O68</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="T68" s="0" t="n">
         <f aca="false">S68-P68</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3647,23 +3647,23 @@
       </c>
       <c r="P69" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D69,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E69,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F69,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G69,$A$2:$A$70,0)),0))</f>
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="Q69" s="0" t="n">
         <f aca="false">P69+O69</f>
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="R69" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A69)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A69)),IF(COUNTIF($E$2:$E$70,$A69)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A69)),IF(COUNTIF($F$2:$F$70,$A69)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A69)),IF(COUNTIF($G$2:$G$70,$A69)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A69)))</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="S69" s="0" t="n">
         <f aca="false">R69-O69</f>
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="T69" s="0" t="n">
         <f aca="false">S69-P69</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3694,19 +3694,19 @@
       </c>
       <c r="P70" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D70,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E70,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F70,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G70,$A$2:$A$70,0)),0))</f>
-        <v>47</v>
+        <v>46.5</v>
       </c>
       <c r="Q70" s="0" t="n">
         <f aca="false">P70+O70</f>
-        <v>47</v>
+        <v>46.5</v>
       </c>
       <c r="R70" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A70)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A70)),IF(COUNTIF($E$2:$E$70,$A70)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A70)),IF(COUNTIF($F$2:$F$70,$A70)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A70)),IF(COUNTIF($G$2:$G$70,$A70)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A70)))</f>
-        <v>47</v>
+        <v>46.5</v>
       </c>
       <c r="S70" s="0" t="n">
         <f aca="false">R70-O70</f>
-        <v>47</v>
+        <v>46.5</v>
       </c>
       <c r="T70" s="0" t="n">
         <f aca="false">S70-P70</f>
@@ -3735,19 +3735,19 @@
       </c>
       <c r="P71" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D71,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E71,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F71,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G71,$A$2:$A$70,0)),0))</f>
-        <v>56</v>
+        <v>55.5</v>
       </c>
       <c r="Q71" s="0" t="n">
         <f aca="false">P71+O71</f>
-        <v>56</v>
+        <v>55.5</v>
       </c>
       <c r="R71" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A71)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A71)),IF(COUNTIF($E$2:$E$70,$A71)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A71)),IF(COUNTIF($F$2:$F$70,$A71)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A71)),IF(COUNTIF($G$2:$G$70,$A71)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A71)))</f>
-        <v>64.25</v>
+        <v>63.75</v>
       </c>
       <c r="S71" s="0" t="n">
         <f aca="false">R71-O71</f>
-        <v>64.25</v>
+        <v>63.75</v>
       </c>
       <c r="T71" s="0" t="n">
         <f aca="false">S71-P71</f>
@@ -3760,7 +3760,7 @@
       </c>
       <c r="O73" s="0" t="n">
         <f aca="false">MAX(Q2:Q70)</f>
-        <v>64.25</v>
+        <v>63.75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Crash terrace waterproofing by two days
</commit_message>
<xml_diff>
--- a/AC Tasks.xlsx
+++ b/AC Tasks.xlsx
@@ -890,11 +890,11 @@
         <v>24</v>
       </c>
       <c r="H4" s="0" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O4" s="0" t="n">
         <f aca="false">IF(H4&lt;&gt;"",H4,IF(AND(I4&lt;&gt;"",J4&lt;&gt;""),(I4+J4)/2,0))</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="P4" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D4,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E4,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F4,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G4,$A$2:$A$70,0)),0))</f>
@@ -902,11 +902,11 @@
       </c>
       <c r="Q4" s="0" t="n">
         <f aca="false">P4+O4</f>
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="R4" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A4)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A4)),IF(COUNTIF($E$2:$E$70,$A4)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A4)),IF(COUNTIF($F$2:$F$70,$A4)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A4)),IF(COUNTIF($G$2:$G$70,$A4)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A4)))</f>
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="S4" s="0" t="n">
         <f aca="false">R4-O4</f>
@@ -939,19 +939,19 @@
       </c>
       <c r="P5" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D5,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E5,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F5,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G5,$A$2:$A$70,0)),0))</f>
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="Q5" s="0" t="n">
         <f aca="false">P5+O5</f>
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="R5" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A5)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A5)),IF(COUNTIF($E$2:$E$70,$A5)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A5)),IF(COUNTIF($F$2:$F$70,$A5)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A5)),IF(COUNTIF($G$2:$G$70,$A5)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A5)))</f>
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="S5" s="0" t="n">
         <f aca="false">R5-O5</f>
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="T5" s="0" t="n">
         <f aca="false">S5-P5</f>
@@ -986,19 +986,19 @@
       </c>
       <c r="P6" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D6,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E6,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F6,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G6,$A$2:$A$70,0)),0))</f>
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="Q6" s="0" t="n">
         <f aca="false">P6+O6</f>
-        <v>25.5</v>
+        <v>23.5</v>
       </c>
       <c r="R6" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A6)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A6)),IF(COUNTIF($E$2:$E$70,$A6)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A6)),IF(COUNTIF($F$2:$F$70,$A6)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A6)),IF(COUNTIF($G$2:$G$70,$A6)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A6)))</f>
-        <v>25.5</v>
+        <v>23.5</v>
       </c>
       <c r="S6" s="0" t="n">
         <f aca="false">R6-O6</f>
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="T6" s="0" t="n">
         <f aca="false">S6-P6</f>
@@ -1030,19 +1030,19 @@
       </c>
       <c r="P7" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D7,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E7,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F7,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G7,$A$2:$A$70,0)),0))</f>
-        <v>25.5</v>
+        <v>23.5</v>
       </c>
       <c r="Q7" s="0" t="n">
         <f aca="false">P7+O7</f>
-        <v>35.5</v>
+        <v>33.5</v>
       </c>
       <c r="R7" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A7)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A7)),IF(COUNTIF($E$2:$E$70,$A7)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A7)),IF(COUNTIF($F$2:$F$70,$A7)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A7)),IF(COUNTIF($G$2:$G$70,$A7)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A7)))</f>
-        <v>35.5</v>
+        <v>33.5</v>
       </c>
       <c r="S7" s="0" t="n">
         <f aca="false">R7-O7</f>
-        <v>25.5</v>
+        <v>23.5</v>
       </c>
       <c r="T7" s="0" t="n">
         <f aca="false">S7-P7</f>
@@ -1071,19 +1071,19 @@
       </c>
       <c r="P8" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D8,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E8,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F8,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G8,$A$2:$A$70,0)),0))</f>
-        <v>25.5</v>
+        <v>23.5</v>
       </c>
       <c r="Q8" s="0" t="n">
         <f aca="false">P8+O8</f>
-        <v>30.5</v>
+        <v>28.5</v>
       </c>
       <c r="R8" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A8)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A8)),IF(COUNTIF($E$2:$E$70,$A8)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A8)),IF(COUNTIF($F$2:$F$70,$A8)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A8)),IF(COUNTIF($G$2:$G$70,$A8)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A8)))</f>
-        <v>35.5</v>
+        <v>33.5</v>
       </c>
       <c r="S8" s="0" t="n">
         <f aca="false">R8-O8</f>
-        <v>30.5</v>
+        <v>28.5</v>
       </c>
       <c r="T8" s="0" t="n">
         <f aca="false">S8-P8</f>
@@ -1115,19 +1115,19 @@
       </c>
       <c r="P9" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D9,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E9,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F9,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G9,$A$2:$A$70,0)),0))</f>
-        <v>35.5</v>
+        <v>33.5</v>
       </c>
       <c r="Q9" s="0" t="n">
         <f aca="false">P9+O9</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="R9" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A9)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A9)),IF(COUNTIF($E$2:$E$70,$A9)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A9)),IF(COUNTIF($F$2:$F$70,$A9)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A9)),IF(COUNTIF($G$2:$G$70,$A9)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A9)))</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="S9" s="0" t="n">
         <f aca="false">R9-O9</f>
-        <v>35.5</v>
+        <v>33.5</v>
       </c>
       <c r="T9" s="0" t="n">
         <f aca="false">S9-P9</f>
@@ -1156,19 +1156,19 @@
       </c>
       <c r="P10" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D10,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E10,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F10,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G10,$A$2:$A$70,0)),0))</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="Q10" s="0" t="n">
         <f aca="false">P10+O10</f>
-        <v>46.5</v>
+        <v>44.5</v>
       </c>
       <c r="R10" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A10)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A10)),IF(COUNTIF($E$2:$E$70,$A10)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A10)),IF(COUNTIF($F$2:$F$70,$A10)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A10)),IF(COUNTIF($G$2:$G$70,$A10)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A10)))</f>
-        <v>46.5</v>
+        <v>44.5</v>
       </c>
       <c r="S10" s="0" t="n">
         <f aca="false">R10-O10</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="T10" s="0" t="n">
         <f aca="false">S10-P10</f>
@@ -1202,15 +1202,15 @@
       </c>
       <c r="R11" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A11)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A11)),IF(COUNTIF($E$2:$E$70,$A11)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A11)),IF(COUNTIF($F$2:$F$70,$A11)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A11)),IF(COUNTIF($G$2:$G$70,$A11)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A11)))</f>
-        <v>4.5</v>
+        <v>2.5</v>
       </c>
       <c r="S11" s="0" t="n">
         <f aca="false">R11-O11</f>
-        <v>4.5</v>
+        <v>2.5</v>
       </c>
       <c r="T11" s="0" t="n">
         <f aca="false">S11-P11</f>
-        <v>4.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1246,15 +1246,15 @@
       </c>
       <c r="R12" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A12)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A12)),IF(COUNTIF($E$2:$E$70,$A12)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A12)),IF(COUNTIF($F$2:$F$70,$A12)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A12)),IF(COUNTIF($G$2:$G$70,$A12)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A12)))</f>
-        <v>7.5</v>
+        <v>5.5</v>
       </c>
       <c r="S12" s="0" t="n">
         <f aca="false">R12-O12</f>
-        <v>4.5</v>
+        <v>2.5</v>
       </c>
       <c r="T12" s="0" t="n">
         <f aca="false">S12-P12</f>
-        <v>4.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1287,15 +1287,15 @@
       </c>
       <c r="R13" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A13)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A13)),IF(COUNTIF($E$2:$E$70,$A13)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A13)),IF(COUNTIF($F$2:$F$70,$A13)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A13)),IF(COUNTIF($G$2:$G$70,$A13)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A13)))</f>
-        <v>22.5</v>
+        <v>20.5</v>
       </c>
       <c r="S13" s="0" t="n">
         <f aca="false">R13-O13</f>
-        <v>12.5</v>
+        <v>10.5</v>
       </c>
       <c r="T13" s="0" t="n">
         <f aca="false">S13-P13</f>
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1328,15 +1328,15 @@
       </c>
       <c r="R14" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A14)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A14)),IF(COUNTIF($E$2:$E$70,$A14)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A14)),IF(COUNTIF($F$2:$F$70,$A14)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A14)),IF(COUNTIF($G$2:$G$70,$A14)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A14)))</f>
-        <v>22.5</v>
+        <v>20.5</v>
       </c>
       <c r="S14" s="0" t="n">
         <f aca="false">R14-O14</f>
-        <v>17.5</v>
+        <v>15.5</v>
       </c>
       <c r="T14" s="0" t="n">
         <f aca="false">S14-P14</f>
-        <v>14.5</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1375,15 +1375,15 @@
       </c>
       <c r="R15" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A15)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A15)),IF(COUNTIF($E$2:$E$70,$A15)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A15)),IF(COUNTIF($F$2:$F$70,$A15)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A15)),IF(COUNTIF($G$2:$G$70,$A15)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A15)))</f>
-        <v>20.5</v>
+        <v>18.5</v>
       </c>
       <c r="S15" s="0" t="n">
         <f aca="false">R15-O15</f>
-        <v>7.5</v>
+        <v>5.5</v>
       </c>
       <c r="T15" s="0" t="n">
         <f aca="false">S15-P15</f>
-        <v>4.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1416,15 +1416,15 @@
       </c>
       <c r="R16" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A16)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A16)),IF(COUNTIF($E$2:$E$70,$A16)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A16)),IF(COUNTIF($F$2:$F$70,$A16)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A16)),IF(COUNTIF($G$2:$G$70,$A16)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A16)))</f>
-        <v>25.5</v>
+        <v>23.5</v>
       </c>
       <c r="S16" s="0" t="n">
         <f aca="false">R16-O16</f>
-        <v>20.5</v>
+        <v>18.5</v>
       </c>
       <c r="T16" s="0" t="n">
         <f aca="false">S16-P16</f>
-        <v>4.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1457,15 +1457,15 @@
       </c>
       <c r="R17" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A17)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A17)),IF(COUNTIF($E$2:$E$70,$A17)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A17)),IF(COUNTIF($F$2:$F$70,$A17)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A17)),IF(COUNTIF($G$2:$G$70,$A17)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A17)))</f>
-        <v>35.5</v>
+        <v>33.5</v>
       </c>
       <c r="S17" s="0" t="n">
         <f aca="false">R17-O17</f>
-        <v>25.5</v>
+        <v>23.5</v>
       </c>
       <c r="T17" s="0" t="n">
         <f aca="false">S17-P17</f>
-        <v>4.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1501,15 +1501,15 @@
       </c>
       <c r="R18" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A18)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A18)),IF(COUNTIF($E$2:$E$70,$A18)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A18)),IF(COUNTIF($F$2:$F$70,$A18)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A18)),IF(COUNTIF($G$2:$G$70,$A18)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A18)))</f>
-        <v>25.5</v>
+        <v>23.5</v>
       </c>
       <c r="S18" s="0" t="n">
         <f aca="false">R18-O18</f>
-        <v>22.5</v>
+        <v>20.5</v>
       </c>
       <c r="T18" s="0" t="n">
         <f aca="false">S18-P18</f>
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1542,15 +1542,15 @@
       </c>
       <c r="R19" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A19)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A19)),IF(COUNTIF($E$2:$E$70,$A19)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A19)),IF(COUNTIF($F$2:$F$70,$A19)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A19)),IF(COUNTIF($G$2:$G$70,$A19)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A19)))</f>
-        <v>35.5</v>
+        <v>33.5</v>
       </c>
       <c r="S19" s="0" t="n">
         <f aca="false">R19-O19</f>
-        <v>25.5</v>
+        <v>23.5</v>
       </c>
       <c r="T19" s="0" t="n">
         <f aca="false">S19-P19</f>
-        <v>9.5</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1583,15 +1583,15 @@
       </c>
       <c r="R20" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A20)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A20)),IF(COUNTIF($E$2:$E$70,$A20)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A20)),IF(COUNTIF($F$2:$F$70,$A20)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A20)),IF(COUNTIF($G$2:$G$70,$A20)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A20)))</f>
-        <v>46.5</v>
+        <v>44.5</v>
       </c>
       <c r="S20" s="0" t="n">
         <f aca="false">R20-O20</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="T20" s="0" t="n">
         <f aca="false">S20-P20</f>
-        <v>4.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1630,15 +1630,15 @@
       </c>
       <c r="R21" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A21)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A21)),IF(COUNTIF($E$2:$E$70,$A21)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A21)),IF(COUNTIF($F$2:$F$70,$A21)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A21)),IF(COUNTIF($G$2:$G$70,$A21)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A21)))</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="S21" s="0" t="n">
         <f aca="false">R21-O21</f>
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="T21" s="0" t="n">
         <f aca="false">S21-P21</f>
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1674,15 +1674,15 @@
       </c>
       <c r="R22" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A22)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A22)),IF(COUNTIF($E$2:$E$70,$A22)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A22)),IF(COUNTIF($F$2:$F$70,$A22)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A22)),IF(COUNTIF($G$2:$G$70,$A22)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A22)))</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="S22" s="0" t="n">
         <f aca="false">R22-O22</f>
-        <v>35.5</v>
+        <v>33.5</v>
       </c>
       <c r="T22" s="0" t="n">
         <f aca="false">S22-P22</f>
-        <v>4.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1712,15 +1712,15 @@
       </c>
       <c r="R23" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A23)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A23)),IF(COUNTIF($E$2:$E$70,$A23)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A23)),IF(COUNTIF($F$2:$F$70,$A23)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A23)),IF(COUNTIF($G$2:$G$70,$A23)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A23)))</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="S23" s="0" t="n">
         <f aca="false">R23-O23</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="T23" s="0" t="n">
         <f aca="false">S23-P23</f>
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1753,15 +1753,15 @@
       </c>
       <c r="R24" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A24)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A24)),IF(COUNTIF($E$2:$E$70,$A24)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A24)),IF(COUNTIF($F$2:$F$70,$A24)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A24)),IF(COUNTIF($G$2:$G$70,$A24)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A24)))</f>
-        <v>35.5</v>
+        <v>33.5</v>
       </c>
       <c r="S24" s="0" t="n">
         <f aca="false">R24-O24</f>
-        <v>19.5</v>
+        <v>17.5</v>
       </c>
       <c r="T24" s="0" t="n">
         <f aca="false">S24-P24</f>
-        <v>19.5</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1794,15 +1794,15 @@
       </c>
       <c r="R25" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A25)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A25)),IF(COUNTIF($E$2:$E$70,$A25)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A25)),IF(COUNTIF($F$2:$F$70,$A25)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A25)),IF(COUNTIF($G$2:$G$70,$A25)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A25)))</f>
-        <v>11.5</v>
+        <v>9.5</v>
       </c>
       <c r="S25" s="0" t="n">
         <f aca="false">R25-O25</f>
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
       <c r="T25" s="0" t="n">
         <f aca="false">S25-P25</f>
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1835,15 +1835,15 @@
       </c>
       <c r="R26" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A26)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A26)),IF(COUNTIF($E$2:$E$70,$A26)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A26)),IF(COUNTIF($F$2:$F$70,$A26)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A26)),IF(COUNTIF($G$2:$G$70,$A26)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A26)))</f>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="S26" s="0" t="n">
         <f aca="false">R26-O26</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="T26" s="0" t="n">
         <f aca="false">S26-P26</f>
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1876,15 +1876,15 @@
       </c>
       <c r="R27" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A27)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A27)),IF(COUNTIF($E$2:$E$70,$A27)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A27)),IF(COUNTIF($F$2:$F$70,$A27)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A27)),IF(COUNTIF($G$2:$G$70,$A27)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A27)))</f>
-        <v>40.5</v>
+        <v>38.5</v>
       </c>
       <c r="S27" s="0" t="n">
         <f aca="false">R27-O27</f>
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="T27" s="0" t="n">
         <f aca="false">S27-P27</f>
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1917,15 +1917,15 @@
       </c>
       <c r="R28" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A28)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A28)),IF(COUNTIF($E$2:$E$70,$A28)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A28)),IF(COUNTIF($F$2:$F$70,$A28)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A28)),IF(COUNTIF($G$2:$G$70,$A28)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A28)))</f>
-        <v>40.5</v>
+        <v>38.5</v>
       </c>
       <c r="S28" s="0" t="n">
         <f aca="false">R28-O28</f>
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="T28" s="0" t="n">
         <f aca="false">S28-P28</f>
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1958,15 +1958,15 @@
       </c>
       <c r="R29" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A29)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A29)),IF(COUNTIF($E$2:$E$70,$A29)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A29)),IF(COUNTIF($F$2:$F$70,$A29)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A29)),IF(COUNTIF($G$2:$G$70,$A29)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A29)))</f>
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="S29" s="0" t="n">
         <f aca="false">R29-O29</f>
-        <v>11.5</v>
+        <v>9.5</v>
       </c>
       <c r="T29" s="0" t="n">
         <f aca="false">S29-P29</f>
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1999,15 +1999,15 @@
       </c>
       <c r="R30" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A30)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A30)),IF(COUNTIF($E$2:$E$70,$A30)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A30)),IF(COUNTIF($F$2:$F$70,$A30)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A30)),IF(COUNTIF($G$2:$G$70,$A30)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A30)))</f>
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="S30" s="0" t="n">
         <f aca="false">R30-O30</f>
-        <v>11.5</v>
+        <v>9.5</v>
       </c>
       <c r="T30" s="0" t="n">
         <f aca="false">S30-P30</f>
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2043,15 +2043,15 @@
       </c>
       <c r="R31" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A31)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A31)),IF(COUNTIF($E$2:$E$70,$A31)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A31)),IF(COUNTIF($F$2:$F$70,$A31)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A31)),IF(COUNTIF($G$2:$G$70,$A31)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A31)))</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="S31" s="0" t="n">
         <f aca="false">R31-O31</f>
-        <v>40.5</v>
+        <v>38.5</v>
       </c>
       <c r="T31" s="0" t="n">
         <f aca="false">S31-P31</f>
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2084,15 +2084,15 @@
       </c>
       <c r="R32" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A32)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A32)),IF(COUNTIF($E$2:$E$70,$A32)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A32)),IF(COUNTIF($F$2:$F$70,$A32)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A32)),IF(COUNTIF($G$2:$G$70,$A32)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A32)))</f>
-        <v>53.75</v>
+        <v>51.75</v>
       </c>
       <c r="S32" s="0" t="n">
         <f aca="false">R32-O32</f>
-        <v>41.25</v>
+        <v>39.25</v>
       </c>
       <c r="T32" s="0" t="n">
         <f aca="false">S32-P32</f>
-        <v>32.75</v>
+        <v>30.75</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2125,15 +2125,15 @@
       </c>
       <c r="R33" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A33)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A33)),IF(COUNTIF($E$2:$E$70,$A33)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A33)),IF(COUNTIF($F$2:$F$70,$A33)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A33)),IF(COUNTIF($G$2:$G$70,$A33)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A33)))</f>
-        <v>35.5</v>
+        <v>33.5</v>
       </c>
       <c r="S33" s="0" t="n">
         <f aca="false">R33-O33</f>
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="T33" s="0" t="n">
         <f aca="false">S33-P33</f>
-        <v>14.5</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2175,15 +2175,15 @@
       </c>
       <c r="R34" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A34)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A34)),IF(COUNTIF($E$2:$E$70,$A34)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A34)),IF(COUNTIF($F$2:$F$70,$A34)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A34)),IF(COUNTIF($G$2:$G$70,$A34)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A34)))</f>
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="S34" s="0" t="n">
         <f aca="false">R34-O34</f>
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="T34" s="0" t="n">
         <f aca="false">S34-P34</f>
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2216,15 +2216,15 @@
       </c>
       <c r="R35" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A35)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A35)),IF(COUNTIF($E$2:$E$70,$A35)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A35)),IF(COUNTIF($F$2:$F$70,$A35)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A35)),IF(COUNTIF($G$2:$G$70,$A35)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A35)))</f>
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="S35" s="0" t="n">
         <f aca="false">R35-O35</f>
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="T35" s="0" t="n">
         <f aca="false">S35-P35</f>
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2260,15 +2260,15 @@
       </c>
       <c r="R36" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A36)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A36)),IF(COUNTIF($E$2:$E$70,$A36)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A36)),IF(COUNTIF($F$2:$F$70,$A36)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A36)),IF(COUNTIF($G$2:$G$70,$A36)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A36)))</f>
-        <v>63.75</v>
+        <v>61.75</v>
       </c>
       <c r="S36" s="0" t="n">
         <f aca="false">R36-O36</f>
-        <v>53.75</v>
+        <v>51.75</v>
       </c>
       <c r="T36" s="0" t="n">
         <f aca="false">S36-P36</f>
-        <v>32.75</v>
+        <v>30.75</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2304,15 +2304,15 @@
       </c>
       <c r="R37" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A37)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A37)),IF(COUNTIF($E$2:$E$70,$A37)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A37)),IF(COUNTIF($F$2:$F$70,$A37)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A37)),IF(COUNTIF($G$2:$G$70,$A37)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A37)))</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="S37" s="0" t="n">
         <f aca="false">R37-O37</f>
-        <v>35.5</v>
+        <v>33.5</v>
       </c>
       <c r="T37" s="0" t="n">
         <f aca="false">S37-P37</f>
-        <v>14.5</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2345,15 +2345,15 @@
       </c>
       <c r="R38" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A38)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A38)),IF(COUNTIF($E$2:$E$70,$A38)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A38)),IF(COUNTIF($F$2:$F$70,$A38)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A38)),IF(COUNTIF($G$2:$G$70,$A38)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A38)))</f>
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="S38" s="0" t="n">
         <f aca="false">R38-O38</f>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="T38" s="0" t="n">
         <f aca="false">S38-P38</f>
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2386,15 +2386,15 @@
       </c>
       <c r="R39" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A39)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A39)),IF(COUNTIF($E$2:$E$70,$A39)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A39)),IF(COUNTIF($F$2:$F$70,$A39)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A39)),IF(COUNTIF($G$2:$G$70,$A39)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A39)))</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="S39" s="0" t="n">
         <f aca="false">R39-O39</f>
-        <v>40.5</v>
+        <v>38.5</v>
       </c>
       <c r="T39" s="0" t="n">
         <f aca="false">S39-P39</f>
-        <v>34.5</v>
+        <v>32.5</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2433,15 +2433,15 @@
       </c>
       <c r="R40" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A40)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A40)),IF(COUNTIF($E$2:$E$70,$A40)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A40)),IF(COUNTIF($F$2:$F$70,$A40)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A40)),IF(COUNTIF($G$2:$G$70,$A40)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A40)))</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="S40" s="0" t="n">
         <f aca="false">R40-O40</f>
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="T40" s="0" t="n">
         <f aca="false">S40-P40</f>
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2474,15 +2474,15 @@
       </c>
       <c r="R41" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A41)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A41)),IF(COUNTIF($E$2:$E$70,$A41)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A41)),IF(COUNTIF($F$2:$F$70,$A41)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A41)),IF(COUNTIF($G$2:$G$70,$A41)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A41)))</f>
-        <v>46.5</v>
+        <v>44.5</v>
       </c>
       <c r="S41" s="0" t="n">
         <f aca="false">R41-O41</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="T41" s="0" t="n">
         <f aca="false">S41-P41</f>
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2512,15 +2512,15 @@
       </c>
       <c r="R42" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A42)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A42)),IF(COUNTIF($E$2:$E$70,$A42)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A42)),IF(COUNTIF($F$2:$F$70,$A42)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A42)),IF(COUNTIF($G$2:$G$70,$A42)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A42)))</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="S42" s="0" t="n">
         <f aca="false">R42-O42</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="T42" s="0" t="n">
         <f aca="false">S42-P42</f>
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2553,15 +2553,15 @@
       </c>
       <c r="R43" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A43)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A43)),IF(COUNTIF($E$2:$E$70,$A43)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A43)),IF(COUNTIF($F$2:$F$70,$A43)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A43)),IF(COUNTIF($G$2:$G$70,$A43)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A43)))</f>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="S43" s="0" t="n">
         <f aca="false">R43-O43</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="T43" s="0" t="n">
         <f aca="false">S43-P43</f>
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2594,15 +2594,15 @@
       </c>
       <c r="R44" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A44)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A44)),IF(COUNTIF($E$2:$E$70,$A44)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A44)),IF(COUNTIF($F$2:$F$70,$A44)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A44)),IF(COUNTIF($G$2:$G$70,$A44)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A44)))</f>
-        <v>25.5</v>
+        <v>23.5</v>
       </c>
       <c r="S44" s="0" t="n">
         <f aca="false">R44-O44</f>
-        <v>15.5</v>
+        <v>13.5</v>
       </c>
       <c r="T44" s="0" t="n">
         <f aca="false">S44-P44</f>
-        <v>15.5</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2635,15 +2635,15 @@
       </c>
       <c r="R45" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A45)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A45)),IF(COUNTIF($E$2:$E$70,$A45)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A45)),IF(COUNTIF($F$2:$F$70,$A45)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A45)),IF(COUNTIF($G$2:$G$70,$A45)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A45)))</f>
-        <v>25.5</v>
+        <v>23.5</v>
       </c>
       <c r="S45" s="0" t="n">
         <f aca="false">R45-O45</f>
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
       <c r="T45" s="0" t="n">
         <f aca="false">S45-P45</f>
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2676,15 +2676,15 @@
       </c>
       <c r="R46" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A46)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A46)),IF(COUNTIF($E$2:$E$70,$A46)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A46)),IF(COUNTIF($F$2:$F$70,$A46)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A46)),IF(COUNTIF($G$2:$G$70,$A46)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A46)))</f>
-        <v>25.5</v>
+        <v>23.5</v>
       </c>
       <c r="S46" s="0" t="n">
         <f aca="false">R46-O46</f>
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
       <c r="T46" s="0" t="n">
         <f aca="false">S46-P46</f>
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2723,15 +2723,15 @@
       </c>
       <c r="R47" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A47)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A47)),IF(COUNTIF($E$2:$E$70,$A47)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A47)),IF(COUNTIF($F$2:$F$70,$A47)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A47)),IF(COUNTIF($G$2:$G$70,$A47)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A47)))</f>
-        <v>30.5</v>
+        <v>28.5</v>
       </c>
       <c r="S47" s="0" t="n">
         <f aca="false">R47-O47</f>
-        <v>25.5</v>
+        <v>23.5</v>
       </c>
       <c r="T47" s="0" t="n">
         <f aca="false">S47-P47</f>
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2767,15 +2767,15 @@
       </c>
       <c r="R48" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A48)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A48)),IF(COUNTIF($E$2:$E$70,$A48)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A48)),IF(COUNTIF($F$2:$F$70,$A48)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A48)),IF(COUNTIF($G$2:$G$70,$A48)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A48)))</f>
-        <v>16.5</v>
+        <v>14.5</v>
       </c>
       <c r="S48" s="0" t="n">
         <f aca="false">R48-O48</f>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="T48" s="0" t="n">
         <f aca="false">S48-P48</f>
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2808,15 +2808,15 @@
       </c>
       <c r="R49" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A49)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A49)),IF(COUNTIF($E$2:$E$70,$A49)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A49)),IF(COUNTIF($F$2:$F$70,$A49)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A49)),IF(COUNTIF($G$2:$G$70,$A49)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A49)))</f>
-        <v>63.75</v>
+        <v>61.75</v>
       </c>
       <c r="S49" s="0" t="n">
         <f aca="false">R49-O49</f>
-        <v>58.75</v>
+        <v>56.75</v>
       </c>
       <c r="T49" s="0" t="n">
         <f aca="false">S49-P49</f>
-        <v>43.75</v>
+        <v>41.75</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2855,15 +2855,15 @@
       </c>
       <c r="R50" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A50)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A50)),IF(COUNTIF($E$2:$E$70,$A50)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A50)),IF(COUNTIF($F$2:$F$70,$A50)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A50)),IF(COUNTIF($G$2:$G$70,$A50)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A50)))</f>
-        <v>40.5</v>
+        <v>38.5</v>
       </c>
       <c r="S50" s="0" t="n">
         <f aca="false">R50-O50</f>
-        <v>16.5</v>
+        <v>14.5</v>
       </c>
       <c r="T50" s="0" t="n">
         <f aca="false">S50-P50</f>
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2896,15 +2896,15 @@
       </c>
       <c r="R51" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A51)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A51)),IF(COUNTIF($E$2:$E$70,$A51)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A51)),IF(COUNTIF($F$2:$F$70,$A51)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A51)),IF(COUNTIF($G$2:$G$70,$A51)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A51)))</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="S51" s="0" t="n">
         <f aca="false">R51-O51</f>
-        <v>40.5</v>
+        <v>38.5</v>
       </c>
       <c r="T51" s="0" t="n">
         <f aca="false">S51-P51</f>
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2940,15 +2940,15 @@
       </c>
       <c r="R52" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A52)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A52)),IF(COUNTIF($E$2:$E$70,$A52)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A52)),IF(COUNTIF($F$2:$F$70,$A52)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A52)),IF(COUNTIF($G$2:$G$70,$A52)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A52)))</f>
-        <v>35.5</v>
+        <v>33.5</v>
       </c>
       <c r="S52" s="0" t="n">
         <f aca="false">R52-O52</f>
-        <v>26.5</v>
+        <v>24.5</v>
       </c>
       <c r="T52" s="0" t="n">
         <f aca="false">S52-P52</f>
-        <v>11.5</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2984,15 +2984,15 @@
       </c>
       <c r="R53" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A53)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A53)),IF(COUNTIF($E$2:$E$70,$A53)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A53)),IF(COUNTIF($F$2:$F$70,$A53)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A53)),IF(COUNTIF($G$2:$G$70,$A53)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A53)))</f>
-        <v>63.75</v>
+        <v>61.75</v>
       </c>
       <c r="S53" s="0" t="n">
         <f aca="false">R53-O53</f>
-        <v>60.75</v>
+        <v>58.75</v>
       </c>
       <c r="T53" s="0" t="n">
         <f aca="false">S53-P53</f>
-        <v>45.75</v>
+        <v>43.75</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3025,15 +3025,15 @@
       </c>
       <c r="R54" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A54)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A54)),IF(COUNTIF($E$2:$E$70,$A54)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A54)),IF(COUNTIF($F$2:$F$70,$A54)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A54)),IF(COUNTIF($G$2:$G$70,$A54)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A54)))</f>
-        <v>35.5</v>
+        <v>33.5</v>
       </c>
       <c r="S54" s="0" t="n">
         <f aca="false">R54-O54</f>
-        <v>30.5</v>
+        <v>28.5</v>
       </c>
       <c r="T54" s="0" t="n">
         <f aca="false">S54-P54</f>
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3069,15 +3069,15 @@
       </c>
       <c r="R55" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A55)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A55)),IF(COUNTIF($E$2:$E$70,$A55)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A55)),IF(COUNTIF($F$2:$F$70,$A55)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A55)),IF(COUNTIF($G$2:$G$70,$A55)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A55)))</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="S55" s="0" t="n">
         <f aca="false">R55-O55</f>
-        <v>35.5</v>
+        <v>33.5</v>
       </c>
       <c r="T55" s="0" t="n">
         <f aca="false">S55-P55</f>
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3113,15 +3113,15 @@
       </c>
       <c r="R56" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A56)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A56)),IF(COUNTIF($E$2:$E$70,$A56)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A56)),IF(COUNTIF($F$2:$F$70,$A56)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A56)),IF(COUNTIF($G$2:$G$70,$A56)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A56)))</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="S56" s="0" t="n">
         <f aca="false">R56-O56</f>
-        <v>35.5</v>
+        <v>33.5</v>
       </c>
       <c r="T56" s="0" t="n">
         <f aca="false">S56-P56</f>
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3154,15 +3154,15 @@
       </c>
       <c r="R57" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A57)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A57)),IF(COUNTIF($E$2:$E$70,$A57)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A57)),IF(COUNTIF($F$2:$F$70,$A57)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A57)),IF(COUNTIF($G$2:$G$70,$A57)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A57)))</f>
-        <v>46.5</v>
+        <v>44.5</v>
       </c>
       <c r="S57" s="0" t="n">
         <f aca="false">R57-O57</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="T57" s="0" t="n">
         <f aca="false">S57-P57</f>
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3228,19 +3228,19 @@
       </c>
       <c r="P59" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D59,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E59,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F59,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G59,$A$2:$A$70,0)),0))</f>
-        <v>55.5</v>
+        <v>53.5</v>
       </c>
       <c r="Q59" s="0" t="n">
         <f aca="false">P59+O59</f>
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="R59" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A59)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A59)),IF(COUNTIF($E$2:$E$70,$A59)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A59)),IF(COUNTIF($F$2:$F$70,$A59)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A59)),IF(COUNTIF($G$2:$G$70,$A59)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A59)))</f>
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="S59" s="0" t="n">
         <f aca="false">R59-O59</f>
-        <v>55.5</v>
+        <v>53.5</v>
       </c>
       <c r="T59" s="0" t="n">
         <f aca="false">S59-P59</f>
@@ -3274,15 +3274,15 @@
       </c>
       <c r="R60" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A60)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A60)),IF(COUNTIF($E$2:$E$70,$A60)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A60)),IF(COUNTIF($F$2:$F$70,$A60)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A60)),IF(COUNTIF($G$2:$G$70,$A60)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A60)))</f>
-        <v>29.5</v>
+        <v>27.5</v>
       </c>
       <c r="S60" s="0" t="n">
         <f aca="false">R60-O60</f>
-        <v>29.5</v>
+        <v>27.5</v>
       </c>
       <c r="T60" s="0" t="n">
         <f aca="false">S60-P60</f>
-        <v>29.5</v>
+        <v>27.5</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3318,15 +3318,15 @@
       </c>
       <c r="R61" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A61)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A61)),IF(COUNTIF($E$2:$E$70,$A61)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A61)),IF(COUNTIF($F$2:$F$70,$A61)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A61)),IF(COUNTIF($G$2:$G$70,$A61)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A61)))</f>
-        <v>50.5</v>
+        <v>48.5</v>
       </c>
       <c r="S61" s="0" t="n">
         <f aca="false">R61-O61</f>
-        <v>29.5</v>
+        <v>27.5</v>
       </c>
       <c r="T61" s="0" t="n">
         <f aca="false">S61-P61</f>
-        <v>29.5</v>
+        <v>27.5</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3354,19 +3354,19 @@
       </c>
       <c r="P62" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D62,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E62,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F62,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G62,$A$2:$A$70,0)),0))</f>
-        <v>50.5</v>
+        <v>48.5</v>
       </c>
       <c r="Q62" s="0" t="n">
         <f aca="false">P62+O62</f>
-        <v>55.5</v>
+        <v>53.5</v>
       </c>
       <c r="R62" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A62)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A62)),IF(COUNTIF($E$2:$E$70,$A62)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A62)),IF(COUNTIF($F$2:$F$70,$A62)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A62)),IF(COUNTIF($G$2:$G$70,$A62)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A62)))</f>
-        <v>55.5</v>
+        <v>53.5</v>
       </c>
       <c r="S62" s="0" t="n">
         <f aca="false">R62-O62</f>
-        <v>50.5</v>
+        <v>48.5</v>
       </c>
       <c r="T62" s="0" t="n">
         <f aca="false">S62-P62</f>
@@ -3398,19 +3398,19 @@
       </c>
       <c r="P63" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D63,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E63,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F63,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G63,$A$2:$A$70,0)),0))</f>
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="Q63" s="0" t="n">
         <f aca="false">P63+O63</f>
-        <v>63.75</v>
+        <v>61.75</v>
       </c>
       <c r="R63" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A63)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A63)),IF(COUNTIF($E$2:$E$70,$A63)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A63)),IF(COUNTIF($F$2:$F$70,$A63)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A63)),IF(COUNTIF($G$2:$G$70,$A63)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A63)))</f>
-        <v>63.75</v>
+        <v>61.75</v>
       </c>
       <c r="S63" s="0" t="n">
         <f aca="false">R63-O63</f>
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="T63" s="0" t="n">
         <f aca="false">S63-P63</f>
@@ -3436,19 +3436,19 @@
       </c>
       <c r="P64" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D64,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E64,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F64,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G64,$A$2:$A$70,0)),0))</f>
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="Q64" s="0" t="n">
         <f aca="false">P64+O64</f>
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="R64" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A64)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A64)),IF(COUNTIF($E$2:$E$70,$A64)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A64)),IF(COUNTIF($F$2:$F$70,$A64)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A64)),IF(COUNTIF($G$2:$G$70,$A64)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A64)))</f>
-        <v>63.75</v>
+        <v>61.75</v>
       </c>
       <c r="S64" s="0" t="n">
         <f aca="false">R64-O64</f>
-        <v>63.75</v>
+        <v>61.75</v>
       </c>
       <c r="T64" s="0" t="n">
         <f aca="false">S64-P64</f>
@@ -3477,19 +3477,19 @@
       </c>
       <c r="P65" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D65,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E65,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F65,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G65,$A$2:$A$70,0)),0))</f>
-        <v>46.5</v>
+        <v>44.5</v>
       </c>
       <c r="Q65" s="0" t="n">
         <f aca="false">P65+O65</f>
-        <v>50.5</v>
+        <v>48.5</v>
       </c>
       <c r="R65" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A65)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A65)),IF(COUNTIF($E$2:$E$70,$A65)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A65)),IF(COUNTIF($F$2:$F$70,$A65)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A65)),IF(COUNTIF($G$2:$G$70,$A65)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A65)))</f>
-        <v>50.5</v>
+        <v>48.5</v>
       </c>
       <c r="S65" s="0" t="n">
         <f aca="false">R65-O65</f>
-        <v>46.5</v>
+        <v>44.5</v>
       </c>
       <c r="T65" s="0" t="n">
         <f aca="false">S65-P65</f>
@@ -3529,15 +3529,15 @@
       </c>
       <c r="R66" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A66)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A66)),IF(COUNTIF($E$2:$E$70,$A66)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A66)),IF(COUNTIF($F$2:$F$70,$A66)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A66)),IF(COUNTIF($G$2:$G$70,$A66)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A66)))</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="S66" s="0" t="n">
         <f aca="false">R66-O66</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="T66" s="0" t="n">
         <f aca="false">S66-P66</f>
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3576,15 +3576,15 @@
       </c>
       <c r="R67" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A67)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A67)),IF(COUNTIF($E$2:$E$70,$A67)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A67)),IF(COUNTIF($F$2:$F$70,$A67)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A67)),IF(COUNTIF($G$2:$G$70,$A67)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A67)))</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="S67" s="0" t="n">
         <f aca="false">R67-O67</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="T67" s="0" t="n">
         <f aca="false">S67-P67</f>
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3606,19 +3606,19 @@
       </c>
       <c r="P68" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D68,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E68,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F68,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G68,$A$2:$A$70,0)),0))</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="Q68" s="0" t="n">
         <f aca="false">P68+O68</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="R68" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A68)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A68)),IF(COUNTIF($E$2:$E$70,$A68)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A68)),IF(COUNTIF($F$2:$F$70,$A68)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A68)),IF(COUNTIF($G$2:$G$70,$A68)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A68)))</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="S68" s="0" t="n">
         <f aca="false">R68-O68</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="T68" s="0" t="n">
         <f aca="false">S68-P68</f>
@@ -3655,15 +3655,15 @@
       </c>
       <c r="R69" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A69)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A69)),IF(COUNTIF($E$2:$E$70,$A69)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A69)),IF(COUNTIF($F$2:$F$70,$A69)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A69)),IF(COUNTIF($G$2:$G$70,$A69)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A69)))</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="S69" s="0" t="n">
         <f aca="false">R69-O69</f>
-        <v>45.5</v>
+        <v>43.5</v>
       </c>
       <c r="T69" s="0" t="n">
         <f aca="false">S69-P69</f>
-        <v>4.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3694,19 +3694,19 @@
       </c>
       <c r="P70" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D70,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E70,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F70,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G70,$A$2:$A$70,0)),0))</f>
-        <v>46.5</v>
+        <v>44.5</v>
       </c>
       <c r="Q70" s="0" t="n">
         <f aca="false">P70+O70</f>
-        <v>46.5</v>
+        <v>44.5</v>
       </c>
       <c r="R70" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A70)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A70)),IF(COUNTIF($E$2:$E$70,$A70)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A70)),IF(COUNTIF($F$2:$F$70,$A70)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A70)),IF(COUNTIF($G$2:$G$70,$A70)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A70)))</f>
-        <v>46.5</v>
+        <v>44.5</v>
       </c>
       <c r="S70" s="0" t="n">
         <f aca="false">R70-O70</f>
-        <v>46.5</v>
+        <v>44.5</v>
       </c>
       <c r="T70" s="0" t="n">
         <f aca="false">S70-P70</f>
@@ -3735,19 +3735,19 @@
       </c>
       <c r="P71" s="0" t="n">
         <f aca="false">MAX(IFERROR(INDEX($Q$2:$Q$70,MATCH(D71,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(E71,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(F71,$A$2:$A$70,0)),0),IFERROR(INDEX($Q$2:$Q$70,MATCH(G71,$A$2:$A$70,0)),0))</f>
-        <v>55.5</v>
+        <v>53.5</v>
       </c>
       <c r="Q71" s="0" t="n">
         <f aca="false">P71+O71</f>
-        <v>55.5</v>
+        <v>53.5</v>
       </c>
       <c r="R71" s="0" t="n">
         <f aca="false">MIN(IF(COUNTIF($D$2:$D$70,$A71)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$D$2:$D$70,$A71)),IF(COUNTIF($E$2:$E$70,$A71)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$E$2:$E$70,$A71)),IF(COUNTIF($F$2:$F$70,$A71)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$F$2:$F$70,$A71)),IF(COUNTIF($G$2:$G$70,$A71)=0,$O$73,_xlfn.MINIFS($S$2:$S$70,$G$2:$G$70,$A71)))</f>
-        <v>63.75</v>
+        <v>61.75</v>
       </c>
       <c r="S71" s="0" t="n">
         <f aca="false">R71-O71</f>
-        <v>63.75</v>
+        <v>61.75</v>
       </c>
       <c r="T71" s="0" t="n">
         <f aca="false">S71-P71</f>
@@ -3760,7 +3760,7 @@
       </c>
       <c r="O73" s="0" t="n">
         <f aca="false">MAX(Q2:Q70)</f>
-        <v>63.75</v>
+        <v>61.75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>